<commit_message>
Fixed vocabulary loading and audio loading
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\icass\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B12DB0-6CFB-42E0-BF04-677B7CED62FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EABCD64F-D494-4C32-BDCD-E9F0B9FF64C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="2655" windowWidth="38640" windowHeight="21120" xr2:uid="{C22C0A01-2830-40B6-936A-3C340C04517B}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>KEY</t>
   </si>
   <si>
-    <t xml:space="preserve">ALBUMS </t>
-  </si>
-  <si>
     <t>Albums</t>
   </si>
   <si>
@@ -1119,6 +1116,9 @@
   </si>
   <si>
     <t>Actualizar</t>
+  </si>
+  <si>
+    <t>ALBUMS</t>
   </si>
 </sst>
 </file>
@@ -1537,2187 +1537,2187 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B3" t="s">
         <v>306</v>
       </c>
-      <c r="B3" t="s">
-        <v>307</v>
-      </c>
       <c r="C3" t="str">
-        <f>_xlfn.TRANSLATE(B3,$B$2,$C$2)</f>
+        <f t="shared" ref="C3:C22" si="0">_xlfn.TRANSLATE(B3,$B$2,$C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" t="s">
         <v>308</v>
       </c>
-      <c r="B4" t="s">
-        <v>309</v>
-      </c>
       <c r="C4" t="str">
-        <f>_xlfn.TRANSLATE(B4,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista al final de la cola</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5" t="s">
         <v>237</v>
       </c>
-      <c r="B5" t="s">
-        <v>238</v>
-      </c>
       <c r="C5" t="str">
-        <f>_xlfn.TRANSLATE(B5,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista a la cola</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B6" t="s">
         <v>225</v>
       </c>
-      <c r="B6" t="s">
-        <v>226</v>
-      </c>
       <c r="C6" t="str">
-        <f>_xlfn.TRANSLATE(B6,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B7" t="s">
         <v>239</v>
       </c>
-      <c r="B7" t="s">
-        <v>240</v>
-      </c>
       <c r="C7" t="str">
-        <f>_xlfn.TRANSLATE(B7,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la cola</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" t="s">
         <v>243</v>
       </c>
-      <c r="B8" t="s">
-        <v>244</v>
-      </c>
       <c r="C8" t="str">
-        <f>_xlfn.TRANSLATE(B8,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la biblioteca</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" t="str">
-        <f>_xlfn.TRANSLATE(B9,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a los que me gusta</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" t="str">
-        <f>_xlfn.TRANSLATE(B10,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la cola</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" t="str">
-        <f>_xlfn.TRANSLATE(B11,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Álbum</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>360</v>
+      </c>
+      <c r="B12" t="s">
         <v>5</v>
       </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
       <c r="C12" t="str">
-        <f>_xlfn.TRANSLATE(B12,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Álbumes</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" t="s">
         <v>169</v>
       </c>
-      <c r="B13" t="s">
-        <v>170</v>
-      </c>
       <c r="C13" t="str">
-        <f>_xlfn.TRANSLATE(B13,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Álbumes y sencillos</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>297</v>
+      </c>
+      <c r="B14" t="s">
         <v>298</v>
       </c>
-      <c r="B14" t="s">
-        <v>299</v>
-      </c>
       <c r="C14" t="str">
-        <f>_xlfn.TRANSLATE(B14,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Todos</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>260</v>
+      </c>
+      <c r="B15" t="s">
         <v>261</v>
       </c>
-      <c r="B15" t="s">
-        <v>262</v>
-      </c>
       <c r="C15" t="str">
-        <f>_xlfn.TRANSLATE(B15,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Abril</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>188</v>
+      </c>
+      <c r="B16" t="s">
         <v>189</v>
       </c>
-      <c r="B16" t="s">
-        <v>190</v>
-      </c>
       <c r="C16" t="str">
-        <f>_xlfn.TRANSLATE(B16,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Artista</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" t="s">
         <v>111</v>
       </c>
-      <c r="B17" t="s">
-        <v>112</v>
-      </c>
       <c r="C17" t="str">
-        <f>_xlfn.TRANSLATE(B17,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Artistas</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>268</v>
+      </c>
+      <c r="B18" t="s">
         <v>269</v>
       </c>
-      <c r="B18" t="s">
-        <v>270</v>
-      </c>
       <c r="C18" t="str">
-        <f>_xlfn.TRANSLATE(B18,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Agosto</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" t="s">
         <v>253</v>
       </c>
-      <c r="B19" t="s">
-        <v>254</v>
-      </c>
       <c r="C19" t="str">
-        <f>_xlfn.TRANSLATE(B19,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Minutos medios por canción</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B20" t="s">
         <v>209</v>
       </c>
-      <c r="B20" t="s">
-        <v>210</v>
-      </c>
       <c r="C20" t="str">
-        <f>_xlfn.TRANSLATE(B20,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>por</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>292</v>
+      </c>
+      <c r="B21" t="s">
         <v>293</v>
       </c>
-      <c r="B21" t="s">
-        <v>294</v>
-      </c>
       <c r="C21" t="str">
-        <f>_xlfn.TRANSLATE(B21,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Cancelar</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" t="s">
         <v>153</v>
       </c>
-      <c r="B22" t="s">
-        <v>154</v>
-      </c>
       <c r="C22" t="str">
-        <f>_xlfn.TRANSLATE(B22,$B$2,$C$2)</f>
+        <f t="shared" si="0"/>
         <v>Cambiar contraseña</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>23</v>
-      </c>
-      <c r="C23" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C24" t="str">
-        <f>_xlfn.TRANSLATE(B24,$B$2,$C$2)</f>
+        <f t="shared" ref="C24:C30" si="1">_xlfn.TRANSLATE(B24,$B$2,$C$2)</f>
         <v>Topo comunitario</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>248</v>
+      </c>
+      <c r="B25" t="s">
         <v>249</v>
       </c>
-      <c r="B25" t="s">
-        <v>250</v>
-      </c>
       <c r="C25" t="str">
-        <f>_xlfn.TRANSLATE(B25,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>URL de la lista de copiar</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26" t="str">
-        <f>_xlfn.TRANSLATE(B26,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>Copiar la URL de la canción</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>294</v>
+      </c>
+      <c r="B27" t="s">
         <v>295</v>
       </c>
-      <c r="B27" t="s">
-        <v>296</v>
-      </c>
       <c r="C27" t="str">
-        <f>_xlfn.TRANSLATE(B27,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>Crear</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>303</v>
+      </c>
+      <c r="B28" t="s">
         <v>304</v>
       </c>
-      <c r="B28" t="s">
-        <v>305</v>
-      </c>
       <c r="C28" t="str">
-        <f>_xlfn.TRANSLATE(B28,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>Crear...</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>190</v>
+      </c>
+      <c r="B29" t="s">
         <v>191</v>
       </c>
-      <c r="B29" t="s">
-        <v>192</v>
-      </c>
       <c r="C29" t="str">
-        <f>_xlfn.TRANSLATE(B29,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>Fecha añadida</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>276</v>
+      </c>
+      <c r="B30" t="s">
         <v>277</v>
       </c>
-      <c r="B30" t="s">
-        <v>278</v>
-      </c>
       <c r="C30" t="str">
-        <f>_xlfn.TRANSLATE(B30,$B$2,$C$2)</f>
+        <f t="shared" si="1"/>
         <v>Diciembre</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B31" t="s">
+        <v>356</v>
+      </c>
+      <c r="C31" t="s">
         <v>357</v>
-      </c>
-      <c r="C31" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" t="s">
         <v>211</v>
       </c>
-      <c r="B32" t="s">
-        <v>212</v>
-      </c>
       <c r="C32" t="str">
-        <f>_xlfn.TRANSLATE(B32,$B$2,$C$2)</f>
+        <f t="shared" ref="C32:C63" si="2">_xlfn.TRANSLATE(B32,$B$2,$C$2)</f>
         <v>Disco</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" t="s">
         <v>151</v>
       </c>
-      <c r="B33" t="s">
-        <v>152</v>
-      </c>
       <c r="C33" t="str">
-        <f>_xlfn.TRANSLATE(B33,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Nombre de Muestra</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>200</v>
+      </c>
+      <c r="B34" t="s">
         <v>201</v>
       </c>
-      <c r="B34" t="s">
-        <v>202</v>
-      </c>
       <c r="C34" t="str">
-        <f>_xlfn.TRANSLATE(B34,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargar</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>158</v>
+      </c>
+      <c r="B35" t="s">
         <v>159</v>
       </c>
-      <c r="B35" t="s">
-        <v>160</v>
-      </c>
       <c r="C35" t="str">
-        <f>_xlfn.TRANSLATE(B35,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descarga la app para escuchar offline</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B36" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C36" t="str">
-        <f>_xlfn.TRANSLATE(B36,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>309</v>
+      </c>
+      <c r="B37" t="s">
         <v>310</v>
       </c>
-      <c r="B37" t="s">
-        <v>311</v>
-      </c>
       <c r="C37" t="str">
-        <f>_xlfn.TRANSLATE(B37,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Lista de descargas al dispositivo</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C38" t="str">
-        <f>_xlfn.TRANSLATE(B38,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargar medios al dispositivo</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C39" t="str">
-        <f>_xlfn.TRANSLATE(B39,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargar mp</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>228</v>
+      </c>
+      <c r="B40" t="s">
         <v>229</v>
       </c>
-      <c r="B40" t="s">
-        <v>230</v>
-      </c>
       <c r="C40" t="str">
-        <f>_xlfn.TRANSLATE(B40,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargar canción al dispositivo</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>311</v>
+      </c>
+      <c r="B41" t="s">
         <v>312</v>
       </c>
-      <c r="B41" t="s">
-        <v>313</v>
-      </c>
       <c r="C41" t="str">
-        <f>_xlfn.TRANSLATE(B41,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargar ZIP</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" t="s">
         <v>85</v>
       </c>
-      <c r="B42" t="s">
-        <v>86</v>
-      </c>
       <c r="C42" t="str">
-        <f>_xlfn.TRANSLATE(B42,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargas</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>192</v>
+      </c>
+      <c r="B43" t="s">
         <v>193</v>
       </c>
-      <c r="B43" t="s">
-        <v>194</v>
-      </c>
       <c r="C43" t="str">
-        <f>_xlfn.TRANSLATE(B43,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Duración</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>283</v>
+      </c>
+      <c r="B44" t="s">
         <v>284</v>
       </c>
-      <c r="B44" t="s">
-        <v>285</v>
-      </c>
       <c r="C44" t="str">
-        <f>_xlfn.TRANSLATE(B44,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Energía</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C45" t="str">
-        <f>_xlfn.TRANSLATE(B45,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B46" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C46" t="str">
-        <f>_xlfn.TRANSLATE(B46,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Error</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" t="str">
-        <f>_xlfn.TRANSLATE(B47,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C48" t="str">
-        <f>_xlfn.TRANSLATE(B48,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C49" t="str">
-        <f>_xlfn.TRANSLATE(B49,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>92</v>
+      </c>
+      <c r="B50" t="s">
         <v>93</v>
       </c>
-      <c r="B50" t="s">
-        <v>94</v>
-      </c>
       <c r="C50" t="str">
-        <f>_xlfn.TRANSLATE(B50,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Álbumes destacados</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" t="s">
         <v>95</v>
       </c>
-      <c r="B51" t="s">
-        <v>96</v>
-      </c>
       <c r="C51" t="str">
-        <f>_xlfn.TRANSLATE(B51,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Listas destacadas</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>256</v>
+      </c>
+      <c r="B52" t="s">
         <v>257</v>
       </c>
-      <c r="B52" t="s">
-        <v>258</v>
-      </c>
       <c r="C52" t="str">
-        <f>_xlfn.TRANSLATE(B52,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Febrero</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>285</v>
+      </c>
+      <c r="B53" t="s">
         <v>286</v>
       </c>
-      <c r="B53" t="s">
-        <v>287</v>
-      </c>
       <c r="C53" t="str">
-        <f>_xlfn.TRANSLATE(B53,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Enfoque</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C54" t="str">
-        <f>_xlfn.TRANSLATE(B54,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Amigos</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>130</v>
+      </c>
+      <c r="B55" t="s">
         <v>131</v>
       </c>
-      <c r="B55" t="s">
-        <v>132</v>
-      </c>
       <c r="C55" t="str">
-        <f>_xlfn.TRANSLATE(B55,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Lista de amigos</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>118</v>
+      </c>
+      <c r="B56" t="s">
         <v>119</v>
       </c>
-      <c r="B56" t="s">
-        <v>120</v>
-      </c>
       <c r="C56" t="str">
-        <f>_xlfn.TRANSLATE(B56,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B57" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C57" t="str">
-        <f>_xlfn.TRANSLATE(B57,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Estadísticas de Friends</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C58" t="str">
-        <f>_xlfn.TRANSLATE(B58,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>General</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C59" t="str">
-        <f>_xlfn.TRANSLATE(B59,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Estadísticas generales</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>250</v>
+      </c>
+      <c r="B60" t="s">
         <v>251</v>
       </c>
-      <c r="B60" t="s">
-        <v>252</v>
-      </c>
       <c r="C60" t="str">
-        <f>_xlfn.TRANSLATE(B60,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Obtén información</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B61" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C61" t="str">
-        <f>_xlfn.TRANSLATE(B61,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Ir al álbum</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B62" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C62" t="str">
-        <f>_xlfn.TRANSLATE(B62,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Ir a artista</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B63" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C63" t="str">
-        <f>_xlfn.TRANSLATE(B63,$B$2,$C$2)</f>
+        <f t="shared" si="2"/>
         <v>Joyas ocultas que olvidaste</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" t="s">
         <v>71</v>
       </c>
-      <c r="B64" t="s">
-        <v>72</v>
-      </c>
       <c r="C64" t="str">
-        <f>_xlfn.TRANSLATE(B64,$B$2,$C$2)</f>
+        <f t="shared" ref="C64:C95" si="3">_xlfn.TRANSLATE(B64,$B$2,$C$2)</f>
         <v>Inicio</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>254</v>
+      </c>
+      <c r="B65" t="s">
         <v>255</v>
       </c>
-      <c r="B65" t="s">
-        <v>256</v>
-      </c>
       <c r="C65" t="str">
-        <f>_xlfn.TRANSLATE(B65,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Enero</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>266</v>
+      </c>
+      <c r="B66" t="s">
         <v>267</v>
       </c>
-      <c r="B66" t="s">
-        <v>268</v>
-      </c>
       <c r="C66" t="str">
-        <f>_xlfn.TRANSLATE(B66,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Julio</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>264</v>
+      </c>
+      <c r="B67" t="s">
         <v>265</v>
       </c>
-      <c r="B67" t="s">
-        <v>266</v>
-      </c>
       <c r="C67" t="str">
-        <f>_xlfn.TRANSLATE(B67,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Junio</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>204</v>
+      </c>
+      <c r="B68" t="s">
         <v>205</v>
       </c>
-      <c r="B68" t="s">
-        <v>206</v>
-      </c>
       <c r="C68" t="str">
-        <f>_xlfn.TRANSLATE(B68,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Idioma</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B69" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C69" t="str">
-        <f>_xlfn.TRANSLATE(B69,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Últimas descargas</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>116</v>
+      </c>
+      <c r="B70" t="s">
         <v>117</v>
       </c>
-      <c r="B70" t="s">
-        <v>118</v>
-      </c>
       <c r="C70" t="str">
-        <f>_xlfn.TRANSLATE(B70,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Nivel</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>72</v>
+      </c>
+      <c r="B71" t="s">
         <v>73</v>
       </c>
-      <c r="B71" t="s">
-        <v>74</v>
-      </c>
       <c r="C71" t="str">
-        <f>_xlfn.TRANSLATE(B71,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Biblioteca</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>176</v>
+      </c>
+      <c r="B72" t="s">
         <v>177</v>
       </c>
-      <c r="B72" t="s">
-        <v>178</v>
-      </c>
       <c r="C72" t="str">
-        <f>_xlfn.TRANSLATE(B72,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Como</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>98</v>
+      </c>
+      <c r="B73" t="s">
         <v>99</v>
       </c>
-      <c r="B73" t="s">
-        <v>100</v>
-      </c>
       <c r="C73" t="str">
-        <f>_xlfn.TRANSLATE(B73,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Canciones que me gustaban</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>174</v>
+      </c>
+      <c r="B74" t="s">
         <v>175</v>
       </c>
-      <c r="B74" t="s">
-        <v>176</v>
-      </c>
       <c r="C74" t="str">
-        <f>_xlfn.TRANSLATE(B74,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Cerrar sesión</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>178</v>
+      </c>
+      <c r="B75" t="s">
         <v>179</v>
       </c>
-      <c r="B75" t="s">
-        <v>180</v>
-      </c>
       <c r="C75" t="str">
-        <f>_xlfn.TRANSLATE(B75,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Letra</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>258</v>
+      </c>
+      <c r="B76" t="s">
         <v>259</v>
       </c>
-      <c r="B76" t="s">
-        <v>260</v>
-      </c>
       <c r="C76" t="str">
-        <f>_xlfn.TRANSLATE(B76,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Marzo</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>262</v>
+      </c>
+      <c r="B77" t="s">
         <v>263</v>
       </c>
-      <c r="B77" t="s">
-        <v>264</v>
-      </c>
       <c r="C77" t="str">
-        <f>_xlfn.TRANSLATE(B77,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Mayo</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>184</v>
+      </c>
+      <c r="B78" t="s">
         <v>185</v>
       </c>
-      <c r="B78" t="s">
-        <v>186</v>
-      </c>
       <c r="C78" t="str">
-        <f>_xlfn.TRANSLATE(B78,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Actas</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>214</v>
+      </c>
+      <c r="B79" t="s">
         <v>215</v>
       </c>
-      <c r="B79" t="s">
-        <v>216</v>
-      </c>
       <c r="C79" t="str">
-        <f>_xlfn.TRANSLATE(B79,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Minutos escuchados</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>222</v>
+      </c>
+      <c r="B80" t="s">
         <v>223</v>
       </c>
-      <c r="B80" t="s">
-        <v>224</v>
-      </c>
       <c r="C80" t="str">
-        <f>_xlfn.TRANSLATE(B80,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Minutos escuchados por día</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B81" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C81" t="str">
-        <f>_xlfn.TRANSLATE(B81,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Canciones para cuando te sientas</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>182</v>
+      </c>
+      <c r="B82" t="s">
         <v>183</v>
       </c>
-      <c r="B82" t="s">
-        <v>184</v>
-      </c>
       <c r="C82" t="str">
-        <f>_xlfn.TRANSLATE(B82,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Más opciones</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>162</v>
+      </c>
+      <c r="B83" t="s">
         <v>163</v>
       </c>
-      <c r="B83" t="s">
-        <v>164</v>
-      </c>
       <c r="C83" t="str">
-        <f>_xlfn.TRANSLATE(B83,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Más canciones de</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>100</v>
+      </c>
+      <c r="B84" t="s">
         <v>101</v>
       </c>
-      <c r="B84" t="s">
-        <v>102</v>
-      </c>
       <c r="C84" t="str">
-        <f>_xlfn.TRANSLATE(B84,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Más escuchado</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>216</v>
+      </c>
+      <c r="B85" t="s">
         <v>217</v>
       </c>
-      <c r="B85" t="s">
-        <v>218</v>
-      </c>
       <c r="C85" t="str">
-        <f>_xlfn.TRANSLATE(B85,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbumes más escuchados</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>218</v>
+      </c>
+      <c r="B86" t="s">
         <v>219</v>
       </c>
-      <c r="B86" t="s">
-        <v>220</v>
-      </c>
       <c r="C86" t="str">
-        <f>_xlfn.TRANSLATE(B86,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Artistas más escuchados</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>220</v>
+      </c>
+      <c r="B87" t="s">
         <v>221</v>
       </c>
-      <c r="B87" t="s">
-        <v>222</v>
-      </c>
       <c r="C87" t="str">
-        <f>_xlfn.TRANSLATE(B87,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Canciones más escuchadas</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>186</v>
+      </c>
+      <c r="B88" t="s">
         <v>187</v>
       </c>
-      <c r="B88" t="s">
-        <v>188</v>
-      </c>
       <c r="C88" t="str">
-        <f>_xlfn.TRANSLATE(B88,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Nombre</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>154</v>
+      </c>
+      <c r="B89" t="s">
         <v>155</v>
       </c>
-      <c r="B89" t="s">
-        <v>156</v>
-      </c>
       <c r="C89" t="str">
-        <f>_xlfn.TRANSLATE(B89,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Introducir nueva contraseña</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B90" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C90" t="str">
-        <f>_xlfn.TRANSLATE(B90,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Nueva lista de reproducción</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B91" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C91" t="str">
-        <f>_xlfn.TRANSLATE(B91,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>315</v>
+      </c>
+      <c r="B92" t="s">
         <v>316</v>
       </c>
-      <c r="B92" t="s">
-        <v>317</v>
-      </c>
       <c r="C92" t="str">
-        <f>_xlfn.TRANSLATE(B92,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>146</v>
+      </c>
+      <c r="B93" t="s">
         <v>147</v>
       </c>
-      <c r="B93" t="s">
-        <v>148</v>
-      </c>
       <c r="C93" t="str">
-        <f>_xlfn.TRANSLATE(B93,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>No hay datos registrados.</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>180</v>
+      </c>
+      <c r="B94" t="s">
         <v>181</v>
       </c>
-      <c r="B94" t="s">
-        <v>182</v>
-      </c>
       <c r="C94" t="str">
-        <f>_xlfn.TRANSLATE(B94,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Letra no disponible</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>323</v>
+      </c>
+      <c r="B95" t="s">
         <v>324</v>
       </c>
-      <c r="B95" t="s">
-        <v>325</v>
-      </c>
       <c r="C95" t="str">
-        <f>_xlfn.TRANSLATE(B95,$B$2,$C$2)</f>
+        <f t="shared" si="3"/>
         <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>313</v>
+      </c>
+      <c r="B96" t="s">
         <v>314</v>
       </c>
-      <c r="B96" t="s">
-        <v>315</v>
-      </c>
       <c r="C96" t="str">
-        <f>_xlfn.TRANSLATE(B96,$B$2,$C$2)</f>
+        <f t="shared" ref="C96:C127" si="4">_xlfn.TRANSLATE(B96,$B$2,$C$2)</f>
         <v>Sin resultados</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B97" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C97" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>317</v>
+      </c>
+      <c r="B98" t="s">
         <v>318</v>
       </c>
-      <c r="B98" t="s">
-        <v>319</v>
-      </c>
       <c r="C98" t="str">
-        <f>_xlfn.TRANSLATE(B98,$B$2,$C$2)</f>
+        <f t="shared" ref="C98:C129" si="5">_xlfn.TRANSLATE(B98,$B$2,$C$2)</f>
         <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B99" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C99" t="str">
-        <f>_xlfn.TRANSLATE(B99,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Sin estado</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>321</v>
+      </c>
+      <c r="B100" t="s">
         <v>322</v>
       </c>
-      <c r="B100" t="s">
-        <v>323</v>
-      </c>
       <c r="C100" t="str">
-        <f>_xlfn.TRANSLATE(B100,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>319</v>
+      </c>
+      <c r="B101" t="s">
         <v>320</v>
       </c>
-      <c r="B101" t="s">
-        <v>321</v>
-      </c>
       <c r="C101" t="str">
-        <f>_xlfn.TRANSLATE(B101,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>274</v>
+      </c>
+      <c r="B102" t="s">
         <v>275</v>
       </c>
-      <c r="B102" t="s">
-        <v>276</v>
-      </c>
       <c r="C102" t="str">
-        <f>_xlfn.TRANSLATE(B102,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Noviembre</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>272</v>
+      </c>
+      <c r="B103" t="s">
         <v>273</v>
       </c>
-      <c r="B103" t="s">
-        <v>274</v>
-      </c>
       <c r="C103" t="str">
-        <f>_xlfn.TRANSLATE(B103,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Octubre</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>232</v>
+      </c>
+      <c r="B104" t="s">
         <v>233</v>
       </c>
-      <c r="B104" t="s">
-        <v>234</v>
-      </c>
       <c r="C104" t="str">
-        <f>_xlfn.TRANSLATE(B104,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Lista abierta</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>234</v>
+      </c>
+      <c r="B105" t="s">
         <v>235</v>
       </c>
-      <c r="B105" t="s">
-        <v>236</v>
-      </c>
       <c r="C105" t="str">
-        <f>_xlfn.TRANSLATE(B105,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Canción abierta</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
+        <v>287</v>
+      </c>
+      <c r="B106" t="s">
         <v>288</v>
       </c>
-      <c r="B106" t="s">
-        <v>289</v>
-      </c>
       <c r="C106" t="str">
-        <f>_xlfn.TRANSLATE(B106,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Partido</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B107" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C107" t="str">
-        <f>_xlfn.TRANSLATE(B107,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Canción de pausa</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
+        <v>128</v>
+      </c>
+      <c r="B108" t="s">
         <v>129</v>
       </c>
-      <c r="B108" t="s">
-        <v>130</v>
-      </c>
       <c r="C108" t="str">
-        <f>_xlfn.TRANSLATE(B108,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Solicitudes pendientes</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>246</v>
+      </c>
+      <c r="B109" t="s">
         <v>247</v>
       </c>
-      <c r="B109" t="s">
-        <v>248</v>
-      </c>
       <c r="C109" t="str">
-        <f>_xlfn.TRANSLATE(B109,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Pin</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>82</v>
+      </c>
+      <c r="B110" t="s">
         <v>83</v>
       </c>
-      <c r="B110" t="s">
-        <v>84</v>
-      </c>
       <c r="C110" t="str">
-        <f>_xlfn.TRANSLATE(B110,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Listas fijadas</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>196</v>
+      </c>
+      <c r="B111" t="s">
         <v>197</v>
       </c>
-      <c r="B111" t="s">
-        <v>198</v>
-      </c>
       <c r="C111" t="str">
-        <f>_xlfn.TRANSLATE(B111,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Título del álbum</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>198</v>
+      </c>
+      <c r="B112" t="s">
         <v>199</v>
       </c>
-      <c r="B112" t="s">
-        <v>200</v>
-      </c>
       <c r="C112" t="str">
-        <f>_xlfn.TRANSLATE(B112,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Nombre artístico</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
+        <v>301</v>
+      </c>
+      <c r="B113" t="s">
         <v>302</v>
       </c>
-      <c r="B113" t="s">
-        <v>303</v>
-      </c>
       <c r="C113" t="str">
-        <f>_xlfn.TRANSLATE(B113,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Mi lista de reproducción perfecta</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>194</v>
+      </c>
+      <c r="B114" t="s">
         <v>195</v>
       </c>
-      <c r="B114" t="s">
-        <v>196</v>
-      </c>
       <c r="C114" t="str">
-        <f>_xlfn.TRANSLATE(B114,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Título de la canción</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>230</v>
+      </c>
+      <c r="B115" t="s">
         <v>231</v>
       </c>
-      <c r="B115" t="s">
-        <v>232</v>
-      </c>
       <c r="C115" t="str">
-        <f>_xlfn.TRANSLATE(B115,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Lista de reproducción</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B116" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C116" t="str">
-        <f>_xlfn.TRANSLATE(B116,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Reproducir medios</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B117" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C117" t="str">
-        <f>_xlfn.TRANSLATE(B117,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Juego a continuación</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B118" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C118" t="str">
-        <f>_xlfn.TRANSLATE(B118,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Tocar canción</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B119" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C119" t="str">
-        <f>_xlfn.TRANSLATE(B119,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Listas de reproducción</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B120" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C120" t="str">
-        <f>_xlfn.TRANSLATE(B120,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Selecciones rápidas</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>80</v>
+      </c>
+      <c r="B121" t="s">
         <v>81</v>
       </c>
-      <c r="B121" t="s">
-        <v>82</v>
-      </c>
       <c r="C121" t="str">
-        <f>_xlfn.TRANSLATE(B121,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Radio</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
+        <v>136</v>
+      </c>
+      <c r="B122" t="s">
         <v>137</v>
       </c>
-      <c r="B122" t="s">
-        <v>138</v>
-      </c>
       <c r="C122" t="str">
-        <f>_xlfn.TRANSLATE(B122,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>No se han encontrado estaciones</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
+        <v>138</v>
+      </c>
+      <c r="B123" t="s">
         <v>139</v>
       </c>
-      <c r="B123" t="s">
-        <v>140</v>
-      </c>
       <c r="C123" t="str">
-        <f>_xlfn.TRANSLATE(B123,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>140</v>
+      </c>
+      <c r="B124" t="s">
         <v>141</v>
       </c>
-      <c r="B124" t="s">
-        <v>142</v>
-      </c>
       <c r="C124" t="str">
-        <f>_xlfn.TRANSLATE(B124,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Busca emisoras, géneros, países...</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>112</v>
+      </c>
+      <c r="B125" t="s">
         <v>113</v>
       </c>
-      <c r="B125" t="s">
-        <v>114</v>
-      </c>
       <c r="C125" t="str">
-        <f>_xlfn.TRANSLATE(B125,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Emisoras de radio</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
+        <v>102</v>
+      </c>
+      <c r="B126" t="s">
         <v>103</v>
       </c>
-      <c r="B126" t="s">
-        <v>104</v>
-      </c>
       <c r="C126" t="str">
-        <f>_xlfn.TRANSLATE(B126,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Mezcla reciente</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
+        <v>88</v>
+      </c>
+      <c r="B127" t="s">
         <v>89</v>
       </c>
-      <c r="B127" t="s">
-        <v>90</v>
-      </c>
       <c r="C127" t="str">
-        <f>_xlfn.TRANSLATE(B127,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Jugado recientemente</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B128" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C128" t="str">
-        <f>_xlfn.TRANSLATE(B128,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Jugado recientemente</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B129" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C129" t="str">
-        <f>_xlfn.TRANSLATE(B129,$B$2,$C$2)</f>
+        <f t="shared" si="5"/>
         <v>Registro</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B130" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C130" t="str">
-        <f>_xlfn.TRANSLATE(B130,$B$2,$C$2)</f>
+        <f t="shared" ref="C130:C161" si="6">_xlfn.TRANSLATE(B130,$B$2,$C$2)</f>
         <v>Registrado</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B131" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C131" t="str">
-        <f>_xlfn.TRANSLATE(B131,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Registrando...</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
+        <v>170</v>
+      </c>
+      <c r="B132" t="s">
         <v>171</v>
       </c>
-      <c r="B132" t="s">
-        <v>172</v>
-      </c>
       <c r="C132" t="str">
-        <f>_xlfn.TRANSLATE(B132,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Artistas relacionados</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
+        <v>281</v>
+      </c>
+      <c r="B133" t="s">
         <v>282</v>
       </c>
-      <c r="B133" t="s">
-        <v>283</v>
-      </c>
       <c r="C133" t="str">
-        <f>_xlfn.TRANSLATE(B133,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Relajado</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
+        <v>240</v>
+      </c>
+      <c r="B134" t="s">
         <v>241</v>
       </c>
-      <c r="B134" t="s">
-        <v>242</v>
-      </c>
       <c r="C134" t="str">
-        <f>_xlfn.TRANSLATE(B134,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Eliminar de la biblioteca</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B135" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C135" t="str">
-        <f>_xlfn.TRANSLATE(B135,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Quitar de me gusta</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
+        <v>226</v>
+      </c>
+      <c r="B136" t="s">
         <v>227</v>
       </c>
-      <c r="B136" t="s">
-        <v>228</v>
-      </c>
       <c r="C136" t="str">
-        <f>_xlfn.TRANSLATE(B136,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Eliminar de la lista de reproducción</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
+        <v>43</v>
+      </c>
+      <c r="B137" t="s">
         <v>44</v>
       </c>
-      <c r="B137" t="s">
-        <v>45</v>
-      </c>
       <c r="C137" t="str">
-        <f>_xlfn.TRANSLATE(B137,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Eliminar de la cola</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
+        <v>156</v>
+      </c>
+      <c r="B138" t="s">
         <v>157</v>
       </c>
-      <c r="B138" t="s">
-        <v>158</v>
-      </c>
       <c r="C138" t="str">
-        <f>_xlfn.TRANSLATE(B138,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Repetir nueva contraseña</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
+        <v>74</v>
+      </c>
+      <c r="B139" t="s">
         <v>75</v>
       </c>
-      <c r="B139" t="s">
-        <v>76</v>
-      </c>
       <c r="C139" t="str">
-        <f>_xlfn.TRANSLATE(B139,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Búsqueda</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
+        <v>86</v>
+      </c>
+      <c r="B140" t="s">
         <v>87</v>
       </c>
-      <c r="B140" t="s">
-        <v>88</v>
-      </c>
       <c r="C140" t="str">
-        <f>_xlfn.TRANSLATE(B140,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Busca artistas, canciones, álbumes...</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
+        <v>106</v>
+      </c>
+      <c r="B141" t="s">
         <v>107</v>
       </c>
-      <c r="B141" t="s">
-        <v>108</v>
-      </c>
       <c r="C141" t="str">
-        <f>_xlfn.TRANSLATE(B141,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Parece que el silencio también es música...</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
+        <v>108</v>
+      </c>
+      <c r="B142" t="s">
         <v>109</v>
       </c>
-      <c r="B142" t="s">
-        <v>110</v>
-      </c>
       <c r="C142" t="str">
-        <f>_xlfn.TRANSLATE(B142,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
+        <v>104</v>
+      </c>
+      <c r="B143" t="s">
         <v>105</v>
       </c>
-      <c r="B143" t="s">
-        <v>106</v>
-      </c>
       <c r="C143" t="str">
-        <f>_xlfn.TRANSLATE(B143,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Buscar en la biblioteca</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>126</v>
+      </c>
+      <c r="B144" t="s">
         <v>127</v>
       </c>
-      <c r="B144" t="s">
-        <v>128</v>
-      </c>
       <c r="C144" t="str">
-        <f>_xlfn.TRANSLATE(B144,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Usuarios de búsqueda</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
+        <v>134</v>
+      </c>
+      <c r="B145" t="s">
         <v>135</v>
       </c>
-      <c r="B145" t="s">
-        <v>136</v>
-      </c>
       <c r="C145" t="str">
-        <f>_xlfn.TRANSLATE(B145,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Enviar canción actual</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
+        <v>270</v>
+      </c>
+      <c r="B146" t="s">
         <v>271</v>
       </c>
-      <c r="B146" t="s">
-        <v>272</v>
-      </c>
       <c r="C146" t="str">
-        <f>_xlfn.TRANSLATE(B146,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Septiembre</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
+        <v>76</v>
+      </c>
+      <c r="B147" t="s">
         <v>77</v>
       </c>
-      <c r="B147" t="s">
-        <v>78</v>
-      </c>
       <c r="C147" t="str">
-        <f>_xlfn.TRANSLATE(B147,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Escenarios</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B148" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C148" t="str">
-        <f>_xlfn.TRANSLATE(B148,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Compartir canción</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
+        <v>120</v>
+      </c>
+      <c r="B149" t="s">
         <v>121</v>
       </c>
-      <c r="B149" t="s">
-        <v>122</v>
-      </c>
       <c r="C149" t="str">
-        <f>_xlfn.TRANSLATE(B149,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones compartidas para ti</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
+        <v>122</v>
+      </c>
+      <c r="B150" t="s">
         <v>123</v>
       </c>
-      <c r="B150" t="s">
-        <v>124</v>
-      </c>
       <c r="C150" t="str">
-        <f>_xlfn.TRANSLATE(B150,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Compartido desde</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
+        <v>144</v>
+      </c>
+      <c r="B151" t="s">
         <v>145</v>
       </c>
-      <c r="B151" t="s">
-        <v>146</v>
-      </c>
       <c r="C151" t="str">
-        <f>_xlfn.TRANSLATE(B151,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Mostrando datos de</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B152" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C152" t="str">
-        <f>_xlfn.TRANSLATE(B152,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canción</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B153" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C153" t="str">
-        <f>_xlfn.TRANSLATE(B153,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B154" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C154" t="str">
-        <f>_xlfn.TRANSLATE(B154,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones Solo para ti</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>160</v>
+      </c>
+      <c r="B155" t="s">
         <v>161</v>
       </c>
-      <c r="B155" t="s">
-        <v>162</v>
-      </c>
       <c r="C155" t="str">
-        <f>_xlfn.TRANSLATE(B155,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones de</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>212</v>
+      </c>
+      <c r="B156" t="s">
         <v>213</v>
       </c>
-      <c r="B156" t="s">
-        <v>214</v>
-      </c>
       <c r="C156" t="str">
-        <f>_xlfn.TRANSLATE(B156,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones escuchadas</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>142</v>
+      </c>
+      <c r="B157" t="s">
         <v>143</v>
       </c>
-      <c r="B157" t="s">
-        <v>144</v>
-      </c>
       <c r="C157" t="str">
-        <f>_xlfn.TRANSLATE(B157,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Estadísticas</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>78</v>
+      </c>
+      <c r="B158" t="s">
         <v>79</v>
       </c>
-      <c r="B158" t="s">
-        <v>80</v>
-      </c>
       <c r="C158" t="str">
-        <f>_xlfn.TRANSLATE(B158,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Estadísticas</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B159" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C159" t="str">
-        <f>_xlfn.TRANSLATE(B159,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>¡Para</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
+        <v>172</v>
+      </c>
+      <c r="B160" t="s">
         <v>173</v>
       </c>
-      <c r="B160" t="s">
-        <v>174</v>
-      </c>
       <c r="C160" t="str">
-        <f>_xlfn.TRANSLATE(B160,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>a</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
+        <v>166</v>
+      </c>
+      <c r="B161" t="s">
         <v>167</v>
       </c>
-      <c r="B161" t="s">
-        <v>168</v>
-      </c>
       <c r="C161" t="str">
-        <f>_xlfn.TRANSLATE(B161,$B$2,$C$2)</f>
+        <f t="shared" si="6"/>
         <v>Álbumes destacados</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>164</v>
+      </c>
+      <c r="B162" t="s">
         <v>165</v>
       </c>
-      <c r="B162" t="s">
-        <v>166</v>
-      </c>
       <c r="C162" t="str">
-        <f>_xlfn.TRANSLATE(B162,$B$2,$C$2)</f>
+        <f t="shared" ref="C162:C193" si="7">_xlfn.TRANSLATE(B162,$B$2,$C$2)</f>
         <v>Canciones principales</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
+        <v>244</v>
+      </c>
+      <c r="B163" t="s">
         <v>245</v>
       </c>
-      <c r="B163" t="s">
-        <v>246</v>
-      </c>
       <c r="C163" t="str">
-        <f>_xlfn.TRANSLATE(B163,$B$2,$C$2)</f>
+        <f t="shared" si="7"/>
         <v>Desclavar</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
+        <v>346</v>
+      </c>
+      <c r="B164" t="s">
         <v>347</v>
       </c>
-      <c r="B164" t="s">
-        <v>348</v>
-      </c>
       <c r="C164" t="str">
-        <f>_xlfn.TRANSLATE(B164,$B$2,$C$2)</f>
+        <f t="shared" si="7"/>
         <v>Desregistrar</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B165" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C165" t="str">
-        <f>_xlfn.TRANSLATE(B165,$B$2,$C$2)</f>
+        <f t="shared" si="7"/>
         <v>No registrado</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B166" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C166" t="str">
-        <f>_xlfn.TRANSLATE(B166,$B$2,$C$2)</f>
+        <f t="shared" si="7"/>
         <v>Dejar de registrarse...</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
+        <v>202</v>
+      </c>
+      <c r="B167" t="s">
         <v>203</v>
       </c>
-      <c r="B167" t="s">
-        <v>204</v>
-      </c>
       <c r="C167" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B168" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C168" t="str">
-        <f>_xlfn.TRANSLATE(B168,$B$2,$C$2)</f>
+        <f t="shared" ref="C168:C190" si="8">_xlfn.TRANSLATE(B168,$B$2,$C$2)</f>
         <v>Actualizando...</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
+        <v>325</v>
+      </c>
+      <c r="B169" t="s">
         <v>326</v>
       </c>
-      <c r="B169" t="s">
-        <v>327</v>
-      </c>
       <c r="C169" t="str">
-        <f>_xlfn.TRANSLATE(B169,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Subida</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B170" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C170" t="str">
-        <f>_xlfn.TRANSLATE(B170,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Usuario</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
+        <v>148</v>
+      </c>
+      <c r="B171" t="s">
         <v>149</v>
       </c>
-      <c r="B171" t="s">
-        <v>150</v>
-      </c>
       <c r="C171" t="str">
-        <f>_xlfn.TRANSLATE(B171,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Configuración de usuario</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B172" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C172" t="str">
-        <f>_xlfn.TRANSLATE(B172,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Estadísticas de usuario</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>124</v>
+      </c>
+      <c r="B173" t="s">
         <v>125</v>
       </c>
-      <c r="B173" t="s">
-        <v>126</v>
-      </c>
       <c r="C173" t="str">
-        <f>_xlfn.TRANSLATE(B173,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Usuarios y amigos</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>132</v>
+      </c>
+      <c r="B174" t="s">
         <v>133</v>
       </c>
-      <c r="B174" t="s">
-        <v>134</v>
-      </c>
       <c r="C174" t="str">
-        <f>_xlfn.TRANSLATE(B174,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Lista de usuarios</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>331</v>
+      </c>
+      <c r="B175" t="s">
         <v>332</v>
       </c>
-      <c r="B175" t="s">
-        <v>333</v>
-      </c>
       <c r="C175" t="str">
-        <f>_xlfn.TRANSLATE(B175,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Vídeos</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>90</v>
+      </c>
+      <c r="B176" t="s">
         <v>91</v>
       </c>
-      <c r="B176" t="s">
-        <v>92</v>
-      </c>
       <c r="C176" t="str">
-        <f>_xlfn.TRANSLATE(B176,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>También puede que te interese</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
+        <v>289</v>
+      </c>
+      <c r="B177" t="s">
         <v>290</v>
       </c>
-      <c r="B177" t="s">
-        <v>291</v>
-      </c>
       <c r="C177" t="str">
-        <f>_xlfn.TRANSLATE(B177,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Tu</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
+        <v>96</v>
+      </c>
+      <c r="B178" t="s">
         <v>97</v>
       </c>
-      <c r="B178" t="s">
-        <v>98</v>
-      </c>
       <c r="C178" t="str">
-        <f>_xlfn.TRANSLATE(B178,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Tus álbumes y listas de reproducción</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
+        <v>114</v>
+      </c>
+      <c r="B179" t="s">
         <v>115</v>
       </c>
-      <c r="B179" t="s">
-        <v>116</v>
-      </c>
       <c r="C179" t="str">
-        <f>_xlfn.TRANSLATE(B179,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v>Vídeos de YouTube</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C180" t="str">
-        <f>_xlfn.TRANSLATE(B180,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C181" t="str">
-        <f>_xlfn.TRANSLATE(B181,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C182" t="str">
-        <f>_xlfn.TRANSLATE(B182,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C183" t="str">
-        <f>_xlfn.TRANSLATE(B183,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C184" t="str">
-        <f>_xlfn.TRANSLATE(B184,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C185" t="str">
-        <f>_xlfn.TRANSLATE(B185,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C186" t="str">
-        <f>_xlfn.TRANSLATE(B186,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C187" t="str">
-        <f>_xlfn.TRANSLATE(B187,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C188" t="str">
-        <f>_xlfn.TRANSLATE(B188,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C189" t="str">
-        <f>_xlfn.TRANSLATE(B189,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C190" t="str">
-        <f>_xlfn.TRANSLATE(B190,$B$2,$C$2)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(downloads): add completed column to track download progress
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\icass\rockit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicorebo18\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EABCD64F-D494-4C32-BDCD-E9F0B9FF64C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2A4016-6E70-4A46-87C2-5E7E28F5BDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="2655" windowWidth="38640" windowHeight="21120" xr2:uid="{C22C0A01-2830-40B6-936A-3C340C04517B}"/>
+    <workbookView xWindow="-28920" yWindow="780" windowWidth="29040" windowHeight="15720" xr2:uid="{C22C0A01-2830-40B6-936A-3C340C04517B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="363">
   <si>
     <t>Español</t>
   </si>
@@ -1119,6 +1119,12 @@
   </si>
   <si>
     <t>ALBUMS</t>
+  </si>
+  <si>
+    <t>SAVING</t>
+  </si>
+  <si>
+    <t>Saving…</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1197,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1508,7 +1514,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EAF2166-6392-4C77-B9D6-7F4DF776B7D5}">
   <dimension ref="A1:C190"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
     <col min="2" max="2" width="44.7109375" customWidth="1"/>
@@ -1543,7 +1549,7 @@
         <v>306</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C22" si="0">_xlfn.TRANSLATE(B3,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B3,$B$2,$C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
     </row>
@@ -1555,7 +1561,7 @@
         <v>308</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B4,$B$2,$C$2)</f>
         <v>Añadir lista al final de la cola</v>
       </c>
     </row>
@@ -1567,7 +1573,7 @@
         <v>237</v>
       </c>
       <c r="C5" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B5,$B$2,$C$2)</f>
         <v>Añadir lista a la cola</v>
       </c>
     </row>
@@ -1579,7 +1585,7 @@
         <v>225</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B6,$B$2,$C$2)</f>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
     </row>
@@ -1591,7 +1597,7 @@
         <v>239</v>
       </c>
       <c r="C7" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B7,$B$2,$C$2)</f>
         <v>Añadir canción a la cola</v>
       </c>
     </row>
@@ -1603,7 +1609,7 @@
         <v>243</v>
       </c>
       <c r="C8" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B8,$B$2,$C$2)</f>
         <v>Añadir a la biblioteca</v>
       </c>
     </row>
@@ -1615,7 +1621,7 @@
         <v>41</v>
       </c>
       <c r="C9" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B9,$B$2,$C$2)</f>
         <v>Añadir a los que me gusta</v>
       </c>
     </row>
@@ -1627,7 +1633,7 @@
         <v>42</v>
       </c>
       <c r="C10" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B10,$B$2,$C$2)</f>
         <v>Añadir a la cola</v>
       </c>
     </row>
@@ -1639,7 +1645,7 @@
         <v>11</v>
       </c>
       <c r="C11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B11,$B$2,$C$2)</f>
         <v>Álbum</v>
       </c>
     </row>
@@ -1651,7 +1657,7 @@
         <v>5</v>
       </c>
       <c r="C12" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B12,$B$2,$C$2)</f>
         <v>Álbumes</v>
       </c>
     </row>
@@ -1663,7 +1669,7 @@
         <v>169</v>
       </c>
       <c r="C13" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B13,$B$2,$C$2)</f>
         <v>Álbumes y sencillos</v>
       </c>
     </row>
@@ -1675,7 +1681,7 @@
         <v>298</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B14,$B$2,$C$2)</f>
         <v>Todos</v>
       </c>
     </row>
@@ -1687,7 +1693,7 @@
         <v>261</v>
       </c>
       <c r="C15" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B15,$B$2,$C$2)</f>
         <v>Abril</v>
       </c>
     </row>
@@ -1699,7 +1705,7 @@
         <v>189</v>
       </c>
       <c r="C16" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B16,$B$2,$C$2)</f>
         <v>Artista</v>
       </c>
     </row>
@@ -1711,7 +1717,7 @@
         <v>111</v>
       </c>
       <c r="C17" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B17,$B$2,$C$2)</f>
         <v>Artistas</v>
       </c>
     </row>
@@ -1723,7 +1729,7 @@
         <v>269</v>
       </c>
       <c r="C18" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B18,$B$2,$C$2)</f>
         <v>Agosto</v>
       </c>
     </row>
@@ -1735,7 +1741,7 @@
         <v>253</v>
       </c>
       <c r="C19" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B19,$B$2,$C$2)</f>
         <v>Minutos medios por canción</v>
       </c>
     </row>
@@ -1747,7 +1753,7 @@
         <v>209</v>
       </c>
       <c r="C20" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B20,$B$2,$C$2)</f>
         <v>por</v>
       </c>
     </row>
@@ -1759,7 +1765,7 @@
         <v>293</v>
       </c>
       <c r="C21" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B21,$B$2,$C$2)</f>
         <v>Cancelar</v>
       </c>
     </row>
@@ -1771,7 +1777,7 @@
         <v>153</v>
       </c>
       <c r="C22" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE(B22,$B$2,$C$2)</f>
         <v>Cambiar contraseña</v>
       </c>
     </row>
@@ -1794,7 +1800,7 @@
         <v>55</v>
       </c>
       <c r="C24" t="str">
-        <f t="shared" ref="C24:C30" si="1">_xlfn.TRANSLATE(B24,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B24,$B$2,$C$2)</f>
         <v>Topo comunitario</v>
       </c>
     </row>
@@ -1806,7 +1812,7 @@
         <v>249</v>
       </c>
       <c r="C25" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B25,$B$2,$C$2)</f>
         <v>URL de la lista de copiar</v>
       </c>
     </row>
@@ -1818,7 +1824,7 @@
         <v>45</v>
       </c>
       <c r="C26" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B26,$B$2,$C$2)</f>
         <v>Copiar la URL de la canción</v>
       </c>
     </row>
@@ -1830,7 +1836,7 @@
         <v>295</v>
       </c>
       <c r="C27" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B27,$B$2,$C$2)</f>
         <v>Crear</v>
       </c>
     </row>
@@ -1842,7 +1848,7 @@
         <v>304</v>
       </c>
       <c r="C28" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B28,$B$2,$C$2)</f>
         <v>Crear...</v>
       </c>
     </row>
@@ -1854,7 +1860,7 @@
         <v>191</v>
       </c>
       <c r="C29" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B29,$B$2,$C$2)</f>
         <v>Fecha añadida</v>
       </c>
     </row>
@@ -1866,7 +1872,7 @@
         <v>277</v>
       </c>
       <c r="C30" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE(B30,$B$2,$C$2)</f>
         <v>Diciembre</v>
       </c>
     </row>
@@ -1889,7 +1895,7 @@
         <v>211</v>
       </c>
       <c r="C32" t="str">
-        <f t="shared" ref="C32:C63" si="2">_xlfn.TRANSLATE(B32,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B32,$B$2,$C$2)</f>
         <v>Disco</v>
       </c>
     </row>
@@ -1901,7 +1907,7 @@
         <v>151</v>
       </c>
       <c r="C33" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B33,$B$2,$C$2)</f>
         <v>Nombre de Muestra</v>
       </c>
     </row>
@@ -1913,7 +1919,7 @@
         <v>201</v>
       </c>
       <c r="C34" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B34,$B$2,$C$2)</f>
         <v>Descargar</v>
       </c>
     </row>
@@ -1925,7 +1931,7 @@
         <v>159</v>
       </c>
       <c r="C35" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B35,$B$2,$C$2)</f>
         <v>Descarga la app para escuchar offline</v>
       </c>
     </row>
@@ -1937,7 +1943,7 @@
         <v>207</v>
       </c>
       <c r="C36" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B36,$B$2,$C$2)</f>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
     </row>
@@ -1949,7 +1955,7 @@
         <v>310</v>
       </c>
       <c r="C37" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B37,$B$2,$C$2)</f>
         <v>Lista de descargas al dispositivo</v>
       </c>
     </row>
@@ -1961,7 +1967,7 @@
         <v>19</v>
       </c>
       <c r="C38" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B38,$B$2,$C$2)</f>
         <v>Descargar medios al dispositivo</v>
       </c>
     </row>
@@ -1973,7 +1979,7 @@
         <v>46</v>
       </c>
       <c r="C39" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B39,$B$2,$C$2)</f>
         <v>Descargar mp</v>
       </c>
     </row>
@@ -1985,7 +1991,7 @@
         <v>229</v>
       </c>
       <c r="C40" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B40,$B$2,$C$2)</f>
         <v>Descargar canción al dispositivo</v>
       </c>
     </row>
@@ -1997,7 +2003,7 @@
         <v>312</v>
       </c>
       <c r="C41" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B41,$B$2,$C$2)</f>
         <v>Descargar ZIP</v>
       </c>
     </row>
@@ -2009,7 +2015,7 @@
         <v>85</v>
       </c>
       <c r="C42" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B42,$B$2,$C$2)</f>
         <v>Descargas</v>
       </c>
     </row>
@@ -2021,7 +2027,7 @@
         <v>193</v>
       </c>
       <c r="C43" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B43,$B$2,$C$2)</f>
         <v>Duración</v>
       </c>
     </row>
@@ -2033,7 +2039,7 @@
         <v>284</v>
       </c>
       <c r="C44" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B44,$B$2,$C$2)</f>
         <v>Energía</v>
       </c>
     </row>
@@ -2045,7 +2051,7 @@
         <v>66</v>
       </c>
       <c r="C45" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B45,$B$2,$C$2)</f>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
     </row>
@@ -2057,7 +2063,7 @@
         <v>336</v>
       </c>
       <c r="C46" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B46,$B$2,$C$2)</f>
         <v>Error</v>
       </c>
     </row>
@@ -2069,7 +2075,7 @@
         <v>68</v>
       </c>
       <c r="C47" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B47,$B$2,$C$2)</f>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
     </row>
@@ -2081,7 +2087,7 @@
         <v>68</v>
       </c>
       <c r="C48" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B48,$B$2,$C$2)</f>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
     </row>
@@ -2093,7 +2099,7 @@
         <v>66</v>
       </c>
       <c r="C49" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B49,$B$2,$C$2)</f>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
     </row>
@@ -2105,7 +2111,7 @@
         <v>93</v>
       </c>
       <c r="C50" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B50,$B$2,$C$2)</f>
         <v>Álbumes destacados</v>
       </c>
     </row>
@@ -2117,7 +2123,7 @@
         <v>95</v>
       </c>
       <c r="C51" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B51,$B$2,$C$2)</f>
         <v>Listas destacadas</v>
       </c>
     </row>
@@ -2129,7 +2135,7 @@
         <v>257</v>
       </c>
       <c r="C52" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B52,$B$2,$C$2)</f>
         <v>Febrero</v>
       </c>
     </row>
@@ -2141,7 +2147,7 @@
         <v>286</v>
       </c>
       <c r="C53" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B53,$B$2,$C$2)</f>
         <v>Enfoque</v>
       </c>
     </row>
@@ -2153,7 +2159,7 @@
         <v>62</v>
       </c>
       <c r="C54" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B54,$B$2,$C$2)</f>
         <v>Amigos</v>
       </c>
     </row>
@@ -2165,7 +2171,7 @@
         <v>131</v>
       </c>
       <c r="C55" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B55,$B$2,$C$2)</f>
         <v>Lista de amigos</v>
       </c>
     </row>
@@ -2177,7 +2183,7 @@
         <v>119</v>
       </c>
       <c r="C56" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B56,$B$2,$C$2)</f>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
     </row>
@@ -2189,7 +2195,7 @@
         <v>65</v>
       </c>
       <c r="C57" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B57,$B$2,$C$2)</f>
         <v>Estadísticas de Friends</v>
       </c>
     </row>
@@ -2201,7 +2207,7 @@
         <v>61</v>
       </c>
       <c r="C58" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B58,$B$2,$C$2)</f>
         <v>General</v>
       </c>
     </row>
@@ -2213,7 +2219,7 @@
         <v>64</v>
       </c>
       <c r="C59" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B59,$B$2,$C$2)</f>
         <v>Estadísticas generales</v>
       </c>
     </row>
@@ -2225,7 +2231,7 @@
         <v>251</v>
       </c>
       <c r="C60" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B60,$B$2,$C$2)</f>
         <v>Obtén información</v>
       </c>
     </row>
@@ -2237,7 +2243,7 @@
         <v>48</v>
       </c>
       <c r="C61" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B61,$B$2,$C$2)</f>
         <v>Ir al álbum</v>
       </c>
     </row>
@@ -2249,7 +2255,7 @@
         <v>47</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B62,$B$2,$C$2)</f>
         <v>Ir a artista</v>
       </c>
     </row>
@@ -2261,7 +2267,7 @@
         <v>279</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE(B63,$B$2,$C$2)</f>
         <v>Joyas ocultas que olvidaste</v>
       </c>
     </row>
@@ -2273,7 +2279,7 @@
         <v>71</v>
       </c>
       <c r="C64" t="str">
-        <f t="shared" ref="C64:C95" si="3">_xlfn.TRANSLATE(B64,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B64,$B$2,$C$2)</f>
         <v>Inicio</v>
       </c>
     </row>
@@ -2285,7 +2291,7 @@
         <v>255</v>
       </c>
       <c r="C65" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B65,$B$2,$C$2)</f>
         <v>Enero</v>
       </c>
     </row>
@@ -2297,7 +2303,7 @@
         <v>267</v>
       </c>
       <c r="C66" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B66,$B$2,$C$2)</f>
         <v>Julio</v>
       </c>
     </row>
@@ -2309,7 +2315,7 @@
         <v>265</v>
       </c>
       <c r="C67" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B67,$B$2,$C$2)</f>
         <v>Junio</v>
       </c>
     </row>
@@ -2321,7 +2327,7 @@
         <v>205</v>
       </c>
       <c r="C68" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B68,$B$2,$C$2)</f>
         <v>Idioma</v>
       </c>
     </row>
@@ -2333,7 +2339,7 @@
         <v>206</v>
       </c>
       <c r="C69" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B69,$B$2,$C$2)</f>
         <v>Últimas descargas</v>
       </c>
     </row>
@@ -2345,7 +2351,7 @@
         <v>117</v>
       </c>
       <c r="C70" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B70,$B$2,$C$2)</f>
         <v>Nivel</v>
       </c>
     </row>
@@ -2357,7 +2363,7 @@
         <v>73</v>
       </c>
       <c r="C71" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B71,$B$2,$C$2)</f>
         <v>Biblioteca</v>
       </c>
     </row>
@@ -2369,7 +2375,7 @@
         <v>177</v>
       </c>
       <c r="C72" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B72,$B$2,$C$2)</f>
         <v>Como</v>
       </c>
     </row>
@@ -2381,7 +2387,7 @@
         <v>99</v>
       </c>
       <c r="C73" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B73,$B$2,$C$2)</f>
         <v>Canciones que me gustaban</v>
       </c>
     </row>
@@ -2393,7 +2399,7 @@
         <v>175</v>
       </c>
       <c r="C74" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B74,$B$2,$C$2)</f>
         <v>Cerrar sesión</v>
       </c>
     </row>
@@ -2405,7 +2411,7 @@
         <v>179</v>
       </c>
       <c r="C75" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B75,$B$2,$C$2)</f>
         <v>Letra</v>
       </c>
     </row>
@@ -2417,7 +2423,7 @@
         <v>259</v>
       </c>
       <c r="C76" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B76,$B$2,$C$2)</f>
         <v>Marzo</v>
       </c>
     </row>
@@ -2429,7 +2435,7 @@
         <v>263</v>
       </c>
       <c r="C77" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B77,$B$2,$C$2)</f>
         <v>Mayo</v>
       </c>
     </row>
@@ -2441,7 +2447,7 @@
         <v>185</v>
       </c>
       <c r="C78" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B78,$B$2,$C$2)</f>
         <v>Actas</v>
       </c>
     </row>
@@ -2453,7 +2459,7 @@
         <v>215</v>
       </c>
       <c r="C79" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B79,$B$2,$C$2)</f>
         <v>Minutos escuchados</v>
       </c>
     </row>
@@ -2465,7 +2471,7 @@
         <v>223</v>
       </c>
       <c r="C80" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B80,$B$2,$C$2)</f>
         <v>Minutos escuchados por día</v>
       </c>
     </row>
@@ -2477,7 +2483,7 @@
         <v>280</v>
       </c>
       <c r="C81" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B81,$B$2,$C$2)</f>
         <v>Canciones para cuando te sientas</v>
       </c>
     </row>
@@ -2489,7 +2495,7 @@
         <v>183</v>
       </c>
       <c r="C82" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B82,$B$2,$C$2)</f>
         <v>Más opciones</v>
       </c>
     </row>
@@ -2501,7 +2507,7 @@
         <v>163</v>
       </c>
       <c r="C83" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B83,$B$2,$C$2)</f>
         <v>Más canciones de</v>
       </c>
     </row>
@@ -2513,7 +2519,7 @@
         <v>101</v>
       </c>
       <c r="C84" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B84,$B$2,$C$2)</f>
         <v>Más escuchado</v>
       </c>
     </row>
@@ -2525,7 +2531,7 @@
         <v>217</v>
       </c>
       <c r="C85" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B85,$B$2,$C$2)</f>
         <v>Álbumes más escuchados</v>
       </c>
     </row>
@@ -2537,7 +2543,7 @@
         <v>219</v>
       </c>
       <c r="C86" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B86,$B$2,$C$2)</f>
         <v>Artistas más escuchados</v>
       </c>
     </row>
@@ -2549,7 +2555,7 @@
         <v>221</v>
       </c>
       <c r="C87" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B87,$B$2,$C$2)</f>
         <v>Canciones más escuchadas</v>
       </c>
     </row>
@@ -2561,7 +2567,7 @@
         <v>187</v>
       </c>
       <c r="C88" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B88,$B$2,$C$2)</f>
         <v>Nombre</v>
       </c>
     </row>
@@ -2573,7 +2579,7 @@
         <v>155</v>
       </c>
       <c r="C89" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B89,$B$2,$C$2)</f>
         <v>Introducir nueva contraseña</v>
       </c>
     </row>
@@ -2585,7 +2591,7 @@
         <v>296</v>
       </c>
       <c r="C90" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B90,$B$2,$C$2)</f>
         <v>Nueva lista de reproducción</v>
       </c>
     </row>
@@ -2597,7 +2603,7 @@
         <v>291</v>
       </c>
       <c r="C91" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B91,$B$2,$C$2)</f>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
     </row>
@@ -2609,7 +2615,7 @@
         <v>316</v>
       </c>
       <c r="C92" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B92,$B$2,$C$2)</f>
         <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
     </row>
@@ -2621,7 +2627,7 @@
         <v>147</v>
       </c>
       <c r="C93" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B93,$B$2,$C$2)</f>
         <v>No hay datos registrados.</v>
       </c>
     </row>
@@ -2633,7 +2639,7 @@
         <v>181</v>
       </c>
       <c r="C94" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B94,$B$2,$C$2)</f>
         <v>Letra no disponible</v>
       </c>
     </row>
@@ -2645,7 +2651,7 @@
         <v>324</v>
       </c>
       <c r="C95" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE(B95,$B$2,$C$2)</f>
         <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
     </row>
@@ -2657,7 +2663,7 @@
         <v>314</v>
       </c>
       <c r="C96" t="str">
-        <f t="shared" ref="C96:C127" si="4">_xlfn.TRANSLATE(B96,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B96,$B$2,$C$2)</f>
         <v>Sin resultados</v>
       </c>
     </row>
@@ -2680,7 +2686,7 @@
         <v>318</v>
       </c>
       <c r="C98" t="str">
-        <f t="shared" ref="C98:C129" si="5">_xlfn.TRANSLATE(B98,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B98,$B$2,$C$2)</f>
         <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
     </row>
@@ -2692,7 +2698,7 @@
         <v>354</v>
       </c>
       <c r="C99" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B99,$B$2,$C$2)</f>
         <v>Sin estado</v>
       </c>
     </row>
@@ -2704,7 +2710,7 @@
         <v>322</v>
       </c>
       <c r="C100" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B100,$B$2,$C$2)</f>
         <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
     </row>
@@ -2716,7 +2722,7 @@
         <v>320</v>
       </c>
       <c r="C101" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B101,$B$2,$C$2)</f>
         <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
     </row>
@@ -2728,7 +2734,7 @@
         <v>275</v>
       </c>
       <c r="C102" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B102,$B$2,$C$2)</f>
         <v>Noviembre</v>
       </c>
     </row>
@@ -2740,7 +2746,7 @@
         <v>273</v>
       </c>
       <c r="C103" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B103,$B$2,$C$2)</f>
         <v>Octubre</v>
       </c>
     </row>
@@ -2752,7 +2758,7 @@
         <v>233</v>
       </c>
       <c r="C104" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B104,$B$2,$C$2)</f>
         <v>Lista abierta</v>
       </c>
     </row>
@@ -2764,7 +2770,7 @@
         <v>235</v>
       </c>
       <c r="C105" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B105,$B$2,$C$2)</f>
         <v>Canción abierta</v>
       </c>
     </row>
@@ -2776,7 +2782,7 @@
         <v>288</v>
       </c>
       <c r="C106" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B106,$B$2,$C$2)</f>
         <v>Partido</v>
       </c>
     </row>
@@ -2788,7 +2794,7 @@
         <v>36</v>
       </c>
       <c r="C107" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B107,$B$2,$C$2)</f>
         <v>Canción de pausa</v>
       </c>
     </row>
@@ -2800,7 +2806,7 @@
         <v>129</v>
       </c>
       <c r="C108" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B108,$B$2,$C$2)</f>
         <v>Solicitudes pendientes</v>
       </c>
     </row>
@@ -2812,7 +2818,7 @@
         <v>247</v>
       </c>
       <c r="C109" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B109,$B$2,$C$2)</f>
         <v>Pin</v>
       </c>
     </row>
@@ -2824,7 +2830,7 @@
         <v>83</v>
       </c>
       <c r="C110" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B110,$B$2,$C$2)</f>
         <v>Listas fijadas</v>
       </c>
     </row>
@@ -2836,7 +2842,7 @@
         <v>197</v>
       </c>
       <c r="C111" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B111,$B$2,$C$2)</f>
         <v>Título del álbum</v>
       </c>
     </row>
@@ -2848,7 +2854,7 @@
         <v>199</v>
       </c>
       <c r="C112" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B112,$B$2,$C$2)</f>
         <v>Nombre artístico</v>
       </c>
     </row>
@@ -2860,7 +2866,7 @@
         <v>302</v>
       </c>
       <c r="C113" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B113,$B$2,$C$2)</f>
         <v>Mi lista de reproducción perfecta</v>
       </c>
     </row>
@@ -2872,7 +2878,7 @@
         <v>195</v>
       </c>
       <c r="C114" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B114,$B$2,$C$2)</f>
         <v>Título de la canción</v>
       </c>
     </row>
@@ -2884,7 +2890,7 @@
         <v>231</v>
       </c>
       <c r="C115" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B115,$B$2,$C$2)</f>
         <v>Lista de reproducción</v>
       </c>
     </row>
@@ -2896,7 +2902,7 @@
         <v>18</v>
       </c>
       <c r="C116" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B116,$B$2,$C$2)</f>
         <v>Reproducir medios</v>
       </c>
     </row>
@@ -2908,7 +2914,7 @@
         <v>38</v>
       </c>
       <c r="C117" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B117,$B$2,$C$2)</f>
         <v>Juego a continuación</v>
       </c>
     </row>
@@ -2920,7 +2926,7 @@
         <v>37</v>
       </c>
       <c r="C118" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B118,$B$2,$C$2)</f>
         <v>Tocar canción</v>
       </c>
     </row>
@@ -2932,7 +2938,7 @@
         <v>13</v>
       </c>
       <c r="C119" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B119,$B$2,$C$2)</f>
         <v>Listas de reproducción</v>
       </c>
     </row>
@@ -2944,7 +2950,7 @@
         <v>53</v>
       </c>
       <c r="C120" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B120,$B$2,$C$2)</f>
         <v>Selecciones rápidas</v>
       </c>
     </row>
@@ -2956,7 +2962,7 @@
         <v>81</v>
       </c>
       <c r="C121" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B121,$B$2,$C$2)</f>
         <v>Radio</v>
       </c>
     </row>
@@ -2968,7 +2974,7 @@
         <v>137</v>
       </c>
       <c r="C122" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B122,$B$2,$C$2)</f>
         <v>No se han encontrado estaciones</v>
       </c>
     </row>
@@ -2980,7 +2986,7 @@
         <v>139</v>
       </c>
       <c r="C123" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B123,$B$2,$C$2)</f>
         <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
     </row>
@@ -2992,7 +2998,7 @@
         <v>141</v>
       </c>
       <c r="C124" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B124,$B$2,$C$2)</f>
         <v>Busca emisoras, géneros, países...</v>
       </c>
     </row>
@@ -3004,7 +3010,7 @@
         <v>113</v>
       </c>
       <c r="C125" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B125,$B$2,$C$2)</f>
         <v>Emisoras de radio</v>
       </c>
     </row>
@@ -3016,7 +3022,7 @@
         <v>103</v>
       </c>
       <c r="C126" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B126,$B$2,$C$2)</f>
         <v>Mezcla reciente</v>
       </c>
     </row>
@@ -3028,7 +3034,7 @@
         <v>89</v>
       </c>
       <c r="C127" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B127,$B$2,$C$2)</f>
         <v>Jugado recientemente</v>
       </c>
     </row>
@@ -3040,7 +3046,7 @@
         <v>54</v>
       </c>
       <c r="C128" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B128,$B$2,$C$2)</f>
         <v>Jugado recientemente</v>
       </c>
     </row>
@@ -3052,7 +3058,7 @@
         <v>349</v>
       </c>
       <c r="C129" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE(B129,$B$2,$C$2)</f>
         <v>Registro</v>
       </c>
     </row>
@@ -3064,7 +3070,7 @@
         <v>350</v>
       </c>
       <c r="C130" t="str">
-        <f t="shared" ref="C130:C161" si="6">_xlfn.TRANSLATE(B130,$B$2,$C$2)</f>
+        <f>_xlfn.TRANSLATE(B130,$B$2,$C$2)</f>
         <v>Registrado</v>
       </c>
     </row>
@@ -3076,7 +3082,7 @@
         <v>351</v>
       </c>
       <c r="C131" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B131,$B$2,$C$2)</f>
         <v>Registrando...</v>
       </c>
     </row>
@@ -3088,7 +3094,7 @@
         <v>171</v>
       </c>
       <c r="C132" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B132,$B$2,$C$2)</f>
         <v>Artistas relacionados</v>
       </c>
     </row>
@@ -3100,7 +3106,7 @@
         <v>282</v>
       </c>
       <c r="C133" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B133,$B$2,$C$2)</f>
         <v>Relajado</v>
       </c>
     </row>
@@ -3112,7 +3118,7 @@
         <v>241</v>
       </c>
       <c r="C134" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B134,$B$2,$C$2)</f>
         <v>Eliminar de la biblioteca</v>
       </c>
     </row>
@@ -3124,7 +3130,7 @@
         <v>40</v>
       </c>
       <c r="C135" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B135,$B$2,$C$2)</f>
         <v>Quitar de me gusta</v>
       </c>
     </row>
@@ -3136,7 +3142,7 @@
         <v>227</v>
       </c>
       <c r="C136" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B136,$B$2,$C$2)</f>
         <v>Eliminar de la lista de reproducción</v>
       </c>
     </row>
@@ -3148,7 +3154,7 @@
         <v>44</v>
       </c>
       <c r="C137" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B137,$B$2,$C$2)</f>
         <v>Eliminar de la cola</v>
       </c>
     </row>
@@ -3160,564 +3166,570 @@
         <v>157</v>
       </c>
       <c r="C138" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B138,$B$2,$C$2)</f>
         <v>Repetir nueva contraseña</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>74</v>
+        <v>361</v>
       </c>
       <c r="B139" t="s">
-        <v>75</v>
+        <v>362</v>
       </c>
       <c r="C139" t="str">
-        <f t="shared" si="6"/>
-        <v>Búsqueda</v>
+        <f>_xlfn.TRANSLATE(B139,$B$2,$C$2)</f>
+        <v>Guardando...</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="B140" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C140" t="str">
-        <f t="shared" si="6"/>
-        <v>Busca artistas, canciones, álbumes...</v>
+        <f>_xlfn.TRANSLATE(B140,$B$2,$C$2)</f>
+        <v>Búsqueda</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="B141" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="C141" t="str">
-        <f t="shared" si="6"/>
-        <v>Parece que el silencio también es música...</v>
+        <f>_xlfn.TRANSLATE(B141,$B$2,$C$2)</f>
+        <v>Busca artistas, canciones, álbumes...</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B142" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C142" t="str">
-        <f t="shared" si="6"/>
-        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
+        <f>_xlfn.TRANSLATE(B142,$B$2,$C$2)</f>
+        <v>Parece que el silencio también es música...</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B143" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C143" t="str">
-        <f t="shared" si="6"/>
-        <v>Buscar en la biblioteca</v>
+        <f>_xlfn.TRANSLATE(B143,$B$2,$C$2)</f>
+        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="B144" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="C144" t="str">
-        <f t="shared" si="6"/>
-        <v>Usuarios de búsqueda</v>
+        <f>_xlfn.TRANSLATE(B144,$B$2,$C$2)</f>
+        <v>Buscar en la biblioteca</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B145" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C145" t="str">
-        <f t="shared" si="6"/>
-        <v>Enviar canción actual</v>
+        <f>_xlfn.TRANSLATE(B145,$B$2,$C$2)</f>
+        <v>Usuarios de búsqueda</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>270</v>
+        <v>134</v>
       </c>
       <c r="B146" t="s">
-        <v>271</v>
+        <v>135</v>
       </c>
       <c r="C146" t="str">
-        <f t="shared" si="6"/>
-        <v>Septiembre</v>
+        <f>_xlfn.TRANSLATE(B146,$B$2,$C$2)</f>
+        <v>Enviar canción actual</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>76</v>
+        <v>270</v>
       </c>
       <c r="B147" t="s">
-        <v>77</v>
+        <v>271</v>
       </c>
       <c r="C147" t="str">
-        <f t="shared" si="6"/>
-        <v>Escenarios</v>
+        <f>_xlfn.TRANSLATE(B147,$B$2,$C$2)</f>
+        <v>Septiembre</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="B148" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="C148" t="str">
-        <f t="shared" si="6"/>
-        <v>Compartir canción</v>
+        <f>_xlfn.TRANSLATE(B148,$B$2,$C$2)</f>
+        <v>Escenarios</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>120</v>
+        <v>31</v>
       </c>
       <c r="B149" t="s">
-        <v>121</v>
+        <v>39</v>
       </c>
       <c r="C149" t="str">
-        <f t="shared" si="6"/>
-        <v>Canciones compartidas para ti</v>
+        <f>_xlfn.TRANSLATE(B149,$B$2,$C$2)</f>
+        <v>Compartir canción</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B150" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C150" t="str">
-        <f t="shared" si="6"/>
-        <v>Compartido desde</v>
+        <f>_xlfn.TRANSLATE(B150,$B$2,$C$2)</f>
+        <v>Canciones compartidas para ti</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="B151" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="C151" t="str">
-        <f t="shared" si="6"/>
-        <v>Mostrando datos de</v>
+        <f>_xlfn.TRANSLATE(B151,$B$2,$C$2)</f>
+        <v>Compartido desde</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="B152" t="s">
-        <v>15</v>
+        <v>145</v>
       </c>
       <c r="C152" t="str">
-        <f t="shared" si="6"/>
-        <v>Canción</v>
+        <f>_xlfn.TRANSLATE(B152,$B$2,$C$2)</f>
+        <v>Mostrando datos de</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B153" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C153" t="str">
-        <f t="shared" si="6"/>
-        <v>Canciones</v>
+        <f>_xlfn.TRANSLATE(B153,$B$2,$C$2)</f>
+        <v>Canción</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>330</v>
+        <v>9</v>
       </c>
       <c r="B154" t="s">
-        <v>278</v>
+        <v>14</v>
       </c>
       <c r="C154" t="str">
-        <f t="shared" si="6"/>
-        <v>Canciones Solo para ti</v>
+        <f>_xlfn.TRANSLATE(B154,$B$2,$C$2)</f>
+        <v>Canciones</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>160</v>
+        <v>330</v>
       </c>
       <c r="B155" t="s">
-        <v>161</v>
+        <v>278</v>
       </c>
       <c r="C155" t="str">
-        <f t="shared" si="6"/>
-        <v>Canciones de</v>
+        <f>_xlfn.TRANSLATE(B155,$B$2,$C$2)</f>
+        <v>Canciones Solo para ti</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>212</v>
+        <v>160</v>
       </c>
       <c r="B156" t="s">
-        <v>213</v>
+        <v>161</v>
       </c>
       <c r="C156" t="str">
-        <f t="shared" si="6"/>
-        <v>Canciones escuchadas</v>
+        <f>_xlfn.TRANSLATE(B156,$B$2,$C$2)</f>
+        <v>Canciones de</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>142</v>
+        <v>212</v>
       </c>
       <c r="B157" t="s">
-        <v>143</v>
+        <v>213</v>
       </c>
       <c r="C157" t="str">
-        <f t="shared" si="6"/>
-        <v>Estadísticas</v>
+        <f>_xlfn.TRANSLATE(B157,$B$2,$C$2)</f>
+        <v>Canciones escuchadas</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>78</v>
+        <v>142</v>
       </c>
       <c r="B158" t="s">
-        <v>79</v>
+        <v>143</v>
       </c>
       <c r="C158" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE(B158,$B$2,$C$2)</f>
         <v>Estadísticas</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>333</v>
+        <v>78</v>
       </c>
       <c r="B159" t="s">
-        <v>335</v>
+        <v>79</v>
       </c>
       <c r="C159" t="str">
-        <f t="shared" si="6"/>
-        <v>¡Para</v>
+        <f>_xlfn.TRANSLATE(B159,$B$2,$C$2)</f>
+        <v>Estadísticas</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>172</v>
+        <v>333</v>
       </c>
       <c r="B160" t="s">
-        <v>173</v>
+        <v>335</v>
       </c>
       <c r="C160" t="str">
-        <f t="shared" si="6"/>
-        <v>a</v>
+        <f>_xlfn.TRANSLATE(B160,$B$2,$C$2)</f>
+        <v>¡Para</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B161" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C161" t="str">
-        <f t="shared" si="6"/>
-        <v>Álbumes destacados</v>
+        <f>_xlfn.TRANSLATE(B161,$B$2,$C$2)</f>
+        <v>a</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C162" t="str">
-        <f t="shared" ref="C162:C193" si="7">_xlfn.TRANSLATE(B162,$B$2,$C$2)</f>
-        <v>Canciones principales</v>
+        <f>_xlfn.TRANSLATE(B162,$B$2,$C$2)</f>
+        <v>Álbumes destacados</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>244</v>
+        <v>164</v>
       </c>
       <c r="B163" t="s">
-        <v>245</v>
+        <v>165</v>
       </c>
       <c r="C163" t="str">
-        <f t="shared" si="7"/>
-        <v>Desclavar</v>
+        <f>_xlfn.TRANSLATE(B163,$B$2,$C$2)</f>
+        <v>Canciones principales</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>346</v>
+        <v>244</v>
       </c>
       <c r="B164" t="s">
-        <v>347</v>
+        <v>245</v>
       </c>
       <c r="C164" t="str">
-        <f t="shared" si="7"/>
-        <v>Desregistrar</v>
+        <f>_xlfn.TRANSLATE(B164,$B$2,$C$2)</f>
+        <v>Desclavar</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="B165" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C165" t="str">
-        <f t="shared" si="7"/>
-        <v>No registrado</v>
+        <f>_xlfn.TRANSLATE(B165,$B$2,$C$2)</f>
+        <v>Desregistrar</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B166" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="C166" t="str">
-        <f t="shared" si="7"/>
-        <v>Dejar de registrarse...</v>
+        <f>_xlfn.TRANSLATE(B166,$B$2,$C$2)</f>
+        <v>No registrado</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>202</v>
+        <v>341</v>
       </c>
       <c r="B167" t="s">
-        <v>203</v>
-      </c>
-      <c r="C167" t="s">
-        <v>359</v>
+        <v>352</v>
+      </c>
+      <c r="C167" t="str">
+        <f>_xlfn.TRANSLATE(B167,$B$2,$C$2)</f>
+        <v>Dejar de registrarse...</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>340</v>
+        <v>202</v>
       </c>
       <c r="B168" t="s">
-        <v>358</v>
-      </c>
-      <c r="C168" t="str">
-        <f t="shared" ref="C168:C190" si="8">_xlfn.TRANSLATE(B168,$B$2,$C$2)</f>
-        <v>Actualizando...</v>
+        <v>203</v>
+      </c>
+      <c r="C168" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="B169" t="s">
-        <v>326</v>
+        <v>358</v>
       </c>
       <c r="C169" t="str">
-        <f t="shared" si="8"/>
-        <v>Subida</v>
+        <f>_xlfn.TRANSLATE(B169,$B$2,$C$2)</f>
+        <v>Actualizando...</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>7</v>
+        <v>325</v>
       </c>
       <c r="B170" t="s">
-        <v>12</v>
+        <v>326</v>
       </c>
       <c r="C170" t="str">
-        <f t="shared" si="8"/>
-        <v>Usuario</v>
+        <f>_xlfn.TRANSLATE(B170,$B$2,$C$2)</f>
+        <v>Subida</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>148</v>
+        <v>7</v>
       </c>
       <c r="B171" t="s">
-        <v>149</v>
+        <v>12</v>
       </c>
       <c r="C171" t="str">
-        <f t="shared" si="8"/>
-        <v>Configuración de usuario</v>
+        <f>_xlfn.TRANSLATE(B171,$B$2,$C$2)</f>
+        <v>Usuario</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>58</v>
+        <v>148</v>
       </c>
       <c r="B172" t="s">
-        <v>63</v>
+        <v>149</v>
       </c>
       <c r="C172" t="str">
-        <f t="shared" si="8"/>
-        <v>Estadísticas de usuario</v>
+        <f>_xlfn.TRANSLATE(B172,$B$2,$C$2)</f>
+        <v>Configuración de usuario</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>124</v>
+        <v>58</v>
       </c>
       <c r="B173" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
       <c r="C173" t="str">
-        <f t="shared" si="8"/>
-        <v>Usuarios y amigos</v>
+        <f>_xlfn.TRANSLATE(B173,$B$2,$C$2)</f>
+        <v>Estadísticas de usuario</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="B174" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C174" t="str">
-        <f t="shared" si="8"/>
-        <v>Lista de usuarios</v>
+        <f>_xlfn.TRANSLATE(B174,$B$2,$C$2)</f>
+        <v>Usuarios y amigos</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>331</v>
+        <v>132</v>
       </c>
       <c r="B175" t="s">
-        <v>332</v>
+        <v>133</v>
       </c>
       <c r="C175" t="str">
-        <f t="shared" si="8"/>
-        <v>Vídeos</v>
+        <f>_xlfn.TRANSLATE(B175,$B$2,$C$2)</f>
+        <v>Lista de usuarios</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>90</v>
+        <v>331</v>
       </c>
       <c r="B176" t="s">
-        <v>91</v>
+        <v>332</v>
       </c>
       <c r="C176" t="str">
-        <f t="shared" si="8"/>
-        <v>También puede que te interese</v>
+        <f>_xlfn.TRANSLATE(B176,$B$2,$C$2)</f>
+        <v>Vídeos</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>289</v>
+        <v>90</v>
       </c>
       <c r="B177" t="s">
-        <v>290</v>
+        <v>91</v>
       </c>
       <c r="C177" t="str">
-        <f t="shared" si="8"/>
-        <v>Tu</v>
+        <f>_xlfn.TRANSLATE(B177,$B$2,$C$2)</f>
+        <v>También puede que te interese</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>96</v>
+        <v>289</v>
       </c>
       <c r="B178" t="s">
-        <v>97</v>
+        <v>290</v>
       </c>
       <c r="C178" t="str">
-        <f t="shared" si="8"/>
-        <v>Tus álbumes y listas de reproducción</v>
+        <f>_xlfn.TRANSLATE(B178,$B$2,$C$2)</f>
+        <v>Tu</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
+        <v>96</v>
+      </c>
+      <c r="B179" t="s">
+        <v>97</v>
+      </c>
+      <c r="C179" t="str">
+        <f>_xlfn.TRANSLATE(B179,$B$2,$C$2)</f>
+        <v>Tus álbumes y listas de reproducción</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
         <v>114</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B180" t="s">
         <v>115</v>
       </c>
-      <c r="C179" t="str">
-        <f t="shared" si="8"/>
+      <c r="C180" t="str">
+        <f>_xlfn.TRANSLATE(B180,$B$2,$C$2)</f>
         <v>Vídeos de YouTube</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C180" t="str">
-        <f t="shared" si="8"/>
-        <v/>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C181" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B181,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C182" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B182,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C183" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B183,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C184" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B184,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C185" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B185,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C186" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B186,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C187" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B187,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C188" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B188,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C189" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B189,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C190" t="str">
-        <f t="shared" si="8"/>
+        <f>_xlfn.TRANSLATE(B190,$B$2,$C$2)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor media handling and enums for improved consistency and clarity
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\icass\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC16839-EC62-4D4D-8F27-BE025F7ED06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A31E6F-183C-41EF-BA42-C3726195E78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="379">
   <si>
     <t>KEY</t>
   </si>
@@ -1158,6 +1158,18 @@
   </si>
   <si>
     <t>Media progress</t>
+  </si>
+  <si>
+    <t>GETTING_INFO</t>
+  </si>
+  <si>
+    <t>Getting info</t>
+  </si>
+  <si>
+    <t>CLICK_TO_DOWNLOAD</t>
+  </si>
+  <si>
+    <t>Click to download</t>
   </si>
 </sst>
 </file>
@@ -1497,7 +1509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C188"/>
+  <dimension ref="A1:D224"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
@@ -3083,7 +3095,7 @@
         <v>262</v>
       </c>
       <c r="C132" t="str">
-        <f t="shared" ref="C132:C188" si="2">_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
+        <f t="shared" ref="C132:C195" si="2">_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
         <v>Artistas relacionados</v>
       </c>
     </row>
@@ -3757,6 +3769,232 @@
       <c r="C188" t="str">
         <f t="shared" si="2"/>
         <v>Progreso de los medios</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>375</v>
+      </c>
+      <c r="B189" t="s">
+        <v>376</v>
+      </c>
+      <c r="C189" t="str">
+        <f t="shared" si="2"/>
+        <v>Obteniendo información</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>377</v>
+      </c>
+      <c r="B190" t="s">
+        <v>378</v>
+      </c>
+      <c r="C190" t="str">
+        <f t="shared" si="2"/>
+        <v>Haz clic para descargar</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C192" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="193" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C193" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="194" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C194" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="195" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C195" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="D195" t="str">
+        <f>_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C196" t="str">
+        <f t="shared" ref="C196:C224" si="3">_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C197" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="198" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C198" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="199" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C199" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="200" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C200" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="201" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C201" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="202" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C202" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="203" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C203" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="204" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C204" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="205" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C205" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="206" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C206" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="207" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C207" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="208" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C208" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="209" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C209" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="210" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C210" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="211" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C211" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="212" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C212" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="213" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C213" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="214" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C214" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="215" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C215" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="216" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C216" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="217" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C217" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="218" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C218" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="219" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C219" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="220" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C220" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="221" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C221" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="222" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C222" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="223" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C223" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="224" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C224" t="str">
+        <f t="shared" si="3"/>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update Vocabulary.xlsx with new content
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicorebo18\rockit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DE7F14-5F1C-4B25-A049-2ACDA78604B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3BF0727-71CB-48A8-9F1B-1A66C47D781D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="1170" windowWidth="16410" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="481">
   <si>
     <t>KEY</t>
   </si>
@@ -1412,7 +1412,70 @@
     <t>Return back home</t>
   </si>
   <si>
-    <t>Para</t>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>ToDo</t>
+  </si>
+  <si>
+    <t>MEDIA_ADDED_TO_LIBRARY</t>
+  </si>
+  <si>
+    <t>Media added to library</t>
+  </si>
+  <si>
+    <t>FAILED_TO_ADD_MEDIA_TO_LIBRARY</t>
+  </si>
+  <si>
+    <t>Failed to add media to library</t>
+  </si>
+  <si>
+    <t>FAILED_TO_FETCH_PLAYLISTS</t>
+  </si>
+  <si>
+    <t>Failed to fetch playlists</t>
+  </si>
+  <si>
+    <t>ADDED_TO_PLAYLIST</t>
+  </si>
+  <si>
+    <t>Added to playlist</t>
+  </si>
+  <si>
+    <t>FAILED_TO_ADD_MEDIA_TO_PLAYLIST</t>
+  </si>
+  <si>
+    <t>Failed to add media to playlist</t>
+  </si>
+  <si>
+    <t>ERROR_SEARCHING</t>
+  </si>
+  <si>
+    <t>ERROR_GETTING_DOWNLOADS</t>
+  </si>
+  <si>
+    <t>ERROR_GETTING_USER</t>
+  </si>
+  <si>
+    <t>Error searching</t>
+  </si>
+  <si>
+    <t>Error getting downloads</t>
+  </si>
+  <si>
+    <t>Error getting user</t>
+  </si>
+  <si>
+    <t>LANGUAGE_CHANGE_FAILED</t>
+  </si>
+  <si>
+    <t>Language change failed</t>
+  </si>
+  <si>
+    <t>NEW_VERSION_AVAILABLE</t>
+  </si>
+  <si>
+    <t>New version available</t>
   </si>
 </sst>
 </file>
@@ -1468,10 +1531,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D232" totalsRowShown="0">
-  <autoFilter ref="A2:D232" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D229">
-    <sortCondition ref="A2:A229"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D255" totalsRowShown="0">
+  <autoFilter ref="A2:D255" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D255">
+    <sortCondition ref="A2:A255"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="KEY"/>
@@ -1772,8 +1835,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D232"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D255"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.7109375" customWidth="1"/>
@@ -1859,407 +1922,407 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>455</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>456</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir canción a la lista de reproducción</v>
+        <v>Añadir medios a la lista de reproducción</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter une chanson à la playlist</v>
+        <v>Ajouter un média à une playlist</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir canción a la cola</v>
+        <v>Añadir canción a la lista de reproducción</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter une chanson à la file d’attente</v>
+        <v>Ajouter une chanson à la playlist</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir a la biblioteca</v>
+        <v>Añadir canción a la cola</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter à la bibliothèque</v>
+        <v>Ajouter une chanson à la file d’attente</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir a los que me gusta</v>
+        <v>Añadir a la biblioteca</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter aux aimés</v>
+        <v>Ajouter à la bibliothèque</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir a la cola</v>
+        <v>Añadir a los que me gusta</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter à la file d’attente</v>
+        <v>Ajouter aux aimés</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>Añadir Build</v>
+        <v>Añadir a la cola</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
-        <v>Ajouter une construction</v>
+        <v>Ajouter à la file d’attente</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>467</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>468</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
-        <v>Archivo APK</v>
+        <v>Añadido a la lista de reproducción</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
-        <v>Fichier APK</v>
+        <v>Ajouté à la playlist</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>Gestiona tus builds de Android</v>
+        <v>Añadir Build</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="0"/>
-        <v>Gérez vos versions Android</v>
+        <v>Ajouter une construction</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>Construcciones</v>
+        <v>Archivo APK</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="0"/>
-        <v>Constructions</v>
+        <v>Fichier APK</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>Cancelar</v>
+        <v>Gestiona tus builds de Android</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="0"/>
-        <v>Annuler</v>
+        <v>Gérez vos versions Android</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
-        <v>Descripción</v>
+        <v>Construcciones</v>
       </c>
       <c r="D16" t="str">
         <f t="shared" si="0"/>
-        <v>Description</v>
+        <v>Constructions</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
-        <v>Aquí entra la descripción...</v>
+        <v>Cancelar</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="0"/>
-        <v>Voici la description...</v>
+        <v>Annuler</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
-        <v>Enter Version</v>
+        <v>Descripción</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="0"/>
-        <v>Enter Version</v>
+        <v>Description</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas novedades</v>
+        <v>Aquí entra la descripción...</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="0"/>
-        <v>Dernières nouvelles</v>
+        <v>Voici la description...</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
-        <v>Aún no hay builds</v>
+        <v>Enter Version</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="0"/>
-        <v>Pas encore de builds</v>
+        <v>Enter Version</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
-        <v>Solo APK</v>
+        <v>Últimas novedades</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="0"/>
-        <v>Seul APK</v>
+        <v>Dernières nouvelles</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
-        <v>Opcional</v>
+        <v>Aún no hay builds</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="0"/>
-        <v>Optionnel</v>
+        <v>Pas encore de builds</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" ref="C23:D42" si="1">_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
-        <v>Leer Fallido</v>
+        <v>Solo APK</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="1"/>
-        <v>Lire Échec</v>
+        <v>Seul APK</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="1"/>
-        <v>Obligatorio</v>
+        <v>Opcional</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="1"/>
-        <v>Obligatoire</v>
+        <v>Optionnel</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>Seleccionar APK</v>
+        <v>Leer Fallido</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="1"/>
-        <v>Sélectionner APK</v>
+        <v>Lire Échec</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="1"/>
-        <v>Seleccionados</v>
+        <v>Obligatorio</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="1"/>
-        <v>Sélectionné</v>
+        <v>Obligatoire</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="1"/>
-        <v>Próximamente</v>
+        <v>Seleccionar APK</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="1"/>
-        <v>Bientôt</v>
+        <v>Sélectionner APK</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="1"/>
-        <v>Configuración de plataformas</v>
+        <v>Seleccionados</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="1"/>
-        <v>Réglages de la plateforme</v>
+        <v>Sélectionné</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="1"/>
-        <v>Escenarios</v>
+        <v>Próximamente</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" si="1"/>
-        <v>Décors</v>
+        <v>Bientôt</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="1"/>
-        <v>Construcciones</v>
+        <v>Configuración de plataformas</v>
       </c>
       <c r="D30" t="str">
         <f t="shared" si="1"/>
-        <v>Constructions</v>
+        <v>Réglages de la plateforme</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B31" t="s">
         <v>60</v>
@@ -2275,3224 +2338,3518 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="1"/>
-        <v>Usuarios</v>
+        <v>Construcciones</v>
       </c>
       <c r="D32" t="str">
         <f t="shared" si="1"/>
-        <v>Utilisateurs</v>
+        <v>Constructions</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="1"/>
-        <v>Compilación de subida</v>
+        <v>Escenarios</v>
       </c>
       <c r="D33" t="str">
         <f t="shared" si="1"/>
-        <v>Upload Build</v>
+        <v>Décors</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B34" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="1"/>
-        <v>Fallido en la subida</v>
+        <v>Usuarios</v>
       </c>
       <c r="D34" t="str">
         <f t="shared" si="1"/>
-        <v>Téléchargement échoué</v>
+        <v>Utilisateurs</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="1"/>
-        <v>Sube tu primera construcción</v>
+        <v>Compilación de subida</v>
       </c>
       <c r="D35" t="str">
         <f t="shared" si="1"/>
-        <v>Téléchargez votre première compilation</v>
+        <v>Upload Build</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="1"/>
-        <v>Subir nueva versión</v>
+        <v>Fallido en la subida</v>
       </c>
       <c r="D36" t="str">
         <f t="shared" si="1"/>
-        <v>Télécharger une nouvelle version</v>
+        <v>Téléchargement échoué</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B37" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="1"/>
-        <v>Éxito en la subida</v>
+        <v>Sube tu primera construcción</v>
       </c>
       <c r="D37" t="str">
         <f t="shared" si="1"/>
-        <v>Succès de la télévision</v>
+        <v>Téléchargez votre première compilation</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="1"/>
-        <v>Subiendo algo...</v>
+        <v>Subir nueva versión</v>
       </c>
       <c r="D38" t="str">
         <f t="shared" si="1"/>
-        <v>Téléchargement...</v>
+        <v>Télécharger une nouvelle version</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="1"/>
-        <v>Próximamente</v>
+        <v>Éxito en la subida</v>
       </c>
       <c r="D39" t="str">
         <f t="shared" si="1"/>
-        <v>Bientôt</v>
+        <v>Succès de la télévision</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="1"/>
-        <v>Gestionar los usuarios de la plataforma</v>
+        <v>Subiendo algo...</v>
       </c>
       <c r="D40" t="str">
         <f t="shared" si="1"/>
-        <v>Gérer les utilisateurs de la plateforme</v>
+        <v>Téléchargement...</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="1"/>
-        <v>Usuarios</v>
+        <v>Próximamente</v>
       </c>
       <c r="D41" t="str">
         <f t="shared" si="1"/>
-        <v>Utilisateurs</v>
+        <v>Bientôt</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="1"/>
-        <v>Versión</v>
+        <v>Gestionar los usuarios de la plataforma</v>
       </c>
       <c r="D42" t="str">
         <f t="shared" si="1"/>
-        <v>Version</v>
+        <v>Gérer les utilisateurs de la plateforme</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B43" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" ref="C43:D62" si="2">_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
-        <v>Álbum</v>
+        <v>Usuarios</v>
       </c>
       <c r="D43" t="str">
         <f t="shared" si="2"/>
-        <v>Album</v>
+        <v>Utilisateurs</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B44" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="2"/>
-        <v>Álbumes</v>
+        <v>Versión</v>
       </c>
       <c r="D44" t="str">
         <f t="shared" si="2"/>
-        <v>Albums</v>
+        <v>Version</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="2"/>
-        <v>Álbumes y sencillos</v>
+        <v>Álbum</v>
       </c>
       <c r="D45" t="str">
         <f t="shared" si="2"/>
-        <v>Albums et singles</v>
+        <v>Album</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="2"/>
-        <v>Todos</v>
+        <v>Álbumes</v>
       </c>
       <c r="D46" t="str">
         <f t="shared" si="2"/>
-        <v>Tous</v>
+        <v>Albums</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="2"/>
-        <v>Abril</v>
+        <v>Álbumes y sencillos</v>
       </c>
       <c r="D47" t="str">
         <f t="shared" si="2"/>
-        <v>Avril</v>
+        <v>Albums et singles</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="2"/>
-        <v>Artista</v>
+        <v>Todos</v>
       </c>
       <c r="D48" t="str">
         <f t="shared" si="2"/>
-        <v>Artiste</v>
+        <v>Tous</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="2"/>
-        <v>Artistas</v>
+        <v>Abril</v>
       </c>
       <c r="D49" t="str">
         <f t="shared" si="2"/>
-        <v>Artistes</v>
+        <v>Avril</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C50" t="str">
         <f t="shared" si="2"/>
-        <v>Agosto</v>
+        <v>Artista</v>
       </c>
       <c r="D50" t="str">
         <f t="shared" si="2"/>
-        <v>Août</v>
+        <v>Artiste</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="2"/>
-        <v>Minutos medios por canción</v>
+        <v>Artistas</v>
       </c>
       <c r="D51" t="str">
         <f t="shared" si="2"/>
-        <v>Minutes moyennes par chanson</v>
+        <v>Artistes</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="2"/>
-        <v>por</v>
+        <v>Agosto</v>
       </c>
       <c r="D52" t="str">
         <f t="shared" si="2"/>
-        <v>par</v>
+        <v>Août</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B53" t="s">
-        <v>32</v>
+        <v>100</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="2"/>
-        <v>Cancelar</v>
+        <v>Minutos medios por canción</v>
       </c>
       <c r="D53" t="str">
         <f t="shared" si="2"/>
-        <v>Annuler</v>
+        <v>Minutes moyennes par chanson</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="2"/>
-        <v>Cambiar contraseña</v>
+        <v>por</v>
       </c>
       <c r="D54" t="str">
         <f t="shared" si="2"/>
-        <v>Changer le mot de passe</v>
+        <v>par</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>107</v>
+        <v>32</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="2"/>
-        <v>Descargas claras</v>
+        <v>Cancelar</v>
       </c>
       <c r="D55" t="str">
         <f t="shared" si="2"/>
-        <v>Téléchargements clairs</v>
+        <v>Annuler</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="2"/>
-        <v>Haz clic para descargar</v>
+        <v>Cambiar contraseña</v>
       </c>
       <c r="D56" t="str">
         <f t="shared" si="2"/>
-        <v>Cliquez pour télécharger</v>
+        <v>Changer le mot de passe</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B57" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="2"/>
-        <v>Topo comunitario</v>
+        <v>Descargas claras</v>
       </c>
       <c r="D57" t="str">
         <f t="shared" si="2"/>
-        <v>Sommet communautaire</v>
+        <v>Téléchargements clairs</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="2"/>
-        <v>URL de la lista de copiar</v>
+        <v>Haz clic para descargar</v>
       </c>
       <c r="D58" t="str">
         <f t="shared" si="2"/>
-        <v>URL de la liste de copie</v>
+        <v>Cliquez pour télécharger</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="2"/>
-        <v>Copiar la URL de la canción</v>
+        <v>Topo comunitario</v>
       </c>
       <c r="D59" t="str">
         <f t="shared" si="2"/>
-        <v>Copier l’URL de la chanson</v>
+        <v>Sommet communautaire</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B60" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="2"/>
-        <v>Crear</v>
+        <v>URL de la lista de copiar</v>
       </c>
       <c r="D60" t="str">
         <f t="shared" si="2"/>
-        <v>Créer</v>
+        <v>URL de la liste de copie</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B61" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="2"/>
-        <v>Crear...</v>
+        <v>Copiar la URL de la canción</v>
       </c>
       <c r="D61" t="str">
         <f t="shared" si="2"/>
-        <v>Créer...</v>
+        <v>Copier l’URL de la chanson</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C62" t="str">
         <f t="shared" si="2"/>
-        <v>Fecha añadida</v>
+        <v>Crear</v>
       </c>
       <c r="D62" t="str">
         <f t="shared" si="2"/>
-        <v>Date ajoutée</v>
+        <v>Créer</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B63" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C63" t="str">
         <f t="shared" ref="C63:D82" si="3">_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
-        <v>Diciembre</v>
+        <v>Crear...</v>
       </c>
       <c r="D63" t="str">
         <f t="shared" si="3"/>
-        <v>Décembre</v>
+        <v>Créer...</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B64" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C64" t="str">
         <f t="shared" si="3"/>
-        <v>Tu dispositivo no soporta al trabajador de servicio</v>
+        <v>Fecha añadida</v>
       </c>
       <c r="D64" t="str">
         <f t="shared" si="3"/>
-        <v>Votre appareil ne prend pas en charge l’assistant de service</v>
+        <v>Date ajoutée</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B65" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C65" t="str">
         <f t="shared" si="3"/>
-        <v>Disco</v>
+        <v>Diciembre</v>
       </c>
       <c r="D65" t="str">
         <f t="shared" si="3"/>
-        <v>Disque</v>
+        <v>Décembre</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C66" t="str">
         <f t="shared" si="3"/>
-        <v>Nombre de Muestra</v>
+        <v>Tu dispositivo no soporta al trabajador de servicio</v>
       </c>
       <c r="D66" t="str">
         <f t="shared" si="3"/>
-        <v>Nom d’affichage</v>
+        <v>Votre appareil ne prend pas en charge l’assistant de service</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B67" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C67" t="str">
         <f t="shared" si="3"/>
-        <v>Descargar</v>
+        <v>Disco</v>
       </c>
       <c r="D67" t="str">
         <f t="shared" si="3"/>
-        <v>Télécharger</v>
+        <v>Disque</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B68" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C68" t="str">
         <f t="shared" si="3"/>
-        <v>Descarga la app para escuchar offline</v>
+        <v>Nombre de Muestra</v>
       </c>
       <c r="D68" t="str">
         <f t="shared" si="3"/>
-        <v>Téléchargez l’application pour une écoute hors ligne</v>
+        <v>Nom d’affichage</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B69" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C69" t="str">
         <f t="shared" si="3"/>
-        <v>Introduce una URL de Spotify o YouTube Music</v>
+        <v>Descargar</v>
       </c>
       <c r="D69" t="str">
         <f t="shared" si="3"/>
-        <v>Saisissez une URL Spotify ou YouTube Music</v>
+        <v>Télécharger</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B70" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C70" t="str">
         <f t="shared" si="3"/>
-        <v>Lista de descargas al dispositivo</v>
+        <v>Descarga la app para escuchar offline</v>
       </c>
       <c r="D70" t="str">
         <f t="shared" si="3"/>
-        <v>Liste de téléchargement vers l’appareil</v>
+        <v>Téléchargez l’application pour une écoute hors ligne</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B71" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C71" t="str">
         <f t="shared" si="3"/>
-        <v>Descargar medios al dispositivo</v>
+        <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
       <c r="D71" t="str">
         <f t="shared" si="3"/>
-        <v>Télécharger des médias sur l’appareil</v>
+        <v>Saisissez une URL Spotify ou YouTube Music</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B72" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C72" t="str">
         <f t="shared" si="3"/>
-        <v>Descargar mp</v>
+        <v>Lista de descargas al dispositivo</v>
       </c>
       <c r="D72" t="str">
         <f t="shared" si="3"/>
-        <v>Télécharger le MP</v>
+        <v>Liste de téléchargement vers l’appareil</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B73" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C73" t="str">
         <f t="shared" si="3"/>
-        <v>Descargar canción al dispositivo</v>
+        <v>Descargar medios al dispositivo</v>
       </c>
       <c r="D73" t="str">
         <f t="shared" si="3"/>
-        <v>Télécharger la chanson sur l’appareil</v>
+        <v>Télécharger des médias sur l’appareil</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B74" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C74" t="str">
         <f t="shared" si="3"/>
-        <v>Descarga iniciada</v>
+        <v>Descargar mp</v>
       </c>
       <c r="D74" t="str">
         <f t="shared" si="3"/>
-        <v>Téléchargement lancé</v>
+        <v>Télécharger le MP</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B75" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C75" t="str">
         <f t="shared" si="3"/>
-        <v>Descargar ZIP</v>
+        <v>Descargar canción al dispositivo</v>
       </c>
       <c r="D75" t="str">
         <f t="shared" si="3"/>
-        <v>Télécharger ZIP</v>
+        <v>Télécharger la chanson sur l’appareil</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C76" t="str">
         <f t="shared" si="3"/>
-        <v>Descargas</v>
+        <v>Descarga iniciada</v>
       </c>
       <c r="D76" t="str">
         <f t="shared" si="3"/>
-        <v>Téléchargements</v>
+        <v>Téléchargement lancé</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B77" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C77" t="str">
         <f t="shared" si="3"/>
-        <v>Duración</v>
+        <v>Descargar ZIP</v>
       </c>
       <c r="D77" t="str">
         <f t="shared" si="3"/>
-        <v>Durée</v>
+        <v>Télécharger ZIP</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B78" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="3"/>
-        <v>Energía</v>
+        <v>Descargas</v>
       </c>
       <c r="D78" t="str">
         <f t="shared" si="3"/>
-        <v>Énergie</v>
+        <v>Téléchargements</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B79" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C79" t="str">
         <f t="shared" si="3"/>
-        <v>Introduce un nombre para tu nueva lista de reproducción</v>
+        <v>Duración</v>
       </c>
       <c r="D79" t="str">
         <f t="shared" si="3"/>
-        <v>Saisissez un nom pour votre nouvelle playlist</v>
+        <v>Durée</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B80" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C80" t="str">
         <f t="shared" si="3"/>
-        <v>Error</v>
+        <v>Energía</v>
       </c>
       <c r="D80" t="str">
         <f t="shared" si="3"/>
-        <v>Erreur</v>
+        <v>Énergie</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B81" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C81" t="str">
         <f t="shared" si="3"/>
-        <v>Lenguaje de cambio de error</v>
+        <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D81" t="str">
         <f t="shared" si="3"/>
-        <v>Langage de changement d’erreur</v>
+        <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B82" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C82" t="str">
         <f t="shared" si="3"/>
-        <v>Error al crear tu nueva lista de reproducción</v>
+        <v>Error</v>
       </c>
       <c r="D82" t="str">
         <f t="shared" si="3"/>
-        <v>Erreur lors de la création de votre nouvelle playlist</v>
+        <v>Erreur</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B83" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C83" t="str">
         <f t="shared" ref="C83:D102" si="4">_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
-        <v>Error al crear tu nueva lista de reproducción</v>
+        <v>Lenguaje de cambio de error</v>
       </c>
       <c r="D83" t="str">
         <f t="shared" si="4"/>
-        <v>Erreur lors de la création de votre nouvelle playlist</v>
+        <v>Langage de changement d’erreur</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B84" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C84" t="str">
         <f t="shared" si="4"/>
-        <v>Introduce un nombre para tu nueva lista de reproducción</v>
+        <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D84" t="str">
         <f t="shared" si="4"/>
-        <v>Saisissez un nom pour votre nouvelle playlist</v>
+        <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B85" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C85" t="str">
         <f t="shared" si="4"/>
-        <v>Cola de obtención de errores</v>
+        <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D85" t="str">
         <f t="shared" si="4"/>
-        <v>File d’attente d’obtention d’erreurs</v>
+        <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B86" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="C86" t="str">
         <f t="shared" si="4"/>
-        <v>Error al dar like a medios</v>
+        <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D86" t="str">
         <f t="shared" si="4"/>
-        <v>Erreur d’appréciation des médias</v>
+        <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>168</v>
+        <v>472</v>
       </c>
       <c r="B87" t="s">
-        <v>169</v>
+        <v>475</v>
       </c>
       <c r="C87" t="str">
         <f t="shared" si="4"/>
-        <v>Error al iniciar la descarga</v>
+        <v>Error al obtener descargas</v>
       </c>
       <c r="D87" t="str">
         <f t="shared" si="4"/>
-        <v>Erreur au démarrage du téléchargement</v>
+        <v>Erreur de téléchargement</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B88" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C88" t="str">
         <f t="shared" si="4"/>
-        <v>Error al dejar de dar like a los medios</v>
+        <v>Cola de obtención de errores</v>
       </c>
       <c r="D88" t="str">
         <f t="shared" si="4"/>
-        <v>Erreur de non-like des médias</v>
+        <v>File d’attente d’obtention d’erreurs</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>172</v>
+        <v>473</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>476</v>
       </c>
       <c r="C89" t="str">
         <f t="shared" si="4"/>
-        <v>No cambiaron el idioma</v>
+        <v>Usuario que obtiene errores</v>
       </c>
       <c r="D89" t="str">
         <f t="shared" si="4"/>
-        <v>Échec de changer de langue</v>
+        <v>Utilisateur d’obtention d’erreurs</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B90" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C90" t="str">
         <f t="shared" si="4"/>
-        <v>Álbumes destacados</v>
+        <v>Error al dar like a medios</v>
       </c>
       <c r="D90" t="str">
         <f t="shared" si="4"/>
-        <v>Albums en vedette</v>
+        <v>Erreur d’appréciation des médias</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>176</v>
+        <v>471</v>
       </c>
       <c r="B91" t="s">
-        <v>177</v>
+        <v>474</v>
       </c>
       <c r="C91" t="str">
         <f t="shared" si="4"/>
-        <v>Listas destacadas</v>
+        <v>Búsqueda de errores</v>
       </c>
       <c r="D91" t="str">
         <f t="shared" si="4"/>
-        <v>Listes en vedette</v>
+        <v>Recherche d’erreurs</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="B92" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C92" t="str">
         <f t="shared" si="4"/>
-        <v>Febrero</v>
+        <v>Error al iniciar la descarga</v>
       </c>
       <c r="D92" t="str">
         <f t="shared" si="4"/>
-        <v>Février</v>
+        <v>Erreur au démarrage du téléchargement</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B93" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="C93" t="str">
         <f t="shared" si="4"/>
-        <v>Enfoque</v>
+        <v>Error al dejar de dar like a los medios</v>
       </c>
       <c r="D93" t="str">
         <f t="shared" si="4"/>
-        <v>Focus</v>
+        <v>Erreur de non-like des médias</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>182</v>
+        <v>463</v>
       </c>
       <c r="B94" t="s">
-        <v>183</v>
+        <v>464</v>
       </c>
       <c r="C94" t="str">
         <f t="shared" si="4"/>
-        <v>Amigos</v>
+        <v>No se añadió contenido a la biblioteca</v>
       </c>
       <c r="D94" t="str">
         <f t="shared" si="4"/>
-        <v>Amis</v>
+        <v>Échec d’ajouter des médias à la bibliothèque</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>184</v>
+        <v>469</v>
       </c>
       <c r="B95" t="s">
-        <v>185</v>
+        <v>470</v>
       </c>
       <c r="C95" t="str">
         <f t="shared" si="4"/>
-        <v>Lista de amigos</v>
+        <v>No se añadió contenido a la lista de reproducción</v>
       </c>
       <c r="D95" t="str">
         <f t="shared" si="4"/>
-        <v>Liste d’amis</v>
+        <v>Échec d’ajouter des médias à la playlist</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="B96" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="C96" t="str">
         <f t="shared" si="4"/>
-        <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
+        <v>No cambiaron el idioma</v>
       </c>
       <c r="D96" t="str">
         <f t="shared" si="4"/>
-        <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
+        <v>Échec de changer de langue</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>188</v>
+        <v>465</v>
       </c>
       <c r="B97" t="s">
-        <v>189</v>
+        <v>466</v>
       </c>
       <c r="C97" t="str">
         <f t="shared" si="4"/>
-        <v>Estadísticas de Friends</v>
+        <v>No se han conseguido las listas de reproducción</v>
       </c>
       <c r="D97" t="str">
         <f t="shared" si="4"/>
-        <v>Statistiques de Friends</v>
+        <v>Échec à récupérer les playlists</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="B98" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="C98" t="str">
         <f t="shared" si="4"/>
-        <v>General</v>
+        <v>Álbumes destacados</v>
       </c>
       <c r="D98" t="str">
         <f t="shared" si="4"/>
-        <v>Généralités</v>
+        <v>Albums en vedette</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="B99" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="C99" t="str">
         <f t="shared" si="4"/>
-        <v>Estadísticas generales</v>
+        <v>Listas destacadas</v>
       </c>
       <c r="D99" t="str">
         <f t="shared" si="4"/>
-        <v>Statistiques générales</v>
+        <v>Listes en vedette</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="B100" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="C100" t="str">
         <f t="shared" si="4"/>
-        <v>Obtén información</v>
+        <v>Febrero</v>
       </c>
       <c r="D100" t="str">
         <f t="shared" si="4"/>
-        <v>Obtenez des infos</v>
+        <v>Février</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>196</v>
+        <v>180</v>
       </c>
       <c r="B101" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="C101" t="str">
         <f t="shared" si="4"/>
-        <v>Obteniendo información</v>
+        <v>Enfoque</v>
       </c>
       <c r="D101" t="str">
         <f t="shared" si="4"/>
-        <v>Obtenir des infos</v>
+        <v>Focus</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="B102" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="4"/>
-        <v>Ir al álbum</v>
+        <v>Amigos</v>
       </c>
       <c r="D102" t="str">
         <f t="shared" si="4"/>
-        <v>Aller à l’album</v>
+        <v>Amis</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="B103" t="s">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="C103" t="str">
         <f t="shared" ref="C103:D122" si="5">_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
-        <v>Ir a artista</v>
+        <v>Lista de amigos</v>
       </c>
       <c r="D103" t="str">
         <f t="shared" si="5"/>
-        <v>Aller à l’artiste</v>
+        <v>Liste d’amis</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="B104" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="C104" t="str">
         <f t="shared" si="5"/>
-        <v>Joyas ocultas que olvidaste</v>
+        <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
       <c r="D104" t="str">
         <f t="shared" si="5"/>
-        <v>Des perles cachées que tu as oubliées</v>
+        <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="B105" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="C105" t="str">
         <f t="shared" si="5"/>
-        <v>Inicio</v>
+        <v>Estadísticas de Friends</v>
       </c>
       <c r="D105" t="str">
         <f t="shared" si="5"/>
-        <v>Accueil</v>
+        <v>Statistiques de Friends</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="B106" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="C106" t="str">
         <f t="shared" si="5"/>
-        <v>Enero</v>
+        <v>General</v>
       </c>
       <c r="D106" t="str">
         <f t="shared" si="5"/>
-        <v>Janvier</v>
+        <v>Généralités</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="B107" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="5"/>
-        <v>Julio</v>
+        <v>Estadísticas generales</v>
       </c>
       <c r="D107" t="str">
         <f t="shared" si="5"/>
-        <v>Juillet</v>
+        <v>Statistiques générales</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="B108" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="C108" t="str">
         <f t="shared" si="5"/>
-        <v>Junio</v>
+        <v>Obtén información</v>
       </c>
       <c r="D108" t="str">
         <f t="shared" si="5"/>
-        <v>Juin</v>
+        <v>Obtenez des infos</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="B109" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="C109" t="str">
         <f t="shared" si="5"/>
-        <v>Idioma</v>
+        <v>Obteniendo información</v>
       </c>
       <c r="D109" t="str">
         <f t="shared" si="5"/>
-        <v>Langue</v>
+        <v>Obtenir des infos</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="B110" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="5"/>
-        <v>Cambio de idioma</v>
+        <v>Ir al álbum</v>
       </c>
       <c r="D110" t="str">
         <f t="shared" si="5"/>
-        <v>Changement de langue</v>
+        <v>Aller à l’album</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="B111" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="C111" t="str">
         <f t="shared" si="5"/>
-        <v>Últimas descargas</v>
+        <v>Ir a artista</v>
       </c>
       <c r="D111" t="str">
         <f t="shared" si="5"/>
-        <v>Derniers téléchargements</v>
+        <v>Aller à l’artiste</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="B112" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="C112" t="str">
         <f t="shared" si="5"/>
-        <v>Nivel</v>
+        <v>Joyas ocultas que olvidaste</v>
       </c>
       <c r="D112" t="str">
         <f t="shared" si="5"/>
-        <v>Niveau</v>
+        <v>Des perles cachées que tu as oubliées</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="B113" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="C113" t="str">
         <f t="shared" si="5"/>
-        <v>Biblioteca</v>
+        <v>Inicio</v>
       </c>
       <c r="D113" t="str">
         <f t="shared" si="5"/>
-        <v>Bibliothèque</v>
+        <v>Accueil</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="B114" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="C114" t="str">
         <f t="shared" si="5"/>
-        <v>Como</v>
+        <v>Enero</v>
       </c>
       <c r="D114" t="str">
         <f t="shared" si="5"/>
-        <v>Comme</v>
+        <v>Janvier</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="B115" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="5"/>
-        <v>Canciones que me gustaban</v>
+        <v>Julio</v>
       </c>
       <c r="D115" t="str">
         <f t="shared" si="5"/>
-        <v>Chansons appréciées</v>
+        <v>Juillet</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="B116" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="C116" t="str">
         <f t="shared" si="5"/>
-        <v>Cerrar sesión</v>
+        <v>Junio</v>
       </c>
       <c r="D116" t="str">
         <f t="shared" si="5"/>
-        <v>Déconnexion</v>
+        <v>Juin</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="B117" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="C117" t="str">
         <f t="shared" si="5"/>
-        <v>Letra</v>
+        <v>Idioma</v>
       </c>
       <c r="D117" t="str">
         <f t="shared" si="5"/>
-        <v>Paroles</v>
+        <v>Langue</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>230</v>
+        <v>477</v>
       </c>
       <c r="B118" t="s">
-        <v>231</v>
+        <v>478</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="5"/>
-        <v>Marzo</v>
+        <v>El cambio de idioma fracasó</v>
       </c>
       <c r="D118" t="str">
         <f t="shared" si="5"/>
-        <v>Mars</v>
+        <v>Échec du changement linguistique</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="B119" t="s">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="C119" t="str">
         <f t="shared" si="5"/>
-        <v>Mayo</v>
+        <v>Cambio de idioma</v>
       </c>
       <c r="D119" t="str">
         <f t="shared" si="5"/>
-        <v>Mai</v>
+        <v>Changement de langue</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="B120" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C120" t="str">
         <f t="shared" si="5"/>
-        <v>Progreso de los medios</v>
+        <v>Últimas descargas</v>
       </c>
       <c r="D120" t="str">
         <f t="shared" si="5"/>
-        <v>Progrès des médias</v>
+        <v>Derniers téléchargements</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>236</v>
+        <v>218</v>
       </c>
       <c r="B121" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="C121" t="str">
         <f t="shared" si="5"/>
-        <v>Actas</v>
+        <v>Nivel</v>
       </c>
       <c r="D121" t="str">
         <f t="shared" si="5"/>
-        <v>Procès-verbal</v>
+        <v>Niveau</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>238</v>
+        <v>220</v>
       </c>
       <c r="B122" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
       <c r="C122" t="str">
         <f t="shared" si="5"/>
-        <v>Minutos escuchados</v>
+        <v>Biblioteca</v>
       </c>
       <c r="D122" t="str">
         <f t="shared" si="5"/>
-        <v>Minutes écoutées</v>
+        <v>Bibliothèque</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
       <c r="B123" t="s">
-        <v>241</v>
+        <v>223</v>
       </c>
       <c r="C123" t="str">
         <f t="shared" ref="C123:D142" si="6">_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
-        <v>Minutos escuchados por día</v>
+        <v>Como</v>
       </c>
       <c r="D123" t="str">
         <f t="shared" si="6"/>
-        <v>Minutes écoutées par jour</v>
+        <v>Comme</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="B124" t="s">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="C124" t="str">
         <f t="shared" si="6"/>
-        <v>Canciones para cuando te sientas</v>
+        <v>Canciones que me gustaban</v>
       </c>
       <c r="D124" t="str">
         <f t="shared" si="6"/>
-        <v>Chansons pour quand tu te sens</v>
+        <v>Chansons appréciées</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>244</v>
+        <v>226</v>
       </c>
       <c r="B125" t="s">
-        <v>245</v>
+        <v>227</v>
       </c>
       <c r="C125" t="str">
         <f t="shared" si="6"/>
-        <v>Más opciones</v>
+        <v>Cerrar sesión</v>
       </c>
       <c r="D125" t="str">
         <f t="shared" si="6"/>
-        <v>Plus d’options</v>
+        <v>Déconnexion</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="B126" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="C126" t="str">
         <f t="shared" si="6"/>
-        <v>Más canciones de</v>
+        <v>Letra</v>
       </c>
       <c r="D126" t="str">
         <f t="shared" si="6"/>
-        <v>Plus de chansons de</v>
+        <v>Paroles</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="B127" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="C127" t="str">
         <f t="shared" si="6"/>
-        <v>Más escuchado</v>
+        <v>Marzo</v>
       </c>
       <c r="D127" t="str">
         <f t="shared" si="6"/>
-        <v>Les plus écoutés</v>
+        <v>Mars</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="B128" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="C128" t="str">
         <f t="shared" si="6"/>
-        <v>Álbumes más escuchados</v>
+        <v>Mayo</v>
       </c>
       <c r="D128" t="str">
         <f t="shared" si="6"/>
-        <v>Albums les plus écoutés</v>
+        <v>Mai</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>252</v>
+        <v>461</v>
       </c>
       <c r="B129" t="s">
-        <v>253</v>
+        <v>462</v>
       </c>
       <c r="C129" t="str">
         <f t="shared" si="6"/>
-        <v>Artistas más escuchados</v>
+        <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D129" t="str">
         <f t="shared" si="6"/>
-        <v>Artistes les plus écoutés</v>
+        <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="B130" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="C130" t="str">
         <f t="shared" si="6"/>
-        <v>Canciones más escuchadas</v>
+        <v>Progreso de los medios</v>
       </c>
       <c r="D130" t="str">
         <f t="shared" si="6"/>
-        <v>Chansons les plus écoutées</v>
+        <v>Progrès des médias</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="B131" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="C131" t="str">
         <f t="shared" si="6"/>
-        <v>Nombre</v>
+        <v>Actas</v>
       </c>
       <c r="D131" t="str">
         <f t="shared" si="6"/>
-        <v>Nom</v>
+        <v>Procès-verbal</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="B132" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="C132" t="str">
         <f t="shared" si="6"/>
-        <v>Introducir nueva contraseña</v>
+        <v>Minutos escuchados</v>
       </c>
       <c r="D132" t="str">
         <f t="shared" si="6"/>
-        <v>Entrer un nouveau mot de passe</v>
+        <v>Minutes écoutées</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="B133" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="C133" t="str">
         <f t="shared" si="6"/>
-        <v>Nueva lista de reproducción</v>
+        <v>Minutos escuchados por día</v>
       </c>
       <c r="D133" t="str">
         <f t="shared" si="6"/>
-        <v>Nouvelle playlist</v>
+        <v>Minutes écoutées par jour</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="B134" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C134" t="str">
         <f t="shared" si="6"/>
-        <v>Nuevo nombre de la lista de reproducción</v>
+        <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D134" t="str">
         <f t="shared" si="6"/>
-        <v>Nouveau nom de la playlist</v>
+        <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="B135" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="C135" t="str">
         <f t="shared" si="6"/>
-        <v>Próximos medios</v>
+        <v>Más opciones</v>
       </c>
       <c r="D135" t="str">
         <f t="shared" si="6"/>
-        <v>Médias suivants</v>
+        <v>Plus d’options</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="B136" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="C136" t="str">
         <f t="shared" si="6"/>
-        <v>Todavía no hay álbumes en tu biblioteca</v>
+        <v>Más canciones de</v>
       </c>
       <c r="D136" t="str">
         <f t="shared" si="6"/>
-        <v>Aucun album dans ta bibliothèque pour l’instant</v>
+        <v>Plus de chansons de</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="B137" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="C137" t="str">
         <f t="shared" si="6"/>
-        <v>No hay datos registrados.</v>
+        <v>Más escuchado</v>
       </c>
       <c r="D137" t="str">
         <f t="shared" si="6"/>
-        <v>Aucune donnée enregistrée.</v>
+        <v>Les plus écoutés</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="B138" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="C138" t="str">
         <f t="shared" si="6"/>
-        <v>Letra no disponible</v>
+        <v>Álbumes más escuchados</v>
       </c>
       <c r="D138" t="str">
         <f t="shared" si="6"/>
-        <v>Paroles non disponibles</v>
+        <v>Albums les plus écoutés</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="B139" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="C139" t="str">
         <f t="shared" si="6"/>
-        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
+        <v>Artistas más escuchados</v>
       </c>
       <c r="D139" t="str">
         <f t="shared" si="6"/>
-        <v>Pas encore de playlists dans votre bibliothèque</v>
+        <v>Artistes les plus écoutés</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="B140" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="C140" t="str">
         <f t="shared" si="6"/>
-        <v>No hay repetición</v>
+        <v>Canciones más escuchadas</v>
       </c>
       <c r="D140" t="str">
         <f t="shared" si="6"/>
-        <v>Pas de répétition</v>
+        <v>Chansons les plus écoutées</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="B141" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="C141" t="str">
         <f t="shared" si="6"/>
-        <v>Sin resultados</v>
+        <v>Nombre</v>
       </c>
       <c r="D141" t="str">
         <f t="shared" si="6"/>
-        <v>Aucun résultat</v>
+        <v>Nom</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="B142" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
       <c r="C142" t="str">
         <f t="shared" si="6"/>
-        <v>Sin trabajador de servicios</v>
+        <v>Introducir nueva contraseña</v>
       </c>
       <c r="D142" t="str">
         <f t="shared" si="6"/>
-        <v>Aucun travailleur de services</v>
+        <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="B143" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="C143" t="str">
         <f t="shared" ref="C143:D162" si="7">_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
-        <v>Todavía no hay canciones en tu biblioteca</v>
+        <v>Nueva lista de reproducción</v>
       </c>
       <c r="D143" t="str">
         <f t="shared" si="7"/>
-        <v>Pas encore de chansons dans ta bibliothèque</v>
+        <v>Nouvelle playlist</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="B144" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="C144" t="str">
         <f t="shared" si="7"/>
-        <v>Sin estado</v>
+        <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D144" t="str">
         <f t="shared" si="7"/>
-        <v>Aucun État</v>
+        <v>Nouveau nom de la playlist</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="B145" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
       <c r="C145" t="str">
         <f t="shared" si="7"/>
-        <v>Todavía no hay estaciones en tu biblioteca</v>
+        <v>Próximos medios</v>
       </c>
       <c r="D145" t="str">
         <f t="shared" si="7"/>
-        <v>Pas encore de stations dans votre bibliothèque</v>
+        <v>Médias suivants</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>286</v>
+        <v>266</v>
       </c>
       <c r="B146" t="s">
-        <v>287</v>
+        <v>267</v>
       </c>
       <c r="C146" t="str">
         <f t="shared" si="7"/>
-        <v>Todavía no hay vídeos en tu biblioteca</v>
+        <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
       <c r="D146" t="str">
         <f t="shared" si="7"/>
-        <v>Pas encore de vidéos dans ta bibliothèque</v>
+        <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>288</v>
+        <v>268</v>
       </c>
       <c r="B147" t="s">
-        <v>289</v>
+        <v>269</v>
       </c>
       <c r="C147" t="str">
         <f t="shared" si="7"/>
-        <v>Noviembre</v>
+        <v>No hay datos registrados.</v>
       </c>
       <c r="D147" t="str">
         <f t="shared" si="7"/>
-        <v>Novembre</v>
+        <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="B148" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
       <c r="C148" t="str">
         <f t="shared" si="7"/>
-        <v>Octubre</v>
+        <v>Letra no disponible</v>
       </c>
       <c r="D148" t="str">
         <f t="shared" si="7"/>
-        <v>Octobre</v>
+        <v>Paroles non disponibles</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>292</v>
+        <v>272</v>
       </c>
       <c r="B149" t="s">
-        <v>293</v>
+        <v>273</v>
       </c>
       <c r="C149" t="str">
         <f t="shared" si="7"/>
-        <v>Lista abierta</v>
+        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D149" t="str">
         <f t="shared" si="7"/>
-        <v>Liste ouverte</v>
+        <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>294</v>
+        <v>274</v>
       </c>
       <c r="B150" t="s">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="C150" t="str">
         <f t="shared" si="7"/>
-        <v>Canción abierta</v>
+        <v>No hay repetición</v>
       </c>
       <c r="D150" t="str">
         <f t="shared" si="7"/>
-        <v>Chanson d’ouverture</v>
+        <v>Pas de répétition</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="B151" t="s">
-        <v>297</v>
+        <v>277</v>
       </c>
       <c r="C151" t="str">
         <f t="shared" si="7"/>
-        <v>Partido</v>
+        <v>Sin resultados</v>
       </c>
       <c r="D151" t="str">
         <f t="shared" si="7"/>
-        <v>Parti</v>
+        <v>Aucun résultat</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>298</v>
+        <v>278</v>
       </c>
       <c r="B152" t="s">
-        <v>299</v>
+        <v>279</v>
       </c>
       <c r="C152" t="str">
         <f t="shared" si="7"/>
-        <v>Canción de pausa</v>
+        <v>Sin trabajador de servicios</v>
       </c>
       <c r="D152" t="str">
         <f t="shared" si="7"/>
-        <v>Chanson de pause</v>
+        <v>Aucun travailleur de services</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="B153" t="s">
-        <v>301</v>
+        <v>281</v>
       </c>
       <c r="C153" t="str">
         <f t="shared" si="7"/>
-        <v>Solicitudes pendientes</v>
+        <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D153" t="str">
         <f t="shared" si="7"/>
-        <v>Demandes en attente</v>
+        <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>302</v>
+        <v>282</v>
       </c>
       <c r="B154" t="s">
-        <v>303</v>
+        <v>283</v>
       </c>
       <c r="C154" t="str">
         <f t="shared" si="7"/>
-        <v>Pin</v>
+        <v>Sin estado</v>
       </c>
       <c r="D154" t="str">
         <f t="shared" si="7"/>
-        <v>Épingle</v>
+        <v>Aucun État</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>304</v>
+        <v>284</v>
       </c>
       <c r="B155" t="s">
-        <v>305</v>
+        <v>285</v>
       </c>
       <c r="C155" t="str">
         <f t="shared" si="7"/>
-        <v>Listas fijadas</v>
+        <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D155" t="str">
         <f t="shared" si="7"/>
-        <v>Listes épinglées</v>
+        <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>306</v>
+        <v>286</v>
       </c>
       <c r="B156" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="C156" t="str">
         <f t="shared" si="7"/>
-        <v>Título del álbum</v>
+        <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D156" t="str">
         <f t="shared" si="7"/>
-        <v>Titre de l’album</v>
+        <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="B157" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="C157" t="str">
         <f t="shared" si="7"/>
-        <v>Nombre artístico</v>
+        <v>Noviembre</v>
       </c>
       <c r="D157" t="str">
         <f t="shared" si="7"/>
-        <v>Nom de l’artiste</v>
+        <v>Novembre</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="B158" t="s">
-        <v>311</v>
+        <v>291</v>
       </c>
       <c r="C158" t="str">
         <f t="shared" si="7"/>
-        <v>Mi lista de reproducción perfecta</v>
+        <v>Octubre</v>
       </c>
       <c r="D158" t="str">
         <f t="shared" si="7"/>
-        <v>Ma playlist parfaite</v>
+        <v>Octobre</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="B159" t="s">
-        <v>313</v>
+        <v>293</v>
       </c>
       <c r="C159" t="str">
         <f t="shared" si="7"/>
-        <v>Título de la canción</v>
+        <v>Lista abierta</v>
       </c>
       <c r="D159" t="str">
         <f t="shared" si="7"/>
-        <v>Titre de la chanson</v>
+        <v>Liste ouverte</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="B160" t="s">
-        <v>315</v>
+        <v>295</v>
       </c>
       <c r="C160" t="str">
         <f t="shared" si="7"/>
-        <v>Lista de reproducción</v>
+        <v>Canción abierta</v>
       </c>
       <c r="D160" t="str">
         <f t="shared" si="7"/>
-        <v>Liste des jeux</v>
+        <v>Chanson d’ouverture</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="B161" t="s">
-        <v>317</v>
+        <v>297</v>
       </c>
       <c r="C161" t="str">
         <f t="shared" si="7"/>
-        <v>Reproducir medios</v>
+        <v>Partido</v>
       </c>
       <c r="D161" t="str">
         <f t="shared" si="7"/>
-        <v>Lire les médias</v>
+        <v>Parti</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="B162" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="C162" t="str">
         <f t="shared" si="7"/>
-        <v>Juego a continuación</v>
+        <v>Canción de pausa</v>
       </c>
       <c r="D162" t="str">
         <f t="shared" si="7"/>
-        <v>À jouer à venir</v>
+        <v>Chanson de pause</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="B163" t="s">
-        <v>321</v>
+        <v>301</v>
       </c>
       <c r="C163" t="str">
         <f t="shared" ref="C163:D182" si="8">_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
-        <v>Tocar canción</v>
+        <v>Solicitudes pendientes</v>
       </c>
       <c r="D163" t="str">
         <f t="shared" si="8"/>
-        <v>Jouer la chanson</v>
+        <v>Demandes en attente</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>322</v>
+        <v>302</v>
       </c>
       <c r="B164" t="s">
-        <v>323</v>
+        <v>303</v>
       </c>
       <c r="C164" t="str">
         <f t="shared" si="8"/>
-        <v>Listas de reproducción</v>
+        <v>Pin</v>
       </c>
       <c r="D164" t="str">
         <f t="shared" si="8"/>
-        <v>Playlists</v>
+        <v>Épingle</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>324</v>
+        <v>304</v>
       </c>
       <c r="B165" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C165" t="str">
         <f t="shared" si="8"/>
-        <v>Medios anteriores</v>
+        <v>Listas fijadas</v>
       </c>
       <c r="D165" t="str">
         <f t="shared" si="8"/>
-        <v>Médias précédents</v>
+        <v>Listes épinglées</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>326</v>
+        <v>306</v>
       </c>
       <c r="B166" t="s">
-        <v>327</v>
+        <v>307</v>
       </c>
       <c r="C166" t="str">
         <f t="shared" si="8"/>
-        <v>Selecciones rápidas</v>
+        <v>Título del álbum</v>
       </c>
       <c r="D166" t="str">
         <f t="shared" si="8"/>
-        <v>Choix rapides</v>
+        <v>Titre de l’album</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>328</v>
+        <v>308</v>
       </c>
       <c r="B167" t="s">
-        <v>329</v>
+        <v>309</v>
       </c>
       <c r="C167" t="str">
         <f t="shared" si="8"/>
-        <v>Radio</v>
+        <v>Nombre artístico</v>
       </c>
       <c r="D167" t="str">
         <f t="shared" si="8"/>
-        <v>Radio</v>
+        <v>Nom de l’artiste</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
       <c r="B168" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="C168" t="str">
         <f t="shared" si="8"/>
-        <v>No se han encontrado estaciones</v>
+        <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D168" t="str">
         <f t="shared" si="8"/>
-        <v>Aucune station trouvée</v>
+        <v>Ma playlist parfaite</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
       <c r="B169" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C169" t="str">
         <f t="shared" si="8"/>
-        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
+        <v>Título de la canción</v>
       </c>
       <c r="D169" t="str">
         <f t="shared" si="8"/>
-        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
+        <v>Titre de la chanson</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>334</v>
+        <v>453</v>
       </c>
       <c r="B170" t="s">
-        <v>335</v>
+        <v>454</v>
       </c>
       <c r="C170" t="str">
         <f t="shared" si="8"/>
-        <v>Busca emisoras, géneros, países...</v>
+        <v>Juego</v>
       </c>
       <c r="D170" t="str">
         <f t="shared" si="8"/>
-        <v>Recherche des stations, genres, pays...</v>
+        <v>Jeu</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>336</v>
+        <v>314</v>
       </c>
       <c r="B171" t="s">
-        <v>337</v>
+        <v>315</v>
       </c>
       <c r="C171" t="str">
         <f t="shared" si="8"/>
-        <v>Emisoras de radio</v>
+        <v>Lista de reproducción</v>
       </c>
       <c r="D171" t="str">
         <f t="shared" si="8"/>
-        <v>Radio Stations</v>
+        <v>Liste des jeux</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>338</v>
+        <v>316</v>
       </c>
       <c r="B172" t="s">
-        <v>339</v>
+        <v>317</v>
       </c>
       <c r="C172" t="str">
         <f t="shared" si="8"/>
-        <v>Mezcla reciente</v>
+        <v>Reproducir medios</v>
       </c>
       <c r="D172" t="str">
         <f t="shared" si="8"/>
-        <v>Mix récent</v>
+        <v>Lire les médias</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>340</v>
+        <v>318</v>
       </c>
       <c r="B173" t="s">
-        <v>341</v>
+        <v>319</v>
       </c>
       <c r="C173" t="str">
         <f t="shared" si="8"/>
-        <v>Jugado recientemente</v>
+        <v>Juego a continuación</v>
       </c>
       <c r="D173" t="str">
         <f t="shared" si="8"/>
-        <v>Joué récemment</v>
+        <v>À jouer à venir</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>342</v>
+        <v>320</v>
       </c>
       <c r="B174" t="s">
-        <v>343</v>
+        <v>321</v>
       </c>
       <c r="C174" t="str">
         <f t="shared" si="8"/>
-        <v>Jugado recientemente</v>
+        <v>Tocar canción</v>
       </c>
       <c r="D174" t="str">
         <f t="shared" si="8"/>
-        <v>Récemment joué</v>
+        <v>Jouer la chanson</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
       <c r="B175" t="s">
-        <v>345</v>
+        <v>323</v>
       </c>
       <c r="C175" t="str">
         <f t="shared" si="8"/>
-        <v>Registro</v>
+        <v>Listas de reproducción</v>
       </c>
       <c r="D175" t="str">
         <f t="shared" si="8"/>
-        <v>Registre</v>
+        <v>Playlists</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>346</v>
+        <v>324</v>
       </c>
       <c r="B176" t="s">
-        <v>347</v>
+        <v>325</v>
       </c>
       <c r="C176" t="str">
         <f t="shared" si="8"/>
-        <v>Registrado</v>
+        <v>Medios anteriores</v>
       </c>
       <c r="D176" t="str">
         <f t="shared" si="8"/>
-        <v>Enregistré</v>
+        <v>Médias précédents</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>348</v>
+        <v>326</v>
       </c>
       <c r="B177" t="s">
-        <v>349</v>
+        <v>327</v>
       </c>
       <c r="C177" t="str">
         <f t="shared" si="8"/>
-        <v>Registrando...</v>
+        <v>Selecciones rápidas</v>
       </c>
       <c r="D177" t="str">
         <f t="shared" si="8"/>
-        <v>Enregistrement...</v>
+        <v>Choix rapides</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="B178" t="s">
-        <v>351</v>
+        <v>329</v>
       </c>
       <c r="C178" t="str">
         <f t="shared" si="8"/>
-        <v>Artistas relacionados</v>
+        <v>Radio</v>
       </c>
       <c r="D178" t="str">
         <f t="shared" si="8"/>
-        <v>Artistes associés</v>
+        <v>Radio</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
       <c r="B179" t="s">
-        <v>353</v>
+        <v>331</v>
       </c>
       <c r="C179" t="str">
         <f t="shared" si="8"/>
-        <v>Relajado</v>
+        <v>No se han encontrado estaciones</v>
       </c>
       <c r="D179" t="str">
         <f t="shared" si="8"/>
-        <v>Détendu</v>
+        <v>Aucune station trouvée</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>354</v>
+        <v>332</v>
       </c>
       <c r="B180" t="s">
-        <v>355</v>
+        <v>333</v>
       </c>
       <c r="C180" t="str">
         <f t="shared" si="8"/>
-        <v>Eliminar de la biblioteca</v>
+        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D180" t="str">
         <f t="shared" si="8"/>
-        <v>Retirer de la bibliothèque</v>
+        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>356</v>
+        <v>334</v>
       </c>
       <c r="B181" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="C181" t="str">
         <f t="shared" si="8"/>
-        <v>Quitar de me gusta</v>
+        <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D181" t="str">
         <f t="shared" si="8"/>
-        <v>Retirer de aimé</v>
+        <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>358</v>
+        <v>336</v>
       </c>
       <c r="B182" t="s">
-        <v>359</v>
+        <v>337</v>
       </c>
       <c r="C182" t="str">
         <f t="shared" si="8"/>
-        <v>Eliminar de la lista de reproducción</v>
+        <v>Emisoras de radio</v>
       </c>
       <c r="D182" t="str">
         <f t="shared" si="8"/>
-        <v>Supprimer de la playlist</v>
+        <v>Radio Stations</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>360</v>
+        <v>338</v>
       </c>
       <c r="B183" t="s">
-        <v>361</v>
+        <v>339</v>
       </c>
       <c r="C183" t="str">
         <f t="shared" ref="C183:D202" si="9">_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
-        <v>Eliminar de la cola</v>
+        <v>Mezcla reciente</v>
       </c>
       <c r="D183" t="str">
         <f t="shared" si="9"/>
-        <v>Retirer de la file d’attente</v>
+        <v>Mix récent</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>362</v>
+        <v>340</v>
       </c>
       <c r="B184" t="s">
-        <v>363</v>
+        <v>341</v>
       </c>
       <c r="C184" t="str">
         <f t="shared" si="9"/>
-        <v>Repite todo</v>
+        <v>Jugado recientemente</v>
       </c>
       <c r="D184" t="str">
         <f t="shared" si="9"/>
-        <v>Répétez tout</v>
+        <v>Joué récemment</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>364</v>
+        <v>342</v>
       </c>
       <c r="B185" t="s">
-        <v>365</v>
+        <v>343</v>
       </c>
       <c r="C185" t="str">
         <f t="shared" si="9"/>
-        <v>Repite una</v>
+        <v>Jugado recientemente</v>
       </c>
       <c r="D185" t="str">
         <f t="shared" si="9"/>
-        <v>Répétez-en un</v>
+        <v>Récemment joué</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>366</v>
+        <v>344</v>
       </c>
       <c r="B186" t="s">
-        <v>367</v>
+        <v>345</v>
       </c>
       <c r="C186" t="str">
         <f t="shared" si="9"/>
-        <v>Repetir nueva contraseña</v>
+        <v>Registro</v>
       </c>
       <c r="D186" t="str">
         <f t="shared" si="9"/>
-        <v>Répéter le nouveau mot de passe</v>
+        <v>Registre</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>368</v>
+        <v>346</v>
       </c>
       <c r="B187" t="s">
-        <v>369</v>
+        <v>347</v>
       </c>
       <c r="C187" t="str">
         <f t="shared" si="9"/>
-        <v>Guardando...</v>
+        <v>Registrado</v>
       </c>
       <c r="D187" t="str">
         <f t="shared" si="9"/>
-        <v>Sauver...</v>
+        <v>Enregistré</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>370</v>
+        <v>348</v>
       </c>
       <c r="B188" t="s">
-        <v>371</v>
+        <v>349</v>
       </c>
       <c r="C188" t="str">
         <f t="shared" si="9"/>
-        <v>Búsqueda</v>
+        <v>Registrando...</v>
       </c>
       <c r="D188" t="str">
         <f t="shared" si="9"/>
-        <v>Recherche</v>
+        <v>Enregistrement...</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>372</v>
+        <v>350</v>
       </c>
       <c r="B189" t="s">
-        <v>373</v>
+        <v>351</v>
       </c>
       <c r="C189" t="str">
         <f t="shared" si="9"/>
-        <v>Busca artistas, canciones, álbumes...</v>
+        <v>Artistas relacionados</v>
       </c>
       <c r="D189" t="str">
         <f t="shared" si="9"/>
-        <v>Cherche des artistes, des chansons, des albums...</v>
+        <v>Artistes associés</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>374</v>
+        <v>352</v>
       </c>
       <c r="B190" t="s">
-        <v>375</v>
+        <v>353</v>
       </c>
       <c r="C190" t="str">
         <f t="shared" si="9"/>
-        <v>Parece que el silencio también es música...</v>
+        <v>Relajado</v>
       </c>
       <c r="D190" t="str">
         <f t="shared" si="9"/>
-        <v>Il semble que le silence soit aussi de la musique...</v>
+        <v>Détendu</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>376</v>
+        <v>354</v>
       </c>
       <c r="B191" t="s">
-        <v>377</v>
+        <v>355</v>
       </c>
       <c r="C191" t="str">
         <f t="shared" si="9"/>
-        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
+        <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D191" t="str">
         <f t="shared" si="9"/>
-        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
+        <v>Retirer de la bibliothèque</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>378</v>
+        <v>356</v>
       </c>
       <c r="B192" t="s">
-        <v>379</v>
+        <v>357</v>
       </c>
       <c r="C192" t="str">
         <f t="shared" si="9"/>
-        <v>Buscar en la biblioteca</v>
+        <v>Quitar de me gusta</v>
       </c>
       <c r="D192" t="str">
         <f t="shared" si="9"/>
-        <v>Recherche dans la bibliothèque</v>
+        <v>Retirer de aimé</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>380</v>
+        <v>358</v>
       </c>
       <c r="B193" t="s">
-        <v>381</v>
+        <v>359</v>
       </c>
       <c r="C193" t="str">
         <f t="shared" si="9"/>
-        <v>Usuarios de búsqueda</v>
+        <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D193" t="str">
         <f t="shared" si="9"/>
-        <v>Rechercher les utilisateurs</v>
+        <v>Supprimer de la playlist</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>382</v>
+        <v>360</v>
       </c>
       <c r="B194" t="s">
-        <v>383</v>
+        <v>361</v>
       </c>
       <c r="C194" t="str">
         <f t="shared" si="9"/>
-        <v>Enviar canción actual</v>
+        <v>Eliminar de la cola</v>
       </c>
       <c r="D194" t="str">
         <f t="shared" si="9"/>
-        <v>Envoyer la chanson actuelle</v>
+        <v>Retirer de la file d’attente</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>384</v>
+        <v>362</v>
       </c>
       <c r="B195" t="s">
-        <v>385</v>
+        <v>363</v>
       </c>
       <c r="C195" t="str">
         <f t="shared" si="9"/>
-        <v>Septiembre</v>
+        <v>Repite todo</v>
       </c>
       <c r="D195" t="str">
         <f t="shared" si="9"/>
-        <v>Septembre</v>
+        <v>Répétez tout</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>386</v>
+        <v>364</v>
       </c>
       <c r="B196" t="s">
-        <v>60</v>
+        <v>365</v>
       </c>
       <c r="C196" t="str">
         <f t="shared" si="9"/>
-        <v>Escenarios</v>
+        <v>Repite una</v>
       </c>
       <c r="D196" t="str">
         <f t="shared" si="9"/>
-        <v>Décors</v>
+        <v>Répétez-en un</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>387</v>
+        <v>366</v>
       </c>
       <c r="B197" t="s">
-        <v>388</v>
+        <v>367</v>
       </c>
       <c r="C197" t="str">
         <f t="shared" si="9"/>
-        <v>Compartir canción</v>
+        <v>Repetir nueva contraseña</v>
       </c>
       <c r="D197" t="str">
         <f t="shared" si="9"/>
-        <v>Partager la chanson</v>
+        <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>389</v>
+        <v>457</v>
       </c>
       <c r="B198" t="s">
-        <v>390</v>
+        <v>458</v>
       </c>
       <c r="C198" t="str">
         <f t="shared" si="9"/>
-        <v>Canciones compartidas para ti</v>
+        <v>Regreso a casa</v>
       </c>
       <c r="D198" t="str">
         <f t="shared" si="9"/>
-        <v>Chansons partagées pour vous</v>
+        <v>Retour à la maison</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>391</v>
+        <v>368</v>
       </c>
       <c r="B199" t="s">
-        <v>392</v>
+        <v>369</v>
       </c>
       <c r="C199" t="str">
         <f t="shared" si="9"/>
-        <v>Compartido desde</v>
+        <v>Guardando...</v>
       </c>
       <c r="D199" t="str">
         <f t="shared" si="9"/>
-        <v>Partagé depuis</v>
+        <v>Sauver...</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>393</v>
+        <v>370</v>
       </c>
       <c r="B200" t="s">
-        <v>394</v>
+        <v>371</v>
       </c>
       <c r="C200" t="str">
         <f t="shared" si="9"/>
-        <v>Mostrando datos de</v>
+        <v>Búsqueda</v>
       </c>
       <c r="D200" t="str">
         <f t="shared" si="9"/>
-        <v>Affichage des données de</v>
+        <v>Recherche</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>395</v>
+        <v>372</v>
       </c>
       <c r="B201" t="s">
-        <v>396</v>
+        <v>373</v>
       </c>
       <c r="C201" t="str">
         <f t="shared" si="9"/>
-        <v>Canción</v>
+        <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D201" t="str">
         <f t="shared" si="9"/>
-        <v>Chanson</v>
+        <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="B202" t="s">
-        <v>398</v>
+        <v>375</v>
       </c>
       <c r="C202" t="str">
         <f t="shared" si="9"/>
-        <v>Canciones</v>
+        <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D202" t="str">
         <f t="shared" si="9"/>
-        <v>Chansons</v>
+        <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>399</v>
+        <v>376</v>
       </c>
       <c r="B203" t="s">
-        <v>400</v>
+        <v>377</v>
       </c>
       <c r="C203" t="str">
         <f t="shared" ref="C203:D222" si="10">_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
-        <v>Canciones Solo para ti</v>
+        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D203" t="str">
         <f t="shared" si="10"/>
-        <v>Chansons juste pour toi</v>
+        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>401</v>
+        <v>378</v>
       </c>
       <c r="B204" t="s">
-        <v>402</v>
+        <v>379</v>
       </c>
       <c r="C204" t="str">
         <f t="shared" si="10"/>
-        <v>Canciones de</v>
+        <v>Buscar en la biblioteca</v>
       </c>
       <c r="D204" t="str">
         <f t="shared" si="10"/>
-        <v>Chansons de</v>
+        <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>403</v>
+        <v>380</v>
       </c>
       <c r="B205" t="s">
-        <v>404</v>
+        <v>381</v>
       </c>
       <c r="C205" t="str">
         <f t="shared" si="10"/>
-        <v>Canciones escuchadas</v>
+        <v>Usuarios de búsqueda</v>
       </c>
       <c r="D205" t="str">
         <f t="shared" si="10"/>
-        <v>Chansons écoutées</v>
+        <v>Rechercher les utilisateurs</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>405</v>
+        <v>382</v>
       </c>
       <c r="B206" t="s">
-        <v>406</v>
+        <v>383</v>
       </c>
       <c r="C206" t="str">
         <f t="shared" si="10"/>
-        <v>Estadísticas</v>
+        <v>Enviar canción actual</v>
       </c>
       <c r="D206" t="str">
         <f t="shared" si="10"/>
-        <v>Statistiques</v>
+        <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="B207" t="s">
-        <v>408</v>
+        <v>385</v>
       </c>
       <c r="C207" t="str">
         <f t="shared" si="10"/>
-        <v>Estadísticas</v>
+        <v>Septiembre</v>
       </c>
       <c r="D207" t="str">
         <f t="shared" si="10"/>
-        <v>Statistiques</v>
+        <v>Septembre</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>409</v>
+        <v>386</v>
       </c>
       <c r="B208" t="s">
-        <v>410</v>
-      </c>
-      <c r="C208" t="s">
-        <v>459</v>
+        <v>60</v>
+      </c>
+      <c r="C208" t="str">
+        <f t="shared" si="10"/>
+        <v>Escenarios</v>
       </c>
       <c r="D208" t="str">
         <f t="shared" si="10"/>
-        <v>Arrête</v>
+        <v>Décors</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>411</v>
+        <v>387</v>
       </c>
       <c r="B209" t="s">
-        <v>412</v>
+        <v>388</v>
       </c>
       <c r="C209" t="str">
         <f t="shared" si="10"/>
-        <v>a</v>
+        <v>Compartir canción</v>
       </c>
       <c r="D209" t="str">
         <f t="shared" si="10"/>
-        <v>à</v>
+        <v>Partager la chanson</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>413</v>
+        <v>389</v>
       </c>
       <c r="B210" t="s">
-        <v>414</v>
+        <v>390</v>
       </c>
       <c r="C210" t="str">
         <f t="shared" si="10"/>
-        <v>Álbumes destacados</v>
+        <v>Canciones compartidas para ti</v>
       </c>
       <c r="D210" t="str">
         <f t="shared" si="10"/>
-        <v>Albums phares</v>
+        <v>Chansons partagées pour vous</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>415</v>
+        <v>391</v>
       </c>
       <c r="B211" t="s">
-        <v>416</v>
+        <v>392</v>
       </c>
       <c r="C211" t="str">
         <f t="shared" si="10"/>
-        <v>Canciones principales</v>
+        <v>Compartido desde</v>
       </c>
       <c r="D211" t="str">
         <f t="shared" si="10"/>
-        <v>Meilleures chansons</v>
+        <v>Partagé depuis</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>417</v>
+        <v>393</v>
       </c>
       <c r="B212" t="s">
-        <v>418</v>
+        <v>394</v>
       </c>
       <c r="C212" t="str">
         <f t="shared" si="10"/>
-        <v>Desclavar</v>
+        <v>Mostrando datos de</v>
       </c>
       <c r="D212" t="str">
         <f t="shared" si="10"/>
-        <v>Détacher</v>
+        <v>Affichage des données de</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>419</v>
+        <v>395</v>
       </c>
       <c r="B213" t="s">
-        <v>420</v>
+        <v>396</v>
       </c>
       <c r="C213" t="str">
         <f t="shared" si="10"/>
-        <v>Desregistrar</v>
+        <v>Canción</v>
       </c>
       <c r="D213" t="str">
         <f t="shared" si="10"/>
-        <v>Désinscription</v>
+        <v>Chanson</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>421</v>
+        <v>397</v>
       </c>
       <c r="B214" t="s">
-        <v>422</v>
+        <v>398</v>
       </c>
       <c r="C214" t="str">
         <f t="shared" si="10"/>
-        <v>No registrado</v>
+        <v>Canciones</v>
       </c>
       <c r="D214" t="str">
         <f t="shared" si="10"/>
-        <v>Non enregistré</v>
+        <v>Chansons</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>423</v>
+        <v>399</v>
       </c>
       <c r="B215" t="s">
-        <v>424</v>
+        <v>400</v>
       </c>
       <c r="C215" t="str">
         <f t="shared" si="10"/>
-        <v>Dejar de registrarse...</v>
+        <v>Canciones Solo para ti</v>
       </c>
       <c r="D215" t="str">
         <f t="shared" si="10"/>
-        <v>Désenregistrement...</v>
+        <v>Chansons juste pour toi</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>425</v>
+        <v>401</v>
       </c>
       <c r="B216" t="s">
-        <v>426</v>
+        <v>402</v>
       </c>
       <c r="C216" t="str">
         <f t="shared" si="10"/>
-        <v>Actualización</v>
+        <v>Canciones de</v>
       </c>
       <c r="D216" t="str">
         <f t="shared" si="10"/>
-        <v>Mise à jour</v>
+        <v>Chansons de</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>427</v>
+        <v>403</v>
       </c>
       <c r="B217" t="s">
-        <v>428</v>
+        <v>404</v>
       </c>
       <c r="C217" t="str">
         <f t="shared" si="10"/>
-        <v>Actualizando...</v>
+        <v>Canciones escuchadas</v>
       </c>
       <c r="D217" t="str">
         <f t="shared" si="10"/>
-        <v>Mise à jour...</v>
+        <v>Chansons écoutées</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>429</v>
+        <v>405</v>
       </c>
       <c r="B218" t="s">
-        <v>430</v>
+        <v>406</v>
       </c>
       <c r="C218" t="str">
         <f t="shared" si="10"/>
-        <v>Subida</v>
+        <v>Estadísticas</v>
       </c>
       <c r="D218" t="str">
         <f t="shared" si="10"/>
-        <v>Téléverser</v>
+        <v>Statistiques</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>431</v>
+        <v>407</v>
       </c>
       <c r="B219" t="s">
-        <v>432</v>
+        <v>408</v>
       </c>
       <c r="C219" t="str">
         <f t="shared" si="10"/>
-        <v>Usuario</v>
+        <v>Estadísticas</v>
       </c>
       <c r="D219" t="str">
         <f t="shared" si="10"/>
-        <v>Utilisateur</v>
+        <v>Statistiques</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>433</v>
+        <v>409</v>
       </c>
       <c r="B220" t="s">
-        <v>434</v>
+        <v>410</v>
       </c>
       <c r="C220" t="str">
         <f t="shared" si="10"/>
-        <v>Configuración de usuario</v>
+        <v>¡Para</v>
       </c>
       <c r="D220" t="str">
         <f t="shared" si="10"/>
-        <v>Paramètres utilisateur</v>
+        <v>Arrête</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>435</v>
+        <v>411</v>
       </c>
       <c r="B221" t="s">
-        <v>436</v>
+        <v>412</v>
       </c>
       <c r="C221" t="str">
         <f t="shared" si="10"/>
-        <v>Estadísticas de usuario</v>
+        <v>a</v>
       </c>
       <c r="D221" t="str">
         <f t="shared" si="10"/>
-        <v>Statistiques des utilisateurs</v>
+        <v>à</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>437</v>
+        <v>459</v>
       </c>
       <c r="B222" t="s">
-        <v>438</v>
+        <v>460</v>
       </c>
       <c r="C222" t="str">
         <f t="shared" si="10"/>
-        <v>Usuarios y amigos</v>
+        <v>ToDo</v>
       </c>
       <c r="D222" t="str">
         <f t="shared" si="10"/>
-        <v>Utilisateurs et amis</v>
+        <v>ToDo</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>439</v>
+        <v>413</v>
       </c>
       <c r="B223" t="s">
-        <v>440</v>
+        <v>414</v>
       </c>
       <c r="C223" t="str">
-        <f t="shared" ref="C223:D232" si="11">_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
-        <v>Lista de usuarios</v>
+        <f t="shared" ref="C223:D242" si="11">_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
+        <v>Álbumes destacados</v>
       </c>
       <c r="D223" t="str">
         <f t="shared" si="11"/>
-        <v>Liste des utilisateurs</v>
+        <v>Albums phares</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>441</v>
+        <v>415</v>
       </c>
       <c r="B224" t="s">
-        <v>442</v>
+        <v>416</v>
       </c>
       <c r="C224" t="str">
         <f t="shared" si="11"/>
-        <v>Vídeos</v>
+        <v>Canciones principales</v>
       </c>
       <c r="D224" t="str">
         <f t="shared" si="11"/>
-        <v>Vidéos</v>
+        <v>Meilleures chansons</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>443</v>
+        <v>417</v>
       </c>
       <c r="B225" t="s">
-        <v>444</v>
+        <v>418</v>
       </c>
       <c r="C225" t="str">
         <f t="shared" si="11"/>
-        <v>También puede que te interese</v>
+        <v>Desclavar</v>
       </c>
       <c r="D225" t="str">
         <f t="shared" si="11"/>
-        <v>Ça pourrait aussi te plaire</v>
+        <v>Détacher</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>445</v>
+        <v>419</v>
       </c>
       <c r="B226" t="s">
-        <v>446</v>
+        <v>420</v>
       </c>
       <c r="C226" t="str">
         <f t="shared" si="11"/>
-        <v>Tu</v>
+        <v>Desregistrar</v>
       </c>
       <c r="D226" t="str">
         <f t="shared" si="11"/>
-        <v>Votre</v>
+        <v>Désinscription</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>447</v>
+        <v>421</v>
       </c>
       <c r="B227" t="s">
-        <v>448</v>
+        <v>422</v>
       </c>
       <c r="C227" t="str">
         <f t="shared" si="11"/>
-        <v>Tus álbumes y listas de reproducción</v>
+        <v>No registrado</v>
       </c>
       <c r="D227" t="str">
         <f t="shared" si="11"/>
-        <v>Vos albums et playlists</v>
+        <v>Non enregistré</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>449</v>
+        <v>423</v>
       </c>
       <c r="B228" t="s">
-        <v>450</v>
+        <v>424</v>
       </c>
       <c r="C228" t="str">
         <f t="shared" si="11"/>
-        <v>Tu mezcla</v>
+        <v>Dejar de registrarse...</v>
       </c>
       <c r="D228" t="str">
         <f t="shared" si="11"/>
-        <v>Votre Mix</v>
+        <v>Désenregistrement...</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>451</v>
+        <v>425</v>
       </c>
       <c r="B229" t="s">
-        <v>452</v>
+        <v>426</v>
       </c>
       <c r="C229" t="str">
         <f t="shared" si="11"/>
-        <v>Vídeos de YouTube</v>
+        <v>Actualización</v>
       </c>
       <c r="D229" t="str">
         <f t="shared" si="11"/>
-        <v>Vidéos YouTube</v>
+        <v>Mise à jour</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>453</v>
+        <v>427</v>
       </c>
       <c r="B230" t="s">
-        <v>454</v>
+        <v>428</v>
       </c>
       <c r="C230" t="str">
         <f t="shared" si="11"/>
-        <v>Juego</v>
+        <v>Actualizando...</v>
       </c>
       <c r="D230" t="str">
         <f t="shared" si="11"/>
-        <v>Jeu</v>
+        <v>Mise à jour...</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>455</v>
+        <v>429</v>
       </c>
       <c r="B231" t="s">
-        <v>456</v>
+        <v>430</v>
       </c>
       <c r="C231" t="str">
         <f t="shared" si="11"/>
-        <v>Añadir medios a la lista de reproducción</v>
+        <v>Subida</v>
       </c>
       <c r="D231" t="str">
         <f t="shared" si="11"/>
-        <v>Ajouter un média à une playlist</v>
+        <v>Téléverser</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>457</v>
+        <v>431</v>
       </c>
       <c r="B232" t="s">
-        <v>458</v>
+        <v>432</v>
       </c>
       <c r="C232" t="str">
         <f t="shared" si="11"/>
-        <v>Regreso a casa</v>
+        <v>Usuario</v>
       </c>
       <c r="D232" t="str">
         <f t="shared" si="11"/>
-        <v>Retour à la maison</v>
+        <v>Utilisateur</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>433</v>
+      </c>
+      <c r="B233" t="s">
+        <v>434</v>
+      </c>
+      <c r="C233" t="str">
+        <f t="shared" si="11"/>
+        <v>Configuración de usuario</v>
+      </c>
+      <c r="D233" t="str">
+        <f t="shared" si="11"/>
+        <v>Paramètres utilisateur</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>435</v>
+      </c>
+      <c r="B234" t="s">
+        <v>436</v>
+      </c>
+      <c r="C234" t="str">
+        <f t="shared" si="11"/>
+        <v>Estadísticas de usuario</v>
+      </c>
+      <c r="D234" t="str">
+        <f t="shared" si="11"/>
+        <v>Statistiques des utilisateurs</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>437</v>
+      </c>
+      <c r="B235" t="s">
+        <v>438</v>
+      </c>
+      <c r="C235" t="str">
+        <f t="shared" si="11"/>
+        <v>Usuarios y amigos</v>
+      </c>
+      <c r="D235" t="str">
+        <f t="shared" si="11"/>
+        <v>Utilisateurs et amis</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>439</v>
+      </c>
+      <c r="B236" t="s">
+        <v>440</v>
+      </c>
+      <c r="C236" t="str">
+        <f t="shared" si="11"/>
+        <v>Lista de usuarios</v>
+      </c>
+      <c r="D236" t="str">
+        <f t="shared" si="11"/>
+        <v>Liste des utilisateurs</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>441</v>
+      </c>
+      <c r="B237" t="s">
+        <v>442</v>
+      </c>
+      <c r="C237" t="str">
+        <f t="shared" si="11"/>
+        <v>Vídeos</v>
+      </c>
+      <c r="D237" t="str">
+        <f t="shared" si="11"/>
+        <v>Vidéos</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>443</v>
+      </c>
+      <c r="B238" t="s">
+        <v>444</v>
+      </c>
+      <c r="C238" t="str">
+        <f t="shared" si="11"/>
+        <v>También puede que te interese</v>
+      </c>
+      <c r="D238" t="str">
+        <f t="shared" si="11"/>
+        <v>Ça pourrait aussi te plaire</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>445</v>
+      </c>
+      <c r="B239" t="s">
+        <v>446</v>
+      </c>
+      <c r="C239" t="str">
+        <f t="shared" si="11"/>
+        <v>Tu</v>
+      </c>
+      <c r="D239" t="str">
+        <f t="shared" si="11"/>
+        <v>Votre</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>447</v>
+      </c>
+      <c r="B240" t="s">
+        <v>448</v>
+      </c>
+      <c r="C240" t="str">
+        <f t="shared" si="11"/>
+        <v>Tus álbumes y listas de reproducción</v>
+      </c>
+      <c r="D240" t="str">
+        <f t="shared" si="11"/>
+        <v>Vos albums et playlists</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>449</v>
+      </c>
+      <c r="B241" t="s">
+        <v>450</v>
+      </c>
+      <c r="C241" t="str">
+        <f t="shared" si="11"/>
+        <v>Tu mezcla</v>
+      </c>
+      <c r="D241" t="str">
+        <f t="shared" si="11"/>
+        <v>Votre Mix</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>451</v>
+      </c>
+      <c r="B242" t="s">
+        <v>452</v>
+      </c>
+      <c r="C242" t="str">
+        <f t="shared" si="11"/>
+        <v>Vídeos de YouTube</v>
+      </c>
+      <c r="D242" t="str">
+        <f t="shared" si="11"/>
+        <v>Vidéos YouTube</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>479</v>
+      </c>
+      <c r="B243" t="s">
+        <v>480</v>
+      </c>
+      <c r="C243" t="str">
+        <f t="shared" ref="C243:D255" si="12">_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
+        <v>Nueva versión disponible</v>
+      </c>
+      <c r="D243" t="str">
+        <f t="shared" si="12"/>
+        <v>Nouvelle version disponible</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C244" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D244" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C245" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D245" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C246" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D246" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C247" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D247" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C248" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D248" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C249" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D249" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C250" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D250" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C251" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D251" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C252" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D252" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C253" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D253" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C254" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D254" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C255" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="D255" t="str">
+        <f t="shared" si="12"/>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError sqref="C208" calculatedColumn="1"/>
-  </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Update Vocabulary.xlsx with new content
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Documents\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3BF0727-71CB-48A8-9F1B-1A66C47D781D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ABBC3E3-651B-47D2-9C41-85ABEA1D3D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="1170" windowWidth="16410" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="1170" windowWidth="32490" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="483">
   <si>
     <t>KEY</t>
   </si>
@@ -1476,6 +1476,12 @@
   </si>
   <si>
     <t>New version available</t>
+  </si>
+  <si>
+    <t>Reproducir</t>
+  </si>
+  <si>
+    <t>Reproducir a continuación</t>
   </si>
 </sst>
 </file>
@@ -1880,11 +1886,11 @@
         <v>8</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:D22" si="0">_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
       <c r="D3" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B3,$B$2,D$2)</f>
         <v>Ajouter la liste à la file d’attente de façon aléatoire</v>
       </c>
     </row>
@@ -1896,11 +1902,11 @@
         <v>10</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B4,$B$2,C$2)</f>
         <v>Añadir lista al final de la cola</v>
       </c>
       <c r="D4" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B4,$B$2,D$2)</f>
         <v>Ajouter la liste en bas de la file d’attente</v>
       </c>
     </row>
@@ -1912,11 +1918,11 @@
         <v>12</v>
       </c>
       <c r="C5" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B5,$B$2,C$2)</f>
         <v>Añadir lista a la cola</v>
       </c>
       <c r="D5" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B5,$B$2,D$2)</f>
         <v>Ajouter la liste à la file d’attente</v>
       </c>
     </row>
@@ -1928,11 +1934,11 @@
         <v>456</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B6,$B$2,C$2)</f>
         <v>Añadir medios a la lista de reproducción</v>
       </c>
       <c r="D6" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B6,$B$2,D$2)</f>
         <v>Ajouter un média à une playlist</v>
       </c>
     </row>
@@ -1944,11 +1950,11 @@
         <v>14</v>
       </c>
       <c r="C7" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B7,$B$2,C$2)</f>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
       <c r="D7" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B7,$B$2,D$2)</f>
         <v>Ajouter une chanson à la playlist</v>
       </c>
     </row>
@@ -1960,11 +1966,11 @@
         <v>16</v>
       </c>
       <c r="C8" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B8,$B$2,C$2)</f>
         <v>Añadir canción a la cola</v>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B8,$B$2,D$2)</f>
         <v>Ajouter une chanson à la file d’attente</v>
       </c>
     </row>
@@ -1976,11 +1982,11 @@
         <v>18</v>
       </c>
       <c r="C9" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B9,$B$2,C$2)</f>
         <v>Añadir a la biblioteca</v>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B9,$B$2,D$2)</f>
         <v>Ajouter à la bibliothèque</v>
       </c>
     </row>
@@ -1992,11 +1998,11 @@
         <v>20</v>
       </c>
       <c r="C10" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B10,$B$2,C$2)</f>
         <v>Añadir a los que me gusta</v>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B10,$B$2,D$2)</f>
         <v>Ajouter aux aimés</v>
       </c>
     </row>
@@ -2008,11 +2014,11 @@
         <v>22</v>
       </c>
       <c r="C11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B11,$B$2,C$2)</f>
         <v>Añadir a la cola</v>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B11,$B$2,D$2)</f>
         <v>Ajouter à la file d’attente</v>
       </c>
     </row>
@@ -2024,11 +2030,11 @@
         <v>468</v>
       </c>
       <c r="C12" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B12,$B$2,C$2)</f>
         <v>Añadido a la lista de reproducción</v>
       </c>
       <c r="D12" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B12,$B$2,D$2)</f>
         <v>Ajouté à la playlist</v>
       </c>
     </row>
@@ -2040,11 +2046,11 @@
         <v>24</v>
       </c>
       <c r="C13" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B13,$B$2,C$2)</f>
         <v>Añadir Build</v>
       </c>
       <c r="D13" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B13,$B$2,D$2)</f>
         <v>Ajouter une construction</v>
       </c>
     </row>
@@ -2056,11 +2062,11 @@
         <v>26</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B14,$B$2,C$2)</f>
         <v>Archivo APK</v>
       </c>
       <c r="D14" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B14,$B$2,D$2)</f>
         <v>Fichier APK</v>
       </c>
     </row>
@@ -2072,11 +2078,11 @@
         <v>28</v>
       </c>
       <c r="C15" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B15,$B$2,C$2)</f>
         <v>Gestiona tus builds de Android</v>
       </c>
       <c r="D15" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B15,$B$2,D$2)</f>
         <v>Gérez vos versions Android</v>
       </c>
     </row>
@@ -2088,11 +2094,11 @@
         <v>30</v>
       </c>
       <c r="C16" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B16,$B$2,C$2)</f>
         <v>Construcciones</v>
       </c>
       <c r="D16" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B16,$B$2,D$2)</f>
         <v>Constructions</v>
       </c>
     </row>
@@ -2104,11 +2110,11 @@
         <v>32</v>
       </c>
       <c r="C17" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B17,$B$2,C$2)</f>
         <v>Cancelar</v>
       </c>
       <c r="D17" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B17,$B$2,D$2)</f>
         <v>Annuler</v>
       </c>
     </row>
@@ -2120,11 +2126,11 @@
         <v>34</v>
       </c>
       <c r="C18" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B18,$B$2,C$2)</f>
         <v>Descripción</v>
       </c>
       <c r="D18" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B18,$B$2,D$2)</f>
         <v>Description</v>
       </c>
     </row>
@@ -2136,11 +2142,11 @@
         <v>36</v>
       </c>
       <c r="C19" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B19,$B$2,C$2)</f>
         <v>Aquí entra la descripción...</v>
       </c>
       <c r="D19" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B19,$B$2,D$2)</f>
         <v>Voici la description...</v>
       </c>
     </row>
@@ -2152,11 +2158,11 @@
         <v>38</v>
       </c>
       <c r="C20" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B20,$B$2,C$2)</f>
         <v>Enter Version</v>
       </c>
       <c r="D20" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B20,$B$2,D$2)</f>
         <v>Enter Version</v>
       </c>
     </row>
@@ -2168,11 +2174,11 @@
         <v>40</v>
       </c>
       <c r="C21" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B21,$B$2,C$2)</f>
         <v>Últimas novedades</v>
       </c>
       <c r="D21" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B21,$B$2,D$2)</f>
         <v>Dernières nouvelles</v>
       </c>
     </row>
@@ -2184,11 +2190,11 @@
         <v>42</v>
       </c>
       <c r="C22" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B22,$B$2,C$2)</f>
         <v>Aún no hay builds</v>
       </c>
       <c r="D22" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.TRANSLATE($B22,$B$2,D$2)</f>
         <v>Pas encore de builds</v>
       </c>
     </row>
@@ -2200,11 +2206,11 @@
         <v>44</v>
       </c>
       <c r="C23" t="str">
-        <f t="shared" ref="C23:D42" si="1">_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
         <v>Solo APK</v>
       </c>
       <c r="D23" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B23,$B$2,D$2)</f>
         <v>Seul APK</v>
       </c>
     </row>
@@ -2216,11 +2222,11 @@
         <v>46</v>
       </c>
       <c r="C24" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B24,$B$2,C$2)</f>
         <v>Opcional</v>
       </c>
       <c r="D24" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B24,$B$2,D$2)</f>
         <v>Optionnel</v>
       </c>
     </row>
@@ -2232,11 +2238,11 @@
         <v>48</v>
       </c>
       <c r="C25" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B25,$B$2,C$2)</f>
         <v>Leer Fallido</v>
       </c>
       <c r="D25" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B25,$B$2,D$2)</f>
         <v>Lire Échec</v>
       </c>
     </row>
@@ -2248,11 +2254,11 @@
         <v>50</v>
       </c>
       <c r="C26" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B26,$B$2,C$2)</f>
         <v>Obligatorio</v>
       </c>
       <c r="D26" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B26,$B$2,D$2)</f>
         <v>Obligatoire</v>
       </c>
     </row>
@@ -2264,11 +2270,11 @@
         <v>52</v>
       </c>
       <c r="C27" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B27,$B$2,C$2)</f>
         <v>Seleccionar APK</v>
       </c>
       <c r="D27" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B27,$B$2,D$2)</f>
         <v>Sélectionner APK</v>
       </c>
     </row>
@@ -2280,11 +2286,11 @@
         <v>54</v>
       </c>
       <c r="C28" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B28,$B$2,C$2)</f>
         <v>Seleccionados</v>
       </c>
       <c r="D28" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B28,$B$2,D$2)</f>
         <v>Sélectionné</v>
       </c>
     </row>
@@ -2296,11 +2302,11 @@
         <v>56</v>
       </c>
       <c r="C29" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B29,$B$2,C$2)</f>
         <v>Próximamente</v>
       </c>
       <c r="D29" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B29,$B$2,D$2)</f>
         <v>Bientôt</v>
       </c>
     </row>
@@ -2312,11 +2318,11 @@
         <v>58</v>
       </c>
       <c r="C30" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B30,$B$2,C$2)</f>
         <v>Configuración de plataformas</v>
       </c>
       <c r="D30" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B30,$B$2,D$2)</f>
         <v>Réglages de la plateforme</v>
       </c>
     </row>
@@ -2328,11 +2334,11 @@
         <v>60</v>
       </c>
       <c r="C31" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B31,$B$2,C$2)</f>
         <v>Escenarios</v>
       </c>
       <c r="D31" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B31,$B$2,D$2)</f>
         <v>Décors</v>
       </c>
     </row>
@@ -2344,11 +2350,11 @@
         <v>30</v>
       </c>
       <c r="C32" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B32,$B$2,C$2)</f>
         <v>Construcciones</v>
       </c>
       <c r="D32" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B32,$B$2,D$2)</f>
         <v>Constructions</v>
       </c>
     </row>
@@ -2360,11 +2366,11 @@
         <v>60</v>
       </c>
       <c r="C33" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B33,$B$2,C$2)</f>
         <v>Escenarios</v>
       </c>
       <c r="D33" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B33,$B$2,D$2)</f>
         <v>Décors</v>
       </c>
     </row>
@@ -2376,11 +2382,11 @@
         <v>64</v>
       </c>
       <c r="C34" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B34,$B$2,C$2)</f>
         <v>Usuarios</v>
       </c>
       <c r="D34" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B34,$B$2,D$2)</f>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -2392,11 +2398,11 @@
         <v>66</v>
       </c>
       <c r="C35" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B35,$B$2,C$2)</f>
         <v>Compilación de subida</v>
       </c>
       <c r="D35" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B35,$B$2,D$2)</f>
         <v>Upload Build</v>
       </c>
     </row>
@@ -2408,11 +2414,11 @@
         <v>68</v>
       </c>
       <c r="C36" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B36,$B$2,C$2)</f>
         <v>Fallido en la subida</v>
       </c>
       <c r="D36" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B36,$B$2,D$2)</f>
         <v>Téléchargement échoué</v>
       </c>
     </row>
@@ -2424,11 +2430,11 @@
         <v>70</v>
       </c>
       <c r="C37" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B37,$B$2,C$2)</f>
         <v>Sube tu primera construcción</v>
       </c>
       <c r="D37" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B37,$B$2,D$2)</f>
         <v>Téléchargez votre première compilation</v>
       </c>
     </row>
@@ -2440,11 +2446,11 @@
         <v>72</v>
       </c>
       <c r="C38" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B38,$B$2,C$2)</f>
         <v>Subir nueva versión</v>
       </c>
       <c r="D38" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B38,$B$2,D$2)</f>
         <v>Télécharger une nouvelle version</v>
       </c>
     </row>
@@ -2456,11 +2462,11 @@
         <v>74</v>
       </c>
       <c r="C39" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B39,$B$2,C$2)</f>
         <v>Éxito en la subida</v>
       </c>
       <c r="D39" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B39,$B$2,D$2)</f>
         <v>Succès de la télévision</v>
       </c>
     </row>
@@ -2472,11 +2478,11 @@
         <v>76</v>
       </c>
       <c r="C40" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B40,$B$2,C$2)</f>
         <v>Subiendo algo...</v>
       </c>
       <c r="D40" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B40,$B$2,D$2)</f>
         <v>Téléchargement...</v>
       </c>
     </row>
@@ -2488,11 +2494,11 @@
         <v>56</v>
       </c>
       <c r="C41" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B41,$B$2,C$2)</f>
         <v>Próximamente</v>
       </c>
       <c r="D41" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B41,$B$2,D$2)</f>
         <v>Bientôt</v>
       </c>
     </row>
@@ -2504,11 +2510,11 @@
         <v>79</v>
       </c>
       <c r="C42" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B42,$B$2,C$2)</f>
         <v>Gestionar los usuarios de la plataforma</v>
       </c>
       <c r="D42" t="str">
-        <f t="shared" si="1"/>
+        <f>_xlfn.TRANSLATE($B42,$B$2,D$2)</f>
         <v>Gérer les utilisateurs de la plateforme</v>
       </c>
     </row>
@@ -2520,11 +2526,11 @@
         <v>64</v>
       </c>
       <c r="C43" t="str">
-        <f t="shared" ref="C43:D62" si="2">_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
         <v>Usuarios</v>
       </c>
       <c r="D43" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B43,$B$2,D$2)</f>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -2536,11 +2542,11 @@
         <v>82</v>
       </c>
       <c r="C44" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B44,$B$2,C$2)</f>
         <v>Versión</v>
       </c>
       <c r="D44" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B44,$B$2,D$2)</f>
         <v>Version</v>
       </c>
     </row>
@@ -2552,11 +2558,11 @@
         <v>84</v>
       </c>
       <c r="C45" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B45,$B$2,C$2)</f>
         <v>Álbum</v>
       </c>
       <c r="D45" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B45,$B$2,D$2)</f>
         <v>Album</v>
       </c>
     </row>
@@ -2568,11 +2574,11 @@
         <v>86</v>
       </c>
       <c r="C46" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B46,$B$2,C$2)</f>
         <v>Álbumes</v>
       </c>
       <c r="D46" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B46,$B$2,D$2)</f>
         <v>Albums</v>
       </c>
     </row>
@@ -2584,11 +2590,11 @@
         <v>88</v>
       </c>
       <c r="C47" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B47,$B$2,C$2)</f>
         <v>Álbumes y sencillos</v>
       </c>
       <c r="D47" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B47,$B$2,D$2)</f>
         <v>Albums et singles</v>
       </c>
     </row>
@@ -2600,11 +2606,11 @@
         <v>90</v>
       </c>
       <c r="C48" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B48,$B$2,C$2)</f>
         <v>Todos</v>
       </c>
       <c r="D48" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B48,$B$2,D$2)</f>
         <v>Tous</v>
       </c>
     </row>
@@ -2616,11 +2622,11 @@
         <v>92</v>
       </c>
       <c r="C49" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B49,$B$2,C$2)</f>
         <v>Abril</v>
       </c>
       <c r="D49" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B49,$B$2,D$2)</f>
         <v>Avril</v>
       </c>
     </row>
@@ -2632,11 +2638,11 @@
         <v>94</v>
       </c>
       <c r="C50" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B50,$B$2,C$2)</f>
         <v>Artista</v>
       </c>
       <c r="D50" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B50,$B$2,D$2)</f>
         <v>Artiste</v>
       </c>
     </row>
@@ -2648,11 +2654,11 @@
         <v>96</v>
       </c>
       <c r="C51" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B51,$B$2,C$2)</f>
         <v>Artistas</v>
       </c>
       <c r="D51" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B51,$B$2,D$2)</f>
         <v>Artistes</v>
       </c>
     </row>
@@ -2664,11 +2670,11 @@
         <v>98</v>
       </c>
       <c r="C52" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B52,$B$2,C$2)</f>
         <v>Agosto</v>
       </c>
       <c r="D52" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B52,$B$2,D$2)</f>
         <v>Août</v>
       </c>
     </row>
@@ -2680,11 +2686,11 @@
         <v>100</v>
       </c>
       <c r="C53" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B53,$B$2,C$2)</f>
         <v>Minutos medios por canción</v>
       </c>
       <c r="D53" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B53,$B$2,D$2)</f>
         <v>Minutes moyennes par chanson</v>
       </c>
     </row>
@@ -2696,11 +2702,11 @@
         <v>102</v>
       </c>
       <c r="C54" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B54,$B$2,C$2)</f>
         <v>por</v>
       </c>
       <c r="D54" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B54,$B$2,D$2)</f>
         <v>par</v>
       </c>
     </row>
@@ -2712,11 +2718,11 @@
         <v>32</v>
       </c>
       <c r="C55" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B55,$B$2,C$2)</f>
         <v>Cancelar</v>
       </c>
       <c r="D55" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B55,$B$2,D$2)</f>
         <v>Annuler</v>
       </c>
     </row>
@@ -2728,11 +2734,11 @@
         <v>105</v>
       </c>
       <c r="C56" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B56,$B$2,C$2)</f>
         <v>Cambiar contraseña</v>
       </c>
       <c r="D56" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B56,$B$2,D$2)</f>
         <v>Changer le mot de passe</v>
       </c>
     </row>
@@ -2744,11 +2750,11 @@
         <v>107</v>
       </c>
       <c r="C57" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B57,$B$2,C$2)</f>
         <v>Descargas claras</v>
       </c>
       <c r="D57" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B57,$B$2,D$2)</f>
         <v>Téléchargements clairs</v>
       </c>
     </row>
@@ -2760,11 +2766,11 @@
         <v>109</v>
       </c>
       <c r="C58" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B58,$B$2,C$2)</f>
         <v>Haz clic para descargar</v>
       </c>
       <c r="D58" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B58,$B$2,D$2)</f>
         <v>Cliquez pour télécharger</v>
       </c>
     </row>
@@ -2776,11 +2782,11 @@
         <v>111</v>
       </c>
       <c r="C59" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B59,$B$2,C$2)</f>
         <v>Topo comunitario</v>
       </c>
       <c r="D59" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B59,$B$2,D$2)</f>
         <v>Sommet communautaire</v>
       </c>
     </row>
@@ -2792,11 +2798,11 @@
         <v>113</v>
       </c>
       <c r="C60" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B60,$B$2,C$2)</f>
         <v>URL de la lista de copiar</v>
       </c>
       <c r="D60" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B60,$B$2,D$2)</f>
         <v>URL de la liste de copie</v>
       </c>
     </row>
@@ -2808,11 +2814,11 @@
         <v>115</v>
       </c>
       <c r="C61" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B61,$B$2,C$2)</f>
         <v>Copiar la URL de la canción</v>
       </c>
       <c r="D61" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B61,$B$2,D$2)</f>
         <v>Copier l’URL de la chanson</v>
       </c>
     </row>
@@ -2824,11 +2830,11 @@
         <v>117</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B62,$B$2,C$2)</f>
         <v>Crear</v>
       </c>
       <c r="D62" t="str">
-        <f t="shared" si="2"/>
+        <f>_xlfn.TRANSLATE($B62,$B$2,D$2)</f>
         <v>Créer</v>
       </c>
     </row>
@@ -2840,11 +2846,11 @@
         <v>119</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" ref="C63:D82" si="3">_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
         <v>Crear...</v>
       </c>
       <c r="D63" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B63,$B$2,D$2)</f>
         <v>Créer...</v>
       </c>
     </row>
@@ -2856,11 +2862,11 @@
         <v>121</v>
       </c>
       <c r="C64" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B64,$B$2,C$2)</f>
         <v>Fecha añadida</v>
       </c>
       <c r="D64" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B64,$B$2,D$2)</f>
         <v>Date ajoutée</v>
       </c>
     </row>
@@ -2872,11 +2878,11 @@
         <v>123</v>
       </c>
       <c r="C65" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B65,$B$2,C$2)</f>
         <v>Diciembre</v>
       </c>
       <c r="D65" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B65,$B$2,D$2)</f>
         <v>Décembre</v>
       </c>
     </row>
@@ -2888,11 +2894,11 @@
         <v>125</v>
       </c>
       <c r="C66" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B66,$B$2,C$2)</f>
         <v>Tu dispositivo no soporta al trabajador de servicio</v>
       </c>
       <c r="D66" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B66,$B$2,D$2)</f>
         <v>Votre appareil ne prend pas en charge l’assistant de service</v>
       </c>
     </row>
@@ -2904,11 +2910,11 @@
         <v>127</v>
       </c>
       <c r="C67" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B67,$B$2,C$2)</f>
         <v>Disco</v>
       </c>
       <c r="D67" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B67,$B$2,D$2)</f>
         <v>Disque</v>
       </c>
     </row>
@@ -2920,11 +2926,11 @@
         <v>129</v>
       </c>
       <c r="C68" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B68,$B$2,C$2)</f>
         <v>Nombre de Muestra</v>
       </c>
       <c r="D68" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B68,$B$2,D$2)</f>
         <v>Nom d’affichage</v>
       </c>
     </row>
@@ -2936,11 +2942,11 @@
         <v>131</v>
       </c>
       <c r="C69" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B69,$B$2,C$2)</f>
         <v>Descargar</v>
       </c>
       <c r="D69" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B69,$B$2,D$2)</f>
         <v>Télécharger</v>
       </c>
     </row>
@@ -2952,11 +2958,11 @@
         <v>133</v>
       </c>
       <c r="C70" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B70,$B$2,C$2)</f>
         <v>Descarga la app para escuchar offline</v>
       </c>
       <c r="D70" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B70,$B$2,D$2)</f>
         <v>Téléchargez l’application pour une écoute hors ligne</v>
       </c>
     </row>
@@ -2968,11 +2974,11 @@
         <v>135</v>
       </c>
       <c r="C71" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B71,$B$2,C$2)</f>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
       <c r="D71" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B71,$B$2,D$2)</f>
         <v>Saisissez une URL Spotify ou YouTube Music</v>
       </c>
     </row>
@@ -2984,11 +2990,11 @@
         <v>137</v>
       </c>
       <c r="C72" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B72,$B$2,C$2)</f>
         <v>Lista de descargas al dispositivo</v>
       </c>
       <c r="D72" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B72,$B$2,D$2)</f>
         <v>Liste de téléchargement vers l’appareil</v>
       </c>
     </row>
@@ -3000,11 +3006,11 @@
         <v>139</v>
       </c>
       <c r="C73" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B73,$B$2,C$2)</f>
         <v>Descargar medios al dispositivo</v>
       </c>
       <c r="D73" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B73,$B$2,D$2)</f>
         <v>Télécharger des médias sur l’appareil</v>
       </c>
     </row>
@@ -3016,11 +3022,11 @@
         <v>141</v>
       </c>
       <c r="C74" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B74,$B$2,C$2)</f>
         <v>Descargar mp</v>
       </c>
       <c r="D74" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B74,$B$2,D$2)</f>
         <v>Télécharger le MP</v>
       </c>
     </row>
@@ -3032,11 +3038,11 @@
         <v>143</v>
       </c>
       <c r="C75" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B75,$B$2,C$2)</f>
         <v>Descargar canción al dispositivo</v>
       </c>
       <c r="D75" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B75,$B$2,D$2)</f>
         <v>Télécharger la chanson sur l’appareil</v>
       </c>
     </row>
@@ -3048,11 +3054,11 @@
         <v>145</v>
       </c>
       <c r="C76" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B76,$B$2,C$2)</f>
         <v>Descarga iniciada</v>
       </c>
       <c r="D76" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B76,$B$2,D$2)</f>
         <v>Téléchargement lancé</v>
       </c>
     </row>
@@ -3064,11 +3070,11 @@
         <v>147</v>
       </c>
       <c r="C77" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B77,$B$2,C$2)</f>
         <v>Descargar ZIP</v>
       </c>
       <c r="D77" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B77,$B$2,D$2)</f>
         <v>Télécharger ZIP</v>
       </c>
     </row>
@@ -3080,11 +3086,11 @@
         <v>149</v>
       </c>
       <c r="C78" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B78,$B$2,C$2)</f>
         <v>Descargas</v>
       </c>
       <c r="D78" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B78,$B$2,D$2)</f>
         <v>Téléchargements</v>
       </c>
     </row>
@@ -3096,11 +3102,11 @@
         <v>151</v>
       </c>
       <c r="C79" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B79,$B$2,C$2)</f>
         <v>Duración</v>
       </c>
       <c r="D79" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B79,$B$2,D$2)</f>
         <v>Durée</v>
       </c>
     </row>
@@ -3112,11 +3118,11 @@
         <v>153</v>
       </c>
       <c r="C80" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B80,$B$2,C$2)</f>
         <v>Energía</v>
       </c>
       <c r="D80" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B80,$B$2,D$2)</f>
         <v>Énergie</v>
       </c>
     </row>
@@ -3128,11 +3134,11 @@
         <v>155</v>
       </c>
       <c r="C81" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B81,$B$2,C$2)</f>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D81" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B81,$B$2,D$2)</f>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3144,11 +3150,11 @@
         <v>157</v>
       </c>
       <c r="C82" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B82,$B$2,C$2)</f>
         <v>Error</v>
       </c>
       <c r="D82" t="str">
-        <f t="shared" si="3"/>
+        <f>_xlfn.TRANSLATE($B82,$B$2,D$2)</f>
         <v>Erreur</v>
       </c>
     </row>
@@ -3160,11 +3166,11 @@
         <v>159</v>
       </c>
       <c r="C83" t="str">
-        <f t="shared" ref="C83:D102" si="4">_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
         <v>Lenguaje de cambio de error</v>
       </c>
       <c r="D83" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B83,$B$2,D$2)</f>
         <v>Langage de changement d’erreur</v>
       </c>
     </row>
@@ -3176,11 +3182,11 @@
         <v>161</v>
       </c>
       <c r="C84" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B84,$B$2,C$2)</f>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D84" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B84,$B$2,D$2)</f>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3192,11 +3198,11 @@
         <v>161</v>
       </c>
       <c r="C85" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B85,$B$2,C$2)</f>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D85" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B85,$B$2,D$2)</f>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3208,11 +3214,11 @@
         <v>155</v>
       </c>
       <c r="C86" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B86,$B$2,C$2)</f>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D86" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B86,$B$2,D$2)</f>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3224,11 +3230,11 @@
         <v>475</v>
       </c>
       <c r="C87" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B87,$B$2,C$2)</f>
         <v>Error al obtener descargas</v>
       </c>
       <c r="D87" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B87,$B$2,D$2)</f>
         <v>Erreur de téléchargement</v>
       </c>
     </row>
@@ -3240,11 +3246,11 @@
         <v>165</v>
       </c>
       <c r="C88" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B88,$B$2,C$2)</f>
         <v>Cola de obtención de errores</v>
       </c>
       <c r="D88" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B88,$B$2,D$2)</f>
         <v>File d’attente d’obtention d’erreurs</v>
       </c>
     </row>
@@ -3256,11 +3262,11 @@
         <v>476</v>
       </c>
       <c r="C89" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B89,$B$2,C$2)</f>
         <v>Usuario que obtiene errores</v>
       </c>
       <c r="D89" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B89,$B$2,D$2)</f>
         <v>Utilisateur d’obtention d’erreurs</v>
       </c>
     </row>
@@ -3272,11 +3278,11 @@
         <v>167</v>
       </c>
       <c r="C90" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B90,$B$2,C$2)</f>
         <v>Error al dar like a medios</v>
       </c>
       <c r="D90" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B90,$B$2,D$2)</f>
         <v>Erreur d’appréciation des médias</v>
       </c>
     </row>
@@ -3288,11 +3294,11 @@
         <v>474</v>
       </c>
       <c r="C91" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B91,$B$2,C$2)</f>
         <v>Búsqueda de errores</v>
       </c>
       <c r="D91" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B91,$B$2,D$2)</f>
         <v>Recherche d’erreurs</v>
       </c>
     </row>
@@ -3304,11 +3310,11 @@
         <v>169</v>
       </c>
       <c r="C92" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B92,$B$2,C$2)</f>
         <v>Error al iniciar la descarga</v>
       </c>
       <c r="D92" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B92,$B$2,D$2)</f>
         <v>Erreur au démarrage du téléchargement</v>
       </c>
     </row>
@@ -3320,11 +3326,11 @@
         <v>171</v>
       </c>
       <c r="C93" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B93,$B$2,C$2)</f>
         <v>Error al dejar de dar like a los medios</v>
       </c>
       <c r="D93" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B93,$B$2,D$2)</f>
         <v>Erreur de non-like des médias</v>
       </c>
     </row>
@@ -3336,11 +3342,11 @@
         <v>464</v>
       </c>
       <c r="C94" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B94,$B$2,C$2)</f>
         <v>No se añadió contenido a la biblioteca</v>
       </c>
       <c r="D94" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B94,$B$2,D$2)</f>
         <v>Échec d’ajouter des médias à la bibliothèque</v>
       </c>
     </row>
@@ -3352,11 +3358,11 @@
         <v>470</v>
       </c>
       <c r="C95" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B95,$B$2,C$2)</f>
         <v>No se añadió contenido a la lista de reproducción</v>
       </c>
       <c r="D95" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B95,$B$2,D$2)</f>
         <v>Échec d’ajouter des médias à la playlist</v>
       </c>
     </row>
@@ -3368,11 +3374,11 @@
         <v>173</v>
       </c>
       <c r="C96" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B96,$B$2,C$2)</f>
         <v>No cambiaron el idioma</v>
       </c>
       <c r="D96" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B96,$B$2,D$2)</f>
         <v>Échec de changer de langue</v>
       </c>
     </row>
@@ -3384,11 +3390,11 @@
         <v>466</v>
       </c>
       <c r="C97" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B97,$B$2,C$2)</f>
         <v>No se han conseguido las listas de reproducción</v>
       </c>
       <c r="D97" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B97,$B$2,D$2)</f>
         <v>Échec à récupérer les playlists</v>
       </c>
     </row>
@@ -3400,11 +3406,11 @@
         <v>175</v>
       </c>
       <c r="C98" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B98,$B$2,C$2)</f>
         <v>Álbumes destacados</v>
       </c>
       <c r="D98" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B98,$B$2,D$2)</f>
         <v>Albums en vedette</v>
       </c>
     </row>
@@ -3416,11 +3422,11 @@
         <v>177</v>
       </c>
       <c r="C99" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B99,$B$2,C$2)</f>
         <v>Listas destacadas</v>
       </c>
       <c r="D99" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B99,$B$2,D$2)</f>
         <v>Listes en vedette</v>
       </c>
     </row>
@@ -3432,11 +3438,11 @@
         <v>179</v>
       </c>
       <c r="C100" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B100,$B$2,C$2)</f>
         <v>Febrero</v>
       </c>
       <c r="D100" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B100,$B$2,D$2)</f>
         <v>Février</v>
       </c>
     </row>
@@ -3448,11 +3454,11 @@
         <v>181</v>
       </c>
       <c r="C101" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B101,$B$2,C$2)</f>
         <v>Enfoque</v>
       </c>
       <c r="D101" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B101,$B$2,D$2)</f>
         <v>Focus</v>
       </c>
     </row>
@@ -3464,11 +3470,11 @@
         <v>183</v>
       </c>
       <c r="C102" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B102,$B$2,C$2)</f>
         <v>Amigos</v>
       </c>
       <c r="D102" t="str">
-        <f t="shared" si="4"/>
+        <f>_xlfn.TRANSLATE($B102,$B$2,D$2)</f>
         <v>Amis</v>
       </c>
     </row>
@@ -3480,11 +3486,11 @@
         <v>185</v>
       </c>
       <c r="C103" t="str">
-        <f t="shared" ref="C103:D122" si="5">_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
         <v>Lista de amigos</v>
       </c>
       <c r="D103" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B103,$B$2,D$2)</f>
         <v>Liste d’amis</v>
       </c>
     </row>
@@ -3496,11 +3502,11 @@
         <v>187</v>
       </c>
       <c r="C104" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B104,$B$2,C$2)</f>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
       <c r="D104" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B104,$B$2,D$2)</f>
         <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
       </c>
     </row>
@@ -3512,11 +3518,11 @@
         <v>189</v>
       </c>
       <c r="C105" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B105,$B$2,C$2)</f>
         <v>Estadísticas de Friends</v>
       </c>
       <c r="D105" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B105,$B$2,D$2)</f>
         <v>Statistiques de Friends</v>
       </c>
     </row>
@@ -3528,11 +3534,11 @@
         <v>191</v>
       </c>
       <c r="C106" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B106,$B$2,C$2)</f>
         <v>General</v>
       </c>
       <c r="D106" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B106,$B$2,D$2)</f>
         <v>Généralités</v>
       </c>
     </row>
@@ -3544,11 +3550,11 @@
         <v>193</v>
       </c>
       <c r="C107" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B107,$B$2,C$2)</f>
         <v>Estadísticas generales</v>
       </c>
       <c r="D107" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B107,$B$2,D$2)</f>
         <v>Statistiques générales</v>
       </c>
     </row>
@@ -3560,11 +3566,11 @@
         <v>195</v>
       </c>
       <c r="C108" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B108,$B$2,C$2)</f>
         <v>Obtén información</v>
       </c>
       <c r="D108" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B108,$B$2,D$2)</f>
         <v>Obtenez des infos</v>
       </c>
     </row>
@@ -3576,11 +3582,11 @@
         <v>197</v>
       </c>
       <c r="C109" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B109,$B$2,C$2)</f>
         <v>Obteniendo información</v>
       </c>
       <c r="D109" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B109,$B$2,D$2)</f>
         <v>Obtenir des infos</v>
       </c>
     </row>
@@ -3592,11 +3598,11 @@
         <v>199</v>
       </c>
       <c r="C110" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B110,$B$2,C$2)</f>
         <v>Ir al álbum</v>
       </c>
       <c r="D110" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B110,$B$2,D$2)</f>
         <v>Aller à l’album</v>
       </c>
     </row>
@@ -3608,11 +3614,11 @@
         <v>201</v>
       </c>
       <c r="C111" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B111,$B$2,C$2)</f>
         <v>Ir a artista</v>
       </c>
       <c r="D111" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B111,$B$2,D$2)</f>
         <v>Aller à l’artiste</v>
       </c>
     </row>
@@ -3624,11 +3630,11 @@
         <v>203</v>
       </c>
       <c r="C112" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B112,$B$2,C$2)</f>
         <v>Joyas ocultas que olvidaste</v>
       </c>
       <c r="D112" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B112,$B$2,D$2)</f>
         <v>Des perles cachées que tu as oubliées</v>
       </c>
     </row>
@@ -3640,11 +3646,11 @@
         <v>205</v>
       </c>
       <c r="C113" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B113,$B$2,C$2)</f>
         <v>Inicio</v>
       </c>
       <c r="D113" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B113,$B$2,D$2)</f>
         <v>Accueil</v>
       </c>
     </row>
@@ -3656,11 +3662,11 @@
         <v>207</v>
       </c>
       <c r="C114" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B114,$B$2,C$2)</f>
         <v>Enero</v>
       </c>
       <c r="D114" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B114,$B$2,D$2)</f>
         <v>Janvier</v>
       </c>
     </row>
@@ -3672,11 +3678,11 @@
         <v>209</v>
       </c>
       <c r="C115" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B115,$B$2,C$2)</f>
         <v>Julio</v>
       </c>
       <c r="D115" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B115,$B$2,D$2)</f>
         <v>Juillet</v>
       </c>
     </row>
@@ -3688,11 +3694,11 @@
         <v>211</v>
       </c>
       <c r="C116" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B116,$B$2,C$2)</f>
         <v>Junio</v>
       </c>
       <c r="D116" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B116,$B$2,D$2)</f>
         <v>Juin</v>
       </c>
     </row>
@@ -3704,11 +3710,11 @@
         <v>213</v>
       </c>
       <c r="C117" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B117,$B$2,C$2)</f>
         <v>Idioma</v>
       </c>
       <c r="D117" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B117,$B$2,D$2)</f>
         <v>Langue</v>
       </c>
     </row>
@@ -3720,11 +3726,11 @@
         <v>478</v>
       </c>
       <c r="C118" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B118,$B$2,C$2)</f>
         <v>El cambio de idioma fracasó</v>
       </c>
       <c r="D118" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B118,$B$2,D$2)</f>
         <v>Échec du changement linguistique</v>
       </c>
     </row>
@@ -3736,11 +3742,11 @@
         <v>215</v>
       </c>
       <c r="C119" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B119,$B$2,C$2)</f>
         <v>Cambio de idioma</v>
       </c>
       <c r="D119" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B119,$B$2,D$2)</f>
         <v>Changement de langue</v>
       </c>
     </row>
@@ -3752,11 +3758,11 @@
         <v>217</v>
       </c>
       <c r="C120" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B120,$B$2,C$2)</f>
         <v>Últimas descargas</v>
       </c>
       <c r="D120" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B120,$B$2,D$2)</f>
         <v>Derniers téléchargements</v>
       </c>
     </row>
@@ -3768,11 +3774,11 @@
         <v>219</v>
       </c>
       <c r="C121" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B121,$B$2,C$2)</f>
         <v>Nivel</v>
       </c>
       <c r="D121" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B121,$B$2,D$2)</f>
         <v>Niveau</v>
       </c>
     </row>
@@ -3784,11 +3790,11 @@
         <v>221</v>
       </c>
       <c r="C122" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B122,$B$2,C$2)</f>
         <v>Biblioteca</v>
       </c>
       <c r="D122" t="str">
-        <f t="shared" si="5"/>
+        <f>_xlfn.TRANSLATE($B122,$B$2,D$2)</f>
         <v>Bibliothèque</v>
       </c>
     </row>
@@ -3800,11 +3806,11 @@
         <v>223</v>
       </c>
       <c r="C123" t="str">
-        <f t="shared" ref="C123:D142" si="6">_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
         <v>Como</v>
       </c>
       <c r="D123" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B123,$B$2,D$2)</f>
         <v>Comme</v>
       </c>
     </row>
@@ -3816,11 +3822,11 @@
         <v>225</v>
       </c>
       <c r="C124" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B124,$B$2,C$2)</f>
         <v>Canciones que me gustaban</v>
       </c>
       <c r="D124" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B124,$B$2,D$2)</f>
         <v>Chansons appréciées</v>
       </c>
     </row>
@@ -3832,11 +3838,11 @@
         <v>227</v>
       </c>
       <c r="C125" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B125,$B$2,C$2)</f>
         <v>Cerrar sesión</v>
       </c>
       <c r="D125" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B125,$B$2,D$2)</f>
         <v>Déconnexion</v>
       </c>
     </row>
@@ -3848,11 +3854,11 @@
         <v>229</v>
       </c>
       <c r="C126" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B126,$B$2,C$2)</f>
         <v>Letra</v>
       </c>
       <c r="D126" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B126,$B$2,D$2)</f>
         <v>Paroles</v>
       </c>
     </row>
@@ -3864,11 +3870,11 @@
         <v>231</v>
       </c>
       <c r="C127" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B127,$B$2,C$2)</f>
         <v>Marzo</v>
       </c>
       <c r="D127" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
         <v>Mars</v>
       </c>
     </row>
@@ -3880,11 +3886,11 @@
         <v>233</v>
       </c>
       <c r="C128" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B128,$B$2,C$2)</f>
         <v>Mayo</v>
       </c>
       <c r="D128" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B128,$B$2,D$2)</f>
         <v>Mai</v>
       </c>
     </row>
@@ -3896,11 +3902,11 @@
         <v>462</v>
       </c>
       <c r="C129" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B129,$B$2,C$2)</f>
         <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D129" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B129,$B$2,D$2)</f>
         <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
@@ -3912,11 +3918,11 @@
         <v>235</v>
       </c>
       <c r="C130" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B130,$B$2,C$2)</f>
         <v>Progreso de los medios</v>
       </c>
       <c r="D130" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B130,$B$2,D$2)</f>
         <v>Progrès des médias</v>
       </c>
     </row>
@@ -3928,11 +3934,11 @@
         <v>237</v>
       </c>
       <c r="C131" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B131,$B$2,C$2)</f>
         <v>Actas</v>
       </c>
       <c r="D131" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B131,$B$2,D$2)</f>
         <v>Procès-verbal</v>
       </c>
     </row>
@@ -3944,11 +3950,11 @@
         <v>239</v>
       </c>
       <c r="C132" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
         <v>Minutos escuchados</v>
       </c>
       <c r="D132" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B132,$B$2,D$2)</f>
         <v>Minutes écoutées</v>
       </c>
     </row>
@@ -3960,11 +3966,11 @@
         <v>241</v>
       </c>
       <c r="C133" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B133,$B$2,C$2)</f>
         <v>Minutos escuchados por día</v>
       </c>
       <c r="D133" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B133,$B$2,D$2)</f>
         <v>Minutes écoutées par jour</v>
       </c>
     </row>
@@ -3976,11 +3982,11 @@
         <v>243</v>
       </c>
       <c r="C134" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B134,$B$2,C$2)</f>
         <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D134" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B134,$B$2,D$2)</f>
         <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
@@ -3992,11 +3998,11 @@
         <v>245</v>
       </c>
       <c r="C135" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B135,$B$2,C$2)</f>
         <v>Más opciones</v>
       </c>
       <c r="D135" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B135,$B$2,D$2)</f>
         <v>Plus d’options</v>
       </c>
     </row>
@@ -4008,11 +4014,11 @@
         <v>247</v>
       </c>
       <c r="C136" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B136,$B$2,C$2)</f>
         <v>Más canciones de</v>
       </c>
       <c r="D136" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B136,$B$2,D$2)</f>
         <v>Plus de chansons de</v>
       </c>
     </row>
@@ -4024,11 +4030,11 @@
         <v>249</v>
       </c>
       <c r="C137" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B137,$B$2,C$2)</f>
         <v>Más escuchado</v>
       </c>
       <c r="D137" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B137,$B$2,D$2)</f>
         <v>Les plus écoutés</v>
       </c>
     </row>
@@ -4040,11 +4046,11 @@
         <v>251</v>
       </c>
       <c r="C138" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B138,$B$2,C$2)</f>
         <v>Álbumes más escuchados</v>
       </c>
       <c r="D138" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B138,$B$2,D$2)</f>
         <v>Albums les plus écoutés</v>
       </c>
     </row>
@@ -4056,11 +4062,11 @@
         <v>253</v>
       </c>
       <c r="C139" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B139,$B$2,C$2)</f>
         <v>Artistas más escuchados</v>
       </c>
       <c r="D139" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B139,$B$2,D$2)</f>
         <v>Artistes les plus écoutés</v>
       </c>
     </row>
@@ -4072,11 +4078,11 @@
         <v>255</v>
       </c>
       <c r="C140" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B140,$B$2,C$2)</f>
         <v>Canciones más escuchadas</v>
       </c>
       <c r="D140" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B140,$B$2,D$2)</f>
         <v>Chansons les plus écoutées</v>
       </c>
     </row>
@@ -4088,11 +4094,11 @@
         <v>257</v>
       </c>
       <c r="C141" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B141,$B$2,C$2)</f>
         <v>Nombre</v>
       </c>
       <c r="D141" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
         <v>Nom</v>
       </c>
     </row>
@@ -4104,11 +4110,11 @@
         <v>259</v>
       </c>
       <c r="C142" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B142,$B$2,C$2)</f>
         <v>Introducir nueva contraseña</v>
       </c>
       <c r="D142" t="str">
-        <f t="shared" si="6"/>
+        <f>_xlfn.TRANSLATE($B142,$B$2,D$2)</f>
         <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
@@ -4120,11 +4126,11 @@
         <v>261</v>
       </c>
       <c r="C143" t="str">
-        <f t="shared" ref="C143:D162" si="7">_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
         <v>Nueva lista de reproducción</v>
       </c>
       <c r="D143" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TRANSLATE($B143,$B$2,D$2)</f>
         <v>Nouvelle playlist</v>
       </c>
     </row>
@@ -4136,1715 +4142,1713 @@
         <v>263</v>
       </c>
       <c r="C144" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TRANSLATE($B144,$B$2,C$2)</f>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D144" t="str">
-        <f t="shared" si="7"/>
+        <f>_xlfn.TRANSLATE($B144,$B$2,D$2)</f>
         <v>Nouveau nom de la playlist</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>264</v>
+        <v>479</v>
       </c>
       <c r="B145" t="s">
-        <v>265</v>
+        <v>480</v>
       </c>
       <c r="C145" t="str">
-        <f t="shared" si="7"/>
-        <v>Próximos medios</v>
+        <f>_xlfn.TRANSLATE($B145,$B$2,C$2)</f>
+        <v>Nueva versión disponible</v>
       </c>
       <c r="D145" t="str">
-        <f t="shared" si="7"/>
-        <v>Médias suivants</v>
+        <f>_xlfn.TRANSLATE($B145,$B$2,D$2)</f>
+        <v>Nouvelle version disponible</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B146" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C146" t="str">
-        <f t="shared" si="7"/>
-        <v>Todavía no hay álbumes en tu biblioteca</v>
+        <f>_xlfn.TRANSLATE($B146,$B$2,C$2)</f>
+        <v>Próximos medios</v>
       </c>
       <c r="D146" t="str">
-        <f t="shared" si="7"/>
-        <v>Aucun album dans ta bibliothèque pour l’instant</v>
+        <f>_xlfn.TRANSLATE($B146,$B$2,D$2)</f>
+        <v>Médias suivants</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B147" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C147" t="str">
-        <f t="shared" si="7"/>
-        <v>No hay datos registrados.</v>
+        <f>_xlfn.TRANSLATE($B147,$B$2,C$2)</f>
+        <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
       <c r="D147" t="str">
-        <f t="shared" si="7"/>
-        <v>Aucune donnée enregistrée.</v>
+        <f>_xlfn.TRANSLATE($B147,$B$2,D$2)</f>
+        <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B148" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C148" t="str">
-        <f t="shared" si="7"/>
-        <v>Letra no disponible</v>
+        <f>_xlfn.TRANSLATE($B148,$B$2,C$2)</f>
+        <v>No hay datos registrados.</v>
       </c>
       <c r="D148" t="str">
-        <f t="shared" si="7"/>
-        <v>Paroles non disponibles</v>
+        <f>_xlfn.TRANSLATE($B148,$B$2,D$2)</f>
+        <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B149" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C149" t="str">
-        <f t="shared" si="7"/>
-        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
+        <f>_xlfn.TRANSLATE($B149,$B$2,C$2)</f>
+        <v>Letra no disponible</v>
       </c>
       <c r="D149" t="str">
-        <f t="shared" si="7"/>
-        <v>Pas encore de playlists dans votre bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B149,$B$2,D$2)</f>
+        <v>Paroles non disponibles</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B150" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C150" t="str">
-        <f t="shared" si="7"/>
-        <v>No hay repetición</v>
+        <f>_xlfn.TRANSLATE($B150,$B$2,C$2)</f>
+        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D150" t="str">
-        <f t="shared" si="7"/>
-        <v>Pas de répétition</v>
+        <f>_xlfn.TRANSLATE($B150,$B$2,D$2)</f>
+        <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B151" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C151" t="str">
-        <f t="shared" si="7"/>
-        <v>Sin resultados</v>
+        <f>_xlfn.TRANSLATE($B151,$B$2,C$2)</f>
+        <v>No hay repetición</v>
       </c>
       <c r="D151" t="str">
-        <f t="shared" si="7"/>
-        <v>Aucun résultat</v>
+        <f>_xlfn.TRANSLATE($B151,$B$2,D$2)</f>
+        <v>Pas de répétition</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B152" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C152" t="str">
-        <f t="shared" si="7"/>
-        <v>Sin trabajador de servicios</v>
+        <f>_xlfn.TRANSLATE($B152,$B$2,C$2)</f>
+        <v>Sin resultados</v>
       </c>
       <c r="D152" t="str">
-        <f t="shared" si="7"/>
-        <v>Aucun travailleur de services</v>
+        <f>_xlfn.TRANSLATE($B152,$B$2,D$2)</f>
+        <v>Aucun résultat</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B153" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C153" t="str">
-        <f t="shared" si="7"/>
-        <v>Todavía no hay canciones en tu biblioteca</v>
+        <f>_xlfn.TRANSLATE($B153,$B$2,C$2)</f>
+        <v>Sin trabajador de servicios</v>
       </c>
       <c r="D153" t="str">
-        <f t="shared" si="7"/>
-        <v>Pas encore de chansons dans ta bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B153,$B$2,D$2)</f>
+        <v>Aucun travailleur de services</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B154" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C154" t="str">
-        <f t="shared" si="7"/>
-        <v>Sin estado</v>
+        <f>_xlfn.TRANSLATE($B154,$B$2,C$2)</f>
+        <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D154" t="str">
-        <f t="shared" si="7"/>
-        <v>Aucun État</v>
+        <f>_xlfn.TRANSLATE($B154,$B$2,D$2)</f>
+        <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B155" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C155" t="str">
-        <f t="shared" si="7"/>
-        <v>Todavía no hay estaciones en tu biblioteca</v>
+        <f>_xlfn.TRANSLATE($B155,$B$2,C$2)</f>
+        <v>Sin estado</v>
       </c>
       <c r="D155" t="str">
-        <f t="shared" si="7"/>
-        <v>Pas encore de stations dans votre bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B155,$B$2,D$2)</f>
+        <v>Aucun État</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B156" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C156" t="str">
-        <f t="shared" si="7"/>
-        <v>Todavía no hay vídeos en tu biblioteca</v>
+        <f>_xlfn.TRANSLATE($B156,$B$2,C$2)</f>
+        <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D156" t="str">
-        <f t="shared" si="7"/>
-        <v>Pas encore de vidéos dans ta bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B156,$B$2,D$2)</f>
+        <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B157" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C157" t="str">
-        <f t="shared" si="7"/>
-        <v>Noviembre</v>
+        <f>_xlfn.TRANSLATE($B157,$B$2,C$2)</f>
+        <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D157" t="str">
-        <f t="shared" si="7"/>
-        <v>Novembre</v>
+        <f>_xlfn.TRANSLATE($B157,$B$2,D$2)</f>
+        <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B158" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C158" t="str">
-        <f t="shared" si="7"/>
-        <v>Octubre</v>
+        <f>_xlfn.TRANSLATE($B158,$B$2,C$2)</f>
+        <v>Noviembre</v>
       </c>
       <c r="D158" t="str">
-        <f t="shared" si="7"/>
-        <v>Octobre</v>
+        <f>_xlfn.TRANSLATE($B158,$B$2,D$2)</f>
+        <v>Novembre</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B159" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C159" t="str">
-        <f t="shared" si="7"/>
-        <v>Lista abierta</v>
+        <f>_xlfn.TRANSLATE($B159,$B$2,C$2)</f>
+        <v>Octubre</v>
       </c>
       <c r="D159" t="str">
-        <f t="shared" si="7"/>
-        <v>Liste ouverte</v>
+        <f>_xlfn.TRANSLATE($B159,$B$2,D$2)</f>
+        <v>Octobre</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B160" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C160" t="str">
-        <f t="shared" si="7"/>
-        <v>Canción abierta</v>
+        <f>_xlfn.TRANSLATE($B160,$B$2,C$2)</f>
+        <v>Lista abierta</v>
       </c>
       <c r="D160" t="str">
-        <f t="shared" si="7"/>
-        <v>Chanson d’ouverture</v>
+        <f>_xlfn.TRANSLATE($B160,$B$2,D$2)</f>
+        <v>Liste ouverte</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B161" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C161" t="str">
-        <f t="shared" si="7"/>
-        <v>Partido</v>
+        <f>_xlfn.TRANSLATE($B161,$B$2,C$2)</f>
+        <v>Canción abierta</v>
       </c>
       <c r="D161" t="str">
-        <f t="shared" si="7"/>
-        <v>Parti</v>
+        <f>_xlfn.TRANSLATE($B161,$B$2,D$2)</f>
+        <v>Chanson d’ouverture</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B162" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C162" t="str">
-        <f t="shared" si="7"/>
-        <v>Canción de pausa</v>
+        <f>_xlfn.TRANSLATE($B162,$B$2,C$2)</f>
+        <v>Partido</v>
       </c>
       <c r="D162" t="str">
-        <f t="shared" si="7"/>
-        <v>Chanson de pause</v>
+        <f>_xlfn.TRANSLATE($B162,$B$2,D$2)</f>
+        <v>Parti</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B163" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C163" t="str">
-        <f t="shared" ref="C163:D182" si="8">_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
-        <v>Solicitudes pendientes</v>
+        <f>_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
+        <v>Canción de pausa</v>
       </c>
       <c r="D163" t="str">
-        <f t="shared" si="8"/>
-        <v>Demandes en attente</v>
+        <f>_xlfn.TRANSLATE($B163,$B$2,D$2)</f>
+        <v>Chanson de pause</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B164" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C164" t="str">
-        <f t="shared" si="8"/>
-        <v>Pin</v>
+        <f>_xlfn.TRANSLATE($B164,$B$2,C$2)</f>
+        <v>Solicitudes pendientes</v>
       </c>
       <c r="D164" t="str">
-        <f t="shared" si="8"/>
-        <v>Épingle</v>
+        <f>_xlfn.TRANSLATE($B164,$B$2,D$2)</f>
+        <v>Demandes en attente</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B165" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C165" t="str">
-        <f t="shared" si="8"/>
-        <v>Listas fijadas</v>
+        <f>_xlfn.TRANSLATE($B165,$B$2,C$2)</f>
+        <v>Pin</v>
       </c>
       <c r="D165" t="str">
-        <f t="shared" si="8"/>
-        <v>Listes épinglées</v>
+        <f>_xlfn.TRANSLATE($B165,$B$2,D$2)</f>
+        <v>Épingle</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B166" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C166" t="str">
-        <f t="shared" si="8"/>
-        <v>Título del álbum</v>
+        <f>_xlfn.TRANSLATE($B166,$B$2,C$2)</f>
+        <v>Listas fijadas</v>
       </c>
       <c r="D166" t="str">
-        <f t="shared" si="8"/>
-        <v>Titre de l’album</v>
+        <f>_xlfn.TRANSLATE($B166,$B$2,D$2)</f>
+        <v>Listes épinglées</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B167" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C167" t="str">
-        <f t="shared" si="8"/>
-        <v>Nombre artístico</v>
+        <f>_xlfn.TRANSLATE($B167,$B$2,C$2)</f>
+        <v>Título del álbum</v>
       </c>
       <c r="D167" t="str">
-        <f t="shared" si="8"/>
-        <v>Nom de l’artiste</v>
+        <f>_xlfn.TRANSLATE($B167,$B$2,D$2)</f>
+        <v>Titre de l’album</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B168" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C168" t="str">
-        <f t="shared" si="8"/>
-        <v>Mi lista de reproducción perfecta</v>
+        <f>_xlfn.TRANSLATE($B168,$B$2,C$2)</f>
+        <v>Nombre artístico</v>
       </c>
       <c r="D168" t="str">
-        <f t="shared" si="8"/>
-        <v>Ma playlist parfaite</v>
+        <f>_xlfn.TRANSLATE($B168,$B$2,D$2)</f>
+        <v>Nom de l’artiste</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B169" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C169" t="str">
-        <f t="shared" si="8"/>
-        <v>Título de la canción</v>
+        <f>_xlfn.TRANSLATE($B169,$B$2,C$2)</f>
+        <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D169" t="str">
-        <f t="shared" si="8"/>
-        <v>Titre de la chanson</v>
+        <f>_xlfn.TRANSLATE($B169,$B$2,D$2)</f>
+        <v>Ma playlist parfaite</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>453</v>
+        <v>312</v>
       </c>
       <c r="B170" t="s">
-        <v>454</v>
+        <v>313</v>
       </c>
       <c r="C170" t="str">
-        <f t="shared" si="8"/>
-        <v>Juego</v>
+        <f>_xlfn.TRANSLATE($B170,$B$2,C$2)</f>
+        <v>Título de la canción</v>
       </c>
       <c r="D170" t="str">
-        <f t="shared" si="8"/>
-        <v>Jeu</v>
+        <f>_xlfn.TRANSLATE($B170,$B$2,D$2)</f>
+        <v>Titre de la chanson</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>314</v>
+        <v>453</v>
       </c>
       <c r="B171" t="s">
-        <v>315</v>
-      </c>
-      <c r="C171" t="str">
-        <f t="shared" si="8"/>
-        <v>Lista de reproducción</v>
+        <v>454</v>
+      </c>
+      <c r="C171" t="s">
+        <v>481</v>
       </c>
       <c r="D171" t="str">
-        <f t="shared" si="8"/>
-        <v>Liste des jeux</v>
+        <f>_xlfn.TRANSLATE($B171,$B$2,D$2)</f>
+        <v>Jeu</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B172" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C172" t="str">
-        <f t="shared" si="8"/>
-        <v>Reproducir medios</v>
+        <f>_xlfn.TRANSLATE($B172,$B$2,C$2)</f>
+        <v>Lista de reproducción</v>
       </c>
       <c r="D172" t="str">
-        <f t="shared" si="8"/>
-        <v>Lire les médias</v>
+        <f>_xlfn.TRANSLATE($B172,$B$2,D$2)</f>
+        <v>Liste des jeux</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B173" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C173" t="str">
-        <f t="shared" si="8"/>
-        <v>Juego a continuación</v>
+        <f>_xlfn.TRANSLATE($B173,$B$2,C$2)</f>
+        <v>Reproducir medios</v>
       </c>
       <c r="D173" t="str">
-        <f t="shared" si="8"/>
-        <v>À jouer à venir</v>
+        <f>_xlfn.TRANSLATE($B173,$B$2,D$2)</f>
+        <v>Lire les médias</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B174" t="s">
-        <v>321</v>
-      </c>
-      <c r="C174" t="str">
-        <f t="shared" si="8"/>
-        <v>Tocar canción</v>
+        <v>319</v>
+      </c>
+      <c r="C174" t="s">
+        <v>482</v>
       </c>
       <c r="D174" t="str">
-        <f t="shared" si="8"/>
-        <v>Jouer la chanson</v>
+        <f>_xlfn.TRANSLATE($B174,$B$2,D$2)</f>
+        <v>À jouer à venir</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B175" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C175" t="str">
-        <f t="shared" si="8"/>
-        <v>Listas de reproducción</v>
+        <f>_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
+        <v>Tocar canción</v>
       </c>
       <c r="D175" t="str">
-        <f t="shared" si="8"/>
-        <v>Playlists</v>
+        <f>_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
+        <v>Jouer la chanson</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B176" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C176" t="str">
-        <f t="shared" si="8"/>
-        <v>Medios anteriores</v>
+        <f>_xlfn.TRANSLATE($B176,$B$2,C$2)</f>
+        <v>Listas de reproducción</v>
       </c>
       <c r="D176" t="str">
-        <f t="shared" si="8"/>
-        <v>Médias précédents</v>
+        <f>_xlfn.TRANSLATE($B176,$B$2,D$2)</f>
+        <v>Playlists</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B177" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C177" t="str">
-        <f t="shared" si="8"/>
-        <v>Selecciones rápidas</v>
+        <f>_xlfn.TRANSLATE($B177,$B$2,C$2)</f>
+        <v>Medios anteriores</v>
       </c>
       <c r="D177" t="str">
-        <f t="shared" si="8"/>
-        <v>Choix rapides</v>
+        <f>_xlfn.TRANSLATE($B177,$B$2,D$2)</f>
+        <v>Médias précédents</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B178" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C178" t="str">
-        <f t="shared" si="8"/>
-        <v>Radio</v>
+        <f>_xlfn.TRANSLATE($B178,$B$2,C$2)</f>
+        <v>Selecciones rápidas</v>
       </c>
       <c r="D178" t="str">
-        <f t="shared" si="8"/>
-        <v>Radio</v>
+        <f>_xlfn.TRANSLATE($B178,$B$2,D$2)</f>
+        <v>Choix rapides</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B179" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C179" t="str">
-        <f t="shared" si="8"/>
-        <v>No se han encontrado estaciones</v>
+        <f>_xlfn.TRANSLATE($B179,$B$2,C$2)</f>
+        <v>Radio</v>
       </c>
       <c r="D179" t="str">
-        <f t="shared" si="8"/>
-        <v>Aucune station trouvée</v>
+        <f>_xlfn.TRANSLATE($B179,$B$2,D$2)</f>
+        <v>Radio</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B180" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C180" t="str">
-        <f t="shared" si="8"/>
-        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
+        <f>_xlfn.TRANSLATE($B180,$B$2,C$2)</f>
+        <v>No se han encontrado estaciones</v>
       </c>
       <c r="D180" t="str">
-        <f t="shared" si="8"/>
-        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
+        <f>_xlfn.TRANSLATE($B180,$B$2,D$2)</f>
+        <v>Aucune station trouvée</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B181" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C181" t="str">
-        <f t="shared" si="8"/>
-        <v>Busca emisoras, géneros, países...</v>
+        <f>_xlfn.TRANSLATE($B181,$B$2,C$2)</f>
+        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D181" t="str">
-        <f t="shared" si="8"/>
-        <v>Recherche des stations, genres, pays...</v>
+        <f>_xlfn.TRANSLATE($B181,$B$2,D$2)</f>
+        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B182" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C182" t="str">
-        <f t="shared" si="8"/>
-        <v>Emisoras de radio</v>
+        <f>_xlfn.TRANSLATE($B182,$B$2,C$2)</f>
+        <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D182" t="str">
-        <f t="shared" si="8"/>
-        <v>Radio Stations</v>
+        <f>_xlfn.TRANSLATE($B182,$B$2,D$2)</f>
+        <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B183" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C183" t="str">
-        <f t="shared" ref="C183:D202" si="9">_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
-        <v>Mezcla reciente</v>
+        <f>_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
+        <v>Emisoras de radio</v>
       </c>
       <c r="D183" t="str">
-        <f t="shared" si="9"/>
-        <v>Mix récent</v>
+        <f>_xlfn.TRANSLATE($B183,$B$2,D$2)</f>
+        <v>Radio Stations</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B184" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C184" t="str">
-        <f t="shared" si="9"/>
-        <v>Jugado recientemente</v>
+        <f>_xlfn.TRANSLATE($B184,$B$2,C$2)</f>
+        <v>Mezcla reciente</v>
       </c>
       <c r="D184" t="str">
-        <f t="shared" si="9"/>
-        <v>Joué récemment</v>
+        <f>_xlfn.TRANSLATE($B184,$B$2,D$2)</f>
+        <v>Mix récent</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B185" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C185" t="str">
-        <f t="shared" si="9"/>
+        <f>_xlfn.TRANSLATE($B185,$B$2,C$2)</f>
         <v>Jugado recientemente</v>
       </c>
       <c r="D185" t="str">
-        <f t="shared" si="9"/>
-        <v>Récemment joué</v>
+        <f>_xlfn.TRANSLATE($B185,$B$2,D$2)</f>
+        <v>Joué récemment</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B186" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C186" t="str">
-        <f t="shared" si="9"/>
-        <v>Registro</v>
+        <f>_xlfn.TRANSLATE($B186,$B$2,C$2)</f>
+        <v>Jugado recientemente</v>
       </c>
       <c r="D186" t="str">
-        <f t="shared" si="9"/>
-        <v>Registre</v>
+        <f>_xlfn.TRANSLATE($B186,$B$2,D$2)</f>
+        <v>Récemment joué</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B187" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C187" t="str">
-        <f t="shared" si="9"/>
-        <v>Registrado</v>
+        <f>_xlfn.TRANSLATE($B187,$B$2,C$2)</f>
+        <v>Registro</v>
       </c>
       <c r="D187" t="str">
-        <f t="shared" si="9"/>
-        <v>Enregistré</v>
+        <f>_xlfn.TRANSLATE($B187,$B$2,D$2)</f>
+        <v>Registre</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B188" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C188" t="str">
-        <f t="shared" si="9"/>
-        <v>Registrando...</v>
+        <f>_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
+        <v>Registrado</v>
       </c>
       <c r="D188" t="str">
-        <f t="shared" si="9"/>
-        <v>Enregistrement...</v>
+        <f>_xlfn.TRANSLATE($B188,$B$2,D$2)</f>
+        <v>Enregistré</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B189" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C189" t="str">
-        <f t="shared" si="9"/>
-        <v>Artistas relacionados</v>
+        <f>_xlfn.TRANSLATE($B189,$B$2,C$2)</f>
+        <v>Registrando...</v>
       </c>
       <c r="D189" t="str">
-        <f t="shared" si="9"/>
-        <v>Artistes associés</v>
+        <f>_xlfn.TRANSLATE($B189,$B$2,D$2)</f>
+        <v>Enregistrement...</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B190" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C190" t="str">
-        <f t="shared" si="9"/>
-        <v>Relajado</v>
+        <f>_xlfn.TRANSLATE($B190,$B$2,C$2)</f>
+        <v>Artistas relacionados</v>
       </c>
       <c r="D190" t="str">
-        <f t="shared" si="9"/>
-        <v>Détendu</v>
+        <f>_xlfn.TRANSLATE($B190,$B$2,D$2)</f>
+        <v>Artistes associés</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B191" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C191" t="str">
-        <f t="shared" si="9"/>
-        <v>Eliminar de la biblioteca</v>
+        <f>_xlfn.TRANSLATE($B191,$B$2,C$2)</f>
+        <v>Relajado</v>
       </c>
       <c r="D191" t="str">
-        <f t="shared" si="9"/>
-        <v>Retirer de la bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B191,$B$2,D$2)</f>
+        <v>Détendu</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B192" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C192" t="str">
-        <f t="shared" si="9"/>
-        <v>Quitar de me gusta</v>
+        <f>_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
+        <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D192" t="str">
-        <f t="shared" si="9"/>
-        <v>Retirer de aimé</v>
+        <f>_xlfn.TRANSLATE($B192,$B$2,D$2)</f>
+        <v>Retirer de la bibliothèque</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B193" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C193" t="str">
-        <f t="shared" si="9"/>
-        <v>Eliminar de la lista de reproducción</v>
+        <f>_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
+        <v>Quitar de me gusta</v>
       </c>
       <c r="D193" t="str">
-        <f t="shared" si="9"/>
-        <v>Supprimer de la playlist</v>
+        <f>_xlfn.TRANSLATE($B193,$B$2,D$2)</f>
+        <v>Retirer de aimé</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B194" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C194" t="str">
-        <f t="shared" si="9"/>
-        <v>Eliminar de la cola</v>
+        <f>_xlfn.TRANSLATE($B194,$B$2,C$2)</f>
+        <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D194" t="str">
-        <f t="shared" si="9"/>
-        <v>Retirer de la file d’attente</v>
+        <f>_xlfn.TRANSLATE($B194,$B$2,D$2)</f>
+        <v>Supprimer de la playlist</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B195" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C195" t="str">
-        <f t="shared" si="9"/>
-        <v>Repite todo</v>
+        <f>_xlfn.TRANSLATE($B195,$B$2,C$2)</f>
+        <v>Eliminar de la cola</v>
       </c>
       <c r="D195" t="str">
-        <f t="shared" si="9"/>
-        <v>Répétez tout</v>
+        <f>_xlfn.TRANSLATE($B195,$B$2,D$2)</f>
+        <v>Retirer de la file d’attente</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B196" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C196" t="str">
-        <f t="shared" si="9"/>
-        <v>Repite una</v>
+        <f>_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
+        <v>Repite todo</v>
       </c>
       <c r="D196" t="str">
-        <f t="shared" si="9"/>
-        <v>Répétez-en un</v>
+        <f>_xlfn.TRANSLATE($B196,$B$2,D$2)</f>
+        <v>Répétez tout</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B197" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C197" t="str">
-        <f t="shared" si="9"/>
-        <v>Repetir nueva contraseña</v>
+        <f>_xlfn.TRANSLATE($B197,$B$2,C$2)</f>
+        <v>Repite una</v>
       </c>
       <c r="D197" t="str">
-        <f t="shared" si="9"/>
-        <v>Répéter le nouveau mot de passe</v>
+        <f>_xlfn.TRANSLATE($B197,$B$2,D$2)</f>
+        <v>Répétez-en un</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>457</v>
+        <v>366</v>
       </c>
       <c r="B198" t="s">
-        <v>458</v>
+        <v>367</v>
       </c>
       <c r="C198" t="str">
-        <f t="shared" si="9"/>
-        <v>Regreso a casa</v>
+        <f>_xlfn.TRANSLATE($B198,$B$2,C$2)</f>
+        <v>Repetir nueva contraseña</v>
       </c>
       <c r="D198" t="str">
-        <f t="shared" si="9"/>
-        <v>Retour à la maison</v>
+        <f>_xlfn.TRANSLATE($B198,$B$2,D$2)</f>
+        <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>368</v>
+        <v>457</v>
       </c>
       <c r="B199" t="s">
-        <v>369</v>
+        <v>458</v>
       </c>
       <c r="C199" t="str">
-        <f t="shared" si="9"/>
-        <v>Guardando...</v>
+        <f>_xlfn.TRANSLATE($B199,$B$2,C$2)</f>
+        <v>Regreso a casa</v>
       </c>
       <c r="D199" t="str">
-        <f t="shared" si="9"/>
-        <v>Sauver...</v>
+        <f>_xlfn.TRANSLATE($B199,$B$2,D$2)</f>
+        <v>Retour à la maison</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B200" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C200" t="str">
-        <f t="shared" si="9"/>
-        <v>Búsqueda</v>
+        <f>_xlfn.TRANSLATE($B200,$B$2,C$2)</f>
+        <v>Guardando...</v>
       </c>
       <c r="D200" t="str">
-        <f t="shared" si="9"/>
-        <v>Recherche</v>
+        <f>_xlfn.TRANSLATE($B200,$B$2,D$2)</f>
+        <v>Sauver...</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B201" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C201" t="str">
-        <f t="shared" si="9"/>
-        <v>Busca artistas, canciones, álbumes...</v>
+        <f>_xlfn.TRANSLATE($B201,$B$2,C$2)</f>
+        <v>Búsqueda</v>
       </c>
       <c r="D201" t="str">
-        <f t="shared" si="9"/>
-        <v>Cherche des artistes, des chansons, des albums...</v>
+        <f>_xlfn.TRANSLATE($B201,$B$2,D$2)</f>
+        <v>Recherche</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B202" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C202" t="str">
-        <f t="shared" si="9"/>
-        <v>Parece que el silencio también es música...</v>
+        <f>_xlfn.TRANSLATE($B202,$B$2,C$2)</f>
+        <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D202" t="str">
-        <f t="shared" si="9"/>
-        <v>Il semble que le silence soit aussi de la musique...</v>
+        <f>_xlfn.TRANSLATE($B202,$B$2,D$2)</f>
+        <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B203" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C203" t="str">
-        <f t="shared" ref="C203:D222" si="10">_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
-        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
+        <f>_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
+        <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D203" t="str">
-        <f t="shared" si="10"/>
-        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
+        <f>_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
+        <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B204" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C204" t="str">
-        <f t="shared" si="10"/>
-        <v>Buscar en la biblioteca</v>
+        <f>_xlfn.TRANSLATE($B204,$B$2,C$2)</f>
+        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D204" t="str">
-        <f t="shared" si="10"/>
-        <v>Recherche dans la bibliothèque</v>
+        <f>_xlfn.TRANSLATE($B204,$B$2,D$2)</f>
+        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B205" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C205" t="str">
-        <f t="shared" si="10"/>
-        <v>Usuarios de búsqueda</v>
+        <f>_xlfn.TRANSLATE($B205,$B$2,C$2)</f>
+        <v>Buscar en la biblioteca</v>
       </c>
       <c r="D205" t="str">
-        <f t="shared" si="10"/>
-        <v>Rechercher les utilisateurs</v>
+        <f>_xlfn.TRANSLATE($B205,$B$2,D$2)</f>
+        <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B206" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C206" t="str">
-        <f t="shared" si="10"/>
-        <v>Enviar canción actual</v>
+        <f>_xlfn.TRANSLATE($B206,$B$2,C$2)</f>
+        <v>Usuarios de búsqueda</v>
       </c>
       <c r="D206" t="str">
-        <f t="shared" si="10"/>
-        <v>Envoyer la chanson actuelle</v>
+        <f>_xlfn.TRANSLATE($B206,$B$2,D$2)</f>
+        <v>Rechercher les utilisateurs</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B207" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C207" t="str">
-        <f t="shared" si="10"/>
-        <v>Septiembre</v>
+        <f>_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
+        <v>Enviar canción actual</v>
       </c>
       <c r="D207" t="str">
-        <f t="shared" si="10"/>
-        <v>Septembre</v>
+        <f>_xlfn.TRANSLATE($B207,$B$2,D$2)</f>
+        <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B208" t="s">
-        <v>60</v>
+        <v>385</v>
       </c>
       <c r="C208" t="str">
-        <f t="shared" si="10"/>
-        <v>Escenarios</v>
+        <f>_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
+        <v>Septiembre</v>
       </c>
       <c r="D208" t="str">
-        <f t="shared" si="10"/>
-        <v>Décors</v>
+        <f>_xlfn.TRANSLATE($B208,$B$2,D$2)</f>
+        <v>Septembre</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B209" t="s">
-        <v>388</v>
+        <v>60</v>
       </c>
       <c r="C209" t="str">
-        <f t="shared" si="10"/>
-        <v>Compartir canción</v>
+        <f>_xlfn.TRANSLATE($B209,$B$2,C$2)</f>
+        <v>Escenarios</v>
       </c>
       <c r="D209" t="str">
-        <f t="shared" si="10"/>
-        <v>Partager la chanson</v>
+        <f>_xlfn.TRANSLATE($B209,$B$2,D$2)</f>
+        <v>Décors</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B210" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C210" t="str">
-        <f t="shared" si="10"/>
-        <v>Canciones compartidas para ti</v>
+        <f>_xlfn.TRANSLATE($B210,$B$2,C$2)</f>
+        <v>Compartir canción</v>
       </c>
       <c r="D210" t="str">
-        <f t="shared" si="10"/>
-        <v>Chansons partagées pour vous</v>
+        <f>_xlfn.TRANSLATE($B210,$B$2,D$2)</f>
+        <v>Partager la chanson</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B211" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C211" t="str">
-        <f t="shared" si="10"/>
-        <v>Compartido desde</v>
+        <f>_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
+        <v>Canciones compartidas para ti</v>
       </c>
       <c r="D211" t="str">
-        <f t="shared" si="10"/>
-        <v>Partagé depuis</v>
+        <f>_xlfn.TRANSLATE($B211,$B$2,D$2)</f>
+        <v>Chansons partagées pour vous</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B212" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C212" t="str">
-        <f t="shared" si="10"/>
-        <v>Mostrando datos de</v>
+        <f>_xlfn.TRANSLATE($B212,$B$2,C$2)</f>
+        <v>Compartido desde</v>
       </c>
       <c r="D212" t="str">
-        <f t="shared" si="10"/>
-        <v>Affichage des données de</v>
+        <f>_xlfn.TRANSLATE($B212,$B$2,D$2)</f>
+        <v>Partagé depuis</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B213" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C213" t="str">
-        <f t="shared" si="10"/>
-        <v>Canción</v>
+        <f>_xlfn.TRANSLATE($B213,$B$2,C$2)</f>
+        <v>Mostrando datos de</v>
       </c>
       <c r="D213" t="str">
-        <f t="shared" si="10"/>
-        <v>Chanson</v>
+        <f>_xlfn.TRANSLATE($B213,$B$2,D$2)</f>
+        <v>Affichage des données de</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B214" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C214" t="str">
-        <f t="shared" si="10"/>
-        <v>Canciones</v>
+        <f>_xlfn.TRANSLATE($B214,$B$2,C$2)</f>
+        <v>Canción</v>
       </c>
       <c r="D214" t="str">
-        <f t="shared" si="10"/>
-        <v>Chansons</v>
+        <f>_xlfn.TRANSLATE($B214,$B$2,D$2)</f>
+        <v>Chanson</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B215" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C215" t="str">
-        <f t="shared" si="10"/>
-        <v>Canciones Solo para ti</v>
+        <f>_xlfn.TRANSLATE($B215,$B$2,C$2)</f>
+        <v>Canciones</v>
       </c>
       <c r="D215" t="str">
-        <f t="shared" si="10"/>
-        <v>Chansons juste pour toi</v>
+        <f>_xlfn.TRANSLATE($B215,$B$2,D$2)</f>
+        <v>Chansons</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B216" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C216" t="str">
-        <f t="shared" si="10"/>
-        <v>Canciones de</v>
+        <f>_xlfn.TRANSLATE($B216,$B$2,C$2)</f>
+        <v>Canciones Solo para ti</v>
       </c>
       <c r="D216" t="str">
-        <f t="shared" si="10"/>
-        <v>Chansons de</v>
+        <f>_xlfn.TRANSLATE($B216,$B$2,D$2)</f>
+        <v>Chansons juste pour toi</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B217" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C217" t="str">
-        <f t="shared" si="10"/>
-        <v>Canciones escuchadas</v>
+        <f>_xlfn.TRANSLATE($B217,$B$2,C$2)</f>
+        <v>Canciones de</v>
       </c>
       <c r="D217" t="str">
-        <f t="shared" si="10"/>
-        <v>Chansons écoutées</v>
+        <f>_xlfn.TRANSLATE($B217,$B$2,D$2)</f>
+        <v>Chansons de</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B218" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C218" t="str">
-        <f t="shared" si="10"/>
-        <v>Estadísticas</v>
+        <f>_xlfn.TRANSLATE($B218,$B$2,C$2)</f>
+        <v>Canciones escuchadas</v>
       </c>
       <c r="D218" t="str">
-        <f t="shared" si="10"/>
-        <v>Statistiques</v>
+        <f>_xlfn.TRANSLATE($B218,$B$2,D$2)</f>
+        <v>Chansons écoutées</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B219" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C219" t="str">
-        <f t="shared" si="10"/>
+        <f>_xlfn.TRANSLATE($B219,$B$2,C$2)</f>
         <v>Estadísticas</v>
       </c>
       <c r="D219" t="str">
-        <f t="shared" si="10"/>
+        <f>_xlfn.TRANSLATE($B219,$B$2,D$2)</f>
         <v>Statistiques</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="B220" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C220" t="str">
-        <f t="shared" si="10"/>
-        <v>¡Para</v>
+        <f>_xlfn.TRANSLATE($B220,$B$2,C$2)</f>
+        <v>Estadísticas</v>
       </c>
       <c r="D220" t="str">
-        <f t="shared" si="10"/>
-        <v>Arrête</v>
+        <f>_xlfn.TRANSLATE($B220,$B$2,D$2)</f>
+        <v>Statistiques</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B221" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C221" t="str">
-        <f t="shared" si="10"/>
-        <v>a</v>
+        <f>_xlfn.TRANSLATE($B221,$B$2,C$2)</f>
+        <v>¡Para</v>
       </c>
       <c r="D221" t="str">
-        <f t="shared" si="10"/>
-        <v>à</v>
+        <f>_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
+        <v>Arrête</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>459</v>
+        <v>411</v>
       </c>
       <c r="B222" t="s">
-        <v>460</v>
+        <v>412</v>
       </c>
       <c r="C222" t="str">
-        <f t="shared" si="10"/>
-        <v>ToDo</v>
+        <f>_xlfn.TRANSLATE($B222,$B$2,C$2)</f>
+        <v>a</v>
       </c>
       <c r="D222" t="str">
-        <f t="shared" si="10"/>
-        <v>ToDo</v>
+        <f>_xlfn.TRANSLATE($B222,$B$2,D$2)</f>
+        <v>à</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>413</v>
+        <v>459</v>
       </c>
       <c r="B223" t="s">
-        <v>414</v>
+        <v>460</v>
       </c>
       <c r="C223" t="str">
-        <f t="shared" ref="C223:D242" si="11">_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
-        <v>Álbumes destacados</v>
+        <f>_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
+        <v>ToDo</v>
       </c>
       <c r="D223" t="str">
-        <f t="shared" si="11"/>
-        <v>Albums phares</v>
+        <f>_xlfn.TRANSLATE($B223,$B$2,D$2)</f>
+        <v>ToDo</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B224" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="C224" t="str">
-        <f t="shared" si="11"/>
-        <v>Canciones principales</v>
+        <f>_xlfn.TRANSLATE($B224,$B$2,C$2)</f>
+        <v>Álbumes destacados</v>
       </c>
       <c r="D224" t="str">
-        <f t="shared" si="11"/>
-        <v>Meilleures chansons</v>
+        <f>_xlfn.TRANSLATE($B224,$B$2,D$2)</f>
+        <v>Albums phares</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B225" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C225" t="str">
-        <f t="shared" si="11"/>
-        <v>Desclavar</v>
+        <f>_xlfn.TRANSLATE($B225,$B$2,C$2)</f>
+        <v>Canciones principales</v>
       </c>
       <c r="D225" t="str">
-        <f t="shared" si="11"/>
-        <v>Détacher</v>
+        <f>_xlfn.TRANSLATE($B225,$B$2,D$2)</f>
+        <v>Meilleures chansons</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B226" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C226" t="str">
-        <f t="shared" si="11"/>
-        <v>Desregistrar</v>
+        <f>_xlfn.TRANSLATE($B226,$B$2,C$2)</f>
+        <v>Desclavar</v>
       </c>
       <c r="D226" t="str">
-        <f t="shared" si="11"/>
-        <v>Désinscription</v>
+        <f>_xlfn.TRANSLATE($B226,$B$2,D$2)</f>
+        <v>Détacher</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="B227" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C227" t="str">
-        <f t="shared" si="11"/>
-        <v>No registrado</v>
+        <f>_xlfn.TRANSLATE($B227,$B$2,C$2)</f>
+        <v>Desregistrar</v>
       </c>
       <c r="D227" t="str">
-        <f t="shared" si="11"/>
-        <v>Non enregistré</v>
+        <f>_xlfn.TRANSLATE($B227,$B$2,D$2)</f>
+        <v>Désinscription</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B228" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C228" t="str">
-        <f t="shared" si="11"/>
-        <v>Dejar de registrarse...</v>
+        <f>_xlfn.TRANSLATE($B228,$B$2,C$2)</f>
+        <v>No registrado</v>
       </c>
       <c r="D228" t="str">
-        <f t="shared" si="11"/>
-        <v>Désenregistrement...</v>
+        <f>_xlfn.TRANSLATE($B228,$B$2,D$2)</f>
+        <v>Non enregistré</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B229" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C229" t="str">
-        <f t="shared" si="11"/>
-        <v>Actualización</v>
+        <f>_xlfn.TRANSLATE($B229,$B$2,C$2)</f>
+        <v>Dejar de registrarse...</v>
       </c>
       <c r="D229" t="str">
-        <f t="shared" si="11"/>
-        <v>Mise à jour</v>
+        <f>_xlfn.TRANSLATE($B229,$B$2,D$2)</f>
+        <v>Désenregistrement...</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B230" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C230" t="str">
-        <f t="shared" si="11"/>
-        <v>Actualizando...</v>
+        <f>_xlfn.TRANSLATE($B230,$B$2,C$2)</f>
+        <v>Actualización</v>
       </c>
       <c r="D230" t="str">
-        <f t="shared" si="11"/>
-        <v>Mise à jour...</v>
+        <f>_xlfn.TRANSLATE($B230,$B$2,D$2)</f>
+        <v>Mise à jour</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B231" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C231" t="str">
-        <f t="shared" si="11"/>
-        <v>Subida</v>
+        <f>_xlfn.TRANSLATE($B231,$B$2,C$2)</f>
+        <v>Actualizando...</v>
       </c>
       <c r="D231" t="str">
-        <f t="shared" si="11"/>
-        <v>Téléverser</v>
+        <f>_xlfn.TRANSLATE($B231,$B$2,D$2)</f>
+        <v>Mise à jour...</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B232" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C232" t="str">
-        <f t="shared" si="11"/>
-        <v>Usuario</v>
+        <f>_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
+        <v>Subida</v>
       </c>
       <c r="D232" t="str">
-        <f t="shared" si="11"/>
-        <v>Utilisateur</v>
+        <f>_xlfn.TRANSLATE($B232,$B$2,D$2)</f>
+        <v>Téléverser</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B233" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C233" t="str">
-        <f t="shared" si="11"/>
-        <v>Configuración de usuario</v>
+        <f>_xlfn.TRANSLATE($B233,$B$2,C$2)</f>
+        <v>Usuario</v>
       </c>
       <c r="D233" t="str">
-        <f t="shared" si="11"/>
-        <v>Paramètres utilisateur</v>
+        <f>_xlfn.TRANSLATE($B233,$B$2,D$2)</f>
+        <v>Utilisateur</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B234" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C234" t="str">
-        <f t="shared" si="11"/>
-        <v>Estadísticas de usuario</v>
+        <f>_xlfn.TRANSLATE($B234,$B$2,C$2)</f>
+        <v>Configuración de usuario</v>
       </c>
       <c r="D234" t="str">
-        <f t="shared" si="11"/>
-        <v>Statistiques des utilisateurs</v>
+        <f>_xlfn.TRANSLATE($B234,$B$2,D$2)</f>
+        <v>Paramètres utilisateur</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B235" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C235" t="str">
-        <f t="shared" si="11"/>
-        <v>Usuarios y amigos</v>
+        <f>_xlfn.TRANSLATE($B235,$B$2,C$2)</f>
+        <v>Estadísticas de usuario</v>
       </c>
       <c r="D235" t="str">
-        <f t="shared" si="11"/>
-        <v>Utilisateurs et amis</v>
+        <f>_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
+        <v>Statistiques des utilisateurs</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="B236" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C236" t="str">
-        <f t="shared" si="11"/>
-        <v>Lista de usuarios</v>
+        <f>_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
+        <v>Usuarios y amigos</v>
       </c>
       <c r="D236" t="str">
-        <f t="shared" si="11"/>
-        <v>Liste des utilisateurs</v>
+        <f>_xlfn.TRANSLATE($B236,$B$2,D$2)</f>
+        <v>Utilisateurs et amis</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B237" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C237" t="str">
-        <f t="shared" si="11"/>
-        <v>Vídeos</v>
+        <f>_xlfn.TRANSLATE($B237,$B$2,C$2)</f>
+        <v>Lista de usuarios</v>
       </c>
       <c r="D237" t="str">
-        <f t="shared" si="11"/>
-        <v>Vidéos</v>
+        <f>_xlfn.TRANSLATE($B237,$B$2,D$2)</f>
+        <v>Liste des utilisateurs</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B238" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C238" t="str">
-        <f t="shared" si="11"/>
-        <v>También puede que te interese</v>
+        <f>_xlfn.TRANSLATE($B238,$B$2,C$2)</f>
+        <v>Vídeos</v>
       </c>
       <c r="D238" t="str">
-        <f t="shared" si="11"/>
-        <v>Ça pourrait aussi te plaire</v>
+        <f>_xlfn.TRANSLATE($B238,$B$2,D$2)</f>
+        <v>Vidéos</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B239" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C239" t="str">
-        <f t="shared" si="11"/>
-        <v>Tu</v>
+        <f>_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
+        <v>También puede que te interese</v>
       </c>
       <c r="D239" t="str">
-        <f t="shared" si="11"/>
-        <v>Votre</v>
+        <f>_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
+        <v>Ça pourrait aussi te plaire</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B240" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C240" t="str">
-        <f t="shared" si="11"/>
-        <v>Tus álbumes y listas de reproducción</v>
+        <f>_xlfn.TRANSLATE($B240,$B$2,C$2)</f>
+        <v>Tu</v>
       </c>
       <c r="D240" t="str">
-        <f t="shared" si="11"/>
-        <v>Vos albums et playlists</v>
+        <f>_xlfn.TRANSLATE($B240,$B$2,D$2)</f>
+        <v>Votre</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B241" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C241" t="str">
-        <f t="shared" si="11"/>
-        <v>Tu mezcla</v>
+        <f>_xlfn.TRANSLATE($B241,$B$2,C$2)</f>
+        <v>Tus álbumes y listas de reproducción</v>
       </c>
       <c r="D241" t="str">
-        <f t="shared" si="11"/>
-        <v>Votre Mix</v>
+        <f>_xlfn.TRANSLATE($B241,$B$2,D$2)</f>
+        <v>Vos albums et playlists</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B242" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C242" t="str">
-        <f t="shared" si="11"/>
-        <v>Vídeos de YouTube</v>
+        <f>_xlfn.TRANSLATE($B242,$B$2,C$2)</f>
+        <v>Tu mezcla</v>
       </c>
       <c r="D242" t="str">
-        <f t="shared" si="11"/>
-        <v>Vidéos YouTube</v>
+        <f>_xlfn.TRANSLATE($B242,$B$2,D$2)</f>
+        <v>Votre Mix</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>479</v>
+        <v>451</v>
       </c>
       <c r="B243" t="s">
-        <v>480</v>
+        <v>452</v>
       </c>
       <c r="C243" t="str">
-        <f t="shared" ref="C243:D255" si="12">_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
-        <v>Nueva versión disponible</v>
+        <f>_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
+        <v>Vídeos de YouTube</v>
       </c>
       <c r="D243" t="str">
-        <f t="shared" si="12"/>
-        <v>Nouvelle version disponible</v>
+        <f>_xlfn.TRANSLATE($B243,$B$2,D$2)</f>
+        <v>Vidéos YouTube</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C244" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B244,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D244" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B244,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C245" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B245,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D245" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B245,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C246" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B246,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D246" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B246,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C247" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B247,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D247" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B247,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C248" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B248,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D248" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B248,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C249" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B249,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D249" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B249,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C250" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B250,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D250" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B250,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C251" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B251,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D251" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B251,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C252" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B252,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D252" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B252,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C253" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B253,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D253" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B253,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C254" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B254,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D254" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B254,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C255" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B255,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D255" t="str">
-        <f t="shared" si="12"/>
+        <f>_xlfn.TRANSLATE($B255,$B$2,D$2)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Added keys to vocabulary
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Documents\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ABBC3E3-651B-47D2-9C41-85ABEA1D3D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51927A1-EB4A-4AF5-9075-86B2A334EA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="1170" windowWidth="32490" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="495">
   <si>
     <t>KEY</t>
   </si>
@@ -1482,6 +1482,42 @@
   </si>
   <si>
     <t>Reproducir a continuación</t>
+  </si>
+  <si>
+    <t>STARTING</t>
+  </si>
+  <si>
+    <t>COMPLETED</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>DOWNLOADING</t>
+  </si>
+  <si>
+    <t>RETRY</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Downloading</t>
+  </si>
+  <si>
+    <t>Retry</t>
+  </si>
+  <si>
+    <t>Reintentar</t>
+  </si>
+  <si>
+    <t>Fallido</t>
+  </si>
+  <si>
+    <t>Starting…</t>
   </si>
 </sst>
 </file>
@@ -1886,11 +1922,11 @@
         <v>8</v>
       </c>
       <c r="C3" t="str">
-        <f>_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
+        <f t="shared" ref="C3:D22" si="0">_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
       <c r="D3" t="str">
-        <f>_xlfn.TRANSLATE($B3,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente de façon aléatoire</v>
       </c>
     </row>
@@ -1902,11 +1938,11 @@
         <v>10</v>
       </c>
       <c r="C4" t="str">
-        <f>_xlfn.TRANSLATE($B4,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista al final de la cola</v>
       </c>
       <c r="D4" t="str">
-        <f>_xlfn.TRANSLATE($B4,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste en bas de la file d’attente</v>
       </c>
     </row>
@@ -1918,11 +1954,11 @@
         <v>12</v>
       </c>
       <c r="C5" t="str">
-        <f>_xlfn.TRANSLATE($B5,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista a la cola</v>
       </c>
       <c r="D5" t="str">
-        <f>_xlfn.TRANSLATE($B5,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente</v>
       </c>
     </row>
@@ -1934,11 +1970,11 @@
         <v>456</v>
       </c>
       <c r="C6" t="str">
-        <f>_xlfn.TRANSLATE($B6,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir medios a la lista de reproducción</v>
       </c>
       <c r="D6" t="str">
-        <f>_xlfn.TRANSLATE($B6,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter un média à une playlist</v>
       </c>
     </row>
@@ -1950,11 +1986,11 @@
         <v>14</v>
       </c>
       <c r="C7" t="str">
-        <f>_xlfn.TRANSLATE($B7,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
       <c r="D7" t="str">
-        <f>_xlfn.TRANSLATE($B7,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la playlist</v>
       </c>
     </row>
@@ -1966,11 +2002,11 @@
         <v>16</v>
       </c>
       <c r="C8" t="str">
-        <f>_xlfn.TRANSLATE($B8,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la cola</v>
       </c>
       <c r="D8" t="str">
-        <f>_xlfn.TRANSLATE($B8,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la file d’attente</v>
       </c>
     </row>
@@ -1982,11 +2018,11 @@
         <v>18</v>
       </c>
       <c r="C9" t="str">
-        <f>_xlfn.TRANSLATE($B9,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la biblioteca</v>
       </c>
       <c r="D9" t="str">
-        <f>_xlfn.TRANSLATE($B9,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la bibliothèque</v>
       </c>
     </row>
@@ -1998,11 +2034,11 @@
         <v>20</v>
       </c>
       <c r="C10" t="str">
-        <f>_xlfn.TRANSLATE($B10,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a los que me gusta</v>
       </c>
       <c r="D10" t="str">
-        <f>_xlfn.TRANSLATE($B10,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter aux aimés</v>
       </c>
     </row>
@@ -2014,11 +2050,11 @@
         <v>22</v>
       </c>
       <c r="C11" t="str">
-        <f>_xlfn.TRANSLATE($B11,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la cola</v>
       </c>
       <c r="D11" t="str">
-        <f>_xlfn.TRANSLATE($B11,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la file d’attente</v>
       </c>
     </row>
@@ -2030,11 +2066,11 @@
         <v>468</v>
       </c>
       <c r="C12" t="str">
-        <f>_xlfn.TRANSLATE($B12,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadido a la lista de reproducción</v>
       </c>
       <c r="D12" t="str">
-        <f>_xlfn.TRANSLATE($B12,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouté à la playlist</v>
       </c>
     </row>
@@ -2046,11 +2082,11 @@
         <v>24</v>
       </c>
       <c r="C13" t="str">
-        <f>_xlfn.TRANSLATE($B13,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir Build</v>
       </c>
       <c r="D13" t="str">
-        <f>_xlfn.TRANSLATE($B13,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une construction</v>
       </c>
     </row>
@@ -2062,11 +2098,11 @@
         <v>26</v>
       </c>
       <c r="C14" t="str">
-        <f>_xlfn.TRANSLATE($B14,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Archivo APK</v>
       </c>
       <c r="D14" t="str">
-        <f>_xlfn.TRANSLATE($B14,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Fichier APK</v>
       </c>
     </row>
@@ -2078,11 +2114,11 @@
         <v>28</v>
       </c>
       <c r="C15" t="str">
-        <f>_xlfn.TRANSLATE($B15,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Gestiona tus builds de Android</v>
       </c>
       <c r="D15" t="str">
-        <f>_xlfn.TRANSLATE($B15,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Gérez vos versions Android</v>
       </c>
     </row>
@@ -2094,11 +2130,11 @@
         <v>30</v>
       </c>
       <c r="C16" t="str">
-        <f>_xlfn.TRANSLATE($B16,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Construcciones</v>
       </c>
       <c r="D16" t="str">
-        <f>_xlfn.TRANSLATE($B16,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -2110,11 +2146,11 @@
         <v>32</v>
       </c>
       <c r="C17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Cancelar</v>
       </c>
       <c r="D17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -2126,11 +2162,11 @@
         <v>34</v>
       </c>
       <c r="C18" t="str">
-        <f>_xlfn.TRANSLATE($B18,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Descripción</v>
       </c>
       <c r="D18" t="str">
-        <f>_xlfn.TRANSLATE($B18,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Description</v>
       </c>
     </row>
@@ -2142,11 +2178,11 @@
         <v>36</v>
       </c>
       <c r="C19" t="str">
-        <f>_xlfn.TRANSLATE($B19,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Aquí entra la descripción...</v>
       </c>
       <c r="D19" t="str">
-        <f>_xlfn.TRANSLATE($B19,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Voici la description...</v>
       </c>
     </row>
@@ -2158,11 +2194,11 @@
         <v>38</v>
       </c>
       <c r="C20" t="str">
-        <f>_xlfn.TRANSLATE($B20,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Enter Version</v>
       </c>
       <c r="D20" t="str">
-        <f>_xlfn.TRANSLATE($B20,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Enter Version</v>
       </c>
     </row>
@@ -2174,11 +2210,11 @@
         <v>40</v>
       </c>
       <c r="C21" t="str">
-        <f>_xlfn.TRANSLATE($B21,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Últimas novedades</v>
       </c>
       <c r="D21" t="str">
-        <f>_xlfn.TRANSLATE($B21,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Dernières nouvelles</v>
       </c>
     </row>
@@ -2190,11 +2226,11 @@
         <v>42</v>
       </c>
       <c r="C22" t="str">
-        <f>_xlfn.TRANSLATE($B22,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Aún no hay builds</v>
       </c>
       <c r="D22" t="str">
-        <f>_xlfn.TRANSLATE($B22,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Pas encore de builds</v>
       </c>
     </row>
@@ -2206,11 +2242,11 @@
         <v>44</v>
       </c>
       <c r="C23" t="str">
-        <f>_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
+        <f t="shared" ref="C23:D42" si="1">_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
         <v>Solo APK</v>
       </c>
       <c r="D23" t="str">
-        <f>_xlfn.TRANSLATE($B23,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Seul APK</v>
       </c>
     </row>
@@ -2222,11 +2258,11 @@
         <v>46</v>
       </c>
       <c r="C24" t="str">
-        <f>_xlfn.TRANSLATE($B24,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Opcional</v>
       </c>
       <c r="D24" t="str">
-        <f>_xlfn.TRANSLATE($B24,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Optionnel</v>
       </c>
     </row>
@@ -2238,11 +2274,11 @@
         <v>48</v>
       </c>
       <c r="C25" t="str">
-        <f>_xlfn.TRANSLATE($B25,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Leer Fallido</v>
       </c>
       <c r="D25" t="str">
-        <f>_xlfn.TRANSLATE($B25,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Lire Échec</v>
       </c>
     </row>
@@ -2254,11 +2290,11 @@
         <v>50</v>
       </c>
       <c r="C26" t="str">
-        <f>_xlfn.TRANSLATE($B26,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Obligatorio</v>
       </c>
       <c r="D26" t="str">
-        <f>_xlfn.TRANSLATE($B26,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Obligatoire</v>
       </c>
     </row>
@@ -2270,11 +2306,11 @@
         <v>52</v>
       </c>
       <c r="C27" t="str">
-        <f>_xlfn.TRANSLATE($B27,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Seleccionar APK</v>
       </c>
       <c r="D27" t="str">
-        <f>_xlfn.TRANSLATE($B27,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Sélectionner APK</v>
       </c>
     </row>
@@ -2286,11 +2322,11 @@
         <v>54</v>
       </c>
       <c r="C28" t="str">
-        <f>_xlfn.TRANSLATE($B28,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Seleccionados</v>
       </c>
       <c r="D28" t="str">
-        <f>_xlfn.TRANSLATE($B28,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Sélectionné</v>
       </c>
     </row>
@@ -2302,11 +2338,11 @@
         <v>56</v>
       </c>
       <c r="C29" t="str">
-        <f>_xlfn.TRANSLATE($B29,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Próximamente</v>
       </c>
       <c r="D29" t="str">
-        <f>_xlfn.TRANSLATE($B29,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -2318,11 +2354,11 @@
         <v>58</v>
       </c>
       <c r="C30" t="str">
-        <f>_xlfn.TRANSLATE($B30,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Configuración de plataformas</v>
       </c>
       <c r="D30" t="str">
-        <f>_xlfn.TRANSLATE($B30,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Réglages de la plateforme</v>
       </c>
     </row>
@@ -2334,11 +2370,11 @@
         <v>60</v>
       </c>
       <c r="C31" t="str">
-        <f>_xlfn.TRANSLATE($B31,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Escenarios</v>
       </c>
       <c r="D31" t="str">
-        <f>_xlfn.TRANSLATE($B31,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Décors</v>
       </c>
     </row>
@@ -2350,11 +2386,11 @@
         <v>30</v>
       </c>
       <c r="C32" t="str">
-        <f>_xlfn.TRANSLATE($B32,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Construcciones</v>
       </c>
       <c r="D32" t="str">
-        <f>_xlfn.TRANSLATE($B32,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -2366,11 +2402,11 @@
         <v>60</v>
       </c>
       <c r="C33" t="str">
-        <f>_xlfn.TRANSLATE($B33,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Escenarios</v>
       </c>
       <c r="D33" t="str">
-        <f>_xlfn.TRANSLATE($B33,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Décors</v>
       </c>
     </row>
@@ -2382,11 +2418,11 @@
         <v>64</v>
       </c>
       <c r="C34" t="str">
-        <f>_xlfn.TRANSLATE($B34,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Usuarios</v>
       </c>
       <c r="D34" t="str">
-        <f>_xlfn.TRANSLATE($B34,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -2398,11 +2434,11 @@
         <v>66</v>
       </c>
       <c r="C35" t="str">
-        <f>_xlfn.TRANSLATE($B35,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Compilación de subida</v>
       </c>
       <c r="D35" t="str">
-        <f>_xlfn.TRANSLATE($B35,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Upload Build</v>
       </c>
     </row>
@@ -2414,11 +2450,11 @@
         <v>68</v>
       </c>
       <c r="C36" t="str">
-        <f>_xlfn.TRANSLATE($B36,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Fallido en la subida</v>
       </c>
       <c r="D36" t="str">
-        <f>_xlfn.TRANSLATE($B36,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Téléchargement échoué</v>
       </c>
     </row>
@@ -2430,11 +2466,11 @@
         <v>70</v>
       </c>
       <c r="C37" t="str">
-        <f>_xlfn.TRANSLATE($B37,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Sube tu primera construcción</v>
       </c>
       <c r="D37" t="str">
-        <f>_xlfn.TRANSLATE($B37,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Téléchargez votre première compilation</v>
       </c>
     </row>
@@ -2446,11 +2482,11 @@
         <v>72</v>
       </c>
       <c r="C38" t="str">
-        <f>_xlfn.TRANSLATE($B38,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Subir nueva versión</v>
       </c>
       <c r="D38" t="str">
-        <f>_xlfn.TRANSLATE($B38,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Télécharger une nouvelle version</v>
       </c>
     </row>
@@ -2462,11 +2498,11 @@
         <v>74</v>
       </c>
       <c r="C39" t="str">
-        <f>_xlfn.TRANSLATE($B39,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Éxito en la subida</v>
       </c>
       <c r="D39" t="str">
-        <f>_xlfn.TRANSLATE($B39,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Succès de la télévision</v>
       </c>
     </row>
@@ -2478,11 +2514,11 @@
         <v>76</v>
       </c>
       <c r="C40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Subiendo algo...</v>
       </c>
       <c r="D40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Téléchargement...</v>
       </c>
     </row>
@@ -2494,11 +2530,11 @@
         <v>56</v>
       </c>
       <c r="C41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Próximamente</v>
       </c>
       <c r="D41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -2510,11 +2546,11 @@
         <v>79</v>
       </c>
       <c r="C42" t="str">
-        <f>_xlfn.TRANSLATE($B42,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Gestionar los usuarios de la plataforma</v>
       </c>
       <c r="D42" t="str">
-        <f>_xlfn.TRANSLATE($B42,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Gérer les utilisateurs de la plateforme</v>
       </c>
     </row>
@@ -2526,11 +2562,11 @@
         <v>64</v>
       </c>
       <c r="C43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
+        <f t="shared" ref="C43:D62" si="2">_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
         <v>Usuarios</v>
       </c>
       <c r="D43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -2542,11 +2578,11 @@
         <v>82</v>
       </c>
       <c r="C44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Versión</v>
       </c>
       <c r="D44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Version</v>
       </c>
     </row>
@@ -2558,11 +2594,11 @@
         <v>84</v>
       </c>
       <c r="C45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Álbum</v>
       </c>
       <c r="D45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Album</v>
       </c>
     </row>
@@ -2574,11 +2610,11 @@
         <v>86</v>
       </c>
       <c r="C46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Álbumes</v>
       </c>
       <c r="D46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums</v>
       </c>
     </row>
@@ -2590,11 +2626,11 @@
         <v>88</v>
       </c>
       <c r="C47" t="str">
-        <f>_xlfn.TRANSLATE($B47,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Álbumes y sencillos</v>
       </c>
       <c r="D47" t="str">
-        <f>_xlfn.TRANSLATE($B47,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums et singles</v>
       </c>
     </row>
@@ -2606,11 +2642,11 @@
         <v>90</v>
       </c>
       <c r="C48" t="str">
-        <f>_xlfn.TRANSLATE($B48,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Todos</v>
       </c>
       <c r="D48" t="str">
-        <f>_xlfn.TRANSLATE($B48,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Tous</v>
       </c>
     </row>
@@ -2622,11 +2658,11 @@
         <v>92</v>
       </c>
       <c r="C49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Abril</v>
       </c>
       <c r="D49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Avril</v>
       </c>
     </row>
@@ -2638,11 +2674,11 @@
         <v>94</v>
       </c>
       <c r="C50" t="str">
-        <f>_xlfn.TRANSLATE($B50,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Artista</v>
       </c>
       <c r="D50" t="str">
-        <f>_xlfn.TRANSLATE($B50,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artiste</v>
       </c>
     </row>
@@ -2654,11 +2690,11 @@
         <v>96</v>
       </c>
       <c r="C51" t="str">
-        <f>_xlfn.TRANSLATE($B51,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Artistas</v>
       </c>
       <c r="D51" t="str">
-        <f>_xlfn.TRANSLATE($B51,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artistes</v>
       </c>
     </row>
@@ -2670,11 +2706,11 @@
         <v>98</v>
       </c>
       <c r="C52" t="str">
-        <f>_xlfn.TRANSLATE($B52,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Agosto</v>
       </c>
       <c r="D52" t="str">
-        <f>_xlfn.TRANSLATE($B52,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Août</v>
       </c>
     </row>
@@ -2686,11 +2722,11 @@
         <v>100</v>
       </c>
       <c r="C53" t="str">
-        <f>_xlfn.TRANSLATE($B53,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Minutos medios por canción</v>
       </c>
       <c r="D53" t="str">
-        <f>_xlfn.TRANSLATE($B53,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Minutes moyennes par chanson</v>
       </c>
     </row>
@@ -2702,11 +2738,11 @@
         <v>102</v>
       </c>
       <c r="C54" t="str">
-        <f>_xlfn.TRANSLATE($B54,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>por</v>
       </c>
       <c r="D54" t="str">
-        <f>_xlfn.TRANSLATE($B54,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>par</v>
       </c>
     </row>
@@ -2718,11 +2754,11 @@
         <v>32</v>
       </c>
       <c r="C55" t="str">
-        <f>_xlfn.TRANSLATE($B55,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Cancelar</v>
       </c>
       <c r="D55" t="str">
-        <f>_xlfn.TRANSLATE($B55,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -2734,11 +2770,11 @@
         <v>105</v>
       </c>
       <c r="C56" t="str">
-        <f>_xlfn.TRANSLATE($B56,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Cambiar contraseña</v>
       </c>
       <c r="D56" t="str">
-        <f>_xlfn.TRANSLATE($B56,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Changer le mot de passe</v>
       </c>
     </row>
@@ -2750,11 +2786,11 @@
         <v>107</v>
       </c>
       <c r="C57" t="str">
-        <f>_xlfn.TRANSLATE($B57,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Descargas claras</v>
       </c>
       <c r="D57" t="str">
-        <f>_xlfn.TRANSLATE($B57,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargements clairs</v>
       </c>
     </row>
@@ -2766,11 +2802,11 @@
         <v>109</v>
       </c>
       <c r="C58" t="str">
-        <f>_xlfn.TRANSLATE($B58,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Haz clic para descargar</v>
       </c>
       <c r="D58" t="str">
-        <f>_xlfn.TRANSLATE($B58,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Cliquez pour télécharger</v>
       </c>
     </row>
@@ -2782,11 +2818,11 @@
         <v>111</v>
       </c>
       <c r="C59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Topo comunitario</v>
       </c>
       <c r="D59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sommet communautaire</v>
       </c>
     </row>
@@ -2798,11 +2834,11 @@
         <v>113</v>
       </c>
       <c r="C60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>URL de la lista de copiar</v>
       </c>
       <c r="D60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>URL de la liste de copie</v>
       </c>
     </row>
@@ -2814,11 +2850,11 @@
         <v>115</v>
       </c>
       <c r="C61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Copiar la URL de la canción</v>
       </c>
       <c r="D61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Copier l’URL de la chanson</v>
       </c>
     </row>
@@ -2830,11 +2866,11 @@
         <v>117</v>
       </c>
       <c r="C62" t="str">
-        <f>_xlfn.TRANSLATE($B62,$B$2,C$2)</f>
+        <f t="shared" si="2"/>
         <v>Crear</v>
       </c>
       <c r="D62" t="str">
-        <f>_xlfn.TRANSLATE($B62,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Créer</v>
       </c>
     </row>
@@ -2846,11 +2882,11 @@
         <v>119</v>
       </c>
       <c r="C63" t="str">
-        <f>_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
+        <f t="shared" ref="C63:D82" si="3">_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
         <v>Crear...</v>
       </c>
       <c r="D63" t="str">
-        <f>_xlfn.TRANSLATE($B63,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Créer...</v>
       </c>
     </row>
@@ -2862,11 +2898,11 @@
         <v>121</v>
       </c>
       <c r="C64" t="str">
-        <f>_xlfn.TRANSLATE($B64,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Fecha añadida</v>
       </c>
       <c r="D64" t="str">
-        <f>_xlfn.TRANSLATE($B64,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Date ajoutée</v>
       </c>
     </row>
@@ -2878,11 +2914,11 @@
         <v>123</v>
       </c>
       <c r="C65" t="str">
-        <f>_xlfn.TRANSLATE($B65,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Diciembre</v>
       </c>
       <c r="D65" t="str">
-        <f>_xlfn.TRANSLATE($B65,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Décembre</v>
       </c>
     </row>
@@ -2894,11 +2930,11 @@
         <v>125</v>
       </c>
       <c r="C66" t="str">
-        <f>_xlfn.TRANSLATE($B66,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Tu dispositivo no soporta al trabajador de servicio</v>
       </c>
       <c r="D66" t="str">
-        <f>_xlfn.TRANSLATE($B66,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Votre appareil ne prend pas en charge l’assistant de service</v>
       </c>
     </row>
@@ -2910,11 +2946,11 @@
         <v>127</v>
       </c>
       <c r="C67" t="str">
-        <f>_xlfn.TRANSLATE($B67,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Disco</v>
       </c>
       <c r="D67" t="str">
-        <f>_xlfn.TRANSLATE($B67,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Disque</v>
       </c>
     </row>
@@ -2926,11 +2962,11 @@
         <v>129</v>
       </c>
       <c r="C68" t="str">
-        <f>_xlfn.TRANSLATE($B68,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Nombre de Muestra</v>
       </c>
       <c r="D68" t="str">
-        <f>_xlfn.TRANSLATE($B68,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Nom d’affichage</v>
       </c>
     </row>
@@ -2942,11 +2978,11 @@
         <v>131</v>
       </c>
       <c r="C69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargar</v>
       </c>
       <c r="D69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Télécharger</v>
       </c>
     </row>
@@ -2958,11 +2994,11 @@
         <v>133</v>
       </c>
       <c r="C70" t="str">
-        <f>_xlfn.TRANSLATE($B70,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descarga la app para escuchar offline</v>
       </c>
       <c r="D70" t="str">
-        <f>_xlfn.TRANSLATE($B70,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Téléchargez l’application pour une écoute hors ligne</v>
       </c>
     </row>
@@ -2974,11 +3010,11 @@
         <v>135</v>
       </c>
       <c r="C71" t="str">
-        <f>_xlfn.TRANSLATE($B71,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
       <c r="D71" t="str">
-        <f>_xlfn.TRANSLATE($B71,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Saisissez une URL Spotify ou YouTube Music</v>
       </c>
     </row>
@@ -2990,11 +3026,11 @@
         <v>137</v>
       </c>
       <c r="C72" t="str">
-        <f>_xlfn.TRANSLATE($B72,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Lista de descargas al dispositivo</v>
       </c>
       <c r="D72" t="str">
-        <f>_xlfn.TRANSLATE($B72,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Liste de téléchargement vers l’appareil</v>
       </c>
     </row>
@@ -3006,11 +3042,11 @@
         <v>139</v>
       </c>
       <c r="C73" t="str">
-        <f>_xlfn.TRANSLATE($B73,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargar medios al dispositivo</v>
       </c>
       <c r="D73" t="str">
-        <f>_xlfn.TRANSLATE($B73,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Télécharger des médias sur l’appareil</v>
       </c>
     </row>
@@ -3022,11 +3058,11 @@
         <v>141</v>
       </c>
       <c r="C74" t="str">
-        <f>_xlfn.TRANSLATE($B74,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargar mp</v>
       </c>
       <c r="D74" t="str">
-        <f>_xlfn.TRANSLATE($B74,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Télécharger le MP</v>
       </c>
     </row>
@@ -3038,11 +3074,11 @@
         <v>143</v>
       </c>
       <c r="C75" t="str">
-        <f>_xlfn.TRANSLATE($B75,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargar canción al dispositivo</v>
       </c>
       <c r="D75" t="str">
-        <f>_xlfn.TRANSLATE($B75,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Télécharger la chanson sur l’appareil</v>
       </c>
     </row>
@@ -3054,11 +3090,11 @@
         <v>145</v>
       </c>
       <c r="C76" t="str">
-        <f>_xlfn.TRANSLATE($B76,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descarga iniciada</v>
       </c>
       <c r="D76" t="str">
-        <f>_xlfn.TRANSLATE($B76,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Téléchargement lancé</v>
       </c>
     </row>
@@ -3070,11 +3106,11 @@
         <v>147</v>
       </c>
       <c r="C77" t="str">
-        <f>_xlfn.TRANSLATE($B77,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargar ZIP</v>
       </c>
       <c r="D77" t="str">
-        <f>_xlfn.TRANSLATE($B77,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Télécharger ZIP</v>
       </c>
     </row>
@@ -3086,11 +3122,11 @@
         <v>149</v>
       </c>
       <c r="C78" t="str">
-        <f>_xlfn.TRANSLATE($B78,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Descargas</v>
       </c>
       <c r="D78" t="str">
-        <f>_xlfn.TRANSLATE($B78,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Téléchargements</v>
       </c>
     </row>
@@ -3102,11 +3138,11 @@
         <v>151</v>
       </c>
       <c r="C79" t="str">
-        <f>_xlfn.TRANSLATE($B79,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Duración</v>
       </c>
       <c r="D79" t="str">
-        <f>_xlfn.TRANSLATE($B79,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Durée</v>
       </c>
     </row>
@@ -3118,11 +3154,11 @@
         <v>153</v>
       </c>
       <c r="C80" t="str">
-        <f>_xlfn.TRANSLATE($B80,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Energía</v>
       </c>
       <c r="D80" t="str">
-        <f>_xlfn.TRANSLATE($B80,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Énergie</v>
       </c>
     </row>
@@ -3134,11 +3170,11 @@
         <v>155</v>
       </c>
       <c r="C81" t="str">
-        <f>_xlfn.TRANSLATE($B81,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D81" t="str">
-        <f>_xlfn.TRANSLATE($B81,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3150,11 +3186,11 @@
         <v>157</v>
       </c>
       <c r="C82" t="str">
-        <f>_xlfn.TRANSLATE($B82,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Error</v>
       </c>
       <c r="D82" t="str">
-        <f>_xlfn.TRANSLATE($B82,$B$2,D$2)</f>
+        <f t="shared" si="3"/>
         <v>Erreur</v>
       </c>
     </row>
@@ -3166,11 +3202,11 @@
         <v>159</v>
       </c>
       <c r="C83" t="str">
-        <f>_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
+        <f t="shared" ref="C83:D102" si="4">_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
         <v>Lenguaje de cambio de error</v>
       </c>
       <c r="D83" t="str">
-        <f>_xlfn.TRANSLATE($B83,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Langage de changement d’erreur</v>
       </c>
     </row>
@@ -3182,11 +3218,11 @@
         <v>161</v>
       </c>
       <c r="C84" t="str">
-        <f>_xlfn.TRANSLATE($B84,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D84" t="str">
-        <f>_xlfn.TRANSLATE($B84,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3198,11 +3234,11 @@
         <v>161</v>
       </c>
       <c r="C85" t="str">
-        <f>_xlfn.TRANSLATE($B85,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D85" t="str">
-        <f>_xlfn.TRANSLATE($B85,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3214,11 +3250,11 @@
         <v>155</v>
       </c>
       <c r="C86" t="str">
-        <f>_xlfn.TRANSLATE($B86,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D86" t="str">
-        <f>_xlfn.TRANSLATE($B86,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3230,11 +3266,11 @@
         <v>475</v>
       </c>
       <c r="C87" t="str">
-        <f>_xlfn.TRANSLATE($B87,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al obtener descargas</v>
       </c>
       <c r="D87" t="str">
-        <f>_xlfn.TRANSLATE($B87,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur de téléchargement</v>
       </c>
     </row>
@@ -3246,11 +3282,11 @@
         <v>165</v>
       </c>
       <c r="C88" t="str">
-        <f>_xlfn.TRANSLATE($B88,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Cola de obtención de errores</v>
       </c>
       <c r="D88" t="str">
-        <f>_xlfn.TRANSLATE($B88,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>File d’attente d’obtention d’erreurs</v>
       </c>
     </row>
@@ -3262,11 +3298,11 @@
         <v>476</v>
       </c>
       <c r="C89" t="str">
-        <f>_xlfn.TRANSLATE($B89,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Usuario que obtiene errores</v>
       </c>
       <c r="D89" t="str">
-        <f>_xlfn.TRANSLATE($B89,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Utilisateur d’obtention d’erreurs</v>
       </c>
     </row>
@@ -3278,11 +3314,11 @@
         <v>167</v>
       </c>
       <c r="C90" t="str">
-        <f>_xlfn.TRANSLATE($B90,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al dar like a medios</v>
       </c>
       <c r="D90" t="str">
-        <f>_xlfn.TRANSLATE($B90,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur d’appréciation des médias</v>
       </c>
     </row>
@@ -3294,11 +3330,11 @@
         <v>474</v>
       </c>
       <c r="C91" t="str">
-        <f>_xlfn.TRANSLATE($B91,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Búsqueda de errores</v>
       </c>
       <c r="D91" t="str">
-        <f>_xlfn.TRANSLATE($B91,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Recherche d’erreurs</v>
       </c>
     </row>
@@ -3310,11 +3346,11 @@
         <v>169</v>
       </c>
       <c r="C92" t="str">
-        <f>_xlfn.TRANSLATE($B92,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al iniciar la descarga</v>
       </c>
       <c r="D92" t="str">
-        <f>_xlfn.TRANSLATE($B92,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur au démarrage du téléchargement</v>
       </c>
     </row>
@@ -3326,11 +3362,11 @@
         <v>171</v>
       </c>
       <c r="C93" t="str">
-        <f>_xlfn.TRANSLATE($B93,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Error al dejar de dar like a los medios</v>
       </c>
       <c r="D93" t="str">
-        <f>_xlfn.TRANSLATE($B93,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Erreur de non-like des médias</v>
       </c>
     </row>
@@ -3342,11 +3378,11 @@
         <v>464</v>
       </c>
       <c r="C94" t="str">
-        <f>_xlfn.TRANSLATE($B94,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>No se añadió contenido a la biblioteca</v>
       </c>
       <c r="D94" t="str">
-        <f>_xlfn.TRANSLATE($B94,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Échec d’ajouter des médias à la bibliothèque</v>
       </c>
     </row>
@@ -3358,11 +3394,11 @@
         <v>470</v>
       </c>
       <c r="C95" t="str">
-        <f>_xlfn.TRANSLATE($B95,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>No se añadió contenido a la lista de reproducción</v>
       </c>
       <c r="D95" t="str">
-        <f>_xlfn.TRANSLATE($B95,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Échec d’ajouter des médias à la playlist</v>
       </c>
     </row>
@@ -3374,11 +3410,11 @@
         <v>173</v>
       </c>
       <c r="C96" t="str">
-        <f>_xlfn.TRANSLATE($B96,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>No cambiaron el idioma</v>
       </c>
       <c r="D96" t="str">
-        <f>_xlfn.TRANSLATE($B96,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Échec de changer de langue</v>
       </c>
     </row>
@@ -3390,11 +3426,11 @@
         <v>466</v>
       </c>
       <c r="C97" t="str">
-        <f>_xlfn.TRANSLATE($B97,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>No se han conseguido las listas de reproducción</v>
       </c>
       <c r="D97" t="str">
-        <f>_xlfn.TRANSLATE($B97,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Échec à récupérer les playlists</v>
       </c>
     </row>
@@ -3406,11 +3442,11 @@
         <v>175</v>
       </c>
       <c r="C98" t="str">
-        <f>_xlfn.TRANSLATE($B98,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D98" t="str">
-        <f>_xlfn.TRANSLATE($B98,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Albums en vedette</v>
       </c>
     </row>
@@ -3422,11 +3458,11 @@
         <v>177</v>
       </c>
       <c r="C99" t="str">
-        <f>_xlfn.TRANSLATE($B99,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Listas destacadas</v>
       </c>
       <c r="D99" t="str">
-        <f>_xlfn.TRANSLATE($B99,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Listes en vedette</v>
       </c>
     </row>
@@ -3438,11 +3474,11 @@
         <v>179</v>
       </c>
       <c r="C100" t="str">
-        <f>_xlfn.TRANSLATE($B100,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Febrero</v>
       </c>
       <c r="D100" t="str">
-        <f>_xlfn.TRANSLATE($B100,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Février</v>
       </c>
     </row>
@@ -3454,11 +3490,11 @@
         <v>181</v>
       </c>
       <c r="C101" t="str">
-        <f>_xlfn.TRANSLATE($B101,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Enfoque</v>
       </c>
       <c r="D101" t="str">
-        <f>_xlfn.TRANSLATE($B101,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Focus</v>
       </c>
     </row>
@@ -3470,11 +3506,11 @@
         <v>183</v>
       </c>
       <c r="C102" t="str">
-        <f>_xlfn.TRANSLATE($B102,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Amigos</v>
       </c>
       <c r="D102" t="str">
-        <f>_xlfn.TRANSLATE($B102,$B$2,D$2)</f>
+        <f t="shared" si="4"/>
         <v>Amis</v>
       </c>
     </row>
@@ -3486,11 +3522,11 @@
         <v>185</v>
       </c>
       <c r="C103" t="str">
-        <f>_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
+        <f t="shared" ref="C103:D122" si="5">_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
         <v>Lista de amigos</v>
       </c>
       <c r="D103" t="str">
-        <f>_xlfn.TRANSLATE($B103,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Liste d’amis</v>
       </c>
     </row>
@@ -3502,11 +3538,11 @@
         <v>187</v>
       </c>
       <c r="C104" t="str">
-        <f>_xlfn.TRANSLATE($B104,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
       <c r="D104" t="str">
-        <f>_xlfn.TRANSLATE($B104,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
       </c>
     </row>
@@ -3518,11 +3554,11 @@
         <v>189</v>
       </c>
       <c r="C105" t="str">
-        <f>_xlfn.TRANSLATE($B105,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Estadísticas de Friends</v>
       </c>
       <c r="D105" t="str">
-        <f>_xlfn.TRANSLATE($B105,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Statistiques de Friends</v>
       </c>
     </row>
@@ -3534,11 +3570,11 @@
         <v>191</v>
       </c>
       <c r="C106" t="str">
-        <f>_xlfn.TRANSLATE($B106,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>General</v>
       </c>
       <c r="D106" t="str">
-        <f>_xlfn.TRANSLATE($B106,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Généralités</v>
       </c>
     </row>
@@ -3550,11 +3586,11 @@
         <v>193</v>
       </c>
       <c r="C107" t="str">
-        <f>_xlfn.TRANSLATE($B107,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Estadísticas generales</v>
       </c>
       <c r="D107" t="str">
-        <f>_xlfn.TRANSLATE($B107,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Statistiques générales</v>
       </c>
     </row>
@@ -3566,11 +3602,11 @@
         <v>195</v>
       </c>
       <c r="C108" t="str">
-        <f>_xlfn.TRANSLATE($B108,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Obtén información</v>
       </c>
       <c r="D108" t="str">
-        <f>_xlfn.TRANSLATE($B108,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Obtenez des infos</v>
       </c>
     </row>
@@ -3582,11 +3618,11 @@
         <v>197</v>
       </c>
       <c r="C109" t="str">
-        <f>_xlfn.TRANSLATE($B109,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Obteniendo información</v>
       </c>
       <c r="D109" t="str">
-        <f>_xlfn.TRANSLATE($B109,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Obtenir des infos</v>
       </c>
     </row>
@@ -3598,11 +3634,11 @@
         <v>199</v>
       </c>
       <c r="C110" t="str">
-        <f>_xlfn.TRANSLATE($B110,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Ir al álbum</v>
       </c>
       <c r="D110" t="str">
-        <f>_xlfn.TRANSLATE($B110,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Aller à l’album</v>
       </c>
     </row>
@@ -3614,11 +3650,11 @@
         <v>201</v>
       </c>
       <c r="C111" t="str">
-        <f>_xlfn.TRANSLATE($B111,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Ir a artista</v>
       </c>
       <c r="D111" t="str">
-        <f>_xlfn.TRANSLATE($B111,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Aller à l’artiste</v>
       </c>
     </row>
@@ -3630,11 +3666,11 @@
         <v>203</v>
       </c>
       <c r="C112" t="str">
-        <f>_xlfn.TRANSLATE($B112,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Joyas ocultas que olvidaste</v>
       </c>
       <c r="D112" t="str">
-        <f>_xlfn.TRANSLATE($B112,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Des perles cachées que tu as oubliées</v>
       </c>
     </row>
@@ -3646,11 +3682,11 @@
         <v>205</v>
       </c>
       <c r="C113" t="str">
-        <f>_xlfn.TRANSLATE($B113,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Inicio</v>
       </c>
       <c r="D113" t="str">
-        <f>_xlfn.TRANSLATE($B113,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Accueil</v>
       </c>
     </row>
@@ -3662,11 +3698,11 @@
         <v>207</v>
       </c>
       <c r="C114" t="str">
-        <f>_xlfn.TRANSLATE($B114,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Enero</v>
       </c>
       <c r="D114" t="str">
-        <f>_xlfn.TRANSLATE($B114,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Janvier</v>
       </c>
     </row>
@@ -3678,11 +3714,11 @@
         <v>209</v>
       </c>
       <c r="C115" t="str">
-        <f>_xlfn.TRANSLATE($B115,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Julio</v>
       </c>
       <c r="D115" t="str">
-        <f>_xlfn.TRANSLATE($B115,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Juillet</v>
       </c>
     </row>
@@ -3694,11 +3730,11 @@
         <v>211</v>
       </c>
       <c r="C116" t="str">
-        <f>_xlfn.TRANSLATE($B116,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Junio</v>
       </c>
       <c r="D116" t="str">
-        <f>_xlfn.TRANSLATE($B116,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Juin</v>
       </c>
     </row>
@@ -3710,11 +3746,11 @@
         <v>213</v>
       </c>
       <c r="C117" t="str">
-        <f>_xlfn.TRANSLATE($B117,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Idioma</v>
       </c>
       <c r="D117" t="str">
-        <f>_xlfn.TRANSLATE($B117,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Langue</v>
       </c>
     </row>
@@ -3726,11 +3762,11 @@
         <v>478</v>
       </c>
       <c r="C118" t="str">
-        <f>_xlfn.TRANSLATE($B118,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>El cambio de idioma fracasó</v>
       </c>
       <c r="D118" t="str">
-        <f>_xlfn.TRANSLATE($B118,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec du changement linguistique</v>
       </c>
     </row>
@@ -3742,11 +3778,11 @@
         <v>215</v>
       </c>
       <c r="C119" t="str">
-        <f>_xlfn.TRANSLATE($B119,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Cambio de idioma</v>
       </c>
       <c r="D119" t="str">
-        <f>_xlfn.TRANSLATE($B119,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Changement de langue</v>
       </c>
     </row>
@@ -3758,11 +3794,11 @@
         <v>217</v>
       </c>
       <c r="C120" t="str">
-        <f>_xlfn.TRANSLATE($B120,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Últimas descargas</v>
       </c>
       <c r="D120" t="str">
-        <f>_xlfn.TRANSLATE($B120,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Derniers téléchargements</v>
       </c>
     </row>
@@ -3774,11 +3810,11 @@
         <v>219</v>
       </c>
       <c r="C121" t="str">
-        <f>_xlfn.TRANSLATE($B121,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Nivel</v>
       </c>
       <c r="D121" t="str">
-        <f>_xlfn.TRANSLATE($B121,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Niveau</v>
       </c>
     </row>
@@ -3790,11 +3826,11 @@
         <v>221</v>
       </c>
       <c r="C122" t="str">
-        <f>_xlfn.TRANSLATE($B122,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Biblioteca</v>
       </c>
       <c r="D122" t="str">
-        <f>_xlfn.TRANSLATE($B122,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Bibliothèque</v>
       </c>
     </row>
@@ -3806,11 +3842,11 @@
         <v>223</v>
       </c>
       <c r="C123" t="str">
-        <f>_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
+        <f t="shared" ref="C123:D142" si="6">_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
         <v>Como</v>
       </c>
       <c r="D123" t="str">
-        <f>_xlfn.TRANSLATE($B123,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Comme</v>
       </c>
     </row>
@@ -3822,11 +3858,11 @@
         <v>225</v>
       </c>
       <c r="C124" t="str">
-        <f>_xlfn.TRANSLATE($B124,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones que me gustaban</v>
       </c>
       <c r="D124" t="str">
-        <f>_xlfn.TRANSLATE($B124,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons appréciées</v>
       </c>
     </row>
@@ -3838,11 +3874,11 @@
         <v>227</v>
       </c>
       <c r="C125" t="str">
-        <f>_xlfn.TRANSLATE($B125,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Cerrar sesión</v>
       </c>
       <c r="D125" t="str">
-        <f>_xlfn.TRANSLATE($B125,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Déconnexion</v>
       </c>
     </row>
@@ -3854,11 +3890,11 @@
         <v>229</v>
       </c>
       <c r="C126" t="str">
-        <f>_xlfn.TRANSLATE($B126,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Letra</v>
       </c>
       <c r="D126" t="str">
-        <f>_xlfn.TRANSLATE($B126,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Paroles</v>
       </c>
     </row>
@@ -3870,11 +3906,11 @@
         <v>231</v>
       </c>
       <c r="C127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Marzo</v>
       </c>
       <c r="D127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Mars</v>
       </c>
     </row>
@@ -3886,11 +3922,11 @@
         <v>233</v>
       </c>
       <c r="C128" t="str">
-        <f>_xlfn.TRANSLATE($B128,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Mayo</v>
       </c>
       <c r="D128" t="str">
-        <f>_xlfn.TRANSLATE($B128,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Mai</v>
       </c>
     </row>
@@ -3902,11 +3938,11 @@
         <v>462</v>
       </c>
       <c r="C129" t="str">
-        <f>_xlfn.TRANSLATE($B129,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D129" t="str">
-        <f>_xlfn.TRANSLATE($B129,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
@@ -3918,11 +3954,11 @@
         <v>235</v>
       </c>
       <c r="C130" t="str">
-        <f>_xlfn.TRANSLATE($B130,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Progreso de los medios</v>
       </c>
       <c r="D130" t="str">
-        <f>_xlfn.TRANSLATE($B130,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Progrès des médias</v>
       </c>
     </row>
@@ -3934,11 +3970,11 @@
         <v>237</v>
       </c>
       <c r="C131" t="str">
-        <f>_xlfn.TRANSLATE($B131,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Actas</v>
       </c>
       <c r="D131" t="str">
-        <f>_xlfn.TRANSLATE($B131,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Procès-verbal</v>
       </c>
     </row>
@@ -3950,11 +3986,11 @@
         <v>239</v>
       </c>
       <c r="C132" t="str">
-        <f>_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutos escuchados</v>
       </c>
       <c r="D132" t="str">
-        <f>_xlfn.TRANSLATE($B132,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutes écoutées</v>
       </c>
     </row>
@@ -3966,11 +4002,11 @@
         <v>241</v>
       </c>
       <c r="C133" t="str">
-        <f>_xlfn.TRANSLATE($B133,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutos escuchados por día</v>
       </c>
       <c r="D133" t="str">
-        <f>_xlfn.TRANSLATE($B133,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutes écoutées par jour</v>
       </c>
     </row>
@@ -3982,11 +4018,11 @@
         <v>243</v>
       </c>
       <c r="C134" t="str">
-        <f>_xlfn.TRANSLATE($B134,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D134" t="str">
-        <f>_xlfn.TRANSLATE($B134,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
@@ -3998,11 +4034,11 @@
         <v>245</v>
       </c>
       <c r="C135" t="str">
-        <f>_xlfn.TRANSLATE($B135,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Más opciones</v>
       </c>
       <c r="D135" t="str">
-        <f>_xlfn.TRANSLATE($B135,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Plus d’options</v>
       </c>
     </row>
@@ -4014,11 +4050,11 @@
         <v>247</v>
       </c>
       <c r="C136" t="str">
-        <f>_xlfn.TRANSLATE($B136,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Más canciones de</v>
       </c>
       <c r="D136" t="str">
-        <f>_xlfn.TRANSLATE($B136,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Plus de chansons de</v>
       </c>
     </row>
@@ -4030,11 +4066,11 @@
         <v>249</v>
       </c>
       <c r="C137" t="str">
-        <f>_xlfn.TRANSLATE($B137,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Más escuchado</v>
       </c>
       <c r="D137" t="str">
-        <f>_xlfn.TRANSLATE($B137,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Les plus écoutés</v>
       </c>
     </row>
@@ -4046,11 +4082,11 @@
         <v>251</v>
       </c>
       <c r="C138" t="str">
-        <f>_xlfn.TRANSLATE($B138,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Álbumes más escuchados</v>
       </c>
       <c r="D138" t="str">
-        <f>_xlfn.TRANSLATE($B138,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Albums les plus écoutés</v>
       </c>
     </row>
@@ -4062,11 +4098,11 @@
         <v>253</v>
       </c>
       <c r="C139" t="str">
-        <f>_xlfn.TRANSLATE($B139,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Artistas más escuchados</v>
       </c>
       <c r="D139" t="str">
-        <f>_xlfn.TRANSLATE($B139,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Artistes les plus écoutés</v>
       </c>
     </row>
@@ -4078,11 +4114,11 @@
         <v>255</v>
       </c>
       <c r="C140" t="str">
-        <f>_xlfn.TRANSLATE($B140,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Canciones más escuchadas</v>
       </c>
       <c r="D140" t="str">
-        <f>_xlfn.TRANSLATE($B140,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons les plus écoutées</v>
       </c>
     </row>
@@ -4094,11 +4130,11 @@
         <v>257</v>
       </c>
       <c r="C141" t="str">
-        <f>_xlfn.TRANSLATE($B141,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Nombre</v>
       </c>
       <c r="D141" t="str">
-        <f>_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Nom</v>
       </c>
     </row>
@@ -4110,11 +4146,11 @@
         <v>259</v>
       </c>
       <c r="C142" t="str">
-        <f>_xlfn.TRANSLATE($B142,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Introducir nueva contraseña</v>
       </c>
       <c r="D142" t="str">
-        <f>_xlfn.TRANSLATE($B142,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
@@ -4126,11 +4162,11 @@
         <v>261</v>
       </c>
       <c r="C143" t="str">
-        <f>_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
+        <f t="shared" ref="C143:D162" si="7">_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
         <v>Nueva lista de reproducción</v>
       </c>
       <c r="D143" t="str">
-        <f>_xlfn.TRANSLATE($B143,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Nouvelle playlist</v>
       </c>
     </row>
@@ -4142,11 +4178,11 @@
         <v>263</v>
       </c>
       <c r="C144" t="str">
-        <f>_xlfn.TRANSLATE($B144,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D144" t="str">
-        <f>_xlfn.TRANSLATE($B144,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Nouveau nom de la playlist</v>
       </c>
     </row>
@@ -4158,11 +4194,11 @@
         <v>480</v>
       </c>
       <c r="C145" t="str">
-        <f>_xlfn.TRANSLATE($B145,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Nueva versión disponible</v>
       </c>
       <c r="D145" t="str">
-        <f>_xlfn.TRANSLATE($B145,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Nouvelle version disponible</v>
       </c>
     </row>
@@ -4174,11 +4210,11 @@
         <v>265</v>
       </c>
       <c r="C146" t="str">
-        <f>_xlfn.TRANSLATE($B146,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Próximos medios</v>
       </c>
       <c r="D146" t="str">
-        <f>_xlfn.TRANSLATE($B146,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Médias suivants</v>
       </c>
     </row>
@@ -4190,11 +4226,11 @@
         <v>267</v>
       </c>
       <c r="C147" t="str">
-        <f>_xlfn.TRANSLATE($B147,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
       <c r="D147" t="str">
-        <f>_xlfn.TRANSLATE($B147,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
@@ -4206,11 +4242,11 @@
         <v>269</v>
       </c>
       <c r="C148" t="str">
-        <f>_xlfn.TRANSLATE($B148,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No hay datos registrados.</v>
       </c>
       <c r="D148" t="str">
-        <f>_xlfn.TRANSLATE($B148,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
@@ -4222,11 +4258,11 @@
         <v>271</v>
       </c>
       <c r="C149" t="str">
-        <f>_xlfn.TRANSLATE($B149,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Letra no disponible</v>
       </c>
       <c r="D149" t="str">
-        <f>_xlfn.TRANSLATE($B149,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Paroles non disponibles</v>
       </c>
     </row>
@@ -4238,11 +4274,11 @@
         <v>273</v>
       </c>
       <c r="C150" t="str">
-        <f>_xlfn.TRANSLATE($B150,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D150" t="str">
-        <f>_xlfn.TRANSLATE($B150,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
@@ -4254,11 +4290,11 @@
         <v>275</v>
       </c>
       <c r="C151" t="str">
-        <f>_xlfn.TRANSLATE($B151,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No hay repetición</v>
       </c>
       <c r="D151" t="str">
-        <f>_xlfn.TRANSLATE($B151,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Pas de répétition</v>
       </c>
     </row>
@@ -4270,11 +4306,11 @@
         <v>277</v>
       </c>
       <c r="C152" t="str">
-        <f>_xlfn.TRANSLATE($B152,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Sin resultados</v>
       </c>
       <c r="D152" t="str">
-        <f>_xlfn.TRANSLATE($B152,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Aucun résultat</v>
       </c>
     </row>
@@ -4286,11 +4322,11 @@
         <v>279</v>
       </c>
       <c r="C153" t="str">
-        <f>_xlfn.TRANSLATE($B153,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Sin trabajador de servicios</v>
       </c>
       <c r="D153" t="str">
-        <f>_xlfn.TRANSLATE($B153,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Aucun travailleur de services</v>
       </c>
     </row>
@@ -4302,11 +4338,11 @@
         <v>281</v>
       </c>
       <c r="C154" t="str">
-        <f>_xlfn.TRANSLATE($B154,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D154" t="str">
-        <f>_xlfn.TRANSLATE($B154,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
@@ -4318,11 +4354,11 @@
         <v>283</v>
       </c>
       <c r="C155" t="str">
-        <f>_xlfn.TRANSLATE($B155,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Sin estado</v>
       </c>
       <c r="D155" t="str">
-        <f>_xlfn.TRANSLATE($B155,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Aucun État</v>
       </c>
     </row>
@@ -4334,11 +4370,11 @@
         <v>285</v>
       </c>
       <c r="C156" t="str">
-        <f>_xlfn.TRANSLATE($B156,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D156" t="str">
-        <f>_xlfn.TRANSLATE($B156,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
@@ -4350,11 +4386,11 @@
         <v>287</v>
       </c>
       <c r="C157" t="str">
-        <f>_xlfn.TRANSLATE($B157,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D157" t="str">
-        <f>_xlfn.TRANSLATE($B157,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
@@ -4366,11 +4402,11 @@
         <v>289</v>
       </c>
       <c r="C158" t="str">
-        <f>_xlfn.TRANSLATE($B158,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Noviembre</v>
       </c>
       <c r="D158" t="str">
-        <f>_xlfn.TRANSLATE($B158,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Novembre</v>
       </c>
     </row>
@@ -4382,11 +4418,11 @@
         <v>291</v>
       </c>
       <c r="C159" t="str">
-        <f>_xlfn.TRANSLATE($B159,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Octubre</v>
       </c>
       <c r="D159" t="str">
-        <f>_xlfn.TRANSLATE($B159,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Octobre</v>
       </c>
     </row>
@@ -4398,11 +4434,11 @@
         <v>293</v>
       </c>
       <c r="C160" t="str">
-        <f>_xlfn.TRANSLATE($B160,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Lista abierta</v>
       </c>
       <c r="D160" t="str">
-        <f>_xlfn.TRANSLATE($B160,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Liste ouverte</v>
       </c>
     </row>
@@ -4414,11 +4450,11 @@
         <v>295</v>
       </c>
       <c r="C161" t="str">
-        <f>_xlfn.TRANSLATE($B161,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Canción abierta</v>
       </c>
       <c r="D161" t="str">
-        <f>_xlfn.TRANSLATE($B161,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Chanson d’ouverture</v>
       </c>
     </row>
@@ -4430,11 +4466,11 @@
         <v>297</v>
       </c>
       <c r="C162" t="str">
-        <f>_xlfn.TRANSLATE($B162,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Partido</v>
       </c>
       <c r="D162" t="str">
-        <f>_xlfn.TRANSLATE($B162,$B$2,D$2)</f>
+        <f t="shared" si="7"/>
         <v>Parti</v>
       </c>
     </row>
@@ -4446,11 +4482,11 @@
         <v>299</v>
       </c>
       <c r="C163" t="str">
-        <f>_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
+        <f t="shared" ref="C163:D170" si="8">_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
         <v>Canción de pausa</v>
       </c>
       <c r="D163" t="str">
-        <f>_xlfn.TRANSLATE($B163,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chanson de pause</v>
       </c>
     </row>
@@ -4462,11 +4498,11 @@
         <v>301</v>
       </c>
       <c r="C164" t="str">
-        <f>_xlfn.TRANSLATE($B164,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Solicitudes pendientes</v>
       </c>
       <c r="D164" t="str">
-        <f>_xlfn.TRANSLATE($B164,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Demandes en attente</v>
       </c>
     </row>
@@ -4478,11 +4514,11 @@
         <v>303</v>
       </c>
       <c r="C165" t="str">
-        <f>_xlfn.TRANSLATE($B165,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Pin</v>
       </c>
       <c r="D165" t="str">
-        <f>_xlfn.TRANSLATE($B165,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Épingle</v>
       </c>
     </row>
@@ -4494,11 +4530,11 @@
         <v>305</v>
       </c>
       <c r="C166" t="str">
-        <f>_xlfn.TRANSLATE($B166,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Listas fijadas</v>
       </c>
       <c r="D166" t="str">
-        <f>_xlfn.TRANSLATE($B166,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Listes épinglées</v>
       </c>
     </row>
@@ -4510,11 +4546,11 @@
         <v>307</v>
       </c>
       <c r="C167" t="str">
-        <f>_xlfn.TRANSLATE($B167,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Título del álbum</v>
       </c>
       <c r="D167" t="str">
-        <f>_xlfn.TRANSLATE($B167,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Titre de l’album</v>
       </c>
     </row>
@@ -4526,11 +4562,11 @@
         <v>309</v>
       </c>
       <c r="C168" t="str">
-        <f>_xlfn.TRANSLATE($B168,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Nombre artístico</v>
       </c>
       <c r="D168" t="str">
-        <f>_xlfn.TRANSLATE($B168,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nom de l’artiste</v>
       </c>
     </row>
@@ -4542,11 +4578,11 @@
         <v>311</v>
       </c>
       <c r="C169" t="str">
-        <f>_xlfn.TRANSLATE($B169,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D169" t="str">
-        <f>_xlfn.TRANSLATE($B169,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Ma playlist parfaite</v>
       </c>
     </row>
@@ -4558,11 +4594,11 @@
         <v>313</v>
       </c>
       <c r="C170" t="str">
-        <f>_xlfn.TRANSLATE($B170,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Título de la canción</v>
       </c>
       <c r="D170" t="str">
-        <f>_xlfn.TRANSLATE($B170,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Titre de la chanson</v>
       </c>
     </row>
@@ -4577,7 +4613,7 @@
         <v>481</v>
       </c>
       <c r="D171" t="str">
-        <f>_xlfn.TRANSLATE($B171,$B$2,D$2)</f>
+        <f t="shared" ref="D171:D202" si="9">_xlfn.TRANSLATE($B171,$B$2,D$2)</f>
         <v>Jeu</v>
       </c>
     </row>
@@ -4593,7 +4629,7 @@
         <v>Lista de reproducción</v>
       </c>
       <c r="D172" t="str">
-        <f>_xlfn.TRANSLATE($B172,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Liste des jeux</v>
       </c>
     </row>
@@ -4609,7 +4645,7 @@
         <v>Reproducir medios</v>
       </c>
       <c r="D173" t="str">
-        <f>_xlfn.TRANSLATE($B173,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Lire les médias</v>
       </c>
     </row>
@@ -4624,7 +4660,7 @@
         <v>482</v>
       </c>
       <c r="D174" t="str">
-        <f>_xlfn.TRANSLATE($B174,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>À jouer à venir</v>
       </c>
     </row>
@@ -4636,11 +4672,11 @@
         <v>321</v>
       </c>
       <c r="C175" t="str">
-        <f>_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
+        <f t="shared" ref="C175:C206" si="10">_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
         <v>Tocar canción</v>
       </c>
       <c r="D175" t="str">
-        <f>_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Jouer la chanson</v>
       </c>
     </row>
@@ -4652,11 +4688,11 @@
         <v>323</v>
       </c>
       <c r="C176" t="str">
-        <f>_xlfn.TRANSLATE($B176,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Listas de reproducción</v>
       </c>
       <c r="D176" t="str">
-        <f>_xlfn.TRANSLATE($B176,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Playlists</v>
       </c>
     </row>
@@ -4668,11 +4704,11 @@
         <v>325</v>
       </c>
       <c r="C177" t="str">
-        <f>_xlfn.TRANSLATE($B177,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Medios anteriores</v>
       </c>
       <c r="D177" t="str">
-        <f>_xlfn.TRANSLATE($B177,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Médias précédents</v>
       </c>
     </row>
@@ -4684,11 +4720,11 @@
         <v>327</v>
       </c>
       <c r="C178" t="str">
-        <f>_xlfn.TRANSLATE($B178,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Selecciones rápidas</v>
       </c>
       <c r="D178" t="str">
-        <f>_xlfn.TRANSLATE($B178,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Choix rapides</v>
       </c>
     </row>
@@ -4700,11 +4736,11 @@
         <v>329</v>
       </c>
       <c r="C179" t="str">
-        <f>_xlfn.TRANSLATE($B179,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Radio</v>
       </c>
       <c r="D179" t="str">
-        <f>_xlfn.TRANSLATE($B179,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Radio</v>
       </c>
     </row>
@@ -4716,11 +4752,11 @@
         <v>331</v>
       </c>
       <c r="C180" t="str">
-        <f>_xlfn.TRANSLATE($B180,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>No se han encontrado estaciones</v>
       </c>
       <c r="D180" t="str">
-        <f>_xlfn.TRANSLATE($B180,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucune station trouvée</v>
       </c>
     </row>
@@ -4732,11 +4768,11 @@
         <v>333</v>
       </c>
       <c r="C181" t="str">
-        <f>_xlfn.TRANSLATE($B181,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D181" t="str">
-        <f>_xlfn.TRANSLATE($B181,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
@@ -4748,11 +4784,11 @@
         <v>335</v>
       </c>
       <c r="C182" t="str">
-        <f>_xlfn.TRANSLATE($B182,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D182" t="str">
-        <f>_xlfn.TRANSLATE($B182,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
@@ -4764,11 +4800,11 @@
         <v>337</v>
       </c>
       <c r="C183" t="str">
-        <f>_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Emisoras de radio</v>
       </c>
       <c r="D183" t="str">
-        <f>_xlfn.TRANSLATE($B183,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Radio Stations</v>
       </c>
     </row>
@@ -4780,11 +4816,11 @@
         <v>339</v>
       </c>
       <c r="C184" t="str">
-        <f>_xlfn.TRANSLATE($B184,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Mezcla reciente</v>
       </c>
       <c r="D184" t="str">
-        <f>_xlfn.TRANSLATE($B184,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Mix récent</v>
       </c>
     </row>
@@ -4796,11 +4832,11 @@
         <v>341</v>
       </c>
       <c r="C185" t="str">
-        <f>_xlfn.TRANSLATE($B185,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D185" t="str">
-        <f>_xlfn.TRANSLATE($B185,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Joué récemment</v>
       </c>
     </row>
@@ -4812,11 +4848,11 @@
         <v>343</v>
       </c>
       <c r="C186" t="str">
-        <f>_xlfn.TRANSLATE($B186,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D186" t="str">
-        <f>_xlfn.TRANSLATE($B186,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Récemment joué</v>
       </c>
     </row>
@@ -4828,11 +4864,11 @@
         <v>345</v>
       </c>
       <c r="C187" t="str">
-        <f>_xlfn.TRANSLATE($B187,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Registro</v>
       </c>
       <c r="D187" t="str">
-        <f>_xlfn.TRANSLATE($B187,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Registre</v>
       </c>
     </row>
@@ -4844,11 +4880,11 @@
         <v>347</v>
       </c>
       <c r="C188" t="str">
-        <f>_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Registrado</v>
       </c>
       <c r="D188" t="str">
-        <f>_xlfn.TRANSLATE($B188,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Enregistré</v>
       </c>
     </row>
@@ -4860,11 +4896,11 @@
         <v>349</v>
       </c>
       <c r="C189" t="str">
-        <f>_xlfn.TRANSLATE($B189,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Registrando...</v>
       </c>
       <c r="D189" t="str">
-        <f>_xlfn.TRANSLATE($B189,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Enregistrement...</v>
       </c>
     </row>
@@ -4876,11 +4912,11 @@
         <v>351</v>
       </c>
       <c r="C190" t="str">
-        <f>_xlfn.TRANSLATE($B190,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Artistas relacionados</v>
       </c>
       <c r="D190" t="str">
-        <f>_xlfn.TRANSLATE($B190,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Artistes associés</v>
       </c>
     </row>
@@ -4892,11 +4928,11 @@
         <v>353</v>
       </c>
       <c r="C191" t="str">
-        <f>_xlfn.TRANSLATE($B191,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Relajado</v>
       </c>
       <c r="D191" t="str">
-        <f>_xlfn.TRANSLATE($B191,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Détendu</v>
       </c>
     </row>
@@ -4908,11 +4944,11 @@
         <v>355</v>
       </c>
       <c r="C192" t="str">
-        <f>_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D192" t="str">
-        <f>_xlfn.TRANSLATE($B192,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de la bibliothèque</v>
       </c>
     </row>
@@ -4924,11 +4960,11 @@
         <v>357</v>
       </c>
       <c r="C193" t="str">
-        <f>_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Quitar de me gusta</v>
       </c>
       <c r="D193" t="str">
-        <f>_xlfn.TRANSLATE($B193,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de aimé</v>
       </c>
     </row>
@@ -4940,11 +4976,11 @@
         <v>359</v>
       </c>
       <c r="C194" t="str">
-        <f>_xlfn.TRANSLATE($B194,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D194" t="str">
-        <f>_xlfn.TRANSLATE($B194,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Supprimer de la playlist</v>
       </c>
     </row>
@@ -4956,11 +4992,11 @@
         <v>361</v>
       </c>
       <c r="C195" t="str">
-        <f>_xlfn.TRANSLATE($B195,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Eliminar de la cola</v>
       </c>
       <c r="D195" t="str">
-        <f>_xlfn.TRANSLATE($B195,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de la file d’attente</v>
       </c>
     </row>
@@ -4972,11 +5008,11 @@
         <v>363</v>
       </c>
       <c r="C196" t="str">
-        <f>_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Repite todo</v>
       </c>
       <c r="D196" t="str">
-        <f>_xlfn.TRANSLATE($B196,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répétez tout</v>
       </c>
     </row>
@@ -4988,11 +5024,11 @@
         <v>365</v>
       </c>
       <c r="C197" t="str">
-        <f>_xlfn.TRANSLATE($B197,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Repite una</v>
       </c>
       <c r="D197" t="str">
-        <f>_xlfn.TRANSLATE($B197,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répétez-en un</v>
       </c>
     </row>
@@ -5004,11 +5040,11 @@
         <v>367</v>
       </c>
       <c r="C198" t="str">
-        <f>_xlfn.TRANSLATE($B198,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Repetir nueva contraseña</v>
       </c>
       <c r="D198" t="str">
-        <f>_xlfn.TRANSLATE($B198,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
@@ -5020,11 +5056,11 @@
         <v>458</v>
       </c>
       <c r="C199" t="str">
-        <f>_xlfn.TRANSLATE($B199,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Regreso a casa</v>
       </c>
       <c r="D199" t="str">
-        <f>_xlfn.TRANSLATE($B199,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retour à la maison</v>
       </c>
     </row>
@@ -5036,11 +5072,11 @@
         <v>369</v>
       </c>
       <c r="C200" t="str">
-        <f>_xlfn.TRANSLATE($B200,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Guardando...</v>
       </c>
       <c r="D200" t="str">
-        <f>_xlfn.TRANSLATE($B200,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Sauver...</v>
       </c>
     </row>
@@ -5052,11 +5088,11 @@
         <v>371</v>
       </c>
       <c r="C201" t="str">
-        <f>_xlfn.TRANSLATE($B201,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Búsqueda</v>
       </c>
       <c r="D201" t="str">
-        <f>_xlfn.TRANSLATE($B201,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Recherche</v>
       </c>
     </row>
@@ -5068,11 +5104,11 @@
         <v>373</v>
       </c>
       <c r="C202" t="str">
-        <f>_xlfn.TRANSLATE($B202,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D202" t="str">
-        <f>_xlfn.TRANSLATE($B202,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
@@ -5084,11 +5120,11 @@
         <v>375</v>
       </c>
       <c r="C203" t="str">
-        <f>_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D203" t="str">
-        <f>_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
+        <f t="shared" ref="D203:D234" si="11">_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
         <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
@@ -5100,11 +5136,11 @@
         <v>377</v>
       </c>
       <c r="C204" t="str">
-        <f>_xlfn.TRANSLATE($B204,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D204" t="str">
-        <f>_xlfn.TRANSLATE($B204,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
@@ -5116,11 +5152,11 @@
         <v>379</v>
       </c>
       <c r="C205" t="str">
-        <f>_xlfn.TRANSLATE($B205,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Buscar en la biblioteca</v>
       </c>
       <c r="D205" t="str">
-        <f>_xlfn.TRANSLATE($B205,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
@@ -5132,11 +5168,11 @@
         <v>381</v>
       </c>
       <c r="C206" t="str">
-        <f>_xlfn.TRANSLATE($B206,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Usuarios de búsqueda</v>
       </c>
       <c r="D206" t="str">
-        <f>_xlfn.TRANSLATE($B206,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Rechercher les utilisateurs</v>
       </c>
     </row>
@@ -5148,11 +5184,11 @@
         <v>383</v>
       </c>
       <c r="C207" t="str">
-        <f>_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
+        <f t="shared" ref="C207:C238" si="12">_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
         <v>Enviar canción actual</v>
       </c>
       <c r="D207" t="str">
-        <f>_xlfn.TRANSLATE($B207,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
@@ -5164,11 +5200,11 @@
         <v>385</v>
       </c>
       <c r="C208" t="str">
-        <f>_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Septiembre</v>
       </c>
       <c r="D208" t="str">
-        <f>_xlfn.TRANSLATE($B208,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Septembre</v>
       </c>
     </row>
@@ -5180,11 +5216,11 @@
         <v>60</v>
       </c>
       <c r="C209" t="str">
-        <f>_xlfn.TRANSLATE($B209,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Escenarios</v>
       </c>
       <c r="D209" t="str">
-        <f>_xlfn.TRANSLATE($B209,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Décors</v>
       </c>
     </row>
@@ -5196,11 +5232,11 @@
         <v>388</v>
       </c>
       <c r="C210" t="str">
-        <f>_xlfn.TRANSLATE($B210,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Compartir canción</v>
       </c>
       <c r="D210" t="str">
-        <f>_xlfn.TRANSLATE($B210,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Partager la chanson</v>
       </c>
     </row>
@@ -5212,11 +5248,11 @@
         <v>390</v>
       </c>
       <c r="C211" t="str">
-        <f>_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones compartidas para ti</v>
       </c>
       <c r="D211" t="str">
-        <f>_xlfn.TRANSLATE($B211,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chansons partagées pour vous</v>
       </c>
     </row>
@@ -5228,11 +5264,11 @@
         <v>392</v>
       </c>
       <c r="C212" t="str">
-        <f>_xlfn.TRANSLATE($B212,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Compartido desde</v>
       </c>
       <c r="D212" t="str">
-        <f>_xlfn.TRANSLATE($B212,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Partagé depuis</v>
       </c>
     </row>
@@ -5244,11 +5280,11 @@
         <v>394</v>
       </c>
       <c r="C213" t="str">
-        <f>_xlfn.TRANSLATE($B213,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Mostrando datos de</v>
       </c>
       <c r="D213" t="str">
-        <f>_xlfn.TRANSLATE($B213,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Affichage des données de</v>
       </c>
     </row>
@@ -5260,11 +5296,11 @@
         <v>396</v>
       </c>
       <c r="C214" t="str">
-        <f>_xlfn.TRANSLATE($B214,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canción</v>
       </c>
       <c r="D214" t="str">
-        <f>_xlfn.TRANSLATE($B214,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chanson</v>
       </c>
     </row>
@@ -5276,11 +5312,11 @@
         <v>398</v>
       </c>
       <c r="C215" t="str">
-        <f>_xlfn.TRANSLATE($B215,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones</v>
       </c>
       <c r="D215" t="str">
-        <f>_xlfn.TRANSLATE($B215,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chansons</v>
       </c>
     </row>
@@ -5292,11 +5328,11 @@
         <v>400</v>
       </c>
       <c r="C216" t="str">
-        <f>_xlfn.TRANSLATE($B216,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones Solo para ti</v>
       </c>
       <c r="D216" t="str">
-        <f>_xlfn.TRANSLATE($B216,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chansons juste pour toi</v>
       </c>
     </row>
@@ -5308,11 +5344,11 @@
         <v>402</v>
       </c>
       <c r="C217" t="str">
-        <f>_xlfn.TRANSLATE($B217,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones de</v>
       </c>
       <c r="D217" t="str">
-        <f>_xlfn.TRANSLATE($B217,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chansons de</v>
       </c>
     </row>
@@ -5324,11 +5360,11 @@
         <v>404</v>
       </c>
       <c r="C218" t="str">
-        <f>_xlfn.TRANSLATE($B218,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones escuchadas</v>
       </c>
       <c r="D218" t="str">
-        <f>_xlfn.TRANSLATE($B218,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Chansons écoutées</v>
       </c>
     </row>
@@ -5340,11 +5376,11 @@
         <v>406</v>
       </c>
       <c r="C219" t="str">
-        <f>_xlfn.TRANSLATE($B219,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas</v>
       </c>
       <c r="D219" t="str">
-        <f>_xlfn.TRANSLATE($B219,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -5356,11 +5392,11 @@
         <v>408</v>
       </c>
       <c r="C220" t="str">
-        <f>_xlfn.TRANSLATE($B220,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas</v>
       </c>
       <c r="D220" t="str">
-        <f>_xlfn.TRANSLATE($B220,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -5372,11 +5408,11 @@
         <v>410</v>
       </c>
       <c r="C221" t="str">
-        <f>_xlfn.TRANSLATE($B221,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>¡Para</v>
       </c>
       <c r="D221" t="str">
-        <f>_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Arrête</v>
       </c>
     </row>
@@ -5388,11 +5424,11 @@
         <v>412</v>
       </c>
       <c r="C222" t="str">
-        <f>_xlfn.TRANSLATE($B222,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>a</v>
       </c>
       <c r="D222" t="str">
-        <f>_xlfn.TRANSLATE($B222,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>à</v>
       </c>
     </row>
@@ -5404,11 +5440,11 @@
         <v>460</v>
       </c>
       <c r="C223" t="str">
-        <f>_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>ToDo</v>
       </c>
       <c r="D223" t="str">
-        <f>_xlfn.TRANSLATE($B223,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>ToDo</v>
       </c>
     </row>
@@ -5420,11 +5456,11 @@
         <v>414</v>
       </c>
       <c r="C224" t="str">
-        <f>_xlfn.TRANSLATE($B224,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D224" t="str">
-        <f>_xlfn.TRANSLATE($B224,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Albums phares</v>
       </c>
     </row>
@@ -5436,11 +5472,11 @@
         <v>416</v>
       </c>
       <c r="C225" t="str">
-        <f>_xlfn.TRANSLATE($B225,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones principales</v>
       </c>
       <c r="D225" t="str">
-        <f>_xlfn.TRANSLATE($B225,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Meilleures chansons</v>
       </c>
     </row>
@@ -5452,11 +5488,11 @@
         <v>418</v>
       </c>
       <c r="C226" t="str">
-        <f>_xlfn.TRANSLATE($B226,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Desclavar</v>
       </c>
       <c r="D226" t="str">
-        <f>_xlfn.TRANSLATE($B226,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Détacher</v>
       </c>
     </row>
@@ -5468,11 +5504,11 @@
         <v>420</v>
       </c>
       <c r="C227" t="str">
-        <f>_xlfn.TRANSLATE($B227,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Desregistrar</v>
       </c>
       <c r="D227" t="str">
-        <f>_xlfn.TRANSLATE($B227,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Désinscription</v>
       </c>
     </row>
@@ -5484,11 +5520,11 @@
         <v>422</v>
       </c>
       <c r="C228" t="str">
-        <f>_xlfn.TRANSLATE($B228,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>No registrado</v>
       </c>
       <c r="D228" t="str">
-        <f>_xlfn.TRANSLATE($B228,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Non enregistré</v>
       </c>
     </row>
@@ -5500,11 +5536,11 @@
         <v>424</v>
       </c>
       <c r="C229" t="str">
-        <f>_xlfn.TRANSLATE($B229,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Dejar de registrarse...</v>
       </c>
       <c r="D229" t="str">
-        <f>_xlfn.TRANSLATE($B229,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Désenregistrement...</v>
       </c>
     </row>
@@ -5516,11 +5552,11 @@
         <v>426</v>
       </c>
       <c r="C230" t="str">
-        <f>_xlfn.TRANSLATE($B230,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Actualización</v>
       </c>
       <c r="D230" t="str">
-        <f>_xlfn.TRANSLATE($B230,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Mise à jour</v>
       </c>
     </row>
@@ -5532,11 +5568,11 @@
         <v>428</v>
       </c>
       <c r="C231" t="str">
-        <f>_xlfn.TRANSLATE($B231,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Actualizando...</v>
       </c>
       <c r="D231" t="str">
-        <f>_xlfn.TRANSLATE($B231,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Mise à jour...</v>
       </c>
     </row>
@@ -5548,11 +5584,11 @@
         <v>430</v>
       </c>
       <c r="C232" t="str">
-        <f>_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Subida</v>
       </c>
       <c r="D232" t="str">
-        <f>_xlfn.TRANSLATE($B232,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Téléverser</v>
       </c>
     </row>
@@ -5564,11 +5600,11 @@
         <v>432</v>
       </c>
       <c r="C233" t="str">
-        <f>_xlfn.TRANSLATE($B233,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Usuario</v>
       </c>
       <c r="D233" t="str">
-        <f>_xlfn.TRANSLATE($B233,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Utilisateur</v>
       </c>
     </row>
@@ -5580,11 +5616,11 @@
         <v>434</v>
       </c>
       <c r="C234" t="str">
-        <f>_xlfn.TRANSLATE($B234,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Configuración de usuario</v>
       </c>
       <c r="D234" t="str">
-        <f>_xlfn.TRANSLATE($B234,$B$2,D$2)</f>
+        <f t="shared" si="11"/>
         <v>Paramètres utilisateur</v>
       </c>
     </row>
@@ -5596,11 +5632,11 @@
         <v>436</v>
       </c>
       <c r="C235" t="str">
-        <f>_xlfn.TRANSLATE($B235,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas de usuario</v>
       </c>
       <c r="D235" t="str">
-        <f>_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
+        <f t="shared" ref="D235:D255" si="13">_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
         <v>Statistiques des utilisateurs</v>
       </c>
     </row>
@@ -5612,11 +5648,11 @@
         <v>438</v>
       </c>
       <c r="C236" t="str">
-        <f>_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Usuarios y amigos</v>
       </c>
       <c r="D236" t="str">
-        <f>_xlfn.TRANSLATE($B236,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Utilisateurs et amis</v>
       </c>
     </row>
@@ -5628,11 +5664,11 @@
         <v>440</v>
       </c>
       <c r="C237" t="str">
-        <f>_xlfn.TRANSLATE($B237,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Lista de usuarios</v>
       </c>
       <c r="D237" t="str">
-        <f>_xlfn.TRANSLATE($B237,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Liste des utilisateurs</v>
       </c>
     </row>
@@ -5644,11 +5680,11 @@
         <v>442</v>
       </c>
       <c r="C238" t="str">
-        <f>_xlfn.TRANSLATE($B238,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Vídeos</v>
       </c>
       <c r="D238" t="str">
-        <f>_xlfn.TRANSLATE($B238,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vidéos</v>
       </c>
     </row>
@@ -5660,11 +5696,11 @@
         <v>444</v>
       </c>
       <c r="C239" t="str">
-        <f>_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
+        <f t="shared" ref="C239:C255" si="14">_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
         <v>También puede que te interese</v>
       </c>
       <c r="D239" t="str">
-        <f>_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Ça pourrait aussi te plaire</v>
       </c>
     </row>
@@ -5676,11 +5712,11 @@
         <v>446</v>
       </c>
       <c r="C240" t="str">
-        <f>_xlfn.TRANSLATE($B240,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v>Tu</v>
       </c>
       <c r="D240" t="str">
-        <f>_xlfn.TRANSLATE($B240,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Votre</v>
       </c>
     </row>
@@ -5692,11 +5728,11 @@
         <v>448</v>
       </c>
       <c r="C241" t="str">
-        <f>_xlfn.TRANSLATE($B241,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v>Tus álbumes y listas de reproducción</v>
       </c>
       <c r="D241" t="str">
-        <f>_xlfn.TRANSLATE($B241,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vos albums et playlists</v>
       </c>
     </row>
@@ -5708,11 +5744,11 @@
         <v>450</v>
       </c>
       <c r="C242" t="str">
-        <f>_xlfn.TRANSLATE($B242,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v>Tu mezcla</v>
       </c>
       <c r="D242" t="str">
-        <f>_xlfn.TRANSLATE($B242,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Votre Mix</v>
       </c>
     </row>
@@ -5724,131 +5760,155 @@
         <v>452</v>
       </c>
       <c r="C243" t="str">
-        <f>_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v>Vídeos de YouTube</v>
       </c>
       <c r="D243" t="str">
-        <f>_xlfn.TRANSLATE($B243,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vidéos YouTube</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>483</v>
+      </c>
+      <c r="B244" t="s">
+        <v>494</v>
+      </c>
       <c r="C244" t="str">
-        <f>_xlfn.TRANSLATE($B244,$B$2,C$2)</f>
-        <v/>
+        <f t="shared" si="14"/>
+        <v>Empezando...</v>
       </c>
       <c r="D244" t="str">
-        <f>_xlfn.TRANSLATE($B244,$B$2,D$2)</f>
-        <v/>
+        <f t="shared" si="13"/>
+        <v>Commencer...</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>484</v>
+      </c>
+      <c r="B245" t="s">
+        <v>488</v>
+      </c>
       <c r="C245" t="str">
-        <f>_xlfn.TRANSLATE($B245,$B$2,C$2)</f>
-        <v/>
+        <f t="shared" si="14"/>
+        <v>Completado</v>
       </c>
       <c r="D245" t="str">
-        <f>_xlfn.TRANSLATE($B245,$B$2,D$2)</f>
-        <v/>
+        <f t="shared" si="13"/>
+        <v>Achèvement</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C246" t="str">
-        <f>_xlfn.TRANSLATE($B246,$B$2,C$2)</f>
-        <v/>
+      <c r="A246" t="s">
+        <v>485</v>
+      </c>
+      <c r="B246" t="s">
+        <v>489</v>
+      </c>
+      <c r="C246" t="s">
+        <v>493</v>
       </c>
       <c r="D246" t="str">
-        <f>_xlfn.TRANSLATE($B246,$B$2,D$2)</f>
-        <v/>
+        <f t="shared" si="13"/>
+        <v>Échec</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>486</v>
+      </c>
+      <c r="B247" t="s">
+        <v>490</v>
+      </c>
       <c r="C247" t="str">
-        <f>_xlfn.TRANSLATE($B247,$B$2,C$2)</f>
-        <v/>
+        <f t="shared" si="14"/>
+        <v>Descargando</v>
       </c>
       <c r="D247" t="str">
-        <f>_xlfn.TRANSLATE($B247,$B$2,D$2)</f>
-        <v/>
+        <f t="shared" si="13"/>
+        <v>Téléchargement</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C248" t="str">
-        <f>_xlfn.TRANSLATE($B248,$B$2,C$2)</f>
-        <v/>
+      <c r="A248" t="s">
+        <v>487</v>
+      </c>
+      <c r="B248" t="s">
+        <v>491</v>
+      </c>
+      <c r="C248" t="s">
+        <v>492</v>
       </c>
       <c r="D248" t="str">
-        <f>_xlfn.TRANSLATE($B248,$B$2,D$2)</f>
-        <v/>
+        <f t="shared" si="13"/>
+        <v>Nouvelle tentative</v>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C249" t="str">
-        <f>_xlfn.TRANSLATE($B249,$B$2,C$2)</f>
-        <v/>
-      </c>
       <c r="D249" t="str">
-        <f>_xlfn.TRANSLATE($B249,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C250" t="str">
-        <f>_xlfn.TRANSLATE($B250,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D250" t="str">
-        <f>_xlfn.TRANSLATE($B250,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C251" t="str">
-        <f>_xlfn.TRANSLATE($B251,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D251" t="str">
-        <f>_xlfn.TRANSLATE($B251,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C252" t="str">
-        <f>_xlfn.TRANSLATE($B252,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D252" t="str">
-        <f>_xlfn.TRANSLATE($B252,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C253" t="str">
-        <f>_xlfn.TRANSLATE($B253,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D253" t="str">
-        <f>_xlfn.TRANSLATE($B253,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C254" t="str">
-        <f>_xlfn.TRANSLATE($B254,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D254" t="str">
-        <f>_xlfn.TRANSLATE($B254,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C255" t="str">
-        <f>_xlfn.TRANSLATE($B255,$B$2,C$2)</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="D255" t="str">
-        <f>_xlfn.TRANSLATE($B255,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Added download list to server key
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Documents\rockit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51927A1-EB4A-4AF5-9075-86B2A334EA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A9776E-7A3A-45DC-86BE-4404016ECE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="1170" windowWidth="32490" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="498">
   <si>
     <t>KEY</t>
   </si>
@@ -1518,6 +1518,15 @@
   </si>
   <si>
     <t>Starting…</t>
+  </si>
+  <si>
+    <t>DOWNLOAD_LIST_TO_SERVER</t>
+  </si>
+  <si>
+    <t>Download list to server</t>
+  </si>
+  <si>
+    <t>Descargar list en el servidor</t>
   </si>
 </sst>
 </file>
@@ -5847,9 +5856,18 @@
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>495</v>
+      </c>
+      <c r="B249" t="s">
+        <v>496</v>
+      </c>
+      <c r="C249" t="s">
+        <v>497</v>
+      </c>
       <c r="D249" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v>Liste de téléchargement vers serveur</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add remember me functionality to authentication flow and UI components
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D257" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D258" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D256"/>
   <sortState ref="A3:D256">
     <sortCondition ref="A2:A256"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D257"/>
+  <dimension ref="A1:D258"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5532,6 +5532,26 @@
         <v/>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>REMEMBER_ME</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Remember me</t>
+        </is>
+      </c>
+      <c r="C258">
+        <f>_xlfn.TRANSLATE($B258,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D258">
+        <f>_xlfn.TRANSLATE($B258,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: update version to 0.3.1 and add new vocabulary entries for admin request log
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1EF932-8C16-49E9-8BF1-34481B1096E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4D5D4D-ED2E-47EB-81BA-3730786ECEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="560">
   <si>
     <t>KEY</t>
   </si>
@@ -1723,6 +1723,18 @@
   </si>
   <si>
     <t>Ruta</t>
+  </si>
+  <si>
+    <t>ADMIN_REQUEST_LOG_STATS</t>
+  </si>
+  <si>
+    <t>ADMIN_REQUEST_DESCRIPTION</t>
+  </si>
+  <si>
+    <t>Request Log Stats</t>
+  </si>
+  <si>
+    <t>Server request metrics and analytics</t>
   </si>
 </sst>
 </file>
@@ -1836,8 +1848,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D277" totalsRowShown="0">
-  <autoFilter ref="A2:D277" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D279" totalsRowShown="0">
+  <autoFilter ref="A2:D279" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D277">
     <sortCondition ref="A2:A277"/>
   </sortState>
@@ -2140,7 +2152,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D277"/>
+  <dimension ref="A1:D279"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
@@ -2185,11 +2197,11 @@
         <v>8</v>
       </c>
       <c r="C3" t="str">
-        <f>_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
+        <f t="shared" ref="C3:D22" si="0">_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
       <c r="D3" t="str">
-        <f>_xlfn.TRANSLATE($B3,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente de façon aléatoire</v>
       </c>
     </row>
@@ -2201,11 +2213,11 @@
         <v>10</v>
       </c>
       <c r="C4" t="str">
-        <f>_xlfn.TRANSLATE($B4,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista al final de la cola</v>
       </c>
       <c r="D4" t="str">
-        <f>_xlfn.TRANSLATE($B4,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste en bas de la file d’attente</v>
       </c>
     </row>
@@ -2217,11 +2229,11 @@
         <v>12</v>
       </c>
       <c r="C5" t="str">
-        <f>_xlfn.TRANSLATE($B5,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista a la cola</v>
       </c>
       <c r="D5" t="str">
-        <f>_xlfn.TRANSLATE($B5,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente</v>
       </c>
     </row>
@@ -2233,11 +2245,11 @@
         <v>14</v>
       </c>
       <c r="C6" t="str">
-        <f>_xlfn.TRANSLATE($B6,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir medios a la lista de reproducción</v>
       </c>
       <c r="D6" t="str">
-        <f>_xlfn.TRANSLATE($B6,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter un média à une playlist</v>
       </c>
     </row>
@@ -2249,11 +2261,11 @@
         <v>16</v>
       </c>
       <c r="C7" t="str">
-        <f>_xlfn.TRANSLATE($B7,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
       <c r="D7" t="str">
-        <f>_xlfn.TRANSLATE($B7,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la playlist</v>
       </c>
     </row>
@@ -2265,11 +2277,11 @@
         <v>18</v>
       </c>
       <c r="C8" t="str">
-        <f>_xlfn.TRANSLATE($B8,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la cola</v>
       </c>
       <c r="D8" t="str">
-        <f>_xlfn.TRANSLATE($B8,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la file d’attente</v>
       </c>
     </row>
@@ -2281,11 +2293,11 @@
         <v>20</v>
       </c>
       <c r="C9" t="str">
-        <f>_xlfn.TRANSLATE($B9,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la biblioteca</v>
       </c>
       <c r="D9" t="str">
-        <f>_xlfn.TRANSLATE($B9,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la bibliothèque</v>
       </c>
     </row>
@@ -2297,11 +2309,11 @@
         <v>22</v>
       </c>
       <c r="C10" t="str">
-        <f>_xlfn.TRANSLATE($B10,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a los que me gusta</v>
       </c>
       <c r="D10" t="str">
-        <f>_xlfn.TRANSLATE($B10,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter aux aimés</v>
       </c>
     </row>
@@ -2313,11 +2325,11 @@
         <v>24</v>
       </c>
       <c r="C11" t="str">
-        <f>_xlfn.TRANSLATE($B11,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la cola</v>
       </c>
       <c r="D11" t="str">
-        <f>_xlfn.TRANSLATE($B11,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la file d’attente</v>
       </c>
     </row>
@@ -2329,11 +2341,11 @@
         <v>26</v>
       </c>
       <c r="C12" t="str">
-        <f>_xlfn.TRANSLATE($B12,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadido a la lista de reproducción</v>
       </c>
       <c r="D12" t="str">
-        <f>_xlfn.TRANSLATE($B12,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouté à la playlist</v>
       </c>
     </row>
@@ -2345,11 +2357,11 @@
         <v>28</v>
       </c>
       <c r="C13" t="str">
-        <f>_xlfn.TRANSLATE($B13,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir Build</v>
       </c>
       <c r="D13" t="str">
-        <f>_xlfn.TRANSLATE($B13,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une construction</v>
       </c>
     </row>
@@ -2361,11 +2373,11 @@
         <v>528</v>
       </c>
       <c r="C14" t="str">
-        <f>_xlfn.TRANSLATE($B14,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Anónimo</v>
       </c>
       <c r="D14" t="str">
-        <f>_xlfn.TRANSLATE($B14,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Anonyme</v>
       </c>
     </row>
@@ -2377,11 +2389,11 @@
         <v>30</v>
       </c>
       <c r="C15" t="str">
-        <f>_xlfn.TRANSLATE($B15,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Archivo APK</v>
       </c>
       <c r="D15" t="str">
-        <f>_xlfn.TRANSLATE($B15,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Fichier APK</v>
       </c>
     </row>
@@ -2393,11 +2405,11 @@
         <v>535</v>
       </c>
       <c r="C16" t="str">
-        <f>_xlfn.TRANSLATE($B16,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Tiempo medio de respuesta</v>
       </c>
       <c r="D16" t="str">
-        <f>_xlfn.TRANSLATE($B16,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Temps de réponse moyen</v>
       </c>
     </row>
@@ -2409,11 +2421,11 @@
         <v>552</v>
       </c>
       <c r="C17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Tiempo medio</v>
       </c>
       <c r="D17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Temps moyen</v>
       </c>
     </row>
@@ -2425,11 +2437,11 @@
         <v>32</v>
       </c>
       <c r="C18" t="str">
-        <f>_xlfn.TRANSLATE($B18,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Gestiona tus builds de Android</v>
       </c>
       <c r="D18" t="str">
-        <f>_xlfn.TRANSLATE($B18,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Gérez vos versions Android</v>
       </c>
     </row>
@@ -2441,11 +2453,11 @@
         <v>34</v>
       </c>
       <c r="C19" t="str">
-        <f>_xlfn.TRANSLATE($B19,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Construcciones</v>
       </c>
       <c r="D19" t="str">
-        <f>_xlfn.TRANSLATE($B19,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -2457,11 +2469,11 @@
         <v>36</v>
       </c>
       <c r="C20" t="str">
-        <f>_xlfn.TRANSLATE($B20,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Cancelar</v>
       </c>
       <c r="D20" t="str">
-        <f>_xlfn.TRANSLATE($B20,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -2473,11 +2485,11 @@
         <v>529</v>
       </c>
       <c r="C21" t="str">
-        <f>_xlfn.TRANSLATE($B21,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Conde</v>
       </c>
       <c r="D21" t="str">
-        <f>_xlfn.TRANSLATE($B21,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Comte</v>
       </c>
     </row>
@@ -2489,11 +2501,11 @@
         <v>38</v>
       </c>
       <c r="C22" t="str">
-        <f>_xlfn.TRANSLATE($B22,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Descripción</v>
       </c>
       <c r="D22" t="str">
-        <f>_xlfn.TRANSLATE($B22,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Description</v>
       </c>
     </row>
@@ -2505,11 +2517,11 @@
         <v>40</v>
       </c>
       <c r="C23" t="str">
-        <f>_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
+        <f t="shared" ref="C23:D46" si="1">_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
         <v>Aquí entra la descripción...</v>
       </c>
       <c r="D23" t="str">
-        <f>_xlfn.TRANSLATE($B23,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Voici la description...</v>
       </c>
     </row>
@@ -2521,11 +2533,11 @@
         <v>42</v>
       </c>
       <c r="C24" t="str">
-        <f>_xlfn.TRANSLATE($B24,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Enter Version</v>
       </c>
       <c r="D24" t="str">
-        <f>_xlfn.TRANSLATE($B24,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Enter Version</v>
       </c>
     </row>
@@ -2537,11 +2549,11 @@
         <v>536</v>
       </c>
       <c r="C25" t="str">
-        <f>_xlfn.TRANSLATE($B25,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>No se han cargado las estadísticas</v>
       </c>
       <c r="D25" t="str">
-        <f>_xlfn.TRANSLATE($B25,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Échec de charger les stats</v>
       </c>
     </row>
@@ -2553,11 +2565,11 @@
         <v>537</v>
       </c>
       <c r="C26" t="str">
-        <f>_xlfn.TRANSLATE($B26,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Actividad horaria</v>
       </c>
       <c r="D26" t="str">
-        <f>_xlfn.TRANSLATE($B26,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Activité horaire</v>
       </c>
     </row>
@@ -2569,11 +2581,11 @@
         <v>538</v>
       </c>
       <c r="C27" t="str">
-        <f>_xlfn.TRANSLATE($B27,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Métodos HTTP</v>
       </c>
       <c r="D27" t="str">
-        <f>_xlfn.TRANSLATE($B27,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Méthodes HTTP</v>
       </c>
     </row>
@@ -2585,11 +2597,11 @@
         <v>44</v>
       </c>
       <c r="C28" t="str">
-        <f>_xlfn.TRANSLATE($B28,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Últimas novedades</v>
       </c>
       <c r="D28" t="str">
-        <f>_xlfn.TRANSLATE($B28,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Dernières nouvelles</v>
       </c>
     </row>
@@ -2601,11 +2613,11 @@
         <v>530</v>
       </c>
       <c r="C29" t="str">
-        <f>_xlfn.TRANSLATE($B29,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Max</v>
       </c>
       <c r="D29" t="str">
-        <f>_xlfn.TRANSLATE($B29,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Max</v>
       </c>
     </row>
@@ -2617,11 +2629,11 @@
         <v>531</v>
       </c>
       <c r="C30" t="str">
-        <f>_xlfn.TRANSLATE($B30,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Método</v>
       </c>
       <c r="D30" t="str">
-        <f>_xlfn.TRANSLATE($B30,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Méthode</v>
       </c>
     </row>
@@ -2633,11 +2645,11 @@
         <v>532</v>
       </c>
       <c r="C31" t="str">
-        <f>_xlfn.TRANSLATE($B31,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Min</v>
       </c>
       <c r="D31" t="str">
-        <f>_xlfn.TRANSLATE($B31,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Min</v>
       </c>
     </row>
@@ -2649,11 +2661,11 @@
         <v>46</v>
       </c>
       <c r="C32" t="str">
-        <f>_xlfn.TRANSLATE($B32,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Aún no hay builds</v>
       </c>
       <c r="D32" t="str">
-        <f>_xlfn.TRANSLATE($B32,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Pas encore de builds</v>
       </c>
     </row>
@@ -2665,11 +2677,11 @@
         <v>539</v>
       </c>
       <c r="C33" t="str">
-        <f>_xlfn.TRANSLATE($B33,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>No hay deseje de datos</v>
       </c>
       <c r="D33" t="e" vm="1">
-        <f>_xlfn.TRANSLATE($B33,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -2681,11 +2693,11 @@
         <v>540</v>
       </c>
       <c r="C34" t="str">
-        <f>_xlfn.TRANSLATE($B34,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Aún no hay datos</v>
       </c>
       <c r="D34" t="str">
-        <f>_xlfn.TRANSLATE($B34,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Pas encore de données</v>
       </c>
     </row>
@@ -2697,11 +2709,11 @@
         <v>541</v>
       </c>
       <c r="C35" t="str">
-        <f>_xlfn.TRANSLATE($B35,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Sin estadísticas</v>
       </c>
       <c r="D35" t="str">
-        <f>_xlfn.TRANSLATE($B35,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Pas de statistiques</v>
       </c>
     </row>
@@ -2713,11 +2725,11 @@
         <v>48</v>
       </c>
       <c r="C36" t="str">
-        <f>_xlfn.TRANSLATE($B36,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solo APK</v>
       </c>
       <c r="D36" t="str">
-        <f>_xlfn.TRANSLATE($B36,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Seul APK</v>
       </c>
     </row>
@@ -2729,11 +2741,11 @@
         <v>50</v>
       </c>
       <c r="C37" t="str">
-        <f>_xlfn.TRANSLATE($B37,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Opcional</v>
       </c>
       <c r="D37" t="str">
-        <f>_xlfn.TRANSLATE($B37,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Optionnel</v>
       </c>
     </row>
@@ -2745,11 +2757,11 @@
         <v>542</v>
       </c>
       <c r="C38" t="str">
-        <f>_xlfn.TRANSLATE($B38,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>P50 - P90</v>
       </c>
       <c r="D38" t="str">
-        <f>_xlfn.TRANSLATE($B38,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>P50 - P90</v>
       </c>
     </row>
@@ -2761,11 +2773,11 @@
         <v>543</v>
       </c>
       <c r="C39" t="str">
-        <f>_xlfn.TRANSLATE($B39,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Latencia P95</v>
       </c>
       <c r="D39" t="str">
-        <f>_xlfn.TRANSLATE($B39,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Latence P95</v>
       </c>
     </row>
@@ -2777,11 +2789,11 @@
         <v>533</v>
       </c>
       <c r="C40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>P99</v>
       </c>
       <c r="D40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>P99</v>
       </c>
     </row>
@@ -2793,11 +2805,11 @@
         <v>52</v>
       </c>
       <c r="C41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Leer Fallido</v>
       </c>
       <c r="D41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Lire Échec</v>
       </c>
     </row>
@@ -2809,11 +2821,11 @@
         <v>544</v>
       </c>
       <c r="C42" t="str">
-        <f>_xlfn.TRANSLATE($B42,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes por día</v>
       </c>
       <c r="D42" t="str">
-        <f>_xlfn.TRANSLATE($B42,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Demandes par jour</v>
       </c>
     </row>
@@ -2825,11 +2837,11 @@
         <v>534</v>
       </c>
       <c r="C43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes</v>
       </c>
       <c r="D43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Demandes</v>
       </c>
     </row>
@@ -2841,11 +2853,11 @@
         <v>545</v>
       </c>
       <c r="C44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes a lo largo del tiempo</v>
       </c>
       <c r="D44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Demandes au fil du temps</v>
       </c>
     </row>
@@ -2857,11 +2869,11 @@
         <v>54</v>
       </c>
       <c r="C45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Obligatorio</v>
       </c>
       <c r="D45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Obligatoire</v>
       </c>
     </row>
@@ -2873,11 +2885,11 @@
         <v>553</v>
       </c>
       <c r="C46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Códigos de respuesta</v>
       </c>
       <c r="D46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,D$2)</f>
+        <f t="shared" si="1"/>
         <v>Codes de réponse</v>
       </c>
     </row>
@@ -2892,7 +2904,7 @@
         <v>555</v>
       </c>
       <c r="D47" t="str">
-        <f>_xlfn.TRANSLATE($B47,$B$2,D$2)</f>
+        <f t="shared" ref="D47:D110" si="2">_xlfn.TRANSLATE($B47,$B$2,D$2)</f>
         <v>Itinéraire</v>
       </c>
     </row>
@@ -2904,11 +2916,11 @@
         <v>56</v>
       </c>
       <c r="C48" t="str">
-        <f>_xlfn.TRANSLATE($B48,$B$2,C$2)</f>
+        <f t="shared" ref="C48:C79" si="3">_xlfn.TRANSLATE($B48,$B$2,C$2)</f>
         <v>Seleccionar APK</v>
       </c>
       <c r="D48" t="str">
-        <f>_xlfn.TRANSLATE($B48,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sélectionner APK</v>
       </c>
     </row>
@@ -2920,11 +2932,11 @@
         <v>58</v>
       </c>
       <c r="C49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Seleccionados</v>
       </c>
       <c r="D49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sélectionné</v>
       </c>
     </row>
@@ -2936,11 +2948,11 @@
         <v>60</v>
       </c>
       <c r="C50" t="str">
-        <f>_xlfn.TRANSLATE($B50,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Próximamente</v>
       </c>
       <c r="D50" t="str">
-        <f>_xlfn.TRANSLATE($B50,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -2952,11 +2964,11 @@
         <v>62</v>
       </c>
       <c r="C51" t="str">
-        <f>_xlfn.TRANSLATE($B51,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Configuración de plataformas</v>
       </c>
       <c r="D51" t="str">
-        <f>_xlfn.TRANSLATE($B51,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Réglages de la plateforme</v>
       </c>
     </row>
@@ -2968,11 +2980,11 @@
         <v>64</v>
       </c>
       <c r="C52" t="str">
-        <f>_xlfn.TRANSLATE($B52,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Escenarios</v>
       </c>
       <c r="D52" t="str">
-        <f>_xlfn.TRANSLATE($B52,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Décors</v>
       </c>
     </row>
@@ -2984,11 +2996,11 @@
         <v>34</v>
       </c>
       <c r="C53" t="str">
-        <f>_xlfn.TRANSLATE($B53,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Construcciones</v>
       </c>
       <c r="D53" t="str">
-        <f>_xlfn.TRANSLATE($B53,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -3000,11 +3012,11 @@
         <v>64</v>
       </c>
       <c r="C54" t="str">
-        <f>_xlfn.TRANSLATE($B54,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Escenarios</v>
       </c>
       <c r="D54" t="str">
-        <f>_xlfn.TRANSLATE($B54,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Décors</v>
       </c>
     </row>
@@ -3016,11 +3028,11 @@
         <v>68</v>
       </c>
       <c r="C55" t="str">
-        <f>_xlfn.TRANSLATE($B55,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuarios</v>
       </c>
       <c r="D55" t="str">
-        <f>_xlfn.TRANSLATE($B55,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -3032,11 +3044,11 @@
         <v>546</v>
       </c>
       <c r="C56" t="str">
-        <f>_xlfn.TRANSLATE($B56,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Rutas principales</v>
       </c>
       <c r="D56" t="str">
-        <f>_xlfn.TRANSLATE($B56,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Itinéraires principaux</v>
       </c>
     </row>
@@ -3048,11 +3060,11 @@
         <v>547</v>
       </c>
       <c r="C57" t="str">
-        <f>_xlfn.TRANSLATE($B57,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Solicitudes totales</v>
       </c>
       <c r="D57" t="str">
-        <f>_xlfn.TRANSLATE($B57,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Nombre total de demandes</v>
       </c>
     </row>
@@ -3064,11 +3076,11 @@
         <v>70</v>
       </c>
       <c r="C58" t="str">
-        <f>_xlfn.TRANSLATE($B58,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Compilación de subida</v>
       </c>
       <c r="D58" t="str">
-        <f>_xlfn.TRANSLATE($B58,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Upload Build</v>
       </c>
     </row>
@@ -3080,11 +3092,11 @@
         <v>72</v>
       </c>
       <c r="C59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Fallido en la subida</v>
       </c>
       <c r="D59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement échoué</v>
       </c>
     </row>
@@ -3096,11 +3108,11 @@
         <v>74</v>
       </c>
       <c r="C60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Sube tu primera construcción</v>
       </c>
       <c r="D60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargez votre première compilation</v>
       </c>
     </row>
@@ -3112,11 +3124,11 @@
         <v>76</v>
       </c>
       <c r="C61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Subir nueva versión</v>
       </c>
       <c r="D61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger une nouvelle version</v>
       </c>
     </row>
@@ -3128,11 +3140,11 @@
         <v>78</v>
       </c>
       <c r="C62" t="str">
-        <f>_xlfn.TRANSLATE($B62,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Éxito en la subida</v>
       </c>
       <c r="D62" t="str">
-        <f>_xlfn.TRANSLATE($B62,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Succès de la télévision</v>
       </c>
     </row>
@@ -3144,11 +3156,11 @@
         <v>80</v>
       </c>
       <c r="C63" t="str">
-        <f>_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Subiendo algo...</v>
       </c>
       <c r="D63" t="str">
-        <f>_xlfn.TRANSLATE($B63,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement...</v>
       </c>
     </row>
@@ -3160,11 +3172,11 @@
         <v>481</v>
       </c>
       <c r="C64" t="str">
-        <f>_xlfn.TRANSLATE($B64,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuario</v>
       </c>
       <c r="D64" t="str">
-        <f>_xlfn.TRANSLATE($B64,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateur</v>
       </c>
     </row>
@@ -3176,11 +3188,11 @@
         <v>548</v>
       </c>
       <c r="C65" t="str">
-        <f>_xlfn.TRANSLATE($B65,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Actividad de usuario</v>
       </c>
       <c r="D65" t="str">
-        <f>_xlfn.TRANSLATE($B65,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Activité des utilisateurs</v>
       </c>
     </row>
@@ -3192,11 +3204,11 @@
         <v>60</v>
       </c>
       <c r="C66" t="str">
-        <f>_xlfn.TRANSLATE($B66,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Próximamente</v>
       </c>
       <c r="D66" t="str">
-        <f>_xlfn.TRANSLATE($B66,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -3208,11 +3220,11 @@
         <v>83</v>
       </c>
       <c r="C67" t="str">
-        <f>_xlfn.TRANSLATE($B67,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Gestionar los usuarios de la plataforma</v>
       </c>
       <c r="D67" t="str">
-        <f>_xlfn.TRANSLATE($B67,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Gérer les utilisateurs de la plateforme</v>
       </c>
     </row>
@@ -3224,11 +3236,11 @@
         <v>68</v>
       </c>
       <c r="C68" t="str">
-        <f>_xlfn.TRANSLATE($B68,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuarios</v>
       </c>
       <c r="D68" t="str">
-        <f>_xlfn.TRANSLATE($B68,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -3240,11 +3252,11 @@
         <v>86</v>
       </c>
       <c r="C69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Versión</v>
       </c>
       <c r="D69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Version</v>
       </c>
     </row>
@@ -3256,11 +3268,11 @@
         <v>88</v>
       </c>
       <c r="C70" t="str">
-        <f>_xlfn.TRANSLATE($B70,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbum</v>
       </c>
       <c r="D70" t="str">
-        <f>_xlfn.TRANSLATE($B70,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Album</v>
       </c>
     </row>
@@ -3272,11 +3284,11 @@
         <v>90</v>
       </c>
       <c r="C71" t="str">
-        <f>_xlfn.TRANSLATE($B71,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbumes</v>
       </c>
       <c r="D71" t="str">
-        <f>_xlfn.TRANSLATE($B71,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums</v>
       </c>
     </row>
@@ -3288,11 +3300,11 @@
         <v>92</v>
       </c>
       <c r="C72" t="str">
-        <f>_xlfn.TRANSLATE($B72,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbumes y sencillos</v>
       </c>
       <c r="D72" t="str">
-        <f>_xlfn.TRANSLATE($B72,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums et singles</v>
       </c>
     </row>
@@ -3304,11 +3316,11 @@
         <v>94</v>
       </c>
       <c r="C73" t="str">
-        <f>_xlfn.TRANSLATE($B73,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Todos</v>
       </c>
       <c r="D73" t="str">
-        <f>_xlfn.TRANSLATE($B73,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Tous</v>
       </c>
     </row>
@@ -3320,11 +3332,11 @@
         <v>96</v>
       </c>
       <c r="C74" t="str">
-        <f>_xlfn.TRANSLATE($B74,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Abril</v>
       </c>
       <c r="D74" t="str">
-        <f>_xlfn.TRANSLATE($B74,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Avril</v>
       </c>
     </row>
@@ -3336,11 +3348,11 @@
         <v>98</v>
       </c>
       <c r="C75" t="str">
-        <f>_xlfn.TRANSLATE($B75,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Artista</v>
       </c>
       <c r="D75" t="str">
-        <f>_xlfn.TRANSLATE($B75,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artiste</v>
       </c>
     </row>
@@ -3352,11 +3364,11 @@
         <v>100</v>
       </c>
       <c r="C76" t="str">
-        <f>_xlfn.TRANSLATE($B76,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Artistas</v>
       </c>
       <c r="D76" t="str">
-        <f>_xlfn.TRANSLATE($B76,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artistes</v>
       </c>
     </row>
@@ -3368,11 +3380,11 @@
         <v>102</v>
       </c>
       <c r="C77" t="str">
-        <f>_xlfn.TRANSLATE($B77,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Agosto</v>
       </c>
       <c r="D77" t="str">
-        <f>_xlfn.TRANSLATE($B77,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Août</v>
       </c>
     </row>
@@ -3384,11 +3396,11 @@
         <v>104</v>
       </c>
       <c r="C78" t="str">
-        <f>_xlfn.TRANSLATE($B78,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Minutos medios por canción</v>
       </c>
       <c r="D78" t="str">
-        <f>_xlfn.TRANSLATE($B78,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Minutes moyennes par chanson</v>
       </c>
     </row>
@@ -3400,11 +3412,11 @@
         <v>106</v>
       </c>
       <c r="C79" t="str">
-        <f>_xlfn.TRANSLATE($B79,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>por</v>
       </c>
       <c r="D79" t="str">
-        <f>_xlfn.TRANSLATE($B79,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>par</v>
       </c>
     </row>
@@ -3416,11 +3428,11 @@
         <v>36</v>
       </c>
       <c r="C80" t="str">
-        <f>_xlfn.TRANSLATE($B80,$B$2,C$2)</f>
+        <f t="shared" ref="C80:C98" si="4">_xlfn.TRANSLATE($B80,$B$2,C$2)</f>
         <v>Cancelar</v>
       </c>
       <c r="D80" t="str">
-        <f>_xlfn.TRANSLATE($B80,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -3432,11 +3444,11 @@
         <v>109</v>
       </c>
       <c r="C81" t="str">
-        <f>_xlfn.TRANSLATE($B81,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Cambiar contraseña</v>
       </c>
       <c r="D81" t="str">
-        <f>_xlfn.TRANSLATE($B81,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Changer le mot de passe</v>
       </c>
     </row>
@@ -3448,11 +3460,11 @@
         <v>111</v>
       </c>
       <c r="C82" t="str">
-        <f>_xlfn.TRANSLATE($B82,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descargas claras</v>
       </c>
       <c r="D82" t="str">
-        <f>_xlfn.TRANSLATE($B82,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargements clairs</v>
       </c>
     </row>
@@ -3464,11 +3476,11 @@
         <v>113</v>
       </c>
       <c r="C83" t="str">
-        <f>_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Haz clic para descargar</v>
       </c>
       <c r="D83" t="str">
-        <f>_xlfn.TRANSLATE($B83,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Cliquez pour télécharger</v>
       </c>
     </row>
@@ -3480,11 +3492,11 @@
         <v>115</v>
       </c>
       <c r="C84" t="str">
-        <f>_xlfn.TRANSLATE($B84,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Topo comunitario</v>
       </c>
       <c r="D84" t="str">
-        <f>_xlfn.TRANSLATE($B84,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sommet communautaire</v>
       </c>
     </row>
@@ -3496,11 +3508,11 @@
         <v>117</v>
       </c>
       <c r="C85" t="str">
-        <f>_xlfn.TRANSLATE($B85,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Completado</v>
       </c>
       <c r="D85" t="str">
-        <f>_xlfn.TRANSLATE($B85,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Achèvement</v>
       </c>
     </row>
@@ -3512,11 +3524,11 @@
         <v>119</v>
       </c>
       <c r="C86" t="str">
-        <f>_xlfn.TRANSLATE($B86,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>URL de la lista de copiar</v>
       </c>
       <c r="D86" t="str">
-        <f>_xlfn.TRANSLATE($B86,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>URL de la liste de copie</v>
       </c>
     </row>
@@ -3528,11 +3540,11 @@
         <v>121</v>
       </c>
       <c r="C87" t="str">
-        <f>_xlfn.TRANSLATE($B87,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Copiar la URL de la canción</v>
       </c>
       <c r="D87" t="str">
-        <f>_xlfn.TRANSLATE($B87,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Copier l’URL de la chanson</v>
       </c>
     </row>
@@ -3544,11 +3556,11 @@
         <v>123</v>
       </c>
       <c r="C88" t="str">
-        <f>_xlfn.TRANSLATE($B88,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Crear</v>
       </c>
       <c r="D88" t="str">
-        <f>_xlfn.TRANSLATE($B88,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Créer</v>
       </c>
     </row>
@@ -3560,11 +3572,11 @@
         <v>125</v>
       </c>
       <c r="C89" t="str">
-        <f>_xlfn.TRANSLATE($B89,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Crear...</v>
       </c>
       <c r="D89" t="str">
-        <f>_xlfn.TRANSLATE($B89,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Créer...</v>
       </c>
     </row>
@@ -3576,11 +3588,11 @@
         <v>127</v>
       </c>
       <c r="C90" t="str">
-        <f>_xlfn.TRANSLATE($B90,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Fecha añadida</v>
       </c>
       <c r="D90" t="str">
-        <f>_xlfn.TRANSLATE($B90,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Date ajoutée</v>
       </c>
     </row>
@@ -3592,11 +3604,11 @@
         <v>129</v>
       </c>
       <c r="C91" t="str">
-        <f>_xlfn.TRANSLATE($B91,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Diciembre</v>
       </c>
       <c r="D91" t="str">
-        <f>_xlfn.TRANSLATE($B91,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Décembre</v>
       </c>
     </row>
@@ -3608,11 +3620,11 @@
         <v>131</v>
       </c>
       <c r="C92" t="str">
-        <f>_xlfn.TRANSLATE($B92,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Tu dispositivo no soporta al trabajador de servicio</v>
       </c>
       <c r="D92" t="str">
-        <f>_xlfn.TRANSLATE($B92,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Votre appareil ne prend pas en charge l’assistant de service</v>
       </c>
     </row>
@@ -3624,11 +3636,11 @@
         <v>133</v>
       </c>
       <c r="C93" t="str">
-        <f>_xlfn.TRANSLATE($B93,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Disco</v>
       </c>
       <c r="D93" t="str">
-        <f>_xlfn.TRANSLATE($B93,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Disque</v>
       </c>
     </row>
@@ -3640,11 +3652,11 @@
         <v>135</v>
       </c>
       <c r="C94" t="str">
-        <f>_xlfn.TRANSLATE($B94,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Nombre de Muestra</v>
       </c>
       <c r="D94" t="str">
-        <f>_xlfn.TRANSLATE($B94,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Nom d’affichage</v>
       </c>
     </row>
@@ -3656,11 +3668,11 @@
         <v>137</v>
       </c>
       <c r="C95" t="str">
-        <f>_xlfn.TRANSLATE($B95,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descargar</v>
       </c>
       <c r="D95" t="str">
-        <f>_xlfn.TRANSLATE($B95,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger</v>
       </c>
     </row>
@@ -3672,11 +3684,11 @@
         <v>139</v>
       </c>
       <c r="C96" t="str">
-        <f>_xlfn.TRANSLATE($B96,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descarga la app para escuchar offline</v>
       </c>
       <c r="D96" t="str">
-        <f>_xlfn.TRANSLATE($B96,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargez l’application pour une écoute hors ligne</v>
       </c>
     </row>
@@ -3688,11 +3700,11 @@
         <v>141</v>
       </c>
       <c r="C97" t="str">
-        <f>_xlfn.TRANSLATE($B97,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
       <c r="D97" t="str">
-        <f>_xlfn.TRANSLATE($B97,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Saisissez une URL Spotify ou YouTube Music</v>
       </c>
     </row>
@@ -3704,11 +3716,11 @@
         <v>143</v>
       </c>
       <c r="C98" t="str">
-        <f>_xlfn.TRANSLATE($B98,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Lista de descargas al dispositivo</v>
       </c>
       <c r="D98" t="str">
-        <f>_xlfn.TRANSLATE($B98,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Liste de téléchargement vers l’appareil</v>
       </c>
     </row>
@@ -3723,7 +3735,7 @@
         <v>146</v>
       </c>
       <c r="D99" t="str">
-        <f>_xlfn.TRANSLATE($B99,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Liste de téléchargement vers serveur</v>
       </c>
     </row>
@@ -3735,11 +3747,11 @@
         <v>148</v>
       </c>
       <c r="C100" t="str">
-        <f>_xlfn.TRANSLATE($B100,$B$2,C$2)</f>
+        <f t="shared" ref="C100:C122" si="5">_xlfn.TRANSLATE($B100,$B$2,C$2)</f>
         <v>Descargar medios al dispositivo</v>
       </c>
       <c r="D100" t="str">
-        <f>_xlfn.TRANSLATE($B100,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger des médias sur l’appareil</v>
       </c>
     </row>
@@ -3751,11 +3763,11 @@
         <v>150</v>
       </c>
       <c r="C101" t="str">
-        <f>_xlfn.TRANSLATE($B101,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descargar mp</v>
       </c>
       <c r="D101" t="str">
-        <f>_xlfn.TRANSLATE($B101,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger le MP</v>
       </c>
     </row>
@@ -3767,11 +3779,11 @@
         <v>152</v>
       </c>
       <c r="C102" t="str">
-        <f>_xlfn.TRANSLATE($B102,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descargar canción al dispositivo</v>
       </c>
       <c r="D102" t="str">
-        <f>_xlfn.TRANSLATE($B102,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger la chanson sur l’appareil</v>
       </c>
     </row>
@@ -3783,11 +3795,11 @@
         <v>154</v>
       </c>
       <c r="C103" t="str">
-        <f>_xlfn.TRANSLATE($B103,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descarga iniciada</v>
       </c>
       <c r="D103" t="str">
-        <f>_xlfn.TRANSLATE($B103,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement lancé</v>
       </c>
     </row>
@@ -3799,11 +3811,11 @@
         <v>156</v>
       </c>
       <c r="C104" t="str">
-        <f>_xlfn.TRANSLATE($B104,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descargar ZIP</v>
       </c>
       <c r="D104" t="str">
-        <f>_xlfn.TRANSLATE($B104,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger ZIP</v>
       </c>
     </row>
@@ -3815,11 +3827,11 @@
         <v>158</v>
       </c>
       <c r="C105" t="str">
-        <f>_xlfn.TRANSLATE($B105,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descargando</v>
       </c>
       <c r="D105" t="str">
-        <f>_xlfn.TRANSLATE($B105,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement</v>
       </c>
     </row>
@@ -3831,11 +3843,11 @@
         <v>160</v>
       </c>
       <c r="C106" t="str">
-        <f>_xlfn.TRANSLATE($B106,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Descargas</v>
       </c>
       <c r="D106" t="str">
-        <f>_xlfn.TRANSLATE($B106,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargements</v>
       </c>
     </row>
@@ -3847,11 +3859,11 @@
         <v>162</v>
       </c>
       <c r="C107" t="str">
-        <f>_xlfn.TRANSLATE($B107,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Duración</v>
       </c>
       <c r="D107" t="str">
-        <f>_xlfn.TRANSLATE($B107,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Durée</v>
       </c>
     </row>
@@ -3863,11 +3875,11 @@
         <v>164</v>
       </c>
       <c r="C108" t="str">
-        <f>_xlfn.TRANSLATE($B108,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Energía</v>
       </c>
       <c r="D108" t="str">
-        <f>_xlfn.TRANSLATE($B108,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Énergie</v>
       </c>
     </row>
@@ -3879,11 +3891,11 @@
         <v>166</v>
       </c>
       <c r="C109" t="str">
-        <f>_xlfn.TRANSLATE($B109,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D109" t="str">
-        <f>_xlfn.TRANSLATE($B109,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3895,11 +3907,11 @@
         <v>168</v>
       </c>
       <c r="C110" t="str">
-        <f>_xlfn.TRANSLATE($B110,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error</v>
       </c>
       <c r="D110" t="str">
-        <f>_xlfn.TRANSLATE($B110,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Erreur</v>
       </c>
     </row>
@@ -3911,11 +3923,11 @@
         <v>170</v>
       </c>
       <c r="C111" t="str">
-        <f>_xlfn.TRANSLATE($B111,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Lenguaje de cambio de error</v>
       </c>
       <c r="D111" t="str">
-        <f>_xlfn.TRANSLATE($B111,$B$2,D$2)</f>
+        <f t="shared" ref="D111:D174" si="6">_xlfn.TRANSLATE($B111,$B$2,D$2)</f>
         <v>Langage de changement d’erreur</v>
       </c>
     </row>
@@ -3927,11 +3939,11 @@
         <v>172</v>
       </c>
       <c r="C112" t="str">
-        <f>_xlfn.TRANSLATE($B112,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D112" t="str">
-        <f>_xlfn.TRANSLATE($B112,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3943,11 +3955,11 @@
         <v>172</v>
       </c>
       <c r="C113" t="str">
-        <f>_xlfn.TRANSLATE($B113,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D113" t="str">
-        <f>_xlfn.TRANSLATE($B113,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -3959,11 +3971,11 @@
         <v>166</v>
       </c>
       <c r="C114" t="str">
-        <f>_xlfn.TRANSLATE($B114,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D114" t="str">
-        <f>_xlfn.TRANSLATE($B114,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3975,11 +3987,11 @@
         <v>176</v>
       </c>
       <c r="C115" t="str">
-        <f>_xlfn.TRANSLATE($B115,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al obtener descargas</v>
       </c>
       <c r="D115" t="str">
-        <f>_xlfn.TRANSLATE($B115,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur de téléchargement</v>
       </c>
     </row>
@@ -3991,11 +4003,11 @@
         <v>178</v>
       </c>
       <c r="C116" t="str">
-        <f>_xlfn.TRANSLATE($B116,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al obtener medios</v>
       </c>
       <c r="D116" t="str">
-        <f>_xlfn.TRANSLATE($B116,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur d’obtention de médias</v>
       </c>
     </row>
@@ -4007,11 +4019,11 @@
         <v>180</v>
       </c>
       <c r="C117" t="str">
-        <f>_xlfn.TRANSLATE($B117,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Cola de obtención de errores</v>
       </c>
       <c r="D117" t="str">
-        <f>_xlfn.TRANSLATE($B117,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>File d’attente d’obtention d’erreurs</v>
       </c>
     </row>
@@ -4023,11 +4035,11 @@
         <v>182</v>
       </c>
       <c r="C118" t="str">
-        <f>_xlfn.TRANSLATE($B118,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Usuario que obtiene errores</v>
       </c>
       <c r="D118" t="str">
-        <f>_xlfn.TRANSLATE($B118,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Utilisateur d’obtention d’erreurs</v>
       </c>
     </row>
@@ -4039,11 +4051,11 @@
         <v>184</v>
       </c>
       <c r="C119" t="str">
-        <f>_xlfn.TRANSLATE($B119,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al dar like a medios</v>
       </c>
       <c r="D119" t="str">
-        <f>_xlfn.TRANSLATE($B119,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur d’appréciation des médias</v>
       </c>
     </row>
@@ -4055,11 +4067,11 @@
         <v>186</v>
       </c>
       <c r="C120" t="str">
-        <f>_xlfn.TRANSLATE($B120,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Búsqueda de errores</v>
       </c>
       <c r="D120" t="str">
-        <f>_xlfn.TRANSLATE($B120,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Recherche d’erreurs</v>
       </c>
     </row>
@@ -4071,11 +4083,11 @@
         <v>188</v>
       </c>
       <c r="C121" t="str">
-        <f>_xlfn.TRANSLATE($B121,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al iniciar la descarga</v>
       </c>
       <c r="D121" t="str">
-        <f>_xlfn.TRANSLATE($B121,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur au démarrage du téléchargement</v>
       </c>
     </row>
@@ -4087,11 +4099,11 @@
         <v>190</v>
       </c>
       <c r="C122" t="str">
-        <f>_xlfn.TRANSLATE($B122,$B$2,C$2)</f>
+        <f t="shared" si="5"/>
         <v>Error al dejar de dar like a los medios</v>
       </c>
       <c r="D122" t="str">
-        <f>_xlfn.TRANSLATE($B122,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Erreur de non-like des médias</v>
       </c>
     </row>
@@ -4106,7 +4118,7 @@
         <v>193</v>
       </c>
       <c r="D123" t="str">
-        <f>_xlfn.TRANSLATE($B123,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec</v>
       </c>
     </row>
@@ -4118,11 +4130,11 @@
         <v>195</v>
       </c>
       <c r="C124" t="str">
-        <f>_xlfn.TRANSLATE($B124,$B$2,C$2)</f>
+        <f t="shared" ref="C124:C155" si="7">_xlfn.TRANSLATE($B124,$B$2,C$2)</f>
         <v>No se añadió contenido a la biblioteca</v>
       </c>
       <c r="D124" t="str">
-        <f>_xlfn.TRANSLATE($B124,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec d’ajouter des médias à la bibliothèque</v>
       </c>
     </row>
@@ -4134,11 +4146,11 @@
         <v>197</v>
       </c>
       <c r="C125" t="str">
-        <f>_xlfn.TRANSLATE($B125,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No se añadió contenido a la lista de reproducción</v>
       </c>
       <c r="D125" t="str">
-        <f>_xlfn.TRANSLATE($B125,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec d’ajouter des médias à la playlist</v>
       </c>
     </row>
@@ -4150,11 +4162,11 @@
         <v>199</v>
       </c>
       <c r="C126" t="str">
-        <f>_xlfn.TRANSLATE($B126,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No cambiaron el idioma</v>
       </c>
       <c r="D126" t="str">
-        <f>_xlfn.TRANSLATE($B126,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec de changer de langue</v>
       </c>
     </row>
@@ -4166,11 +4178,11 @@
         <v>201</v>
       </c>
       <c r="C127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No se han conseguido las listas de reproducción</v>
       </c>
       <c r="D127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec à récupérer les playlists</v>
       </c>
     </row>
@@ -4182,11 +4194,11 @@
         <v>203</v>
       </c>
       <c r="C128" t="str">
-        <f>_xlfn.TRANSLATE($B128,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D128" t="str">
-        <f>_xlfn.TRANSLATE($B128,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Albums en vedette</v>
       </c>
     </row>
@@ -4198,11 +4210,11 @@
         <v>205</v>
       </c>
       <c r="C129" t="str">
-        <f>_xlfn.TRANSLATE($B129,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Listas destacadas</v>
       </c>
       <c r="D129" t="str">
-        <f>_xlfn.TRANSLATE($B129,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Listes en vedette</v>
       </c>
     </row>
@@ -4214,11 +4226,11 @@
         <v>207</v>
       </c>
       <c r="C130" t="str">
-        <f>_xlfn.TRANSLATE($B130,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Febrero</v>
       </c>
       <c r="D130" t="str">
-        <f>_xlfn.TRANSLATE($B130,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Février</v>
       </c>
     </row>
@@ -4230,11 +4242,11 @@
         <v>209</v>
       </c>
       <c r="C131" t="str">
-        <f>_xlfn.TRANSLATE($B131,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Enfoque</v>
       </c>
       <c r="D131" t="str">
-        <f>_xlfn.TRANSLATE($B131,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Focus</v>
       </c>
     </row>
@@ -4246,11 +4258,11 @@
         <v>211</v>
       </c>
       <c r="C132" t="str">
-        <f>_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Amigos</v>
       </c>
       <c r="D132" t="str">
-        <f>_xlfn.TRANSLATE($B132,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Amis</v>
       </c>
     </row>
@@ -4262,11 +4274,11 @@
         <v>213</v>
       </c>
       <c r="C133" t="str">
-        <f>_xlfn.TRANSLATE($B133,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Lista de amigos</v>
       </c>
       <c r="D133" t="str">
-        <f>_xlfn.TRANSLATE($B133,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Liste d’amis</v>
       </c>
     </row>
@@ -4278,11 +4290,11 @@
         <v>215</v>
       </c>
       <c r="C134" t="str">
-        <f>_xlfn.TRANSLATE($B134,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
       <c r="D134" t="str">
-        <f>_xlfn.TRANSLATE($B134,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
       </c>
     </row>
@@ -4294,11 +4306,11 @@
         <v>217</v>
       </c>
       <c r="C135" t="str">
-        <f>_xlfn.TRANSLATE($B135,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Estadísticas de Friends</v>
       </c>
       <c r="D135" t="str">
-        <f>_xlfn.TRANSLATE($B135,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Statistiques de Friends</v>
       </c>
     </row>
@@ -4310,11 +4322,11 @@
         <v>219</v>
       </c>
       <c r="C136" t="str">
-        <f>_xlfn.TRANSLATE($B136,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>General</v>
       </c>
       <c r="D136" t="str">
-        <f>_xlfn.TRANSLATE($B136,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Généralités</v>
       </c>
     </row>
@@ -4326,11 +4338,11 @@
         <v>221</v>
       </c>
       <c r="C137" t="str">
-        <f>_xlfn.TRANSLATE($B137,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Estadísticas generales</v>
       </c>
       <c r="D137" t="str">
-        <f>_xlfn.TRANSLATE($B137,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Statistiques générales</v>
       </c>
     </row>
@@ -4342,11 +4354,11 @@
         <v>223</v>
       </c>
       <c r="C138" t="str">
-        <f>_xlfn.TRANSLATE($B138,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Obtén información</v>
       </c>
       <c r="D138" t="str">
-        <f>_xlfn.TRANSLATE($B138,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Obtenez des infos</v>
       </c>
     </row>
@@ -4358,11 +4370,11 @@
         <v>225</v>
       </c>
       <c r="C139" t="str">
-        <f>_xlfn.TRANSLATE($B139,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Obteniendo información</v>
       </c>
       <c r="D139" t="str">
-        <f>_xlfn.TRANSLATE($B139,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Obtenir des infos</v>
       </c>
     </row>
@@ -4374,11 +4386,11 @@
         <v>227</v>
       </c>
       <c r="C140" t="str">
-        <f>_xlfn.TRANSLATE($B140,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Ir al álbum</v>
       </c>
       <c r="D140" t="str">
-        <f>_xlfn.TRANSLATE($B140,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Aller à l’album</v>
       </c>
     </row>
@@ -4390,11 +4402,11 @@
         <v>229</v>
       </c>
       <c r="C141" t="str">
-        <f>_xlfn.TRANSLATE($B141,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Ir a artista</v>
       </c>
       <c r="D141" t="str">
-        <f>_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Aller à l’artiste</v>
       </c>
     </row>
@@ -4406,11 +4418,11 @@
         <v>231</v>
       </c>
       <c r="C142" t="str">
-        <f>_xlfn.TRANSLATE($B142,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Joyas ocultas que olvidaste</v>
       </c>
       <c r="D142" t="str">
-        <f>_xlfn.TRANSLATE($B142,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Des perles cachées que tu as oubliées</v>
       </c>
     </row>
@@ -4422,11 +4434,11 @@
         <v>233</v>
       </c>
       <c r="C143" t="str">
-        <f>_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Inicio</v>
       </c>
       <c r="D143" t="str">
-        <f>_xlfn.TRANSLATE($B143,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Accueil</v>
       </c>
     </row>
@@ -4438,11 +4450,11 @@
         <v>235</v>
       </c>
       <c r="C144" t="str">
-        <f>_xlfn.TRANSLATE($B144,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Enero</v>
       </c>
       <c r="D144" t="str">
-        <f>_xlfn.TRANSLATE($B144,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Janvier</v>
       </c>
     </row>
@@ -4454,11 +4466,11 @@
         <v>237</v>
       </c>
       <c r="C145" t="str">
-        <f>_xlfn.TRANSLATE($B145,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Julio</v>
       </c>
       <c r="D145" t="str">
-        <f>_xlfn.TRANSLATE($B145,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Juillet</v>
       </c>
     </row>
@@ -4470,11 +4482,11 @@
         <v>239</v>
       </c>
       <c r="C146" t="str">
-        <f>_xlfn.TRANSLATE($B146,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Junio</v>
       </c>
       <c r="D146" t="str">
-        <f>_xlfn.TRANSLATE($B146,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Juin</v>
       </c>
     </row>
@@ -4486,11 +4498,11 @@
         <v>241</v>
       </c>
       <c r="C147" t="str">
-        <f>_xlfn.TRANSLATE($B147,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Idioma</v>
       </c>
       <c r="D147" t="str">
-        <f>_xlfn.TRANSLATE($B147,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Langue</v>
       </c>
     </row>
@@ -4502,11 +4514,11 @@
         <v>243</v>
       </c>
       <c r="C148" t="str">
-        <f>_xlfn.TRANSLATE($B148,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>El cambio de idioma fracasó</v>
       </c>
       <c r="D148" t="str">
-        <f>_xlfn.TRANSLATE($B148,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Échec du changement linguistique</v>
       </c>
     </row>
@@ -4518,11 +4530,11 @@
         <v>245</v>
       </c>
       <c r="C149" t="str">
-        <f>_xlfn.TRANSLATE($B149,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Cambio de idioma</v>
       </c>
       <c r="D149" t="str">
-        <f>_xlfn.TRANSLATE($B149,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Changement de langue</v>
       </c>
     </row>
@@ -4534,11 +4546,11 @@
         <v>247</v>
       </c>
       <c r="C150" t="str">
-        <f>_xlfn.TRANSLATE($B150,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Últimas descargas</v>
       </c>
       <c r="D150" t="str">
-        <f>_xlfn.TRANSLATE($B150,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Derniers téléchargements</v>
       </c>
     </row>
@@ -4550,11 +4562,11 @@
         <v>249</v>
       </c>
       <c r="C151" t="str">
-        <f>_xlfn.TRANSLATE($B151,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Nivel</v>
       </c>
       <c r="D151" t="str">
-        <f>_xlfn.TRANSLATE($B151,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Niveau</v>
       </c>
     </row>
@@ -4566,11 +4578,11 @@
         <v>251</v>
       </c>
       <c r="C152" t="str">
-        <f>_xlfn.TRANSLATE($B152,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Biblioteca</v>
       </c>
       <c r="D152" t="str">
-        <f>_xlfn.TRANSLATE($B152,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Bibliothèque</v>
       </c>
     </row>
@@ -4582,11 +4594,11 @@
         <v>253</v>
       </c>
       <c r="C153" t="str">
-        <f>_xlfn.TRANSLATE($B153,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Como</v>
       </c>
       <c r="D153" t="str">
-        <f>_xlfn.TRANSLATE($B153,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Comme</v>
       </c>
     </row>
@@ -4598,11 +4610,11 @@
         <v>255</v>
       </c>
       <c r="C154" t="str">
-        <f>_xlfn.TRANSLATE($B154,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Canciones que me gustaban</v>
       </c>
       <c r="D154" t="str">
-        <f>_xlfn.TRANSLATE($B154,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons appréciées</v>
       </c>
     </row>
@@ -4614,11 +4626,11 @@
         <v>257</v>
       </c>
       <c r="C155" t="str">
-        <f>_xlfn.TRANSLATE($B155,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Cerrar sesión</v>
       </c>
       <c r="D155" t="str">
-        <f>_xlfn.TRANSLATE($B155,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Déconnexion</v>
       </c>
     </row>
@@ -4630,11 +4642,11 @@
         <v>259</v>
       </c>
       <c r="C156" t="str">
-        <f>_xlfn.TRANSLATE($B156,$B$2,C$2)</f>
+        <f t="shared" ref="C156:C187" si="8">_xlfn.TRANSLATE($B156,$B$2,C$2)</f>
         <v>Letra</v>
       </c>
       <c r="D156" t="str">
-        <f>_xlfn.TRANSLATE($B156,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Paroles</v>
       </c>
     </row>
@@ -4646,11 +4658,11 @@
         <v>261</v>
       </c>
       <c r="C157" t="str">
-        <f>_xlfn.TRANSLATE($B157,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Marzo</v>
       </c>
       <c r="D157" t="str">
-        <f>_xlfn.TRANSLATE($B157,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Mars</v>
       </c>
     </row>
@@ -4662,11 +4674,11 @@
         <v>263</v>
       </c>
       <c r="C158" t="str">
-        <f>_xlfn.TRANSLATE($B158,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Mayo</v>
       </c>
       <c r="D158" t="str">
-        <f>_xlfn.TRANSLATE($B158,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Mai</v>
       </c>
     </row>
@@ -4678,11 +4690,11 @@
         <v>265</v>
       </c>
       <c r="C159" t="str">
-        <f>_xlfn.TRANSLATE($B159,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D159" t="str">
-        <f>_xlfn.TRANSLATE($B159,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
@@ -4694,11 +4706,11 @@
         <v>503</v>
       </c>
       <c r="C160" t="str">
-        <f>_xlfn.TRANSLATE($B160,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>A los medios les gustó</v>
       </c>
       <c r="D160" t="str">
-        <f>_xlfn.TRANSLATE($B160,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Les médias appréciaient</v>
       </c>
     </row>
@@ -4710,11 +4722,11 @@
         <v>267</v>
       </c>
       <c r="C161" t="str">
-        <f>_xlfn.TRANSLATE($B161,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Progreso de los medios</v>
       </c>
       <c r="D161" t="str">
-        <f>_xlfn.TRANSLATE($B161,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Progrès des médias</v>
       </c>
     </row>
@@ -4726,11 +4738,11 @@
         <v>269</v>
       </c>
       <c r="C162" t="str">
-        <f>_xlfn.TRANSLATE($B162,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Actas</v>
       </c>
       <c r="D162" t="str">
-        <f>_xlfn.TRANSLATE($B162,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Procès-verbal</v>
       </c>
     </row>
@@ -4742,11 +4754,11 @@
         <v>271</v>
       </c>
       <c r="C163" t="str">
-        <f>_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Minutos escuchados</v>
       </c>
       <c r="D163" t="str">
-        <f>_xlfn.TRANSLATE($B163,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutes écoutées</v>
       </c>
     </row>
@@ -4758,11 +4770,11 @@
         <v>273</v>
       </c>
       <c r="C164" t="str">
-        <f>_xlfn.TRANSLATE($B164,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Minutos escuchados por día</v>
       </c>
       <c r="D164" t="str">
-        <f>_xlfn.TRANSLATE($B164,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Minutes écoutées par jour</v>
       </c>
     </row>
@@ -4774,11 +4786,11 @@
         <v>275</v>
       </c>
       <c r="C165" t="str">
-        <f>_xlfn.TRANSLATE($B165,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D165" t="str">
-        <f>_xlfn.TRANSLATE($B165,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
@@ -4790,11 +4802,11 @@
         <v>277</v>
       </c>
       <c r="C166" t="str">
-        <f>_xlfn.TRANSLATE($B166,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Más opciones</v>
       </c>
       <c r="D166" t="str">
-        <f>_xlfn.TRANSLATE($B166,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Plus d’options</v>
       </c>
     </row>
@@ -4806,11 +4818,11 @@
         <v>279</v>
       </c>
       <c r="C167" t="str">
-        <f>_xlfn.TRANSLATE($B167,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Más canciones de</v>
       </c>
       <c r="D167" t="str">
-        <f>_xlfn.TRANSLATE($B167,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Plus de chansons de</v>
       </c>
     </row>
@@ -4822,11 +4834,11 @@
         <v>281</v>
       </c>
       <c r="C168" t="str">
-        <f>_xlfn.TRANSLATE($B168,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Más escuchado</v>
       </c>
       <c r="D168" t="str">
-        <f>_xlfn.TRANSLATE($B168,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Les plus écoutés</v>
       </c>
     </row>
@@ -4838,11 +4850,11 @@
         <v>283</v>
       </c>
       <c r="C169" t="str">
-        <f>_xlfn.TRANSLATE($B169,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Álbumes más escuchados</v>
       </c>
       <c r="D169" t="str">
-        <f>_xlfn.TRANSLATE($B169,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Albums les plus écoutés</v>
       </c>
     </row>
@@ -4854,11 +4866,11 @@
         <v>285</v>
       </c>
       <c r="C170" t="str">
-        <f>_xlfn.TRANSLATE($B170,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Artistas más escuchados</v>
       </c>
       <c r="D170" t="str">
-        <f>_xlfn.TRANSLATE($B170,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Artistes les plus écoutés</v>
       </c>
     </row>
@@ -4870,11 +4882,11 @@
         <v>287</v>
       </c>
       <c r="C171" t="str">
-        <f>_xlfn.TRANSLATE($B171,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Canciones más escuchadas</v>
       </c>
       <c r="D171" t="str">
-        <f>_xlfn.TRANSLATE($B171,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Chansons les plus écoutées</v>
       </c>
     </row>
@@ -4886,11 +4898,11 @@
         <v>289</v>
       </c>
       <c r="C172" t="str">
-        <f>_xlfn.TRANSLATE($B172,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Nombre</v>
       </c>
       <c r="D172" t="str">
-        <f>_xlfn.TRANSLATE($B172,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Nom</v>
       </c>
     </row>
@@ -4902,11 +4914,11 @@
         <v>291</v>
       </c>
       <c r="C173" t="str">
-        <f>_xlfn.TRANSLATE($B173,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Introducir nueva contraseña</v>
       </c>
       <c r="D173" t="str">
-        <f>_xlfn.TRANSLATE($B173,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
@@ -4918,11 +4930,11 @@
         <v>293</v>
       </c>
       <c r="C174" t="str">
-        <f>_xlfn.TRANSLATE($B174,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Nueva lista de reproducción</v>
       </c>
       <c r="D174" t="str">
-        <f>_xlfn.TRANSLATE($B174,$B$2,D$2)</f>
+        <f t="shared" si="6"/>
         <v>Nouvelle playlist</v>
       </c>
     </row>
@@ -4934,11 +4946,11 @@
         <v>295</v>
       </c>
       <c r="C175" t="str">
-        <f>_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D175" t="str">
-        <f>_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
+        <f t="shared" ref="D175:D238" si="9">_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
         <v>Nouveau nom de la playlist</v>
       </c>
     </row>
@@ -4950,11 +4962,11 @@
         <v>297</v>
       </c>
       <c r="C176" t="str">
-        <f>_xlfn.TRANSLATE($B176,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Nueva versión disponible</v>
       </c>
       <c r="D176" t="str">
-        <f>_xlfn.TRANSLATE($B176,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Nouvelle version disponible</v>
       </c>
     </row>
@@ -4966,11 +4978,11 @@
         <v>299</v>
       </c>
       <c r="C177" t="str">
-        <f>_xlfn.TRANSLATE($B177,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Próximos medios</v>
       </c>
       <c r="D177" t="str">
-        <f>_xlfn.TRANSLATE($B177,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Médias suivants</v>
       </c>
     </row>
@@ -4982,11 +4994,11 @@
         <v>301</v>
       </c>
       <c r="C178" t="str">
-        <f>_xlfn.TRANSLATE($B178,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
       <c r="D178" t="str">
-        <f>_xlfn.TRANSLATE($B178,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
@@ -4998,11 +5010,11 @@
         <v>303</v>
       </c>
       <c r="C179" t="str">
-        <f>_xlfn.TRANSLATE($B179,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>No hay datos registrados.</v>
       </c>
       <c r="D179" t="str">
-        <f>_xlfn.TRANSLATE($B179,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
@@ -5014,11 +5026,11 @@
         <v>305</v>
       </c>
       <c r="C180" t="str">
-        <f>_xlfn.TRANSLATE($B180,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Letra no disponible</v>
       </c>
       <c r="D180" t="str">
-        <f>_xlfn.TRANSLATE($B180,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Paroles non disponibles</v>
       </c>
     </row>
@@ -5030,11 +5042,11 @@
         <v>307</v>
       </c>
       <c r="C181" t="str">
-        <f>_xlfn.TRANSLATE($B181,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D181" t="str">
-        <f>_xlfn.TRANSLATE($B181,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
@@ -5046,11 +5058,11 @@
         <v>309</v>
       </c>
       <c r="C182" t="str">
-        <f>_xlfn.TRANSLATE($B182,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>No hay repetición</v>
       </c>
       <c r="D182" t="str">
-        <f>_xlfn.TRANSLATE($B182,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Pas de répétition</v>
       </c>
     </row>
@@ -5062,11 +5074,11 @@
         <v>311</v>
       </c>
       <c r="C183" t="str">
-        <f>_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Sin resultados</v>
       </c>
       <c r="D183" t="str">
-        <f>_xlfn.TRANSLATE($B183,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucun résultat</v>
       </c>
     </row>
@@ -5078,11 +5090,11 @@
         <v>313</v>
       </c>
       <c r="C184" t="str">
-        <f>_xlfn.TRANSLATE($B184,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Sin trabajador de servicios</v>
       </c>
       <c r="D184" t="str">
-        <f>_xlfn.TRANSLATE($B184,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucun travailleur de services</v>
       </c>
     </row>
@@ -5094,11 +5106,11 @@
         <v>315</v>
       </c>
       <c r="C185" t="str">
-        <f>_xlfn.TRANSLATE($B185,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D185" t="str">
-        <f>_xlfn.TRANSLATE($B185,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
@@ -5110,11 +5122,11 @@
         <v>317</v>
       </c>
       <c r="C186" t="str">
-        <f>_xlfn.TRANSLATE($B186,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Sin estado</v>
       </c>
       <c r="D186" t="str">
-        <f>_xlfn.TRANSLATE($B186,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucun État</v>
       </c>
     </row>
@@ -5126,11 +5138,11 @@
         <v>319</v>
       </c>
       <c r="C187" t="str">
-        <f>_xlfn.TRANSLATE($B187,$B$2,C$2)</f>
+        <f t="shared" si="8"/>
         <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D187" t="str">
-        <f>_xlfn.TRANSLATE($B187,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
@@ -5142,11 +5154,11 @@
         <v>321</v>
       </c>
       <c r="C188" t="str">
-        <f>_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
+        <f t="shared" ref="C188:C201" si="10">_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
         <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D188" t="str">
-        <f>_xlfn.TRANSLATE($B188,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
@@ -5158,11 +5170,11 @@
         <v>323</v>
       </c>
       <c r="C189" t="str">
-        <f>_xlfn.TRANSLATE($B189,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Noviembre</v>
       </c>
       <c r="D189" t="str">
-        <f>_xlfn.TRANSLATE($B189,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Novembre</v>
       </c>
     </row>
@@ -5174,11 +5186,11 @@
         <v>325</v>
       </c>
       <c r="C190" t="str">
-        <f>_xlfn.TRANSLATE($B190,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Octubre</v>
       </c>
       <c r="D190" t="str">
-        <f>_xlfn.TRANSLATE($B190,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Octobre</v>
       </c>
     </row>
@@ -5190,11 +5202,11 @@
         <v>327</v>
       </c>
       <c r="C191" t="str">
-        <f>_xlfn.TRANSLATE($B191,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Lista abierta</v>
       </c>
       <c r="D191" t="str">
-        <f>_xlfn.TRANSLATE($B191,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Liste ouverte</v>
       </c>
     </row>
@@ -5206,11 +5218,11 @@
         <v>329</v>
       </c>
       <c r="C192" t="str">
-        <f>_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Canción abierta</v>
       </c>
       <c r="D192" t="str">
-        <f>_xlfn.TRANSLATE($B192,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Chanson d’ouverture</v>
       </c>
     </row>
@@ -5222,11 +5234,11 @@
         <v>331</v>
       </c>
       <c r="C193" t="str">
-        <f>_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Partido</v>
       </c>
       <c r="D193" t="str">
-        <f>_xlfn.TRANSLATE($B193,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Parti</v>
       </c>
     </row>
@@ -5238,11 +5250,11 @@
         <v>333</v>
       </c>
       <c r="C194" t="str">
-        <f>_xlfn.TRANSLATE($B194,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Canción de pausa</v>
       </c>
       <c r="D194" t="str">
-        <f>_xlfn.TRANSLATE($B194,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Chanson de pause</v>
       </c>
     </row>
@@ -5254,11 +5266,11 @@
         <v>335</v>
       </c>
       <c r="C195" t="str">
-        <f>_xlfn.TRANSLATE($B195,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Solicitudes pendientes</v>
       </c>
       <c r="D195" t="str">
-        <f>_xlfn.TRANSLATE($B195,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Demandes en attente</v>
       </c>
     </row>
@@ -5270,11 +5282,11 @@
         <v>337</v>
       </c>
       <c r="C196" t="str">
-        <f>_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Pin</v>
       </c>
       <c r="D196" t="str">
-        <f>_xlfn.TRANSLATE($B196,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Épingle</v>
       </c>
     </row>
@@ -5286,11 +5298,11 @@
         <v>339</v>
       </c>
       <c r="C197" t="str">
-        <f>_xlfn.TRANSLATE($B197,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Listas fijadas</v>
       </c>
       <c r="D197" t="str">
-        <f>_xlfn.TRANSLATE($B197,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Listes épinglées</v>
       </c>
     </row>
@@ -5302,11 +5314,11 @@
         <v>341</v>
       </c>
       <c r="C198" t="str">
-        <f>_xlfn.TRANSLATE($B198,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Título del álbum</v>
       </c>
       <c r="D198" t="str">
-        <f>_xlfn.TRANSLATE($B198,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Titre de l’album</v>
       </c>
     </row>
@@ -5318,11 +5330,11 @@
         <v>343</v>
       </c>
       <c r="C199" t="str">
-        <f>_xlfn.TRANSLATE($B199,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Nombre artístico</v>
       </c>
       <c r="D199" t="str">
-        <f>_xlfn.TRANSLATE($B199,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Nom de l’artiste</v>
       </c>
     </row>
@@ -5334,11 +5346,11 @@
         <v>345</v>
       </c>
       <c r="C200" t="str">
-        <f>_xlfn.TRANSLATE($B200,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D200" t="str">
-        <f>_xlfn.TRANSLATE($B200,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Ma playlist parfaite</v>
       </c>
     </row>
@@ -5350,11 +5362,11 @@
         <v>347</v>
       </c>
       <c r="C201" t="str">
-        <f>_xlfn.TRANSLATE($B201,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Título de la canción</v>
       </c>
       <c r="D201" t="str">
-        <f>_xlfn.TRANSLATE($B201,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Titre de la chanson</v>
       </c>
     </row>
@@ -5369,7 +5381,7 @@
         <v>350</v>
       </c>
       <c r="D202" t="str">
-        <f>_xlfn.TRANSLATE($B202,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Jeu</v>
       </c>
     </row>
@@ -5384,7 +5396,7 @@
         <v>353</v>
       </c>
       <c r="D203" t="str">
-        <f>_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Liste des jeux</v>
       </c>
     </row>
@@ -5400,7 +5412,7 @@
         <v>Reproducir medios</v>
       </c>
       <c r="D204" t="str">
-        <f>_xlfn.TRANSLATE($B204,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Lire les médias</v>
       </c>
     </row>
@@ -5415,7 +5427,7 @@
         <v>358</v>
       </c>
       <c r="D205" t="str">
-        <f>_xlfn.TRANSLATE($B205,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>À jouer à venir</v>
       </c>
     </row>
@@ -5430,7 +5442,7 @@
         <v>361</v>
       </c>
       <c r="D206" t="str">
-        <f>_xlfn.TRANSLATE($B206,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Jouer la chanson</v>
       </c>
     </row>
@@ -5442,11 +5454,11 @@
         <v>363</v>
       </c>
       <c r="C207" t="str">
-        <f>_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
+        <f t="shared" ref="C207:C230" si="11">_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
         <v>Listas de reproducción</v>
       </c>
       <c r="D207" t="str">
-        <f>_xlfn.TRANSLATE($B207,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Playlists</v>
       </c>
     </row>
@@ -5458,11 +5470,11 @@
         <v>365</v>
       </c>
       <c r="C208" t="str">
-        <f>_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Medios anteriores</v>
       </c>
       <c r="D208" t="str">
-        <f>_xlfn.TRANSLATE($B208,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Médias précédents</v>
       </c>
     </row>
@@ -5474,11 +5486,11 @@
         <v>367</v>
       </c>
       <c r="C209" t="str">
-        <f>_xlfn.TRANSLATE($B209,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Selecciones rápidas</v>
       </c>
       <c r="D209" t="str">
-        <f>_xlfn.TRANSLATE($B209,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Choix rapides</v>
       </c>
     </row>
@@ -5490,11 +5502,11 @@
         <v>369</v>
       </c>
       <c r="C210" t="str">
-        <f>_xlfn.TRANSLATE($B210,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Radio</v>
       </c>
       <c r="D210" t="str">
-        <f>_xlfn.TRANSLATE($B210,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Radio</v>
       </c>
     </row>
@@ -5506,11 +5518,11 @@
         <v>371</v>
       </c>
       <c r="C211" t="str">
-        <f>_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>No se han encontrado estaciones</v>
       </c>
       <c r="D211" t="str">
-        <f>_xlfn.TRANSLATE($B211,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Aucune station trouvée</v>
       </c>
     </row>
@@ -5522,11 +5534,11 @@
         <v>373</v>
       </c>
       <c r="C212" t="str">
-        <f>_xlfn.TRANSLATE($B212,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D212" t="str">
-        <f>_xlfn.TRANSLATE($B212,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
@@ -5538,11 +5550,11 @@
         <v>375</v>
       </c>
       <c r="C213" t="str">
-        <f>_xlfn.TRANSLATE($B213,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D213" t="str">
-        <f>_xlfn.TRANSLATE($B213,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
@@ -5554,11 +5566,11 @@
         <v>377</v>
       </c>
       <c r="C214" t="str">
-        <f>_xlfn.TRANSLATE($B214,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Emisoras de radio</v>
       </c>
       <c r="D214" t="str">
-        <f>_xlfn.TRANSLATE($B214,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Radio Stations</v>
       </c>
     </row>
@@ -5570,11 +5582,11 @@
         <v>379</v>
       </c>
       <c r="C215" t="str">
-        <f>_xlfn.TRANSLATE($B215,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Mezcla reciente</v>
       </c>
       <c r="D215" t="str">
-        <f>_xlfn.TRANSLATE($B215,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Mix récent</v>
       </c>
     </row>
@@ -5586,11 +5598,11 @@
         <v>381</v>
       </c>
       <c r="C216" t="str">
-        <f>_xlfn.TRANSLATE($B216,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D216" t="str">
-        <f>_xlfn.TRANSLATE($B216,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Joué récemment</v>
       </c>
     </row>
@@ -5602,11 +5614,11 @@
         <v>383</v>
       </c>
       <c r="C217" t="str">
-        <f>_xlfn.TRANSLATE($B217,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D217" t="str">
-        <f>_xlfn.TRANSLATE($B217,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Récemment joué</v>
       </c>
     </row>
@@ -5618,11 +5630,11 @@
         <v>385</v>
       </c>
       <c r="C218" t="str">
-        <f>_xlfn.TRANSLATE($B218,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registro</v>
       </c>
       <c r="D218" t="str">
-        <f>_xlfn.TRANSLATE($B218,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Registre</v>
       </c>
     </row>
@@ -5634,11 +5646,11 @@
         <v>387</v>
       </c>
       <c r="C219" t="str">
-        <f>_xlfn.TRANSLATE($B219,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registrado</v>
       </c>
       <c r="D219" t="str">
-        <f>_xlfn.TRANSLATE($B219,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Enregistré</v>
       </c>
     </row>
@@ -5650,11 +5662,11 @@
         <v>389</v>
       </c>
       <c r="C220" t="str">
-        <f>_xlfn.TRANSLATE($B220,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registrando...</v>
       </c>
       <c r="D220" t="str">
-        <f>_xlfn.TRANSLATE($B220,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Enregistrement...</v>
       </c>
     </row>
@@ -5666,11 +5678,11 @@
         <v>391</v>
       </c>
       <c r="C221" t="str">
-        <f>_xlfn.TRANSLATE($B221,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Artistas relacionados</v>
       </c>
       <c r="D221" t="str">
-        <f>_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Artistes associés</v>
       </c>
     </row>
@@ -5682,11 +5694,11 @@
         <v>393</v>
       </c>
       <c r="C222" t="str">
-        <f>_xlfn.TRANSLATE($B222,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Relajado</v>
       </c>
       <c r="D222" t="str">
-        <f>_xlfn.TRANSLATE($B222,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Détendu</v>
       </c>
     </row>
@@ -5698,11 +5710,11 @@
         <v>505</v>
       </c>
       <c r="C223" t="str">
-        <f>_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Recuérdame</v>
       </c>
       <c r="D223" t="str">
-        <f>_xlfn.TRANSLATE($B223,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Souviens-toi de moi</v>
       </c>
     </row>
@@ -5714,11 +5726,11 @@
         <v>395</v>
       </c>
       <c r="C224" t="str">
-        <f>_xlfn.TRANSLATE($B224,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D224" t="str">
-        <f>_xlfn.TRANSLATE($B224,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de la bibliothèque</v>
       </c>
     </row>
@@ -5730,11 +5742,11 @@
         <v>397</v>
       </c>
       <c r="C225" t="str">
-        <f>_xlfn.TRANSLATE($B225,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Quitar de me gusta</v>
       </c>
       <c r="D225" t="str">
-        <f>_xlfn.TRANSLATE($B225,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de aimé</v>
       </c>
     </row>
@@ -5746,11 +5758,11 @@
         <v>399</v>
       </c>
       <c r="C226" t="str">
-        <f>_xlfn.TRANSLATE($B226,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D226" t="str">
-        <f>_xlfn.TRANSLATE($B226,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Supprimer de la playlist</v>
       </c>
     </row>
@@ -5762,11 +5774,11 @@
         <v>401</v>
       </c>
       <c r="C227" t="str">
-        <f>_xlfn.TRANSLATE($B227,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la cola</v>
       </c>
       <c r="D227" t="str">
-        <f>_xlfn.TRANSLATE($B227,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retirer de la file d’attente</v>
       </c>
     </row>
@@ -5778,11 +5790,11 @@
         <v>403</v>
       </c>
       <c r="C228" t="str">
-        <f>_xlfn.TRANSLATE($B228,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repite todo</v>
       </c>
       <c r="D228" t="str">
-        <f>_xlfn.TRANSLATE($B228,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répétez tout</v>
       </c>
     </row>
@@ -5794,11 +5806,11 @@
         <v>405</v>
       </c>
       <c r="C229" t="str">
-        <f>_xlfn.TRANSLATE($B229,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repite una</v>
       </c>
       <c r="D229" t="str">
-        <f>_xlfn.TRANSLATE($B229,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répétez-en un</v>
       </c>
     </row>
@@ -5810,11 +5822,11 @@
         <v>407</v>
       </c>
       <c r="C230" t="str">
-        <f>_xlfn.TRANSLATE($B230,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repetir nueva contraseña</v>
       </c>
       <c r="D230" t="str">
-        <f>_xlfn.TRANSLATE($B230,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
@@ -5829,7 +5841,7 @@
         <v>410</v>
       </c>
       <c r="D231" t="str">
-        <f>_xlfn.TRANSLATE($B231,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Nouvelle tentative</v>
       </c>
     </row>
@@ -5841,11 +5853,11 @@
         <v>412</v>
       </c>
       <c r="C232" t="str">
-        <f>_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
+        <f t="shared" ref="C232:C277" si="12">_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
         <v>Regreso a casa</v>
       </c>
       <c r="D232" t="str">
-        <f>_xlfn.TRANSLATE($B232,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Retour à la maison</v>
       </c>
     </row>
@@ -5857,11 +5869,11 @@
         <v>414</v>
       </c>
       <c r="C233" t="str">
-        <f>_xlfn.TRANSLATE($B233,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Guardando...</v>
       </c>
       <c r="D233" t="str">
-        <f>_xlfn.TRANSLATE($B233,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Sauver...</v>
       </c>
     </row>
@@ -5873,11 +5885,11 @@
         <v>416</v>
       </c>
       <c r="C234" t="str">
-        <f>_xlfn.TRANSLATE($B234,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Búsqueda</v>
       </c>
       <c r="D234" t="str">
-        <f>_xlfn.TRANSLATE($B234,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Recherche</v>
       </c>
     </row>
@@ -5889,11 +5901,11 @@
         <v>418</v>
       </c>
       <c r="C235" t="str">
-        <f>_xlfn.TRANSLATE($B235,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D235" t="str">
-        <f>_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
@@ -5905,11 +5917,11 @@
         <v>420</v>
       </c>
       <c r="C236" t="str">
-        <f>_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D236" t="str">
-        <f>_xlfn.TRANSLATE($B236,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
@@ -5921,11 +5933,11 @@
         <v>422</v>
       </c>
       <c r="C237" t="str">
-        <f>_xlfn.TRANSLATE($B237,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D237" t="str">
-        <f>_xlfn.TRANSLATE($B237,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
@@ -5937,11 +5949,11 @@
         <v>424</v>
       </c>
       <c r="C238" t="str">
-        <f>_xlfn.TRANSLATE($B238,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Buscar en la biblioteca</v>
       </c>
       <c r="D238" t="str">
-        <f>_xlfn.TRANSLATE($B238,$B$2,D$2)</f>
+        <f t="shared" si="9"/>
         <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
@@ -5953,11 +5965,11 @@
         <v>426</v>
       </c>
       <c r="C239" t="str">
-        <f>_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Usuarios de búsqueda</v>
       </c>
       <c r="D239" t="str">
-        <f>_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
+        <f t="shared" ref="D239:D279" si="13">_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
         <v>Rechercher les utilisateurs</v>
       </c>
     </row>
@@ -5969,11 +5981,11 @@
         <v>428</v>
       </c>
       <c r="C240" t="str">
-        <f>_xlfn.TRANSLATE($B240,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Enviar canción actual</v>
       </c>
       <c r="D240" t="str">
-        <f>_xlfn.TRANSLATE($B240,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
@@ -5985,11 +5997,11 @@
         <v>430</v>
       </c>
       <c r="C241" t="str">
-        <f>_xlfn.TRANSLATE($B241,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Septiembre</v>
       </c>
       <c r="D241" t="str">
-        <f>_xlfn.TRANSLATE($B241,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Septembre</v>
       </c>
     </row>
@@ -6001,11 +6013,11 @@
         <v>64</v>
       </c>
       <c r="C242" t="str">
-        <f>_xlfn.TRANSLATE($B242,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Escenarios</v>
       </c>
       <c r="D242" t="str">
-        <f>_xlfn.TRANSLATE($B242,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Décors</v>
       </c>
     </row>
@@ -6017,11 +6029,11 @@
         <v>433</v>
       </c>
       <c r="C243" t="str">
-        <f>_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Compartir canción</v>
       </c>
       <c r="D243" t="str">
-        <f>_xlfn.TRANSLATE($B243,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Partager la chanson</v>
       </c>
     </row>
@@ -6033,11 +6045,11 @@
         <v>435</v>
       </c>
       <c r="C244" t="str">
-        <f>_xlfn.TRANSLATE($B244,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones compartidas para ti</v>
       </c>
       <c r="D244" t="str">
-        <f>_xlfn.TRANSLATE($B244,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chansons partagées pour vous</v>
       </c>
     </row>
@@ -6049,11 +6061,11 @@
         <v>437</v>
       </c>
       <c r="C245" t="str">
-        <f>_xlfn.TRANSLATE($B245,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Compartido desde</v>
       </c>
       <c r="D245" t="str">
-        <f>_xlfn.TRANSLATE($B245,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Partagé depuis</v>
       </c>
     </row>
@@ -6065,11 +6077,11 @@
         <v>439</v>
       </c>
       <c r="C246" t="str">
-        <f>_xlfn.TRANSLATE($B246,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Mostrando datos de</v>
       </c>
       <c r="D246" t="str">
-        <f>_xlfn.TRANSLATE($B246,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Affichage des données de</v>
       </c>
     </row>
@@ -6081,11 +6093,11 @@
         <v>441</v>
       </c>
       <c r="C247" t="str">
-        <f>_xlfn.TRANSLATE($B247,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canción</v>
       </c>
       <c r="D247" t="str">
-        <f>_xlfn.TRANSLATE($B247,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chanson</v>
       </c>
     </row>
@@ -6097,11 +6109,11 @@
         <v>443</v>
       </c>
       <c r="C248" t="str">
-        <f>_xlfn.TRANSLATE($B248,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones</v>
       </c>
       <c r="D248" t="str">
-        <f>_xlfn.TRANSLATE($B248,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chansons</v>
       </c>
     </row>
@@ -6113,11 +6125,11 @@
         <v>445</v>
       </c>
       <c r="C249" t="str">
-        <f>_xlfn.TRANSLATE($B249,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones Solo para ti</v>
       </c>
       <c r="D249" t="str">
-        <f>_xlfn.TRANSLATE($B249,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chansons juste pour toi</v>
       </c>
     </row>
@@ -6129,11 +6141,11 @@
         <v>447</v>
       </c>
       <c r="C250" t="str">
-        <f>_xlfn.TRANSLATE($B250,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones de</v>
       </c>
       <c r="D250" t="str">
-        <f>_xlfn.TRANSLATE($B250,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chansons de</v>
       </c>
     </row>
@@ -6145,11 +6157,11 @@
         <v>449</v>
       </c>
       <c r="C251" t="str">
-        <f>_xlfn.TRANSLATE($B251,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones escuchadas</v>
       </c>
       <c r="D251" t="str">
-        <f>_xlfn.TRANSLATE($B251,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Chansons écoutées</v>
       </c>
     </row>
@@ -6161,11 +6173,11 @@
         <v>451</v>
       </c>
       <c r="C252" t="str">
-        <f>_xlfn.TRANSLATE($B252,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Empezando...</v>
       </c>
       <c r="D252" t="str">
-        <f>_xlfn.TRANSLATE($B252,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Commencer...</v>
       </c>
     </row>
@@ -6177,11 +6189,11 @@
         <v>453</v>
       </c>
       <c r="C253" t="str">
-        <f>_xlfn.TRANSLATE($B253,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas</v>
       </c>
       <c r="D253" t="str">
-        <f>_xlfn.TRANSLATE($B253,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -6193,11 +6205,11 @@
         <v>455</v>
       </c>
       <c r="C254" t="str">
-        <f>_xlfn.TRANSLATE($B254,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas</v>
       </c>
       <c r="D254" t="str">
-        <f>_xlfn.TRANSLATE($B254,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -6209,11 +6221,11 @@
         <v>457</v>
       </c>
       <c r="C255" t="str">
-        <f>_xlfn.TRANSLATE($B255,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>¡Para</v>
       </c>
       <c r="D255" t="str">
-        <f>_xlfn.TRANSLATE($B255,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Arrête</v>
       </c>
     </row>
@@ -6225,11 +6237,11 @@
         <v>459</v>
       </c>
       <c r="C256" t="str">
-        <f>_xlfn.TRANSLATE($B256,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>a</v>
       </c>
       <c r="D256" t="str">
-        <f>_xlfn.TRANSLATE($B256,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>à</v>
       </c>
     </row>
@@ -6241,11 +6253,11 @@
         <v>461</v>
       </c>
       <c r="C257" t="str">
-        <f>_xlfn.TRANSLATE($B257,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>ToDo</v>
       </c>
       <c r="D257" t="str">
-        <f>_xlfn.TRANSLATE($B257,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>ToDo</v>
       </c>
     </row>
@@ -6257,11 +6269,11 @@
         <v>463</v>
       </c>
       <c r="C258" t="str">
-        <f>_xlfn.TRANSLATE($B258,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D258" t="str">
-        <f>_xlfn.TRANSLATE($B258,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Albums phares</v>
       </c>
     </row>
@@ -6273,11 +6285,11 @@
         <v>465</v>
       </c>
       <c r="C259" t="str">
-        <f>_xlfn.TRANSLATE($B259,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Canciones principales</v>
       </c>
       <c r="D259" t="str">
-        <f>_xlfn.TRANSLATE($B259,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Meilleures chansons</v>
       </c>
     </row>
@@ -6289,11 +6301,11 @@
         <v>467</v>
       </c>
       <c r="C260" t="str">
-        <f>_xlfn.TRANSLATE($B260,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Desclavar</v>
       </c>
       <c r="D260" t="str">
-        <f>_xlfn.TRANSLATE($B260,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Détacher</v>
       </c>
     </row>
@@ -6305,11 +6317,11 @@
         <v>469</v>
       </c>
       <c r="C261" t="str">
-        <f>_xlfn.TRANSLATE($B261,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Desregistrar</v>
       </c>
       <c r="D261" t="str">
-        <f>_xlfn.TRANSLATE($B261,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Désinscription</v>
       </c>
     </row>
@@ -6321,11 +6333,11 @@
         <v>471</v>
       </c>
       <c r="C262" t="str">
-        <f>_xlfn.TRANSLATE($B262,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>No registrado</v>
       </c>
       <c r="D262" t="str">
-        <f>_xlfn.TRANSLATE($B262,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Non enregistré</v>
       </c>
     </row>
@@ -6337,11 +6349,11 @@
         <v>473</v>
       </c>
       <c r="C263" t="str">
-        <f>_xlfn.TRANSLATE($B263,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Dejar de registrarse...</v>
       </c>
       <c r="D263" t="str">
-        <f>_xlfn.TRANSLATE($B263,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Désenregistrement...</v>
       </c>
     </row>
@@ -6353,11 +6365,11 @@
         <v>475</v>
       </c>
       <c r="C264" t="str">
-        <f>_xlfn.TRANSLATE($B264,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Actualización</v>
       </c>
       <c r="D264" t="str">
-        <f>_xlfn.TRANSLATE($B264,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Mise à jour</v>
       </c>
     </row>
@@ -6369,11 +6381,11 @@
         <v>477</v>
       </c>
       <c r="C265" t="str">
-        <f>_xlfn.TRANSLATE($B265,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Actualizando...</v>
       </c>
       <c r="D265" t="str">
-        <f>_xlfn.TRANSLATE($B265,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Mise à jour...</v>
       </c>
     </row>
@@ -6385,11 +6397,11 @@
         <v>479</v>
       </c>
       <c r="C266" t="str">
-        <f>_xlfn.TRANSLATE($B266,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Subida</v>
       </c>
       <c r="D266" t="str">
-        <f>_xlfn.TRANSLATE($B266,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Téléverser</v>
       </c>
     </row>
@@ -6401,11 +6413,11 @@
         <v>481</v>
       </c>
       <c r="C267" t="str">
-        <f>_xlfn.TRANSLATE($B267,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Usuario</v>
       </c>
       <c r="D267" t="str">
-        <f>_xlfn.TRANSLATE($B267,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Utilisateur</v>
       </c>
     </row>
@@ -6417,11 +6429,11 @@
         <v>483</v>
       </c>
       <c r="C268" t="str">
-        <f>_xlfn.TRANSLATE($B268,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Configuración de usuario</v>
       </c>
       <c r="D268" t="str">
-        <f>_xlfn.TRANSLATE($B268,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Paramètres utilisateur</v>
       </c>
     </row>
@@ -6433,11 +6445,11 @@
         <v>485</v>
       </c>
       <c r="C269" t="str">
-        <f>_xlfn.TRANSLATE($B269,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Estadísticas de usuario</v>
       </c>
       <c r="D269" t="str">
-        <f>_xlfn.TRANSLATE($B269,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Statistiques des utilisateurs</v>
       </c>
     </row>
@@ -6449,11 +6461,11 @@
         <v>487</v>
       </c>
       <c r="C270" t="str">
-        <f>_xlfn.TRANSLATE($B270,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Usuarios y amigos</v>
       </c>
       <c r="D270" t="str">
-        <f>_xlfn.TRANSLATE($B270,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Utilisateurs et amis</v>
       </c>
     </row>
@@ -6465,11 +6477,11 @@
         <v>489</v>
       </c>
       <c r="C271" t="str">
-        <f>_xlfn.TRANSLATE($B271,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Lista de usuarios</v>
       </c>
       <c r="D271" t="str">
-        <f>_xlfn.TRANSLATE($B271,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Liste des utilisateurs</v>
       </c>
     </row>
@@ -6481,11 +6493,11 @@
         <v>491</v>
       </c>
       <c r="C272" t="str">
-        <f>_xlfn.TRANSLATE($B272,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Vídeos</v>
       </c>
       <c r="D272" t="str">
-        <f>_xlfn.TRANSLATE($B272,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vidéos</v>
       </c>
     </row>
@@ -6497,11 +6509,11 @@
         <v>493</v>
       </c>
       <c r="C273" t="str">
-        <f>_xlfn.TRANSLATE($B273,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>También puede que te interese</v>
       </c>
       <c r="D273" t="str">
-        <f>_xlfn.TRANSLATE($B273,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Ça pourrait aussi te plaire</v>
       </c>
     </row>
@@ -6513,11 +6525,11 @@
         <v>495</v>
       </c>
       <c r="C274" t="str">
-        <f>_xlfn.TRANSLATE($B274,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Tu</v>
       </c>
       <c r="D274" t="str">
-        <f>_xlfn.TRANSLATE($B274,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Votre</v>
       </c>
     </row>
@@ -6529,11 +6541,11 @@
         <v>497</v>
       </c>
       <c r="C275" t="str">
-        <f>_xlfn.TRANSLATE($B275,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Tus álbumes y listas de reproducción</v>
       </c>
       <c r="D275" t="str">
-        <f>_xlfn.TRANSLATE($B275,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vos albums et playlists</v>
       </c>
     </row>
@@ -6545,11 +6557,11 @@
         <v>499</v>
       </c>
       <c r="C276" t="str">
-        <f>_xlfn.TRANSLATE($B276,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Tu mezcla</v>
       </c>
       <c r="D276" t="str">
-        <f>_xlfn.TRANSLATE($B276,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Votre Mix</v>
       </c>
     </row>
@@ -6561,12 +6573,44 @@
         <v>501</v>
       </c>
       <c r="C277" t="str">
-        <f>_xlfn.TRANSLATE($B277,$B$2,C$2)</f>
+        <f t="shared" si="12"/>
         <v>Vídeos de YouTube</v>
       </c>
       <c r="D277" t="str">
-        <f>_xlfn.TRANSLATE($B277,$B$2,D$2)</f>
+        <f t="shared" si="13"/>
         <v>Vidéos YouTube</v>
+      </c>
+    </row>
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>556</v>
+      </c>
+      <c r="B278" t="s">
+        <v>558</v>
+      </c>
+      <c r="C278" t="str">
+        <f t="shared" ref="C278:C279" si="14">_xlfn.TRANSLATE($B278,$B$2,C$2)</f>
+        <v>Estadísticas del registro de solicitudes</v>
+      </c>
+      <c r="D278" t="str">
+        <f t="shared" si="13"/>
+        <v>Statistiques du journal de requêtes</v>
+      </c>
+    </row>
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>557</v>
+      </c>
+      <c r="B279" t="s">
+        <v>559</v>
+      </c>
+      <c r="C279" t="str">
+        <f t="shared" si="14"/>
+        <v>Métricas y análisis de solicitudes de servidor</v>
+      </c>
+      <c r="D279" t="str">
+        <f t="shared" si="13"/>
+        <v>Métriques et analyses de requêtes serveur</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored player ui layout
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E20F6F7A-590F-449F-B03E-C037EF7F22DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546DE8BE-0A3D-4640-A548-70B7BE1853BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5415" yWindow="3825" windowWidth="16410" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -32,40 +32,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="2">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="569">
   <si>
     <t>KEY</t>
   </si>
@@ -1757,6 +1725,21 @@
   </si>
   <si>
     <t>IP</t>
+  </si>
+  <si>
+    <t>QUEUE</t>
+  </si>
+  <si>
+    <t>Queue</t>
+  </si>
+  <si>
+    <t>NO_MEDIA_PLAYING</t>
+  </si>
+  <si>
+    <t>No media playing</t>
+  </si>
+  <si>
+    <t>No se están reproducion medios</t>
   </si>
 </sst>
 </file>
@@ -1811,73 +1794,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
-  <rv s="0">
-    <v>14</v>
-  </rv>
-  <rv s="1">
-    <v>9</v>
-    <v>16</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
-  <s t="_error">
-    <k n="errorType" t="i"/>
-  </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="subType" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D281" totalsRowShown="0">
-  <autoFilter ref="A2:D281" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D283" totalsRowShown="0">
+  <autoFilter ref="A2:D283" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D281">
     <sortCondition ref="A2:A281"/>
   </sortState>
@@ -2180,7 +2099,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D281"/>
+  <dimension ref="A1:D283"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
@@ -2225,11 +2144,11 @@
         <v>8</v>
       </c>
       <c r="C3" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
+        <f t="shared" ref="C3:D27" si="0">_xlfn.TRANSLATE($B3,$B$2,C$2)</f>
         <v>Añadir lista a la cola de forma aleatoria</v>
       </c>
       <c r="D3" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B3,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente de façon aléatoire</v>
       </c>
     </row>
@@ -2241,11 +2160,11 @@
         <v>10</v>
       </c>
       <c r="C4" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B4,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista al final de la cola</v>
       </c>
       <c r="D4" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B4,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste en bas de la file d’attente</v>
       </c>
     </row>
@@ -2257,11 +2176,11 @@
         <v>12</v>
       </c>
       <c r="C5" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B5,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir lista a la cola</v>
       </c>
       <c r="D5" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B5,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter la liste à la file d’attente</v>
       </c>
     </row>
@@ -2273,11 +2192,11 @@
         <v>14</v>
       </c>
       <c r="C6" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B6,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir medios a la lista de reproducción</v>
       </c>
       <c r="D6" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B6,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter un média à une playlist</v>
       </c>
     </row>
@@ -2289,11 +2208,11 @@
         <v>16</v>
       </c>
       <c r="C7" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B7,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la lista de reproducción</v>
       </c>
       <c r="D7" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B7,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la playlist</v>
       </c>
     </row>
@@ -2305,11 +2224,11 @@
         <v>18</v>
       </c>
       <c r="C8" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B8,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir canción a la cola</v>
       </c>
       <c r="D8" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B8,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une chanson à la file d’attente</v>
       </c>
     </row>
@@ -2321,11 +2240,11 @@
         <v>20</v>
       </c>
       <c r="C9" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B9,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la biblioteca</v>
       </c>
       <c r="D9" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B9,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la bibliothèque</v>
       </c>
     </row>
@@ -2337,11 +2256,11 @@
         <v>22</v>
       </c>
       <c r="C10" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B10,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a los que me gusta</v>
       </c>
       <c r="D10" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B10,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter aux aimés</v>
       </c>
     </row>
@@ -2353,11 +2272,11 @@
         <v>24</v>
       </c>
       <c r="C11" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B11,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir a la cola</v>
       </c>
       <c r="D11" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B11,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter à la file d’attente</v>
       </c>
     </row>
@@ -2369,11 +2288,11 @@
         <v>26</v>
       </c>
       <c r="C12" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B12,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadido a la lista de reproducción</v>
       </c>
       <c r="D12" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B12,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouté à la playlist</v>
       </c>
     </row>
@@ -2385,11 +2304,11 @@
         <v>28</v>
       </c>
       <c r="C13" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B13,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Añadir Build</v>
       </c>
       <c r="D13" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B13,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Ajouter une construction</v>
       </c>
     </row>
@@ -2401,11 +2320,11 @@
         <v>528</v>
       </c>
       <c r="C14" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B14,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Anónimo</v>
       </c>
       <c r="D14" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B14,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Anonyme</v>
       </c>
     </row>
@@ -2417,11 +2336,11 @@
         <v>30</v>
       </c>
       <c r="C15" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B15,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Archivo APK</v>
       </c>
       <c r="D15" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B15,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Fichier APK</v>
       </c>
     </row>
@@ -2433,11 +2352,11 @@
         <v>535</v>
       </c>
       <c r="C16" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B16,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Tiempo medio de respuesta</v>
       </c>
       <c r="D16" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B16,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Temps de réponse moyen</v>
       </c>
     </row>
@@ -2449,11 +2368,11 @@
         <v>552</v>
       </c>
       <c r="C17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Tiempo medio</v>
       </c>
       <c r="D17" t="str">
-        <f>_xlfn.TRANSLATE($B17,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Temps moyen</v>
       </c>
     </row>
@@ -2465,11 +2384,11 @@
         <v>32</v>
       </c>
       <c r="C18" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B18,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Gestiona tus builds de Android</v>
       </c>
       <c r="D18" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B18,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Gérez vos versions Android</v>
       </c>
     </row>
@@ -2481,11 +2400,11 @@
         <v>34</v>
       </c>
       <c r="C19" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B19,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Construcciones</v>
       </c>
       <c r="D19" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B19,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -2497,11 +2416,11 @@
         <v>36</v>
       </c>
       <c r="C20" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B20,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Cancelar</v>
       </c>
       <c r="D20" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B20,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -2513,11 +2432,11 @@
         <v>529</v>
       </c>
       <c r="C21" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B21,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Conde</v>
       </c>
       <c r="D21" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B21,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Comte</v>
       </c>
     </row>
@@ -2529,11 +2448,11 @@
         <v>38</v>
       </c>
       <c r="C22" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B22,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Descripción</v>
       </c>
       <c r="D22" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B22,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Description</v>
       </c>
     </row>
@@ -2545,11 +2464,11 @@
         <v>40</v>
       </c>
       <c r="C23" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B23,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Aquí entra la descripción...</v>
       </c>
       <c r="D23" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B23,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Voici la description...</v>
       </c>
     </row>
@@ -2561,11 +2480,11 @@
         <v>42</v>
       </c>
       <c r="C24" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B24,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Enter Version</v>
       </c>
       <c r="D24" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B24,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Enter Version</v>
       </c>
     </row>
@@ -2577,11 +2496,11 @@
         <v>536</v>
       </c>
       <c r="C25" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B25,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>No se han cargado las estadísticas</v>
       </c>
       <c r="D25" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B25,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Échec de charger les stats</v>
       </c>
     </row>
@@ -2593,11 +2512,11 @@
         <v>537</v>
       </c>
       <c r="C26" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B26,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Actividad horaria</v>
       </c>
       <c r="D26" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B26,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Activité horaire</v>
       </c>
     </row>
@@ -2609,11 +2528,11 @@
         <v>538</v>
       </c>
       <c r="C27" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B27,$B$2,C$2)</f>
+        <f t="shared" si="0"/>
         <v>Métodos HTTP</v>
       </c>
       <c r="D27" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B27,$B$2,D$2)</f>
+        <f t="shared" si="0"/>
         <v>Méthodes HTTP</v>
       </c>
     </row>
@@ -2625,7 +2544,7 @@
         <v>563</v>
       </c>
       <c r="C28" t="str">
-        <f>_xlfn.TRANSLATE($B28,$B$2,C$2)</f>
+        <f t="shared" ref="C28:C49" si="1">_xlfn.TRANSLATE($B28,$B$2,C$2)</f>
         <v>IP</v>
       </c>
       <c r="D28" t="s">
@@ -2640,11 +2559,11 @@
         <v>44</v>
       </c>
       <c r="C29" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B29,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Últimas novedades</v>
       </c>
       <c r="D29" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B29,$B$2,D$2)</f>
+        <f t="shared" ref="D29:D92" si="2">_xlfn.TRANSLATE($B29,$B$2,D$2)</f>
         <v>Dernières nouvelles</v>
       </c>
     </row>
@@ -2656,11 +2575,11 @@
         <v>530</v>
       </c>
       <c r="C30" t="str">
-        <f>_xlfn.TRANSLATE($B30,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Max</v>
       </c>
       <c r="D30" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B30,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Max</v>
       </c>
     </row>
@@ -2672,11 +2591,11 @@
         <v>531</v>
       </c>
       <c r="C31" t="str">
-        <f>_xlfn.TRANSLATE($B31,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Método</v>
       </c>
       <c r="D31" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B31,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Méthode</v>
       </c>
     </row>
@@ -2688,11 +2607,11 @@
         <v>532</v>
       </c>
       <c r="C32" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B32,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Min</v>
       </c>
       <c r="D32" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B32,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Min</v>
       </c>
     </row>
@@ -2704,11 +2623,11 @@
         <v>46</v>
       </c>
       <c r="C33" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B33,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Aún no hay builds</v>
       </c>
       <c r="D33" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B33,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Pas encore de builds</v>
       </c>
     </row>
@@ -2720,12 +2639,12 @@
         <v>539</v>
       </c>
       <c r="C34" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B34,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>No hay deseje de datos</v>
       </c>
-      <c r="D34" t="e" vm="2">
-        <f ca="1">_xlfn.TRANSLATE($B34,$B$2,D$2)</f>
-        <v>#VALUE!</v>
+      <c r="D34" t="str">
+        <f t="shared" si="2"/>
+        <v>Pas de descens de données</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -2736,11 +2655,11 @@
         <v>540</v>
       </c>
       <c r="C35" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B35,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Aún no hay datos</v>
       </c>
       <c r="D35" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B35,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Pas encore de données</v>
       </c>
     </row>
@@ -2752,11 +2671,11 @@
         <v>541</v>
       </c>
       <c r="C36" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B36,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Sin estadísticas</v>
       </c>
       <c r="D36" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B36,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Pas de statistiques</v>
       </c>
     </row>
@@ -2768,11 +2687,11 @@
         <v>48</v>
       </c>
       <c r="C37" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B37,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solo APK</v>
       </c>
       <c r="D37" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B37,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Seul APK</v>
       </c>
     </row>
@@ -2784,11 +2703,11 @@
         <v>50</v>
       </c>
       <c r="C38" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B38,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Opcional</v>
       </c>
       <c r="D38" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B38,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Optionnel</v>
       </c>
     </row>
@@ -2800,11 +2719,11 @@
         <v>542</v>
       </c>
       <c r="C39" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B39,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>P50 - P90</v>
       </c>
       <c r="D39" t="str">
-        <f>_xlfn.TRANSLATE($B39,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>P50 - P90</v>
       </c>
     </row>
@@ -2816,11 +2735,11 @@
         <v>543</v>
       </c>
       <c r="C40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Latencia P95</v>
       </c>
       <c r="D40" t="str">
-        <f>_xlfn.TRANSLATE($B40,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Latence P95</v>
       </c>
     </row>
@@ -2832,11 +2751,11 @@
         <v>533</v>
       </c>
       <c r="C41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>P99</v>
       </c>
       <c r="D41" t="str">
-        <f>_xlfn.TRANSLATE($B41,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>P99</v>
       </c>
     </row>
@@ -2848,11 +2767,11 @@
         <v>52</v>
       </c>
       <c r="C42" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B42,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Leer Fallido</v>
       </c>
       <c r="D42" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B42,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Lire Échec</v>
       </c>
     </row>
@@ -2864,11 +2783,11 @@
         <v>544</v>
       </c>
       <c r="C43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes por día</v>
       </c>
       <c r="D43" t="str">
-        <f>_xlfn.TRANSLATE($B43,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Demandes par jour</v>
       </c>
     </row>
@@ -2880,11 +2799,11 @@
         <v>559</v>
       </c>
       <c r="C44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Métricas y análisis de solicitudes de servidor</v>
       </c>
       <c r="D44" t="str">
-        <f>_xlfn.TRANSLATE($B44,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Métriques et analyses de requêtes serveur</v>
       </c>
     </row>
@@ -2896,11 +2815,11 @@
         <v>558</v>
       </c>
       <c r="C45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Estadísticas del registro de solicitudes</v>
       </c>
       <c r="D45" t="str">
-        <f>_xlfn.TRANSLATE($B45,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Statistiques du journal de requêtes</v>
       </c>
     </row>
@@ -2912,11 +2831,11 @@
         <v>534</v>
       </c>
       <c r="C46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes</v>
       </c>
       <c r="D46" t="str">
-        <f>_xlfn.TRANSLATE($B46,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Demandes</v>
       </c>
     </row>
@@ -2928,11 +2847,11 @@
         <v>545</v>
       </c>
       <c r="C47" t="str">
-        <f>_xlfn.TRANSLATE($B47,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Solicitudes a lo largo del tiempo</v>
       </c>
       <c r="D47" t="str">
-        <f>_xlfn.TRANSLATE($B47,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Demandes au fil du temps</v>
       </c>
     </row>
@@ -2944,11 +2863,11 @@
         <v>54</v>
       </c>
       <c r="C48" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B48,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Obligatorio</v>
       </c>
       <c r="D48" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B48,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Obligatoire</v>
       </c>
     </row>
@@ -2960,11 +2879,11 @@
         <v>553</v>
       </c>
       <c r="C49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,C$2)</f>
+        <f t="shared" si="1"/>
         <v>Códigos de respuesta</v>
       </c>
       <c r="D49" t="str">
-        <f>_xlfn.TRANSLATE($B49,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Codes de réponse</v>
       </c>
     </row>
@@ -2979,7 +2898,7 @@
         <v>555</v>
       </c>
       <c r="D50" t="str">
-        <f>_xlfn.TRANSLATE($B50,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Itinéraire</v>
       </c>
     </row>
@@ -2991,11 +2910,11 @@
         <v>56</v>
       </c>
       <c r="C51" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B51,$B$2,C$2)</f>
+        <f t="shared" ref="C51:C82" si="3">_xlfn.TRANSLATE($B51,$B$2,C$2)</f>
         <v>Seleccionar APK</v>
       </c>
       <c r="D51" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B51,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sélectionner APK</v>
       </c>
     </row>
@@ -3007,11 +2926,11 @@
         <v>58</v>
       </c>
       <c r="C52" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B52,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Seleccionados</v>
       </c>
       <c r="D52" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B52,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sélectionné</v>
       </c>
     </row>
@@ -3023,11 +2942,11 @@
         <v>60</v>
       </c>
       <c r="C53" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B53,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Próximamente</v>
       </c>
       <c r="D53" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B53,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -3039,11 +2958,11 @@
         <v>62</v>
       </c>
       <c r="C54" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B54,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Configuración de plataformas</v>
       </c>
       <c r="D54" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B54,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Réglages de la plateforme</v>
       </c>
     </row>
@@ -3055,11 +2974,11 @@
         <v>64</v>
       </c>
       <c r="C55" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B55,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Escenarios</v>
       </c>
       <c r="D55" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B55,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Décors</v>
       </c>
     </row>
@@ -3071,11 +2990,11 @@
         <v>34</v>
       </c>
       <c r="C56" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B56,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Construcciones</v>
       </c>
       <c r="D56" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B56,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Constructions</v>
       </c>
     </row>
@@ -3087,11 +3006,11 @@
         <v>64</v>
       </c>
       <c r="C57" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B57,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Escenarios</v>
       </c>
       <c r="D57" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B57,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Décors</v>
       </c>
     </row>
@@ -3103,11 +3022,11 @@
         <v>68</v>
       </c>
       <c r="C58" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B58,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuarios</v>
       </c>
       <c r="D58" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B58,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -3119,11 +3038,11 @@
         <v>562</v>
       </c>
       <c r="C59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Principales IPs</v>
       </c>
       <c r="D59" t="str">
-        <f>_xlfn.TRANSLATE($B59,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Meilleures IPS</v>
       </c>
     </row>
@@ -3135,11 +3054,11 @@
         <v>546</v>
       </c>
       <c r="C60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Rutas principales</v>
       </c>
       <c r="D60" t="str">
-        <f>_xlfn.TRANSLATE($B60,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Itinéraires principaux</v>
       </c>
     </row>
@@ -3151,11 +3070,11 @@
         <v>547</v>
       </c>
       <c r="C61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Solicitudes totales</v>
       </c>
       <c r="D61" t="str">
-        <f>_xlfn.TRANSLATE($B61,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Nombre total de demandes</v>
       </c>
     </row>
@@ -3167,11 +3086,11 @@
         <v>70</v>
       </c>
       <c r="C62" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B62,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Compilación de subida</v>
       </c>
       <c r="D62" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B62,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Upload Build</v>
       </c>
     </row>
@@ -3183,11 +3102,11 @@
         <v>72</v>
       </c>
       <c r="C63" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B63,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Fallido en la subida</v>
       </c>
       <c r="D63" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B63,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement échoué</v>
       </c>
     </row>
@@ -3199,11 +3118,11 @@
         <v>74</v>
       </c>
       <c r="C64" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B64,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Sube tu primera construcción</v>
       </c>
       <c r="D64" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B64,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargez votre première compilation</v>
       </c>
     </row>
@@ -3215,11 +3134,11 @@
         <v>76</v>
       </c>
       <c r="C65" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B65,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Subir nueva versión</v>
       </c>
       <c r="D65" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B65,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Télécharger une nouvelle version</v>
       </c>
     </row>
@@ -3231,11 +3150,11 @@
         <v>78</v>
       </c>
       <c r="C66" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B66,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Éxito en la subida</v>
       </c>
       <c r="D66" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B66,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Succès de la télévision</v>
       </c>
     </row>
@@ -3247,11 +3166,11 @@
         <v>80</v>
       </c>
       <c r="C67" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B67,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Subiendo algo...</v>
       </c>
       <c r="D67" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B67,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargement...</v>
       </c>
     </row>
@@ -3263,11 +3182,11 @@
         <v>481</v>
       </c>
       <c r="C68" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B68,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuario</v>
       </c>
       <c r="D68" t="str">
-        <f>_xlfn.TRANSLATE($B68,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateur</v>
       </c>
     </row>
@@ -3279,11 +3198,11 @@
         <v>548</v>
       </c>
       <c r="C69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Actividad de usuario</v>
       </c>
       <c r="D69" t="str">
-        <f>_xlfn.TRANSLATE($B69,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Activité des utilisateurs</v>
       </c>
     </row>
@@ -3295,11 +3214,11 @@
         <v>60</v>
       </c>
       <c r="C70" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B70,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Próximamente</v>
       </c>
       <c r="D70" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B70,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Bientôt</v>
       </c>
     </row>
@@ -3311,11 +3230,11 @@
         <v>83</v>
       </c>
       <c r="C71" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B71,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Gestionar los usuarios de la plataforma</v>
       </c>
       <c r="D71" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B71,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Gérer les utilisateurs de la plateforme</v>
       </c>
     </row>
@@ -3327,11 +3246,11 @@
         <v>68</v>
       </c>
       <c r="C72" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B72,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Usuarios</v>
       </c>
       <c r="D72" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B72,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Utilisateurs</v>
       </c>
     </row>
@@ -3343,11 +3262,11 @@
         <v>86</v>
       </c>
       <c r="C73" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B73,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Versión</v>
       </c>
       <c r="D73" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B73,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Version</v>
       </c>
     </row>
@@ -3359,11 +3278,11 @@
         <v>88</v>
       </c>
       <c r="C74" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B74,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbum</v>
       </c>
       <c r="D74" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B74,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Album</v>
       </c>
     </row>
@@ -3375,11 +3294,11 @@
         <v>90</v>
       </c>
       <c r="C75" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B75,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbumes</v>
       </c>
       <c r="D75" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B75,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums</v>
       </c>
     </row>
@@ -3391,11 +3310,11 @@
         <v>92</v>
       </c>
       <c r="C76" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B76,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Álbumes y sencillos</v>
       </c>
       <c r="D76" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B76,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Albums et singles</v>
       </c>
     </row>
@@ -3407,11 +3326,11 @@
         <v>94</v>
       </c>
       <c r="C77" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B77,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Todos</v>
       </c>
       <c r="D77" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B77,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Tous</v>
       </c>
     </row>
@@ -3423,11 +3342,11 @@
         <v>96</v>
       </c>
       <c r="C78" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B78,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Abril</v>
       </c>
       <c r="D78" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B78,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Avril</v>
       </c>
     </row>
@@ -3439,11 +3358,11 @@
         <v>98</v>
       </c>
       <c r="C79" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B79,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Artista</v>
       </c>
       <c r="D79" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B79,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artiste</v>
       </c>
     </row>
@@ -3455,11 +3374,11 @@
         <v>100</v>
       </c>
       <c r="C80" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B80,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Artistas</v>
       </c>
       <c r="D80" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B80,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Artistes</v>
       </c>
     </row>
@@ -3471,11 +3390,11 @@
         <v>102</v>
       </c>
       <c r="C81" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B81,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Agosto</v>
       </c>
       <c r="D81" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B81,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Août</v>
       </c>
     </row>
@@ -3487,11 +3406,11 @@
         <v>104</v>
       </c>
       <c r="C82" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B82,$B$2,C$2)</f>
+        <f t="shared" si="3"/>
         <v>Minutos medios por canción</v>
       </c>
       <c r="D82" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B82,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Minutes moyennes par chanson</v>
       </c>
     </row>
@@ -3503,11 +3422,11 @@
         <v>106</v>
       </c>
       <c r="C83" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
+        <f t="shared" ref="C83:C102" si="4">_xlfn.TRANSLATE($B83,$B$2,C$2)</f>
         <v>por</v>
       </c>
       <c r="D83" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B83,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>par</v>
       </c>
     </row>
@@ -3519,11 +3438,11 @@
         <v>36</v>
       </c>
       <c r="C84" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B84,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Cancelar</v>
       </c>
       <c r="D84" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B84,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Annuler</v>
       </c>
     </row>
@@ -3535,11 +3454,11 @@
         <v>109</v>
       </c>
       <c r="C85" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B85,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Cambiar contraseña</v>
       </c>
       <c r="D85" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B85,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Changer le mot de passe</v>
       </c>
     </row>
@@ -3551,11 +3470,11 @@
         <v>111</v>
       </c>
       <c r="C86" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B86,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descargas claras</v>
       </c>
       <c r="D86" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B86,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Téléchargements clairs</v>
       </c>
     </row>
@@ -3567,11 +3486,11 @@
         <v>113</v>
       </c>
       <c r="C87" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B87,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Haz clic para descargar</v>
       </c>
       <c r="D87" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B87,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Cliquez pour télécharger</v>
       </c>
     </row>
@@ -3583,11 +3502,11 @@
         <v>115</v>
       </c>
       <c r="C88" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B88,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Topo comunitario</v>
       </c>
       <c r="D88" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B88,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Sommet communautaire</v>
       </c>
     </row>
@@ -3599,11 +3518,11 @@
         <v>117</v>
       </c>
       <c r="C89" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B89,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Completado</v>
       </c>
       <c r="D89" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B89,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Achèvement</v>
       </c>
     </row>
@@ -3615,11 +3534,11 @@
         <v>119</v>
       </c>
       <c r="C90" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B90,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>URL de la lista de copiar</v>
       </c>
       <c r="D90" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B90,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>URL de la liste de copie</v>
       </c>
     </row>
@@ -3631,11 +3550,11 @@
         <v>121</v>
       </c>
       <c r="C91" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B91,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Copiar la URL de la canción</v>
       </c>
       <c r="D91" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B91,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Copier l’URL de la chanson</v>
       </c>
     </row>
@@ -3647,11 +3566,11 @@
         <v>123</v>
       </c>
       <c r="C92" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B92,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Crear</v>
       </c>
       <c r="D92" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B92,$B$2,D$2)</f>
+        <f t="shared" si="2"/>
         <v>Créer</v>
       </c>
     </row>
@@ -3663,11 +3582,11 @@
         <v>125</v>
       </c>
       <c r="C93" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B93,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Crear...</v>
       </c>
       <c r="D93" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B93,$B$2,D$2)</f>
+        <f t="shared" ref="D93:D156" si="5">_xlfn.TRANSLATE($B93,$B$2,D$2)</f>
         <v>Créer...</v>
       </c>
     </row>
@@ -3679,11 +3598,11 @@
         <v>127</v>
       </c>
       <c r="C94" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B94,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Fecha añadida</v>
       </c>
       <c r="D94" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B94,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Date ajoutée</v>
       </c>
     </row>
@@ -3695,11 +3614,11 @@
         <v>129</v>
       </c>
       <c r="C95" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B95,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Diciembre</v>
       </c>
       <c r="D95" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B95,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Décembre</v>
       </c>
     </row>
@@ -3711,11 +3630,11 @@
         <v>131</v>
       </c>
       <c r="C96" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B96,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Tu dispositivo no soporta al trabajador de servicio</v>
       </c>
       <c r="D96" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B96,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Votre appareil ne prend pas en charge l’assistant de service</v>
       </c>
     </row>
@@ -3727,11 +3646,11 @@
         <v>133</v>
       </c>
       <c r="C97" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B97,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Disco</v>
       </c>
       <c r="D97" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B97,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Disque</v>
       </c>
     </row>
@@ -3743,11 +3662,11 @@
         <v>135</v>
       </c>
       <c r="C98" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B98,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Nombre de Muestra</v>
       </c>
       <c r="D98" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B98,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Nom d’affichage</v>
       </c>
     </row>
@@ -3759,11 +3678,11 @@
         <v>137</v>
       </c>
       <c r="C99" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B99,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descargar</v>
       </c>
       <c r="D99" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B99,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Télécharger</v>
       </c>
     </row>
@@ -3775,11 +3694,11 @@
         <v>139</v>
       </c>
       <c r="C100" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B100,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Descarga la app para escuchar offline</v>
       </c>
       <c r="D100" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B100,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Téléchargez l’application pour une écoute hors ligne</v>
       </c>
     </row>
@@ -3791,11 +3710,11 @@
         <v>141</v>
       </c>
       <c r="C101" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B101,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Introduce una URL de Spotify o YouTube Music</v>
       </c>
       <c r="D101" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B101,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Saisissez une URL Spotify ou YouTube Music</v>
       </c>
     </row>
@@ -3807,11 +3726,11 @@
         <v>143</v>
       </c>
       <c r="C102" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B102,$B$2,C$2)</f>
+        <f t="shared" si="4"/>
         <v>Lista de descargas al dispositivo</v>
       </c>
       <c r="D102" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B102,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Liste de téléchargement vers l’appareil</v>
       </c>
     </row>
@@ -3826,7 +3745,7 @@
         <v>146</v>
       </c>
       <c r="D103" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B103,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Liste de téléchargement vers serveur</v>
       </c>
     </row>
@@ -3838,11 +3757,11 @@
         <v>148</v>
       </c>
       <c r="C104" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B104,$B$2,C$2)</f>
+        <f t="shared" ref="C104:C126" si="6">_xlfn.TRANSLATE($B104,$B$2,C$2)</f>
         <v>Descargar medios al dispositivo</v>
       </c>
       <c r="D104" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B104,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Télécharger des médias sur l’appareil</v>
       </c>
     </row>
@@ -3854,11 +3773,11 @@
         <v>150</v>
       </c>
       <c r="C105" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B105,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descargar mp</v>
       </c>
       <c r="D105" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B105,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Télécharger le MP</v>
       </c>
     </row>
@@ -3870,11 +3789,11 @@
         <v>152</v>
       </c>
       <c r="C106" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B106,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descargar canción al dispositivo</v>
       </c>
       <c r="D106" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B106,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Télécharger la chanson sur l’appareil</v>
       </c>
     </row>
@@ -3886,11 +3805,11 @@
         <v>154</v>
       </c>
       <c r="C107" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B107,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descarga iniciada</v>
       </c>
       <c r="D107" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B107,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Téléchargement lancé</v>
       </c>
     </row>
@@ -3902,11 +3821,11 @@
         <v>156</v>
       </c>
       <c r="C108" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B108,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descargar ZIP</v>
       </c>
       <c r="D108" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B108,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Télécharger ZIP</v>
       </c>
     </row>
@@ -3918,11 +3837,11 @@
         <v>158</v>
       </c>
       <c r="C109" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B109,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descargando</v>
       </c>
       <c r="D109" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B109,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Téléchargement</v>
       </c>
     </row>
@@ -3934,11 +3853,11 @@
         <v>160</v>
       </c>
       <c r="C110" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B110,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Descargas</v>
       </c>
       <c r="D110" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B110,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Téléchargements</v>
       </c>
     </row>
@@ -3950,11 +3869,11 @@
         <v>162</v>
       </c>
       <c r="C111" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B111,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Duración</v>
       </c>
       <c r="D111" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B111,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Durée</v>
       </c>
     </row>
@@ -3966,11 +3885,11 @@
         <v>164</v>
       </c>
       <c r="C112" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B112,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Energía</v>
       </c>
       <c r="D112" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B112,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Énergie</v>
       </c>
     </row>
@@ -3982,11 +3901,11 @@
         <v>166</v>
       </c>
       <c r="C113" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B113,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D113" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B113,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -3998,11 +3917,11 @@
         <v>168</v>
       </c>
       <c r="C114" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B114,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error</v>
       </c>
       <c r="D114" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B114,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur</v>
       </c>
     </row>
@@ -4014,11 +3933,11 @@
         <v>170</v>
       </c>
       <c r="C115" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B115,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Lenguaje de cambio de error</v>
       </c>
       <c r="D115" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B115,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Langage de changement d’erreur</v>
       </c>
     </row>
@@ -4030,11 +3949,11 @@
         <v>172</v>
       </c>
       <c r="C116" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B116,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D116" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B116,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -4046,11 +3965,11 @@
         <v>172</v>
       </c>
       <c r="C117" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B117,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al crear tu nueva lista de reproducción</v>
       </c>
       <c r="D117" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B117,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur lors de la création de votre nouvelle playlist</v>
       </c>
     </row>
@@ -4062,11 +3981,11 @@
         <v>166</v>
       </c>
       <c r="C118" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B118,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Introduce un nombre para tu nueva lista de reproducción</v>
       </c>
       <c r="D118" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B118,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Saisissez un nom pour votre nouvelle playlist</v>
       </c>
     </row>
@@ -4078,11 +3997,11 @@
         <v>176</v>
       </c>
       <c r="C119" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B119,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al obtener descargas</v>
       </c>
       <c r="D119" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B119,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur de téléchargement</v>
       </c>
     </row>
@@ -4094,11 +4013,11 @@
         <v>178</v>
       </c>
       <c r="C120" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B120,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al obtener medios</v>
       </c>
       <c r="D120" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B120,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur d’obtention de médias</v>
       </c>
     </row>
@@ -4110,11 +4029,11 @@
         <v>180</v>
       </c>
       <c r="C121" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B121,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Cola de obtención de errores</v>
       </c>
       <c r="D121" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B121,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>File d’attente d’obtention d’erreurs</v>
       </c>
     </row>
@@ -4126,11 +4045,11 @@
         <v>182</v>
       </c>
       <c r="C122" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B122,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Usuario que obtiene errores</v>
       </c>
       <c r="D122" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B122,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Utilisateur d’obtention d’erreurs</v>
       </c>
     </row>
@@ -4142,11 +4061,11 @@
         <v>184</v>
       </c>
       <c r="C123" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B123,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al dar like a medios</v>
       </c>
       <c r="D123" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B123,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur d’appréciation des médias</v>
       </c>
     </row>
@@ -4158,11 +4077,11 @@
         <v>186</v>
       </c>
       <c r="C124" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B124,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Búsqueda de errores</v>
       </c>
       <c r="D124" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B124,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Recherche d’erreurs</v>
       </c>
     </row>
@@ -4174,11 +4093,11 @@
         <v>188</v>
       </c>
       <c r="C125" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B125,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al iniciar la descarga</v>
       </c>
       <c r="D125" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B125,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur au démarrage du téléchargement</v>
       </c>
     </row>
@@ -4190,11 +4109,11 @@
         <v>190</v>
       </c>
       <c r="C126" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B126,$B$2,C$2)</f>
+        <f t="shared" si="6"/>
         <v>Error al dejar de dar like a los medios</v>
       </c>
       <c r="D126" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B126,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Erreur de non-like des médias</v>
       </c>
     </row>
@@ -4209,7 +4128,7 @@
         <v>193</v>
       </c>
       <c r="D127" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec</v>
       </c>
     </row>
@@ -4221,11 +4140,11 @@
         <v>195</v>
       </c>
       <c r="C128" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B128,$B$2,C$2)</f>
+        <f t="shared" ref="C128:C159" si="7">_xlfn.TRANSLATE($B128,$B$2,C$2)</f>
         <v>No se añadió contenido a la biblioteca</v>
       </c>
       <c r="D128" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B128,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec d’ajouter des médias à la bibliothèque</v>
       </c>
     </row>
@@ -4237,11 +4156,11 @@
         <v>197</v>
       </c>
       <c r="C129" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B129,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No se añadió contenido a la lista de reproducción</v>
       </c>
       <c r="D129" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B129,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec d’ajouter des médias à la playlist</v>
       </c>
     </row>
@@ -4253,11 +4172,11 @@
         <v>199</v>
       </c>
       <c r="C130" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B130,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No cambiaron el idioma</v>
       </c>
       <c r="D130" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B130,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec de changer de langue</v>
       </c>
     </row>
@@ -4269,11 +4188,11 @@
         <v>201</v>
       </c>
       <c r="C131" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B131,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>No se han conseguido las listas de reproducción</v>
       </c>
       <c r="D131" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B131,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec à récupérer les playlists</v>
       </c>
     </row>
@@ -4285,11 +4204,11 @@
         <v>203</v>
       </c>
       <c r="C132" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B132,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D132" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B132,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Albums en vedette</v>
       </c>
     </row>
@@ -4301,11 +4220,11 @@
         <v>205</v>
       </c>
       <c r="C133" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B133,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Listas destacadas</v>
       </c>
       <c r="D133" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B133,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Listes en vedette</v>
       </c>
     </row>
@@ -4317,11 +4236,11 @@
         <v>207</v>
       </c>
       <c r="C134" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B134,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Febrero</v>
       </c>
       <c r="D134" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B134,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Février</v>
       </c>
     </row>
@@ -4333,11 +4252,11 @@
         <v>209</v>
       </c>
       <c r="C135" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B135,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Enfoque</v>
       </c>
       <c r="D135" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B135,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Focus</v>
       </c>
     </row>
@@ -4349,11 +4268,11 @@
         <v>211</v>
       </c>
       <c r="C136" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B136,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Amigos</v>
       </c>
       <c r="D136" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B136,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Amis</v>
       </c>
     </row>
@@ -4365,11 +4284,11 @@
         <v>213</v>
       </c>
       <c r="C137" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B137,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Lista de amigos</v>
       </c>
       <c r="D137" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B137,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Liste d’amis</v>
       </c>
     </row>
@@ -4381,11 +4300,11 @@
         <v>215</v>
       </c>
       <c r="C138" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B138,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Gana puntos escuchando música, compartiendo canciones, disfrutando de la música con amigos o añadiendo nuevos amigos. ¡Sigue y sube de nivel!</v>
       </c>
       <c r="D138" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B138,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Gagnez des points en écoutant de la musique, en partageant des chansons, en appréciant de la musique avec des amis ou en ajoutant de nouveaux amis. Continue et monte de niveau !</v>
       </c>
     </row>
@@ -4397,11 +4316,11 @@
         <v>217</v>
       </c>
       <c r="C139" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B139,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Estadísticas de Friends</v>
       </c>
       <c r="D139" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B139,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Statistiques de Friends</v>
       </c>
     </row>
@@ -4413,11 +4332,11 @@
         <v>219</v>
       </c>
       <c r="C140" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B140,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>General</v>
       </c>
       <c r="D140" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B140,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Généralités</v>
       </c>
     </row>
@@ -4429,11 +4348,11 @@
         <v>221</v>
       </c>
       <c r="C141" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B141,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Estadísticas generales</v>
       </c>
       <c r="D141" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Statistiques générales</v>
       </c>
     </row>
@@ -4445,11 +4364,11 @@
         <v>223</v>
       </c>
       <c r="C142" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B142,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Obtén información</v>
       </c>
       <c r="D142" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B142,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Obtenez des infos</v>
       </c>
     </row>
@@ -4461,11 +4380,11 @@
         <v>225</v>
       </c>
       <c r="C143" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B143,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Obteniendo información</v>
       </c>
       <c r="D143" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B143,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Obtenir des infos</v>
       </c>
     </row>
@@ -4477,11 +4396,11 @@
         <v>227</v>
       </c>
       <c r="C144" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B144,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Ir al álbum</v>
       </c>
       <c r="D144" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B144,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Aller à l’album</v>
       </c>
     </row>
@@ -4493,11 +4412,11 @@
         <v>229</v>
       </c>
       <c r="C145" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B145,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Ir a artista</v>
       </c>
       <c r="D145" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B145,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Aller à l’artiste</v>
       </c>
     </row>
@@ -4509,11 +4428,11 @@
         <v>231</v>
       </c>
       <c r="C146" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B146,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Joyas ocultas que olvidaste</v>
       </c>
       <c r="D146" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B146,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Des perles cachées que tu as oubliées</v>
       </c>
     </row>
@@ -4525,11 +4444,11 @@
         <v>233</v>
       </c>
       <c r="C147" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B147,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Inicio</v>
       </c>
       <c r="D147" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B147,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Accueil</v>
       </c>
     </row>
@@ -4541,11 +4460,11 @@
         <v>235</v>
       </c>
       <c r="C148" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B148,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Enero</v>
       </c>
       <c r="D148" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B148,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Janvier</v>
       </c>
     </row>
@@ -4557,11 +4476,11 @@
         <v>237</v>
       </c>
       <c r="C149" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B149,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Julio</v>
       </c>
       <c r="D149" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B149,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Juillet</v>
       </c>
     </row>
@@ -4573,11 +4492,11 @@
         <v>239</v>
       </c>
       <c r="C150" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B150,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Junio</v>
       </c>
       <c r="D150" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B150,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Juin</v>
       </c>
     </row>
@@ -4589,11 +4508,11 @@
         <v>241</v>
       </c>
       <c r="C151" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B151,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Idioma</v>
       </c>
       <c r="D151" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B151,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Langue</v>
       </c>
     </row>
@@ -4605,11 +4524,11 @@
         <v>243</v>
       </c>
       <c r="C152" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B152,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>El cambio de idioma fracasó</v>
       </c>
       <c r="D152" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B152,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Échec du changement linguistique</v>
       </c>
     </row>
@@ -4621,11 +4540,11 @@
         <v>245</v>
       </c>
       <c r="C153" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B153,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Cambio de idioma</v>
       </c>
       <c r="D153" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B153,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Changement de langue</v>
       </c>
     </row>
@@ -4637,11 +4556,11 @@
         <v>247</v>
       </c>
       <c r="C154" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B154,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Últimas descargas</v>
       </c>
       <c r="D154" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B154,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Derniers téléchargements</v>
       </c>
     </row>
@@ -4653,11 +4572,11 @@
         <v>249</v>
       </c>
       <c r="C155" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B155,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Nivel</v>
       </c>
       <c r="D155" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B155,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Niveau</v>
       </c>
     </row>
@@ -4669,11 +4588,11 @@
         <v>251</v>
       </c>
       <c r="C156" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B156,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Biblioteca</v>
       </c>
       <c r="D156" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B156,$B$2,D$2)</f>
+        <f t="shared" si="5"/>
         <v>Bibliothèque</v>
       </c>
     </row>
@@ -4685,11 +4604,11 @@
         <v>253</v>
       </c>
       <c r="C157" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B157,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Como</v>
       </c>
       <c r="D157" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B157,$B$2,D$2)</f>
+        <f t="shared" ref="D157:D220" si="8">_xlfn.TRANSLATE($B157,$B$2,D$2)</f>
         <v>Comme</v>
       </c>
     </row>
@@ -4701,11 +4620,11 @@
         <v>255</v>
       </c>
       <c r="C158" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B158,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Canciones que me gustaban</v>
       </c>
       <c r="D158" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B158,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chansons appréciées</v>
       </c>
     </row>
@@ -4717,11 +4636,11 @@
         <v>257</v>
       </c>
       <c r="C159" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B159,$B$2,C$2)</f>
+        <f t="shared" si="7"/>
         <v>Cerrar sesión</v>
       </c>
       <c r="D159" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B159,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Déconnexion</v>
       </c>
     </row>
@@ -4733,11 +4652,11 @@
         <v>259</v>
       </c>
       <c r="C160" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B160,$B$2,C$2)</f>
+        <f t="shared" ref="C160:C191" si="9">_xlfn.TRANSLATE($B160,$B$2,C$2)</f>
         <v>Letra</v>
       </c>
       <c r="D160" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B160,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Paroles</v>
       </c>
     </row>
@@ -4749,11 +4668,11 @@
         <v>261</v>
       </c>
       <c r="C161" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B161,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Marzo</v>
       </c>
       <c r="D161" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B161,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Mars</v>
       </c>
     </row>
@@ -4765,11 +4684,11 @@
         <v>263</v>
       </c>
       <c r="C162" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B162,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Mayo</v>
       </c>
       <c r="D162" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B162,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Mai</v>
       </c>
     </row>
@@ -4781,11 +4700,11 @@
         <v>265</v>
       </c>
       <c r="C163" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B163,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D163" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B163,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
@@ -4797,11 +4716,11 @@
         <v>503</v>
       </c>
       <c r="C164" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B164,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>A los medios les gustó</v>
       </c>
       <c r="D164" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B164,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Les médias appréciaient</v>
       </c>
     </row>
@@ -4813,11 +4732,11 @@
         <v>267</v>
       </c>
       <c r="C165" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B165,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Progreso de los medios</v>
       </c>
       <c r="D165" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B165,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Progrès des médias</v>
       </c>
     </row>
@@ -4829,11 +4748,11 @@
         <v>269</v>
       </c>
       <c r="C166" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B166,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Actas</v>
       </c>
       <c r="D166" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B166,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Procès-verbal</v>
       </c>
     </row>
@@ -4845,11 +4764,11 @@
         <v>271</v>
       </c>
       <c r="C167" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B167,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Minutos escuchados</v>
       </c>
       <c r="D167" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B167,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Minutes écoutées</v>
       </c>
     </row>
@@ -4861,11 +4780,11 @@
         <v>273</v>
       </c>
       <c r="C168" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B168,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Minutos escuchados por día</v>
       </c>
       <c r="D168" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B168,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Minutes écoutées par jour</v>
       </c>
     </row>
@@ -4877,11 +4796,11 @@
         <v>275</v>
       </c>
       <c r="C169" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B169,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D169" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B169,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
@@ -4893,11 +4812,11 @@
         <v>277</v>
       </c>
       <c r="C170" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B170,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Más opciones</v>
       </c>
       <c r="D170" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B170,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Plus d’options</v>
       </c>
     </row>
@@ -4909,11 +4828,11 @@
         <v>279</v>
       </c>
       <c r="C171" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B171,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Más canciones de</v>
       </c>
       <c r="D171" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B171,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Plus de chansons de</v>
       </c>
     </row>
@@ -4925,11 +4844,11 @@
         <v>281</v>
       </c>
       <c r="C172" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B172,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Más escuchado</v>
       </c>
       <c r="D172" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B172,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Les plus écoutés</v>
       </c>
     </row>
@@ -4941,11 +4860,11 @@
         <v>283</v>
       </c>
       <c r="C173" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B173,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Álbumes más escuchados</v>
       </c>
       <c r="D173" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B173,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Albums les plus écoutés</v>
       </c>
     </row>
@@ -4957,11 +4876,11 @@
         <v>285</v>
       </c>
       <c r="C174" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B174,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Artistas más escuchados</v>
       </c>
       <c r="D174" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B174,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Artistes les plus écoutés</v>
       </c>
     </row>
@@ -4973,11 +4892,11 @@
         <v>287</v>
       </c>
       <c r="C175" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Canciones más escuchadas</v>
       </c>
       <c r="D175" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chansons les plus écoutées</v>
       </c>
     </row>
@@ -4989,11 +4908,11 @@
         <v>289</v>
       </c>
       <c r="C176" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B176,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Nombre</v>
       </c>
       <c r="D176" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B176,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nom</v>
       </c>
     </row>
@@ -5005,11 +4924,11 @@
         <v>291</v>
       </c>
       <c r="C177" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B177,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Introducir nueva contraseña</v>
       </c>
       <c r="D177" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B177,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
@@ -5021,11 +4940,11 @@
         <v>293</v>
       </c>
       <c r="C178" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B178,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Nueva lista de reproducción</v>
       </c>
       <c r="D178" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B178,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nouvelle playlist</v>
       </c>
     </row>
@@ -5037,11 +4956,11 @@
         <v>295</v>
       </c>
       <c r="C179" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B179,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D179" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B179,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nouveau nom de la playlist</v>
       </c>
     </row>
@@ -5053,11 +4972,11 @@
         <v>297</v>
       </c>
       <c r="C180" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B180,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Nueva versión disponible</v>
       </c>
       <c r="D180" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B180,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nouvelle version disponible</v>
       </c>
     </row>
@@ -5069,11 +4988,11 @@
         <v>299</v>
       </c>
       <c r="C181" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B181,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Próximos medios</v>
       </c>
       <c r="D181" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B181,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Médias suivants</v>
       </c>
     </row>
@@ -5085,11 +5004,11 @@
         <v>301</v>
       </c>
       <c r="C182" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B182,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Todavía no hay álbumes en tu biblioteca</v>
       </c>
       <c r="D182" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B182,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
@@ -5101,11 +5020,11 @@
         <v>303</v>
       </c>
       <c r="C183" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>No hay datos registrados.</v>
       </c>
       <c r="D183" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B183,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
@@ -5117,11 +5036,11 @@
         <v>305</v>
       </c>
       <c r="C184" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B184,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Letra no disponible</v>
       </c>
       <c r="D184" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B184,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Paroles non disponibles</v>
       </c>
     </row>
@@ -5133,11 +5052,11 @@
         <v>307</v>
       </c>
       <c r="C185" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B185,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D185" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B185,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
@@ -5149,11 +5068,11 @@
         <v>309</v>
       </c>
       <c r="C186" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B186,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>No hay repetición</v>
       </c>
       <c r="D186" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B186,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Pas de répétition</v>
       </c>
     </row>
@@ -5165,11 +5084,11 @@
         <v>311</v>
       </c>
       <c r="C187" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B187,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Sin resultados</v>
       </c>
       <c r="D187" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B187,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucun résultat</v>
       </c>
     </row>
@@ -5181,11 +5100,11 @@
         <v>313</v>
       </c>
       <c r="C188" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Sin trabajador de servicios</v>
       </c>
       <c r="D188" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B188,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucun travailleur de services</v>
       </c>
     </row>
@@ -5197,11 +5116,11 @@
         <v>315</v>
       </c>
       <c r="C189" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B189,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D189" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B189,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
@@ -5213,11 +5132,11 @@
         <v>317</v>
       </c>
       <c r="C190" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B190,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Sin estado</v>
       </c>
       <c r="D190" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B190,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucun État</v>
       </c>
     </row>
@@ -5229,11 +5148,11 @@
         <v>319</v>
       </c>
       <c r="C191" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B191,$B$2,C$2)</f>
+        <f t="shared" si="9"/>
         <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D191" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B191,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
@@ -5245,11 +5164,11 @@
         <v>321</v>
       </c>
       <c r="C192" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
+        <f t="shared" ref="C192:C205" si="10">_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
         <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D192" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B192,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
@@ -5261,11 +5180,11 @@
         <v>323</v>
       </c>
       <c r="C193" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Noviembre</v>
       </c>
       <c r="D193" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B193,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Novembre</v>
       </c>
     </row>
@@ -5277,11 +5196,11 @@
         <v>325</v>
       </c>
       <c r="C194" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B194,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Octubre</v>
       </c>
       <c r="D194" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B194,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Octobre</v>
       </c>
     </row>
@@ -5293,11 +5212,11 @@
         <v>327</v>
       </c>
       <c r="C195" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B195,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Lista abierta</v>
       </c>
       <c r="D195" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B195,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Liste ouverte</v>
       </c>
     </row>
@@ -5309,11 +5228,11 @@
         <v>329</v>
       </c>
       <c r="C196" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Canción abierta</v>
       </c>
       <c r="D196" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B196,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chanson d’ouverture</v>
       </c>
     </row>
@@ -5325,11 +5244,11 @@
         <v>331</v>
       </c>
       <c r="C197" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B197,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Partido</v>
       </c>
       <c r="D197" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B197,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Parti</v>
       </c>
     </row>
@@ -5341,11 +5260,11 @@
         <v>333</v>
       </c>
       <c r="C198" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B198,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Canción de pausa</v>
       </c>
       <c r="D198" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B198,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Chanson de pause</v>
       </c>
     </row>
@@ -5357,11 +5276,11 @@
         <v>335</v>
       </c>
       <c r="C199" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B199,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Solicitudes pendientes</v>
       </c>
       <c r="D199" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B199,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Demandes en attente</v>
       </c>
     </row>
@@ -5373,11 +5292,11 @@
         <v>337</v>
       </c>
       <c r="C200" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B200,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Pin</v>
       </c>
       <c r="D200" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B200,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Épingle</v>
       </c>
     </row>
@@ -5389,11 +5308,11 @@
         <v>339</v>
       </c>
       <c r="C201" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B201,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Listas fijadas</v>
       </c>
       <c r="D201" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B201,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Listes épinglées</v>
       </c>
     </row>
@@ -5405,11 +5324,11 @@
         <v>341</v>
       </c>
       <c r="C202" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B202,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Título del álbum</v>
       </c>
       <c r="D202" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B202,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Titre de l’album</v>
       </c>
     </row>
@@ -5421,11 +5340,11 @@
         <v>343</v>
       </c>
       <c r="C203" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Nombre artístico</v>
       </c>
       <c r="D203" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Nom de l’artiste</v>
       </c>
     </row>
@@ -5437,11 +5356,11 @@
         <v>345</v>
       </c>
       <c r="C204" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B204,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D204" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B204,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Ma playlist parfaite</v>
       </c>
     </row>
@@ -5453,11 +5372,11 @@
         <v>347</v>
       </c>
       <c r="C205" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B205,$B$2,C$2)</f>
+        <f t="shared" si="10"/>
         <v>Título de la canción</v>
       </c>
       <c r="D205" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B205,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Titre de la chanson</v>
       </c>
     </row>
@@ -5472,7 +5391,7 @@
         <v>350</v>
       </c>
       <c r="D206" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B206,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Jeu</v>
       </c>
     </row>
@@ -5487,7 +5406,7 @@
         <v>353</v>
       </c>
       <c r="D207" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B207,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Liste des jeux</v>
       </c>
     </row>
@@ -5499,11 +5418,11 @@
         <v>355</v>
       </c>
       <c r="C208" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
         <v>Reproducir medios</v>
       </c>
       <c r="D208" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B208,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Lire les médias</v>
       </c>
     </row>
@@ -5518,7 +5437,7 @@
         <v>358</v>
       </c>
       <c r="D209" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B209,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>À jouer à venir</v>
       </c>
     </row>
@@ -5533,7 +5452,7 @@
         <v>361</v>
       </c>
       <c r="D210" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B210,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Jouer la chanson</v>
       </c>
     </row>
@@ -5545,11 +5464,11 @@
         <v>363</v>
       </c>
       <c r="C211" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
+        <f t="shared" ref="C211:C234" si="11">_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
         <v>Listas de reproducción</v>
       </c>
       <c r="D211" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B211,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Playlists</v>
       </c>
     </row>
@@ -5561,11 +5480,11 @@
         <v>365</v>
       </c>
       <c r="C212" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B212,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Medios anteriores</v>
       </c>
       <c r="D212" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B212,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Médias précédents</v>
       </c>
     </row>
@@ -5577,11 +5496,11 @@
         <v>367</v>
       </c>
       <c r="C213" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B213,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Selecciones rápidas</v>
       </c>
       <c r="D213" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B213,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Choix rapides</v>
       </c>
     </row>
@@ -5593,11 +5512,11 @@
         <v>369</v>
       </c>
       <c r="C214" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B214,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Radio</v>
       </c>
       <c r="D214" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B214,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Radio</v>
       </c>
     </row>
@@ -5609,11 +5528,11 @@
         <v>371</v>
       </c>
       <c r="C215" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B215,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>No se han encontrado estaciones</v>
       </c>
       <c r="D215" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B215,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Aucune station trouvée</v>
       </c>
     </row>
@@ -5625,11 +5544,11 @@
         <v>373</v>
       </c>
       <c r="C216" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B216,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D216" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B216,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
@@ -5641,11 +5560,11 @@
         <v>375</v>
       </c>
       <c r="C217" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B217,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D217" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B217,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
@@ -5657,11 +5576,11 @@
         <v>377</v>
       </c>
       <c r="C218" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B218,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Emisoras de radio</v>
       </c>
       <c r="D218" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B218,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Radio Stations</v>
       </c>
     </row>
@@ -5673,11 +5592,11 @@
         <v>379</v>
       </c>
       <c r="C219" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B219,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Mezcla reciente</v>
       </c>
       <c r="D219" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B219,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Mix récent</v>
       </c>
     </row>
@@ -5689,11 +5608,11 @@
         <v>381</v>
       </c>
       <c r="C220" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B220,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D220" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B220,$B$2,D$2)</f>
+        <f t="shared" si="8"/>
         <v>Joué récemment</v>
       </c>
     </row>
@@ -5705,11 +5624,11 @@
         <v>383</v>
       </c>
       <c r="C221" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B221,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Jugado recientemente</v>
       </c>
       <c r="D221" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
+        <f t="shared" ref="D221:D281" si="12">_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
         <v>Récemment joué</v>
       </c>
     </row>
@@ -5721,11 +5640,11 @@
         <v>385</v>
       </c>
       <c r="C222" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B222,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registro</v>
       </c>
       <c r="D222" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B222,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Registre</v>
       </c>
     </row>
@@ -5737,11 +5656,11 @@
         <v>387</v>
       </c>
       <c r="C223" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registrado</v>
       </c>
       <c r="D223" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B223,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Enregistré</v>
       </c>
     </row>
@@ -5753,11 +5672,11 @@
         <v>389</v>
       </c>
       <c r="C224" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B224,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Registrando...</v>
       </c>
       <c r="D224" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B224,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Enregistrement...</v>
       </c>
     </row>
@@ -5769,11 +5688,11 @@
         <v>391</v>
       </c>
       <c r="C225" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B225,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Artistas relacionados</v>
       </c>
       <c r="D225" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B225,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Artistes associés</v>
       </c>
     </row>
@@ -5785,11 +5704,11 @@
         <v>393</v>
       </c>
       <c r="C226" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B226,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Relajado</v>
       </c>
       <c r="D226" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B226,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Détendu</v>
       </c>
     </row>
@@ -5801,11 +5720,11 @@
         <v>505</v>
       </c>
       <c r="C227" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B227,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Recuérdame</v>
       </c>
       <c r="D227" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B227,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Souviens-toi de moi</v>
       </c>
     </row>
@@ -5817,11 +5736,11 @@
         <v>395</v>
       </c>
       <c r="C228" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B228,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D228" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B228,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Retirer de la bibliothèque</v>
       </c>
     </row>
@@ -5833,11 +5752,11 @@
         <v>397</v>
       </c>
       <c r="C229" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B229,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Quitar de me gusta</v>
       </c>
       <c r="D229" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B229,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Retirer de aimé</v>
       </c>
     </row>
@@ -5849,11 +5768,11 @@
         <v>399</v>
       </c>
       <c r="C230" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B230,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D230" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B230,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Supprimer de la playlist</v>
       </c>
     </row>
@@ -5865,11 +5784,11 @@
         <v>401</v>
       </c>
       <c r="C231" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B231,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Eliminar de la cola</v>
       </c>
       <c r="D231" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B231,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Retirer de la file d’attente</v>
       </c>
     </row>
@@ -5881,11 +5800,11 @@
         <v>403</v>
       </c>
       <c r="C232" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repite todo</v>
       </c>
       <c r="D232" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B232,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Répétez tout</v>
       </c>
     </row>
@@ -5897,11 +5816,11 @@
         <v>405</v>
       </c>
       <c r="C233" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B233,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repite una</v>
       </c>
       <c r="D233" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B233,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Répétez-en un</v>
       </c>
     </row>
@@ -5913,11 +5832,11 @@
         <v>407</v>
       </c>
       <c r="C234" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B234,$B$2,C$2)</f>
+        <f t="shared" si="11"/>
         <v>Repetir nueva contraseña</v>
       </c>
       <c r="D234" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B234,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
@@ -5932,7 +5851,7 @@
         <v>410</v>
       </c>
       <c r="D235" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Nouvelle tentative</v>
       </c>
     </row>
@@ -5944,11 +5863,11 @@
         <v>412</v>
       </c>
       <c r="C236" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
+        <f t="shared" ref="C236:C281" si="13">_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
         <v>Regreso a casa</v>
       </c>
       <c r="D236" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B236,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Retour à la maison</v>
       </c>
     </row>
@@ -5960,11 +5879,11 @@
         <v>414</v>
       </c>
       <c r="C237" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B237,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Guardando...</v>
       </c>
       <c r="D237" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B237,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Sauver...</v>
       </c>
     </row>
@@ -5976,11 +5895,11 @@
         <v>416</v>
       </c>
       <c r="C238" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B238,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Búsqueda</v>
       </c>
       <c r="D238" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B238,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Recherche</v>
       </c>
     </row>
@@ -5992,11 +5911,11 @@
         <v>418</v>
       </c>
       <c r="C239" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D239" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
@@ -6008,11 +5927,11 @@
         <v>420</v>
       </c>
       <c r="C240" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B240,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D240" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B240,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
@@ -6024,11 +5943,11 @@
         <v>422</v>
       </c>
       <c r="C241" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B241,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D241" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B241,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
@@ -6040,11 +5959,11 @@
         <v>424</v>
       </c>
       <c r="C242" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B242,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Buscar en la biblioteca</v>
       </c>
       <c r="D242" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B242,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
@@ -6056,11 +5975,11 @@
         <v>426</v>
       </c>
       <c r="C243" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Usuarios de búsqueda</v>
       </c>
       <c r="D243" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B243,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Rechercher les utilisateurs</v>
       </c>
     </row>
@@ -6072,11 +5991,11 @@
         <v>428</v>
       </c>
       <c r="C244" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B244,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Enviar canción actual</v>
       </c>
       <c r="D244" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B244,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
@@ -6088,11 +6007,11 @@
         <v>430</v>
       </c>
       <c r="C245" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B245,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Septiembre</v>
       </c>
       <c r="D245" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B245,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Septembre</v>
       </c>
     </row>
@@ -6104,11 +6023,11 @@
         <v>64</v>
       </c>
       <c r="C246" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B246,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Escenarios</v>
       </c>
       <c r="D246" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B246,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Décors</v>
       </c>
     </row>
@@ -6120,11 +6039,11 @@
         <v>433</v>
       </c>
       <c r="C247" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B247,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Compartir canción</v>
       </c>
       <c r="D247" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B247,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Partager la chanson</v>
       </c>
     </row>
@@ -6136,11 +6055,11 @@
         <v>435</v>
       </c>
       <c r="C248" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B248,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones compartidas para ti</v>
       </c>
       <c r="D248" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B248,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chansons partagées pour vous</v>
       </c>
     </row>
@@ -6152,11 +6071,11 @@
         <v>437</v>
       </c>
       <c r="C249" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B249,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Compartido desde</v>
       </c>
       <c r="D249" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B249,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Partagé depuis</v>
       </c>
     </row>
@@ -6168,11 +6087,11 @@
         <v>439</v>
       </c>
       <c r="C250" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B250,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Mostrando datos de</v>
       </c>
       <c r="D250" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B250,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Affichage des données de</v>
       </c>
     </row>
@@ -6184,11 +6103,11 @@
         <v>441</v>
       </c>
       <c r="C251" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B251,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canción</v>
       </c>
       <c r="D251" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B251,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chanson</v>
       </c>
     </row>
@@ -6200,11 +6119,11 @@
         <v>443</v>
       </c>
       <c r="C252" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B252,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones</v>
       </c>
       <c r="D252" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B252,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chansons</v>
       </c>
     </row>
@@ -6216,11 +6135,11 @@
         <v>445</v>
       </c>
       <c r="C253" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B253,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones Solo para ti</v>
       </c>
       <c r="D253" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B253,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chansons juste pour toi</v>
       </c>
     </row>
@@ -6232,11 +6151,11 @@
         <v>447</v>
       </c>
       <c r="C254" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B254,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones de</v>
       </c>
       <c r="D254" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B254,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chansons de</v>
       </c>
     </row>
@@ -6248,11 +6167,11 @@
         <v>449</v>
       </c>
       <c r="C255" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B255,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones escuchadas</v>
       </c>
       <c r="D255" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B255,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Chansons écoutées</v>
       </c>
     </row>
@@ -6264,11 +6183,11 @@
         <v>451</v>
       </c>
       <c r="C256" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B256,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Empezando...</v>
       </c>
       <c r="D256" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B256,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Commencer...</v>
       </c>
     </row>
@@ -6280,11 +6199,11 @@
         <v>453</v>
       </c>
       <c r="C257" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B257,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Estadísticas</v>
       </c>
       <c r="D257" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B257,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -6296,11 +6215,11 @@
         <v>455</v>
       </c>
       <c r="C258" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B258,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Estadísticas</v>
       </c>
       <c r="D258" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B258,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Statistiques</v>
       </c>
     </row>
@@ -6312,11 +6231,11 @@
         <v>457</v>
       </c>
       <c r="C259" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B259,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>¡Para</v>
       </c>
       <c r="D259" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B259,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Arrête</v>
       </c>
     </row>
@@ -6328,11 +6247,11 @@
         <v>459</v>
       </c>
       <c r="C260" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B260,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>a</v>
       </c>
       <c r="D260" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B260,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>à</v>
       </c>
     </row>
@@ -6344,11 +6263,11 @@
         <v>461</v>
       </c>
       <c r="C261" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B261,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>ToDo</v>
       </c>
       <c r="D261" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B261,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>ToDo</v>
       </c>
     </row>
@@ -6360,11 +6279,11 @@
         <v>463</v>
       </c>
       <c r="C262" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B262,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Álbumes destacados</v>
       </c>
       <c r="D262" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B262,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Albums phares</v>
       </c>
     </row>
@@ -6376,11 +6295,11 @@
         <v>465</v>
       </c>
       <c r="C263" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B263,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Canciones principales</v>
       </c>
       <c r="D263" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B263,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Meilleures chansons</v>
       </c>
     </row>
@@ -6392,11 +6311,11 @@
         <v>467</v>
       </c>
       <c r="C264" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B264,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Desclavar</v>
       </c>
       <c r="D264" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B264,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Détacher</v>
       </c>
     </row>
@@ -6408,11 +6327,11 @@
         <v>469</v>
       </c>
       <c r="C265" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B265,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Desregistrar</v>
       </c>
       <c r="D265" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B265,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Désinscription</v>
       </c>
     </row>
@@ -6424,11 +6343,11 @@
         <v>471</v>
       </c>
       <c r="C266" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B266,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>No registrado</v>
       </c>
       <c r="D266" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B266,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Non enregistré</v>
       </c>
     </row>
@@ -6440,11 +6359,11 @@
         <v>473</v>
       </c>
       <c r="C267" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B267,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Dejar de registrarse...</v>
       </c>
       <c r="D267" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B267,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Désenregistrement...</v>
       </c>
     </row>
@@ -6456,11 +6375,11 @@
         <v>475</v>
       </c>
       <c r="C268" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B268,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Actualización</v>
       </c>
       <c r="D268" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B268,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Mise à jour</v>
       </c>
     </row>
@@ -6472,11 +6391,11 @@
         <v>477</v>
       </c>
       <c r="C269" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B269,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Actualizando...</v>
       </c>
       <c r="D269" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B269,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Mise à jour...</v>
       </c>
     </row>
@@ -6488,11 +6407,11 @@
         <v>479</v>
       </c>
       <c r="C270" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B270,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Subida</v>
       </c>
       <c r="D270" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B270,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Téléverser</v>
       </c>
     </row>
@@ -6504,11 +6423,11 @@
         <v>481</v>
       </c>
       <c r="C271" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B271,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Usuario</v>
       </c>
       <c r="D271" t="str">
-        <f>_xlfn.TRANSLATE($B271,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Utilisateur</v>
       </c>
     </row>
@@ -6520,11 +6439,11 @@
         <v>483</v>
       </c>
       <c r="C272" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B272,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Configuración de usuario</v>
       </c>
       <c r="D272" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B272,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Paramètres utilisateur</v>
       </c>
     </row>
@@ -6536,11 +6455,11 @@
         <v>485</v>
       </c>
       <c r="C273" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B273,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Estadísticas de usuario</v>
       </c>
       <c r="D273" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B273,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Statistiques des utilisateurs</v>
       </c>
     </row>
@@ -6552,11 +6471,11 @@
         <v>487</v>
       </c>
       <c r="C274" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B274,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Usuarios y amigos</v>
       </c>
       <c r="D274" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B274,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Utilisateurs et amis</v>
       </c>
     </row>
@@ -6568,11 +6487,11 @@
         <v>489</v>
       </c>
       <c r="C275" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B275,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Lista de usuarios</v>
       </c>
       <c r="D275" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B275,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Liste des utilisateurs</v>
       </c>
     </row>
@@ -6584,11 +6503,11 @@
         <v>491</v>
       </c>
       <c r="C276" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B276,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Vídeos</v>
       </c>
       <c r="D276" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B276,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Vidéos</v>
       </c>
     </row>
@@ -6600,11 +6519,11 @@
         <v>493</v>
       </c>
       <c r="C277" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B277,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>También puede que te interese</v>
       </c>
       <c r="D277" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B277,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Ça pourrait aussi te plaire</v>
       </c>
     </row>
@@ -6616,11 +6535,11 @@
         <v>495</v>
       </c>
       <c r="C278" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B278,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Tu</v>
       </c>
       <c r="D278" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B278,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Votre</v>
       </c>
     </row>
@@ -6632,11 +6551,11 @@
         <v>497</v>
       </c>
       <c r="C279" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B279,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Tus álbumes y listas de reproducción</v>
       </c>
       <c r="D279" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B279,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Vos albums et playlists</v>
       </c>
     </row>
@@ -6648,11 +6567,11 @@
         <v>499</v>
       </c>
       <c r="C280" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B280,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Tu mezcla</v>
       </c>
       <c r="D280" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B280,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Votre Mix</v>
       </c>
     </row>
@@ -6664,12 +6583,43 @@
         <v>501</v>
       </c>
       <c r="C281" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B281,$B$2,C$2)</f>
+        <f t="shared" si="13"/>
         <v>Vídeos de YouTube</v>
       </c>
       <c r="D281" t="str">
-        <f ca="1">_xlfn.TRANSLATE($B281,$B$2,D$2)</f>
+        <f t="shared" si="12"/>
         <v>Vidéos YouTube</v>
+      </c>
+    </row>
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>564</v>
+      </c>
+      <c r="B282" t="s">
+        <v>565</v>
+      </c>
+      <c r="C282" t="str">
+        <f t="shared" ref="C282:C283" si="14">_xlfn.TRANSLATE($B282,$B$2,C$2)</f>
+        <v>Cola</v>
+      </c>
+      <c r="D282" t="str">
+        <f t="shared" ref="D282:D283" si="15">_xlfn.TRANSLATE($B282,$B$2,D$2)</f>
+        <v>File d’attente</v>
+      </c>
+    </row>
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>566</v>
+      </c>
+      <c r="B283" t="s">
+        <v>567</v>
+      </c>
+      <c r="C283" t="s">
+        <v>568</v>
+      </c>
+      <c r="D283" t="str">
+        <f t="shared" si="15"/>
+        <v>Aucun média diffusé</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add LrclibProviderTag component and integrate vocabulary for lyrics attribution
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\icass\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE18371A-2343-4DE7-9048-8EB41C6C8ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C2EA47-6471-423D-8225-0F26961EA73A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="3840" windowWidth="22650" windowHeight="14325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -32,8 +32,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="613">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="617">
   <si>
     <t>KEY</t>
   </si>
@@ -1872,6 +1894,18 @@
   </si>
   <si>
     <t>Waiting for queue setup</t>
+  </si>
+  <si>
+    <t>LYRICS_BY</t>
+  </si>
+  <si>
+    <t>Lyrics by</t>
+  </si>
+  <si>
+    <t>TOP_VIDEOS</t>
+  </si>
+  <si>
+    <t>Top videos</t>
   </si>
 </sst>
 </file>
@@ -1926,11 +1960,67 @@
 </styleSheet>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>14</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_error">
+    <k n="errorType" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D305" totalsRowShown="0">
-  <autoFilter ref="A2:D305" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D305">
-    <sortCondition ref="A2:A305"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A2:D307" totalsRowShown="0">
+  <autoFilter ref="A2:D307" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D307">
+    <sortCondition ref="A2:A307"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="KEY"/>
@@ -2231,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D305"/>
+  <dimension ref="A1:D307"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
@@ -4257,11 +4347,11 @@
         <v>602</v>
       </c>
       <c r="C127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,C$2)</f>
+        <f ca="1">_xlfn.TRANSLATE($B127,$B$2,C$2)</f>
         <v>Error al cargar el archivo multimedia</v>
       </c>
       <c r="D127" t="str">
-        <f>_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
+        <f ca="1">_xlfn.TRANSLATE($B127,$B$2,D$2)</f>
         <v>Erreur de chargement du fichier média</v>
       </c>
     </row>
@@ -4484,7 +4574,7 @@
         <v>Trayecto</v>
       </c>
       <c r="D141" t="str">
-        <f>_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
+        <f ca="1">_xlfn.TRANSLATE($B141,$B$2,D$2)</f>
         <v>Récupération</v>
       </c>
     </row>
@@ -4986,1093 +5076,1093 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>337</v>
+        <v>613</v>
       </c>
       <c r="B173" t="s">
-        <v>338</v>
+        <v>614</v>
       </c>
       <c r="C173" t="str">
         <f>_xlfn.TRANSLATE($B173,$B$2,C$2)</f>
-        <v>Marzo</v>
+        <v>Letra de</v>
       </c>
       <c r="D173" t="str">
         <f>_xlfn.TRANSLATE($B173,$B$2,D$2)</f>
-        <v>Mars</v>
+        <v>Paroles de</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B174" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C174" t="str">
         <f>_xlfn.TRANSLATE($B174,$B$2,C$2)</f>
-        <v>Mayo</v>
+        <v>Marzo</v>
       </c>
       <c r="D174" t="str">
         <f>_xlfn.TRANSLATE($B174,$B$2,D$2)</f>
-        <v>Mai</v>
+        <v>Mars</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B175" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C175" t="str">
         <f>_xlfn.TRANSLATE($B175,$B$2,C$2)</f>
-        <v>Medios añadidos a la biblioteca</v>
+        <v>Mayo</v>
       </c>
       <c r="D175" t="str">
         <f>_xlfn.TRANSLATE($B175,$B$2,D$2)</f>
-        <v>Ajout de médias à la bibliothèque</v>
+        <v>Mai</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B176" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C176" t="str">
         <f>_xlfn.TRANSLATE($B176,$B$2,C$2)</f>
-        <v>A los medios les gustó</v>
+        <v>Medios añadidos a la biblioteca</v>
       </c>
       <c r="D176" t="str">
         <f>_xlfn.TRANSLATE($B176,$B$2,D$2)</f>
-        <v>Les médias appréciaient</v>
+        <v>Ajout de médias à la bibliothèque</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B177" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C177" t="str">
         <f>_xlfn.TRANSLATE($B177,$B$2,C$2)</f>
-        <v>Progreso de los medios</v>
+        <v>A los medios les gustó</v>
       </c>
       <c r="D177" t="str">
         <f>_xlfn.TRANSLATE($B177,$B$2,D$2)</f>
-        <v>Progrès des médias</v>
+        <v>Les médias appréciaient</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B178" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C178" t="str">
         <f>_xlfn.TRANSLATE($B178,$B$2,C$2)</f>
-        <v>Actas</v>
+        <v>Progreso de los medios</v>
       </c>
       <c r="D178" t="str">
         <f>_xlfn.TRANSLATE($B178,$B$2,D$2)</f>
-        <v>Procès-verbal</v>
+        <v>Progrès des médias</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B179" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C179" t="str">
         <f>_xlfn.TRANSLATE($B179,$B$2,C$2)</f>
-        <v>Minutos escuchados</v>
+        <v>Actas</v>
       </c>
       <c r="D179" t="str">
         <f>_xlfn.TRANSLATE($B179,$B$2,D$2)</f>
-        <v>Minutes écoutées</v>
+        <v>Procès-verbal</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B180" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C180" t="str">
         <f>_xlfn.TRANSLATE($B180,$B$2,C$2)</f>
-        <v>Minutos escuchados por día</v>
+        <v>Minutos escuchados</v>
       </c>
       <c r="D180" t="str">
         <f>_xlfn.TRANSLATE($B180,$B$2,D$2)</f>
-        <v>Minutes écoutées par jour</v>
+        <v>Minutes écoutées</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B181" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C181" t="str">
         <f>_xlfn.TRANSLATE($B181,$B$2,C$2)</f>
-        <v>Canciones para cuando te sientas</v>
+        <v>Minutos escuchados por día</v>
       </c>
       <c r="D181" t="str">
         <f>_xlfn.TRANSLATE($B181,$B$2,D$2)</f>
-        <v>Chansons pour quand tu te sens</v>
+        <v>Minutes écoutées par jour</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B182" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C182" t="str">
         <f>_xlfn.TRANSLATE($B182,$B$2,C$2)</f>
-        <v>Más opciones</v>
+        <v>Canciones para cuando te sientas</v>
       </c>
       <c r="D182" t="str">
         <f>_xlfn.TRANSLATE($B182,$B$2,D$2)</f>
-        <v>Plus d’options</v>
+        <v>Chansons pour quand tu te sens</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B183" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C183" t="str">
         <f>_xlfn.TRANSLATE($B183,$B$2,C$2)</f>
-        <v>Más canciones de</v>
+        <v>Más opciones</v>
       </c>
       <c r="D183" t="str">
         <f>_xlfn.TRANSLATE($B183,$B$2,D$2)</f>
-        <v>Plus de chansons de</v>
+        <v>Plus d’options</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B184" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C184" t="str">
         <f>_xlfn.TRANSLATE($B184,$B$2,C$2)</f>
-        <v>Más escuchado</v>
+        <v>Más canciones de</v>
       </c>
       <c r="D184" t="str">
         <f>_xlfn.TRANSLATE($B184,$B$2,D$2)</f>
-        <v>Les plus écoutés</v>
+        <v>Plus de chansons de</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B185" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C185" t="str">
         <f>_xlfn.TRANSLATE($B185,$B$2,C$2)</f>
-        <v>Álbumes más escuchados</v>
+        <v>Más escuchado</v>
       </c>
       <c r="D185" t="str">
         <f>_xlfn.TRANSLATE($B185,$B$2,D$2)</f>
-        <v>Albums les plus écoutés</v>
+        <v>Les plus écoutés</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B186" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C186" t="str">
         <f>_xlfn.TRANSLATE($B186,$B$2,C$2)</f>
-        <v>Artistas más escuchados</v>
+        <v>Álbumes más escuchados</v>
       </c>
       <c r="D186" t="str">
         <f>_xlfn.TRANSLATE($B186,$B$2,D$2)</f>
-        <v>Artistes les plus écoutés</v>
+        <v>Albums les plus écoutés</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B187" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C187" t="str">
         <f>_xlfn.TRANSLATE($B187,$B$2,C$2)</f>
-        <v>Canciones más escuchadas</v>
+        <v>Artistas más escuchados</v>
       </c>
       <c r="D187" t="str">
         <f>_xlfn.TRANSLATE($B187,$B$2,D$2)</f>
-        <v>Chansons les plus écoutées</v>
+        <v>Artistes les plus écoutés</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B188" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C188" t="str">
         <f>_xlfn.TRANSLATE($B188,$B$2,C$2)</f>
-        <v>Nombre</v>
+        <v>Canciones más escuchadas</v>
       </c>
       <c r="D188" t="str">
         <f>_xlfn.TRANSLATE($B188,$B$2,D$2)</f>
-        <v>Nom</v>
+        <v>Chansons les plus écoutées</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B189" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C189" t="str">
         <f>_xlfn.TRANSLATE($B189,$B$2,C$2)</f>
-        <v>Introducir nueva contraseña</v>
+        <v>Nombre</v>
       </c>
       <c r="D189" t="str">
         <f>_xlfn.TRANSLATE($B189,$B$2,D$2)</f>
-        <v>Entrer un nouveau mot de passe</v>
+        <v>Nom</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B190" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C190" t="str">
         <f>_xlfn.TRANSLATE($B190,$B$2,C$2)</f>
-        <v>Nueva lista de reproducción</v>
+        <v>Introducir nueva contraseña</v>
       </c>
       <c r="D190" t="str">
         <f>_xlfn.TRANSLATE($B190,$B$2,D$2)</f>
-        <v>Nouvelle playlist</v>
+        <v>Entrer un nouveau mot de passe</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B191" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C191" t="str">
         <f>_xlfn.TRANSLATE($B191,$B$2,C$2)</f>
-        <v>Nuevo nombre de la lista de reproducción</v>
+        <v>Nueva lista de reproducción</v>
       </c>
       <c r="D191" t="str">
         <f>_xlfn.TRANSLATE($B191,$B$2,D$2)</f>
-        <v>Nouveau nom de la playlist</v>
+        <v>Nouvelle playlist</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B192" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C192" t="str">
         <f>_xlfn.TRANSLATE($B192,$B$2,C$2)</f>
-        <v>Nueva versión disponible</v>
+        <v>Nuevo nombre de la lista de reproducción</v>
       </c>
       <c r="D192" t="str">
         <f>_xlfn.TRANSLATE($B192,$B$2,D$2)</f>
-        <v>Nouvelle version disponible</v>
+        <v>Nouveau nom de la playlist</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B193" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C193" t="str">
         <f>_xlfn.TRANSLATE($B193,$B$2,C$2)</f>
-        <v>Próximos medios</v>
+        <v>Nueva versión disponible</v>
       </c>
       <c r="D193" t="str">
         <f>_xlfn.TRANSLATE($B193,$B$2,D$2)</f>
-        <v>Médias suivants</v>
+        <v>Nouvelle version disponible</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B194" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C194" t="str">
         <f>_xlfn.TRANSLATE($B194,$B$2,C$2)</f>
-        <v>Todavía no hay álbumes en tu biblioteca</v>
+        <v>Próximos medios</v>
       </c>
       <c r="D194" t="str">
         <f>_xlfn.TRANSLATE($B194,$B$2,D$2)</f>
-        <v>Aucun album dans ta bibliothèque pour l’instant</v>
+        <v>Médias suivants</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B195" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C195" t="str">
         <f>_xlfn.TRANSLATE($B195,$B$2,C$2)</f>
-        <v>No hay datos registrados.</v>
+        <v>Todavía no tienes álbumes en tu biblioteca</v>
       </c>
       <c r="D195" t="str">
         <f>_xlfn.TRANSLATE($B195,$B$2,D$2)</f>
-        <v>Aucune donnée enregistrée.</v>
+        <v>Aucun album dans ta bibliothèque pour l’instant</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>605</v>
+        <v>381</v>
       </c>
       <c r="B196" t="s">
-        <v>611</v>
+        <v>382</v>
       </c>
       <c r="C196" t="str">
         <f>_xlfn.TRANSLATE($B196,$B$2,C$2)</f>
-        <v>No se permiten descargas</v>
+        <v>No hay datos registrados.</v>
       </c>
       <c r="D196" t="str">
         <f>_xlfn.TRANSLATE($B196,$B$2,D$2)</f>
-        <v>Aucun téléchargement</v>
+        <v>Aucune donnée enregistrée.</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>383</v>
+        <v>605</v>
       </c>
       <c r="B197" t="s">
-        <v>384</v>
+        <v>611</v>
       </c>
       <c r="C197" t="str">
         <f>_xlfn.TRANSLATE($B197,$B$2,C$2)</f>
-        <v>Letra no disponible</v>
+        <v>No se permiten descargas</v>
       </c>
       <c r="D197" t="str">
         <f>_xlfn.TRANSLATE($B197,$B$2,D$2)</f>
-        <v>Paroles non disponibles</v>
+        <v>Aucun téléchargement</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B198" t="s">
-        <v>386</v>
-      </c>
-      <c r="C198" t="s">
-        <v>387</v>
+        <v>384</v>
+      </c>
+      <c r="C198" t="str">
+        <f>_xlfn.TRANSLATE($B198,$B$2,C$2)</f>
+        <v>Letra no disponible</v>
       </c>
       <c r="D198" t="str">
         <f>_xlfn.TRANSLATE($B198,$B$2,D$2)</f>
-        <v>Aucun média diffusé</v>
+        <v>Paroles non disponibles</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B199" t="s">
-        <v>389</v>
-      </c>
-      <c r="C199" t="str">
-        <f>_xlfn.TRANSLATE($B199,$B$2,C$2)</f>
-        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
+        <v>386</v>
+      </c>
+      <c r="C199" t="s">
+        <v>387</v>
       </c>
       <c r="D199" t="str">
         <f>_xlfn.TRANSLATE($B199,$B$2,D$2)</f>
-        <v>Pas encore de playlists dans votre bibliothèque</v>
+        <v>Aucun média diffusé</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B200" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C200" t="str">
         <f>_xlfn.TRANSLATE($B200,$B$2,C$2)</f>
-        <v>No hay repetición</v>
+        <v>Todavía no hay listas de reproducción en tu biblioteca</v>
       </c>
       <c r="D200" t="str">
         <f>_xlfn.TRANSLATE($B200,$B$2,D$2)</f>
-        <v>Pas de répétition</v>
+        <v>Pas encore de playlists dans votre bibliothèque</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B201" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C201" t="str">
         <f>_xlfn.TRANSLATE($B201,$B$2,C$2)</f>
-        <v>Sin resultados</v>
+        <v>No hay repetición</v>
       </c>
       <c r="D201" t="str">
         <f>_xlfn.TRANSLATE($B201,$B$2,D$2)</f>
-        <v>Aucun résultat</v>
+        <v>Pas de répétition</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B202" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C202" t="str">
         <f>_xlfn.TRANSLATE($B202,$B$2,C$2)</f>
-        <v>Sin trabajador de servicios</v>
+        <v>Sin resultados</v>
       </c>
       <c r="D202" t="str">
         <f>_xlfn.TRANSLATE($B202,$B$2,D$2)</f>
-        <v>Aucun travailleur de services</v>
+        <v>Aucun résultat</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B203" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C203" t="str">
         <f>_xlfn.TRANSLATE($B203,$B$2,C$2)</f>
-        <v>Todavía no hay canciones en tu biblioteca</v>
+        <v>Sin trabajador de servicios</v>
       </c>
       <c r="D203" t="str">
         <f>_xlfn.TRANSLATE($B203,$B$2,D$2)</f>
-        <v>Pas encore de chansons dans ta bibliothèque</v>
+        <v>Aucun travailleur de services</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B204" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C204" t="str">
         <f>_xlfn.TRANSLATE($B204,$B$2,C$2)</f>
-        <v>Sin estado</v>
+        <v>Todavía no hay canciones en tu biblioteca</v>
       </c>
       <c r="D204" t="str">
         <f>_xlfn.TRANSLATE($B204,$B$2,D$2)</f>
-        <v>Aucun État</v>
+        <v>Pas encore de chansons dans ta bibliothèque</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B205" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C205" t="str">
         <f>_xlfn.TRANSLATE($B205,$B$2,C$2)</f>
-        <v>Todavía no hay estaciones en tu biblioteca</v>
+        <v>Sin estado</v>
       </c>
       <c r="D205" t="str">
         <f>_xlfn.TRANSLATE($B205,$B$2,D$2)</f>
-        <v>Pas encore de stations dans votre bibliothèque</v>
+        <v>Aucun État</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B206" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C206" t="str">
         <f>_xlfn.TRANSLATE($B206,$B$2,C$2)</f>
-        <v>Todavía no hay vídeos en tu biblioteca</v>
+        <v>Todavía no hay estaciones en tu biblioteca</v>
       </c>
       <c r="D206" t="str">
         <f>_xlfn.TRANSLATE($B206,$B$2,D$2)</f>
-        <v>Pas encore de vidéos dans ta bibliothèque</v>
+        <v>Pas encore de stations dans votre bibliothèque</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B207" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C207" t="str">
         <f>_xlfn.TRANSLATE($B207,$B$2,C$2)</f>
-        <v>Noviembre</v>
+        <v>Todavía no hay vídeos en tu biblioteca</v>
       </c>
       <c r="D207" t="str">
         <f>_xlfn.TRANSLATE($B207,$B$2,D$2)</f>
-        <v>Novembre</v>
+        <v>Pas encore de vidéos dans ta bibliothèque</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B208" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C208" t="str">
         <f>_xlfn.TRANSLATE($B208,$B$2,C$2)</f>
-        <v>Octubre</v>
+        <v>Noviembre</v>
       </c>
       <c r="D208" t="str">
         <f>_xlfn.TRANSLATE($B208,$B$2,D$2)</f>
-        <v>Octobre</v>
+        <v>Novembre</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B209" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C209" t="str">
         <f>_xlfn.TRANSLATE($B209,$B$2,C$2)</f>
-        <v>Lista abierta</v>
+        <v>Octubre</v>
       </c>
       <c r="D209" t="str">
         <f>_xlfn.TRANSLATE($B209,$B$2,D$2)</f>
-        <v>Liste ouverte</v>
+        <v>Octobre</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B210" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C210" t="str">
         <f>_xlfn.TRANSLATE($B210,$B$2,C$2)</f>
-        <v>Canción abierta</v>
+        <v>Lista abierta</v>
       </c>
       <c r="D210" t="str">
         <f>_xlfn.TRANSLATE($B210,$B$2,D$2)</f>
-        <v>Chanson d’ouverture</v>
+        <v>Liste ouverte</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B211" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C211" t="str">
         <f>_xlfn.TRANSLATE($B211,$B$2,C$2)</f>
-        <v>o crear una cuenta</v>
+        <v>Canción abierta</v>
       </c>
       <c r="D211" t="str">
         <f>_xlfn.TRANSLATE($B211,$B$2,D$2)</f>
-        <v>ou créer un compte</v>
+        <v>Chanson d’ouverture</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B212" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C212" t="str">
         <f>_xlfn.TRANSLATE($B212,$B$2,C$2)</f>
-        <v>O iniciar sesión con una cuenta existente</v>
+        <v>o crear una cuenta</v>
       </c>
       <c r="D212" t="str">
         <f>_xlfn.TRANSLATE($B212,$B$2,D$2)</f>
-        <v>Ou connectez-vous avec un compte existant</v>
+        <v>ou créer un compte</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B213" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C213" t="str">
         <f>_xlfn.TRANSLATE($B213,$B$2,C$2)</f>
-        <v>Partido</v>
+        <v>O iniciar sesión con una cuenta existente</v>
       </c>
       <c r="D213" t="str">
         <f>_xlfn.TRANSLATE($B213,$B$2,D$2)</f>
-        <v>Parti</v>
+        <v>Ou connectez-vous avec un compte existant</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B214" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C214" t="str">
         <f>_xlfn.TRANSLATE($B214,$B$2,C$2)</f>
-        <v>Contraseña</v>
+        <v>Partido</v>
       </c>
       <c r="D214" t="str">
         <f>_xlfn.TRANSLATE($B214,$B$2,D$2)</f>
-        <v>Mot de passe</v>
+        <v>Parti</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B215" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C215" t="str">
         <f>_xlfn.TRANSLATE($B215,$B$2,C$2)</f>
-        <v>Las contraseñas no coinciden</v>
+        <v>Contraseña</v>
       </c>
       <c r="D215" t="str">
         <f>_xlfn.TRANSLATE($B215,$B$2,D$2)</f>
-        <v>Les mots de passe ne correspondent pas</v>
+        <v>Mot de passe</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B216" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C216" t="str">
         <f>_xlfn.TRANSLATE($B216,$B$2,C$2)</f>
-        <v>Canción de pausa</v>
+        <v>Las contraseñas no coinciden</v>
       </c>
       <c r="D216" t="str">
         <f>_xlfn.TRANSLATE($B216,$B$2,D$2)</f>
-        <v>Chanson de pause</v>
+        <v>Les mots de passe ne correspondent pas</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>603</v>
+        <v>422</v>
       </c>
       <c r="B217" t="s">
-        <v>608</v>
+        <v>423</v>
       </c>
       <c r="C217" t="str">
         <f>_xlfn.TRANSLATE($B217,$B$2,C$2)</f>
-        <v>Pendiente</v>
+        <v>Canción de pausa</v>
       </c>
       <c r="D217" t="str">
         <f>_xlfn.TRANSLATE($B217,$B$2,D$2)</f>
-        <v>En attente</v>
+        <v>Chanson de pause</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>424</v>
+        <v>603</v>
       </c>
       <c r="B218" t="s">
-        <v>425</v>
+        <v>608</v>
       </c>
       <c r="C218" t="str">
         <f>_xlfn.TRANSLATE($B218,$B$2,C$2)</f>
-        <v>Solicitudes pendientes</v>
+        <v>Pendiente</v>
       </c>
       <c r="D218" t="str">
         <f>_xlfn.TRANSLATE($B218,$B$2,D$2)</f>
-        <v>Demandes en attente</v>
+        <v>En attente</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B219" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C219" t="str">
         <f>_xlfn.TRANSLATE($B219,$B$2,C$2)</f>
-        <v>Pin</v>
+        <v>Solicitudes pendientes</v>
       </c>
       <c r="D219" t="str">
         <f>_xlfn.TRANSLATE($B219,$B$2,D$2)</f>
-        <v>Épingle</v>
+        <v>Demandes en attente</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B220" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C220" t="str">
         <f>_xlfn.TRANSLATE($B220,$B$2,C$2)</f>
-        <v>Listas fijadas</v>
+        <v>Pin</v>
       </c>
       <c r="D220" t="str">
         <f>_xlfn.TRANSLATE($B220,$B$2,D$2)</f>
-        <v>Listes épinglées</v>
+        <v>Épingle</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B221" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C221" t="str">
         <f>_xlfn.TRANSLATE($B221,$B$2,C$2)</f>
-        <v>Título del álbum</v>
+        <v>Listas fijadas</v>
       </c>
       <c r="D221" t="str">
         <f>_xlfn.TRANSLATE($B221,$B$2,D$2)</f>
-        <v>Titre de l’album</v>
+        <v>Listes épinglées</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B222" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C222" t="str">
         <f>_xlfn.TRANSLATE($B222,$B$2,C$2)</f>
-        <v>Nombre artístico</v>
+        <v>Título del álbum</v>
       </c>
       <c r="D222" t="str">
         <f>_xlfn.TRANSLATE($B222,$B$2,D$2)</f>
-        <v>Nom de l’artiste</v>
+        <v>Titre de l’album</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B223" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C223" t="str">
         <f>_xlfn.TRANSLATE($B223,$B$2,C$2)</f>
-        <v>Mi lista de reproducción perfecta</v>
+        <v>Nombre artístico</v>
       </c>
       <c r="D223" t="str">
         <f>_xlfn.TRANSLATE($B223,$B$2,D$2)</f>
-        <v>Ma playlist parfaite</v>
+        <v>Nom de l’artiste</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B224" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C224" t="str">
         <f>_xlfn.TRANSLATE($B224,$B$2,C$2)</f>
-        <v>Título de la canción</v>
+        <v>Mi lista de reproducción perfecta</v>
       </c>
       <c r="D224" t="str">
         <f>_xlfn.TRANSLATE($B224,$B$2,D$2)</f>
-        <v>Titre de la chanson</v>
+        <v>Ma playlist parfaite</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B225" t="s">
-        <v>439</v>
-      </c>
-      <c r="C225" t="s">
-        <v>440</v>
+        <v>437</v>
+      </c>
+      <c r="C225" t="str">
+        <f>_xlfn.TRANSLATE($B225,$B$2,C$2)</f>
+        <v>Título de la canción</v>
       </c>
       <c r="D225" t="str">
         <f>_xlfn.TRANSLATE($B225,$B$2,D$2)</f>
-        <v>Jeu</v>
+        <v>Titre de la chanson</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="B226" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="C226" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="D226" t="str">
         <f>_xlfn.TRANSLATE($B226,$B$2,D$2)</f>
-        <v>Liste des jeux</v>
+        <v>Jeu</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B227" t="s">
-        <v>445</v>
-      </c>
-      <c r="C227" t="str">
-        <f>_xlfn.TRANSLATE($B227,$B$2,C$2)</f>
-        <v>Reproducir medios</v>
+        <v>442</v>
+      </c>
+      <c r="C227" t="s">
+        <v>443</v>
       </c>
       <c r="D227" t="str">
         <f>_xlfn.TRANSLATE($B227,$B$2,D$2)</f>
-        <v>Lire les médias</v>
+        <v>Liste des jeux</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B228" t="s">
-        <v>447</v>
-      </c>
-      <c r="C228" t="s">
-        <v>448</v>
+        <v>445</v>
+      </c>
+      <c r="C228" t="str">
+        <f>_xlfn.TRANSLATE($B228,$B$2,C$2)</f>
+        <v>Reproducir medios</v>
       </c>
       <c r="D228" t="str">
         <f>_xlfn.TRANSLATE($B228,$B$2,D$2)</f>
-        <v>À jouer à venir</v>
+        <v>Lire les médias</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="B229" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C229" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D229" t="str">
         <f>_xlfn.TRANSLATE($B229,$B$2,D$2)</f>
-        <v>Jouer la chanson</v>
+        <v>À jouer à venir</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="B230" t="s">
-        <v>453</v>
-      </c>
-      <c r="C230" t="str">
-        <f>_xlfn.TRANSLATE($B230,$B$2,C$2)</f>
-        <v>Listas de reproducción</v>
+        <v>450</v>
+      </c>
+      <c r="C230" t="s">
+        <v>451</v>
       </c>
       <c r="D230" t="str">
         <f>_xlfn.TRANSLATE($B230,$B$2,D$2)</f>
-        <v>Playlists</v>
+        <v>Jouer la chanson</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B231" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C231" t="str">
         <f>_xlfn.TRANSLATE($B231,$B$2,C$2)</f>
-        <v>Medios anteriores</v>
+        <v>Listas de reproducción</v>
       </c>
       <c r="D231" t="str">
         <f>_xlfn.TRANSLATE($B231,$B$2,D$2)</f>
-        <v>Médias précédents</v>
+        <v>Playlists</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B232" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C232" t="str">
         <f>_xlfn.TRANSLATE($B232,$B$2,C$2)</f>
-        <v>Cola</v>
+        <v>Medios anteriores</v>
       </c>
       <c r="D232" t="str">
         <f>_xlfn.TRANSLATE($B232,$B$2,D$2)</f>
-        <v>File d’attente</v>
+        <v>Médias précédents</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B233" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C233" t="str">
         <f>_xlfn.TRANSLATE($B233,$B$2,C$2)</f>
-        <v>Selecciones rápidas</v>
+        <v>Cola</v>
       </c>
       <c r="D233" t="str">
         <f>_xlfn.TRANSLATE($B233,$B$2,D$2)</f>
-        <v>Choix rapides</v>
+        <v>File d’attente</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B234" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C234" t="str">
         <f>_xlfn.TRANSLATE($B234,$B$2,C$2)</f>
-        <v>Radio</v>
+        <v>Selecciones rápidas</v>
       </c>
       <c r="D234" t="str">
         <f>_xlfn.TRANSLATE($B234,$B$2,D$2)</f>
-        <v>Radio</v>
+        <v>Choix rapides</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B235" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C235" t="str">
         <f>_xlfn.TRANSLATE($B235,$B$2,C$2)</f>
-        <v>No se han encontrado estaciones</v>
+        <v>Radio</v>
       </c>
       <c r="D235" t="str">
         <f>_xlfn.TRANSLATE($B235,$B$2,D$2)</f>
-        <v>Aucune station trouvée</v>
+        <v>Radio</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B236" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C236" t="str">
         <f>_xlfn.TRANSLATE($B236,$B$2,C$2)</f>
-        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
+        <v>No se han encontrado estaciones</v>
       </c>
       <c r="D236" t="str">
         <f>_xlfn.TRANSLATE($B236,$B$2,D$2)</f>
-        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
+        <v>Aucune station trouvée</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B237" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C237" t="str">
         <f>_xlfn.TRANSLATE($B237,$B$2,C$2)</f>
-        <v>Busca emisoras, géneros, países...</v>
+        <v>Desde samba brasileña hasta rock australiano, ¡busca y sintoniza tu siguiente ritmo favorito!</v>
       </c>
       <c r="D237" t="str">
         <f>_xlfn.TRANSLATE($B237,$B$2,D$2)</f>
-        <v>Recherche des stations, genres, pays...</v>
+        <v>De la samba brésilienne au rock australien, cherchez et écoutez votre prochain beat préféré !</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B238" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C238" t="str">
         <f>_xlfn.TRANSLATE($B238,$B$2,C$2)</f>
-        <v>Emisoras de radio</v>
+        <v>Busca emisoras, géneros, países...</v>
       </c>
       <c r="D238" t="str">
         <f>_xlfn.TRANSLATE($B238,$B$2,D$2)</f>
-        <v>Radio Stations</v>
+        <v>Recherche des stations, genres, pays...</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B239" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C239" t="str">
         <f>_xlfn.TRANSLATE($B239,$B$2,C$2)</f>
-        <v>Mezcla reciente</v>
+        <v>Emisoras de radio</v>
       </c>
       <c r="D239" t="str">
         <f>_xlfn.TRANSLATE($B239,$B$2,D$2)</f>
-        <v>Mix récent</v>
+        <v>Radio Stations</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B240" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="C240" t="str">
         <f>_xlfn.TRANSLATE($B240,$B$2,C$2)</f>
-        <v>Jugado recientemente</v>
+        <v>Mezcla reciente</v>
       </c>
       <c r="D240" t="str">
         <f>_xlfn.TRANSLATE($B240,$B$2,D$2)</f>
-        <v>Joué récemment</v>
+        <v>Mix récent</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B241" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C241" t="str">
         <f>_xlfn.TRANSLATE($B241,$B$2,C$2)</f>
@@ -6080,606 +6170,606 @@
       </c>
       <c r="D241" t="str">
         <f>_xlfn.TRANSLATE($B241,$B$2,D$2)</f>
-        <v>Récemment joué</v>
+        <v>Joué récemment</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B242" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="C242" t="str">
         <f>_xlfn.TRANSLATE($B242,$B$2,C$2)</f>
-        <v>Registro</v>
+        <v>Jugado recientemente</v>
       </c>
       <c r="D242" t="str">
         <f>_xlfn.TRANSLATE($B242,$B$2,D$2)</f>
-        <v>Registre</v>
+        <v>Récemment joué</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B243" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C243" t="str">
         <f>_xlfn.TRANSLATE($B243,$B$2,C$2)</f>
-        <v>Registrado</v>
+        <v>Registro</v>
       </c>
       <c r="D243" t="str">
         <f>_xlfn.TRANSLATE($B243,$B$2,D$2)</f>
-        <v>Enregistré</v>
+        <v>Registre</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B244" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C244" t="str">
         <f>_xlfn.TRANSLATE($B244,$B$2,C$2)</f>
-        <v>Registrando...</v>
+        <v>Registrado</v>
       </c>
       <c r="D244" t="str">
         <f>_xlfn.TRANSLATE($B244,$B$2,D$2)</f>
-        <v>Enregistrement...</v>
+        <v>Enregistré</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B245" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C245" t="str">
         <f>_xlfn.TRANSLATE($B245,$B$2,C$2)</f>
-        <v>Artistas relacionados</v>
+        <v>Registrando...</v>
       </c>
       <c r="D245" t="str">
         <f>_xlfn.TRANSLATE($B245,$B$2,D$2)</f>
-        <v>Artistes associés</v>
+        <v>Enregistrement...</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B246" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C246" t="str">
         <f>_xlfn.TRANSLATE($B246,$B$2,C$2)</f>
-        <v>Relajado</v>
+        <v>Artistas relacionados</v>
       </c>
       <c r="D246" t="str">
         <f>_xlfn.TRANSLATE($B246,$B$2,D$2)</f>
-        <v>Détendu</v>
+        <v>Artistes associés</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B247" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C247" t="str">
         <f>_xlfn.TRANSLATE($B247,$B$2,C$2)</f>
-        <v>Recuérdame</v>
+        <v>Relajado</v>
       </c>
       <c r="D247" t="str">
         <f>_xlfn.TRANSLATE($B247,$B$2,D$2)</f>
-        <v>Souviens-toi de moi</v>
+        <v>Détendu</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B248" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="C248" t="str">
         <f>_xlfn.TRANSLATE($B248,$B$2,C$2)</f>
-        <v>Eliminar de la biblioteca</v>
+        <v>Recuérdame</v>
       </c>
       <c r="D248" t="str">
         <f>_xlfn.TRANSLATE($B248,$B$2,D$2)</f>
-        <v>Retirer de la bibliothèque</v>
+        <v>Souviens-toi de moi</v>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B249" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C249" t="str">
         <f>_xlfn.TRANSLATE($B249,$B$2,C$2)</f>
-        <v>Quitar de me gusta</v>
+        <v>Eliminar de la biblioteca</v>
       </c>
       <c r="D249" t="str">
         <f>_xlfn.TRANSLATE($B249,$B$2,D$2)</f>
-        <v>Retirer de aimé</v>
+        <v>Retirer de la bibliothèque</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B250" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C250" t="str">
         <f>_xlfn.TRANSLATE($B250,$B$2,C$2)</f>
-        <v>Eliminar de la lista de reproducción</v>
+        <v>Quitar de me gusta</v>
       </c>
       <c r="D250" t="str">
         <f>_xlfn.TRANSLATE($B250,$B$2,D$2)</f>
-        <v>Supprimer de la playlist</v>
+        <v>Retirer de aimé</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B251" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C251" t="str">
         <f>_xlfn.TRANSLATE($B251,$B$2,C$2)</f>
-        <v>Eliminar de la cola</v>
+        <v>Eliminar de la lista de reproducción</v>
       </c>
       <c r="D251" t="str">
         <f>_xlfn.TRANSLATE($B251,$B$2,D$2)</f>
-        <v>Retirer de la file d’attente</v>
+        <v>Supprimer de la playlist</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="B252" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C252" t="str">
         <f>_xlfn.TRANSLATE($B252,$B$2,C$2)</f>
-        <v>Repite todo</v>
+        <v>Eliminar de la cola</v>
       </c>
       <c r="D252" t="str">
         <f>_xlfn.TRANSLATE($B252,$B$2,D$2)</f>
-        <v>Répétez tout</v>
+        <v>Retirer de la file d’attente</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B253" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C253" t="str">
         <f>_xlfn.TRANSLATE($B253,$B$2,C$2)</f>
-        <v>Repite una</v>
+        <v>Repite todo</v>
       </c>
       <c r="D253" t="str">
         <f>_xlfn.TRANSLATE($B253,$B$2,D$2)</f>
-        <v>Répétez-en un</v>
+        <v>Répétez tout</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B254" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C254" t="str">
         <f>_xlfn.TRANSLATE($B254,$B$2,C$2)</f>
-        <v>Repetir nueva contraseña</v>
+        <v>Repite una</v>
       </c>
       <c r="D254" t="str">
         <f>_xlfn.TRANSLATE($B254,$B$2,D$2)</f>
-        <v>Répéter le nouveau mot de passe</v>
+        <v>Répétez-en un</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B255" t="s">
-        <v>503</v>
-      </c>
-      <c r="C255" t="s">
-        <v>504</v>
+        <v>501</v>
+      </c>
+      <c r="C255" t="str">
+        <f>_xlfn.TRANSLATE($B255,$B$2,C$2)</f>
+        <v>Repetir nueva contraseña</v>
       </c>
       <c r="D255" t="str">
         <f>_xlfn.TRANSLATE($B255,$B$2,D$2)</f>
-        <v>Nouvelle tentative</v>
+        <v>Répéter le nouveau mot de passe</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B256" t="s">
-        <v>506</v>
-      </c>
-      <c r="C256" t="str">
-        <f>_xlfn.TRANSLATE($B256,$B$2,C$2)</f>
-        <v>Regreso a casa</v>
+        <v>503</v>
+      </c>
+      <c r="C256" t="s">
+        <v>504</v>
       </c>
       <c r="D256" t="str">
         <f>_xlfn.TRANSLATE($B256,$B$2,D$2)</f>
-        <v>Retour à la maison</v>
+        <v>Nouvelle tentative</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B257" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C257" t="str">
         <f>_xlfn.TRANSLATE($B257,$B$2,C$2)</f>
-        <v>Guardando...</v>
+        <v>Regreso a casa</v>
       </c>
       <c r="D257" t="str">
         <f>_xlfn.TRANSLATE($B257,$B$2,D$2)</f>
-        <v>Sauver...</v>
+        <v>Retour à la maison</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B258" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C258" t="str">
         <f>_xlfn.TRANSLATE($B258,$B$2,C$2)</f>
-        <v>Búsqueda</v>
+        <v>Guardando...</v>
       </c>
       <c r="D258" t="str">
         <f>_xlfn.TRANSLATE($B258,$B$2,D$2)</f>
-        <v>Recherche</v>
+        <v>Sauver...</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B259" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C259" t="str">
         <f>_xlfn.TRANSLATE($B259,$B$2,C$2)</f>
-        <v>Busca artistas, canciones, álbumes...</v>
+        <v>Búsqueda</v>
       </c>
       <c r="D259" t="str">
         <f>_xlfn.TRANSLATE($B259,$B$2,D$2)</f>
-        <v>Cherche des artistes, des chansons, des albums...</v>
+        <v>Recherche</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B260" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C260" t="str">
         <f>_xlfn.TRANSLATE($B260,$B$2,C$2)</f>
-        <v>Parece que el silencio también es música...</v>
+        <v>Busca artistas, canciones, álbumes...</v>
       </c>
       <c r="D260" t="str">
         <f>_xlfn.TRANSLATE($B260,$B$2,D$2)</f>
-        <v>Il semble que le silence soit aussi de la musique...</v>
+        <v>Cherche des artistes, des chansons, des albums...</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B261" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C261" t="str">
         <f>_xlfn.TRANSLATE($B261,$B$2,C$2)</f>
-        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
+        <v>Parece que el silencio también es música...</v>
       </c>
       <c r="D261" t="str">
         <f>_xlfn.TRANSLATE($B261,$B$2,D$2)</f>
-        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
+        <v>Il semble que le silence soit aussi de la musique...</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B262" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C262" t="str">
         <f>_xlfn.TRANSLATE($B262,$B$2,C$2)</f>
-        <v>Buscar en la biblioteca</v>
+        <v>Pero no es muy entretenido, ¿verdad? ¡Busca algo que escuchar!</v>
       </c>
       <c r="D262" t="str">
         <f>_xlfn.TRANSLATE($B262,$B$2,D$2)</f>
-        <v>Recherche dans la bibliothèque</v>
+        <v>Mais ce n’est pas très divertissant, n’est-ce pas ? Trouvez quelque chose à écouter !</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B263" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C263" t="str">
         <f>_xlfn.TRANSLATE($B263,$B$2,C$2)</f>
-        <v>Usuarios de búsqueda</v>
+        <v>Buscar en la biblioteca</v>
       </c>
       <c r="D263" t="str">
         <f>_xlfn.TRANSLATE($B263,$B$2,D$2)</f>
-        <v>Rechercher les utilisateurs</v>
+        <v>Recherche dans la bibliothèque</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B264" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C264" t="str">
         <f>_xlfn.TRANSLATE($B264,$B$2,C$2)</f>
-        <v>Enviar canción actual</v>
+        <v>Usuarios de búsqueda</v>
       </c>
       <c r="D264" t="str">
         <f>_xlfn.TRANSLATE($B264,$B$2,D$2)</f>
-        <v>Envoyer la chanson actuelle</v>
+        <v>Rechercher les utilisateurs</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B265" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C265" t="str">
         <f>_xlfn.TRANSLATE($B265,$B$2,C$2)</f>
-        <v>Septiembre</v>
+        <v>Enviar canción actual</v>
       </c>
       <c r="D265" t="str">
         <f>_xlfn.TRANSLATE($B265,$B$2,D$2)</f>
-        <v>Septembre</v>
+        <v>Envoyer la chanson actuelle</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B266" t="s">
-        <v>113</v>
+        <v>524</v>
       </c>
       <c r="C266" t="str">
         <f>_xlfn.TRANSLATE($B266,$B$2,C$2)</f>
-        <v>Escenarios</v>
+        <v>Septiembre</v>
       </c>
       <c r="D266" t="str">
         <f>_xlfn.TRANSLATE($B266,$B$2,D$2)</f>
-        <v>Décors</v>
+        <v>Septembre</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B267" t="s">
-        <v>527</v>
+        <v>113</v>
       </c>
       <c r="C267" t="str">
         <f>_xlfn.TRANSLATE($B267,$B$2,C$2)</f>
-        <v>Compartir canción</v>
+        <v>Escenarios</v>
       </c>
       <c r="D267" t="str">
         <f>_xlfn.TRANSLATE($B267,$B$2,D$2)</f>
-        <v>Partager la chanson</v>
+        <v>Décors</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B268" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C268" t="str">
         <f>_xlfn.TRANSLATE($B268,$B$2,C$2)</f>
-        <v>Canciones compartidas para ti</v>
+        <v>Compartir canción</v>
       </c>
       <c r="D268" t="str">
         <f>_xlfn.TRANSLATE($B268,$B$2,D$2)</f>
-        <v>Chansons partagées pour vous</v>
+        <v>Partager la chanson</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B269" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C269" t="str">
         <f>_xlfn.TRANSLATE($B269,$B$2,C$2)</f>
-        <v>Compartido desde</v>
+        <v>Canciones compartidas para ti</v>
       </c>
       <c r="D269" t="str">
         <f>_xlfn.TRANSLATE($B269,$B$2,D$2)</f>
-        <v>Partagé depuis</v>
+        <v>Chansons partagées pour vous</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B270" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C270" t="str">
         <f>_xlfn.TRANSLATE($B270,$B$2,C$2)</f>
-        <v>Mostrando datos de</v>
+        <v>Compartido desde</v>
       </c>
       <c r="D270" t="str">
         <f>_xlfn.TRANSLATE($B270,$B$2,D$2)</f>
-        <v>Affichage des données de</v>
+        <v>Partagé depuis</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B271" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C271" t="str">
         <f>_xlfn.TRANSLATE($B271,$B$2,C$2)</f>
-        <v>Regístrate</v>
+        <v>Mostrando datos de</v>
       </c>
       <c r="D271" t="str">
         <f>_xlfn.TRANSLATE($B271,$B$2,D$2)</f>
-        <v>Inscrivez-vous</v>
+        <v>Affichage des données de</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B272" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C272" t="str">
         <f>_xlfn.TRANSLATE($B272,$B$2,C$2)</f>
-        <v>Canción</v>
+        <v>Regístrate</v>
       </c>
       <c r="D272" t="str">
         <f>_xlfn.TRANSLATE($B272,$B$2,D$2)</f>
-        <v>Chanson</v>
+        <v>Inscrivez-vous</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B273" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C273" t="str">
         <f>_xlfn.TRANSLATE($B273,$B$2,C$2)</f>
-        <v>Canciones</v>
+        <v>Canción</v>
       </c>
       <c r="D273" t="str">
         <f>_xlfn.TRANSLATE($B273,$B$2,D$2)</f>
-        <v>Chansons</v>
+        <v>Chanson</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B274" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C274" t="str">
         <f>_xlfn.TRANSLATE($B274,$B$2,C$2)</f>
-        <v>Canciones Solo para ti</v>
+        <v>Canciones</v>
       </c>
       <c r="D274" t="str">
         <f>_xlfn.TRANSLATE($B274,$B$2,D$2)</f>
-        <v>Chansons juste pour toi</v>
+        <v>Chansons</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B275" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C275" t="str">
         <f>_xlfn.TRANSLATE($B275,$B$2,C$2)</f>
-        <v>Canciones de</v>
+        <v>Canciones Solo para ti</v>
       </c>
       <c r="D275" t="str">
         <f>_xlfn.TRANSLATE($B275,$B$2,D$2)</f>
-        <v>Chansons de</v>
+        <v>Chansons juste pour toi</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B276" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C276" t="str">
         <f>_xlfn.TRANSLATE($B276,$B$2,C$2)</f>
-        <v>Canciones escuchadas</v>
+        <v>Canciones de</v>
       </c>
       <c r="D276" t="str">
         <f>_xlfn.TRANSLATE($B276,$B$2,D$2)</f>
-        <v>Chansons écoutées</v>
+        <v>Chansons de</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B277" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C277" t="str">
         <f>_xlfn.TRANSLATE($B277,$B$2,C$2)</f>
-        <v>Empezando...</v>
+        <v>Canciones escuchadas</v>
       </c>
       <c r="D277" t="str">
         <f>_xlfn.TRANSLATE($B277,$B$2,D$2)</f>
-        <v>Commencer...</v>
+        <v>Chansons écoutées</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="B278" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C278" t="str">
         <f>_xlfn.TRANSLATE($B278,$B$2,C$2)</f>
-        <v>Estadísticas</v>
+        <v>Empezando...</v>
       </c>
       <c r="D278" t="str">
         <f>_xlfn.TRANSLATE($B278,$B$2,D$2)</f>
-        <v>Statistiques</v>
+        <v>Commencer...</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B279" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C279" t="str">
         <f>_xlfn.TRANSLATE($B279,$B$2,C$2)</f>
@@ -6692,417 +6782,449 @@
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B280" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C280" t="str">
         <f>_xlfn.TRANSLATE($B280,$B$2,C$2)</f>
-        <v>¡Para</v>
+        <v>Estadísticas</v>
       </c>
       <c r="D280" t="str">
         <f>_xlfn.TRANSLATE($B280,$B$2,D$2)</f>
-        <v>Arrête</v>
+        <v>Statistiques</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B281" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C281" t="str">
         <f>_xlfn.TRANSLATE($B281,$B$2,C$2)</f>
-        <v>a</v>
+        <v>¡Para</v>
       </c>
       <c r="D281" t="str">
         <f>_xlfn.TRANSLATE($B281,$B$2,D$2)</f>
-        <v>à</v>
+        <v>Arrête</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B282" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C282" t="str">
         <f>_xlfn.TRANSLATE($B282,$B$2,C$2)</f>
-        <v>ToDo</v>
+        <v>a</v>
       </c>
       <c r="D282" t="str">
         <f>_xlfn.TRANSLATE($B282,$B$2,D$2)</f>
-        <v>ToDo</v>
+        <v>à</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B283" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C283" t="str">
         <f>_xlfn.TRANSLATE($B283,$B$2,C$2)</f>
-        <v>Álbumes destacados</v>
+        <v>ToDo</v>
       </c>
       <c r="D283" t="str">
         <f>_xlfn.TRANSLATE($B283,$B$2,D$2)</f>
-        <v>Albums phares</v>
+        <v>ToDo</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B284" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C284" t="str">
         <f>_xlfn.TRANSLATE($B284,$B$2,C$2)</f>
-        <v>Canciones principales</v>
+        <v>Álbumes destacados</v>
       </c>
       <c r="D284" t="str">
         <f>_xlfn.TRANSLATE($B284,$B$2,D$2)</f>
-        <v>Meilleures chansons</v>
+        <v>Albums phares</v>
       </c>
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B285" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C285" t="str">
         <f>_xlfn.TRANSLATE($B285,$B$2,C$2)</f>
-        <v>Desclavar</v>
+        <v>Canciones principales</v>
       </c>
       <c r="D285" t="str">
         <f>_xlfn.TRANSLATE($B285,$B$2,D$2)</f>
-        <v>Détacher</v>
+        <v>Meilleures chansons</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>564</v>
+        <v>615</v>
       </c>
       <c r="B286" t="s">
-        <v>565</v>
+        <v>616</v>
       </c>
       <c r="C286" t="str">
         <f>_xlfn.TRANSLATE($B286,$B$2,C$2)</f>
-        <v>Desregistrar</v>
+        <v>Vídeos principales</v>
       </c>
       <c r="D286" t="str">
         <f>_xlfn.TRANSLATE($B286,$B$2,D$2)</f>
-        <v>Désinscription</v>
+        <v>Meilleures vidéos</v>
       </c>
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="B287" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="C287" t="str">
         <f>_xlfn.TRANSLATE($B287,$B$2,C$2)</f>
-        <v>No registrado</v>
+        <v>Desclavar</v>
       </c>
       <c r="D287" t="str">
         <f>_xlfn.TRANSLATE($B287,$B$2,D$2)</f>
-        <v>Non enregistré</v>
+        <v>Détacher</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="B288" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="C288" t="str">
         <f>_xlfn.TRANSLATE($B288,$B$2,C$2)</f>
-        <v>Dejar de registrarse...</v>
+        <v>Desregistrar</v>
       </c>
       <c r="D288" t="str">
         <f>_xlfn.TRANSLATE($B288,$B$2,D$2)</f>
-        <v>Désenregistrement...</v>
+        <v>Désinscription</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="B289" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="C289" t="str">
         <f>_xlfn.TRANSLATE($B289,$B$2,C$2)</f>
-        <v>Actualización</v>
+        <v>No registrado</v>
       </c>
       <c r="D289" t="str">
         <f>_xlfn.TRANSLATE($B289,$B$2,D$2)</f>
-        <v>Mise à jour</v>
+        <v>Non enregistré</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="B290" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="C290" t="str">
         <f>_xlfn.TRANSLATE($B290,$B$2,C$2)</f>
-        <v>Actualizando...</v>
+        <v>Dejar de registrarse...</v>
       </c>
       <c r="D290" t="str">
         <f>_xlfn.TRANSLATE($B290,$B$2,D$2)</f>
-        <v>Mise à jour...</v>
+        <v>Désenregistrement...</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="B291" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C291" t="str">
         <f>_xlfn.TRANSLATE($B291,$B$2,C$2)</f>
-        <v>Subida</v>
+        <v>Actualización</v>
       </c>
       <c r="D291" t="str">
         <f>_xlfn.TRANSLATE($B291,$B$2,D$2)</f>
-        <v>Téléverser</v>
+        <v>Mise à jour</v>
       </c>
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="B292" t="s">
-        <v>137</v>
+        <v>573</v>
       </c>
       <c r="C292" t="str">
         <f>_xlfn.TRANSLATE($B292,$B$2,C$2)</f>
-        <v>Usuario</v>
+        <v>Actualizando...</v>
       </c>
       <c r="D292" t="str">
         <f>_xlfn.TRANSLATE($B292,$B$2,D$2)</f>
-        <v>Utilisateur</v>
+        <v>Mise à jour...</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="B293" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="C293" t="str">
         <f>_xlfn.TRANSLATE($B293,$B$2,C$2)</f>
-        <v>Se requiere nombre de usuario y contraseña</v>
+        <v>Subida</v>
       </c>
       <c r="D293" t="str">
         <f>_xlfn.TRANSLATE($B293,$B$2,D$2)</f>
-        <v>Nom d’utilisateur et mot de passe requis</v>
+        <v>Téléverser</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B294" t="s">
-        <v>580</v>
+        <v>137</v>
       </c>
       <c r="C294" t="str">
         <f>_xlfn.TRANSLATE($B294,$B$2,C$2)</f>
-        <v>Configuración de usuario</v>
+        <v>Usuario</v>
       </c>
       <c r="D294" t="str">
         <f>_xlfn.TRANSLATE($B294,$B$2,D$2)</f>
-        <v>Paramètres utilisateur</v>
+        <v>Utilisateur</v>
       </c>
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="B295" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="C295" t="str">
         <f>_xlfn.TRANSLATE($B295,$B$2,C$2)</f>
-        <v>Estadísticas de usuario</v>
+        <v>Se requiere nombre de usuario y contraseña</v>
       </c>
       <c r="D295" t="str">
         <f>_xlfn.TRANSLATE($B295,$B$2,D$2)</f>
-        <v>Statistiques des utilisateurs</v>
+        <v>Nom d’utilisateur et mot de passe requis</v>
       </c>
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="B296" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="C296" t="str">
         <f>_xlfn.TRANSLATE($B296,$B$2,C$2)</f>
-        <v>Nombre de usuario</v>
+        <v>Configuración de usuario</v>
       </c>
       <c r="D296" t="str">
         <f>_xlfn.TRANSLATE($B296,$B$2,D$2)</f>
-        <v>Nom d’utilisateur</v>
+        <v>Paramètres utilisateur</v>
       </c>
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="B297" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="C297" t="str">
         <f>_xlfn.TRANSLATE($B297,$B$2,C$2)</f>
-        <v>Usuarios y amigos</v>
+        <v>Estadísticas de usuario</v>
       </c>
       <c r="D297" t="str">
         <f>_xlfn.TRANSLATE($B297,$B$2,D$2)</f>
-        <v>Utilisateurs et amis</v>
+        <v>Statistiques des utilisateurs</v>
       </c>
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B298" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="C298" t="str">
         <f>_xlfn.TRANSLATE($B298,$B$2,C$2)</f>
-        <v>Lista de usuarios</v>
+        <v>Nombre de usuario</v>
       </c>
       <c r="D298" t="str">
         <f>_xlfn.TRANSLATE($B298,$B$2,D$2)</f>
-        <v>Liste des utilisateurs</v>
+        <v>Nom d’utilisateur</v>
       </c>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="B299" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="C299" t="str">
         <f>_xlfn.TRANSLATE($B299,$B$2,C$2)</f>
-        <v>Vídeos</v>
+        <v>Usuarios y amigos</v>
       </c>
       <c r="D299" t="str">
         <f>_xlfn.TRANSLATE($B299,$B$2,D$2)</f>
-        <v>Vidéos</v>
+        <v>Utilisateurs et amis</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>607</v>
+        <v>587</v>
       </c>
       <c r="B300" t="s">
-        <v>612</v>
+        <v>588</v>
       </c>
       <c r="C300" t="str">
         <f>_xlfn.TRANSLATE($B300,$B$2,C$2)</f>
-        <v>Esperando a que se configure la cola</v>
+        <v>Lista de usuarios</v>
       </c>
       <c r="D300" t="str">
         <f>_xlfn.TRANSLATE($B300,$B$2,D$2)</f>
-        <v>En attente de la mise en place de la file d’attente</v>
+        <v>Liste des utilisateurs</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B301" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C301" t="str">
         <f>_xlfn.TRANSLATE($B301,$B$2,C$2)</f>
-        <v>También puede que te interese</v>
+        <v>Vídeos</v>
       </c>
       <c r="D301" t="str">
         <f>_xlfn.TRANSLATE($B301,$B$2,D$2)</f>
-        <v>Ça pourrait aussi te plaire</v>
+        <v>Vidéos</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>593</v>
+        <v>607</v>
       </c>
       <c r="B302" t="s">
-        <v>594</v>
+        <v>612</v>
       </c>
       <c r="C302" t="str">
         <f>_xlfn.TRANSLATE($B302,$B$2,C$2)</f>
-        <v>Tu</v>
+        <v>Esperando a que se configure la cola</v>
       </c>
       <c r="D302" t="str">
-        <f>_xlfn.TRANSLATE($B302,$B$2,D$2)</f>
-        <v>Votre</v>
+        <f ca="1">_xlfn.TRANSLATE($B302,$B$2,D$2)</f>
+        <v>En attente de la mise en place de la file d’attente</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="B303" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="C303" t="str">
         <f>_xlfn.TRANSLATE($B303,$B$2,C$2)</f>
-        <v>Tus álbumes y listas de reproducción</v>
+        <v>También puede que te interese</v>
       </c>
       <c r="D303" t="str">
         <f>_xlfn.TRANSLATE($B303,$B$2,D$2)</f>
-        <v>Vos albums et playlists</v>
+        <v>Ça pourrait aussi te plaire</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="B304" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="C304" t="str">
-        <f>_xlfn.TRANSLATE($B304,$B$2,C$2)</f>
-        <v>Tu mezcla</v>
+        <f ca="1">_xlfn.TRANSLATE($B304,$B$2,C$2)</f>
+        <v>Tu</v>
       </c>
       <c r="D304" t="str">
-        <f>_xlfn.TRANSLATE($B304,$B$2,D$2)</f>
-        <v>Votre Mix</v>
+        <f ca="1">_xlfn.TRANSLATE($B304,$B$2,D$2)</f>
+        <v>Votre</v>
       </c>
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
+        <v>595</v>
+      </c>
+      <c r="B305" t="s">
+        <v>596</v>
+      </c>
+      <c r="C305" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B305,$B$2,C$2)</f>
+        <v>Tus álbumes y listas de reproducción</v>
+      </c>
+      <c r="D305" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B305,$B$2,D$2)</f>
+        <v>Vos albums et playlists</v>
+      </c>
+    </row>
+    <row r="306" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>597</v>
+      </c>
+      <c r="B306" t="s">
+        <v>598</v>
+      </c>
+      <c r="C306" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B306,$B$2,C$2)</f>
+        <v>Tu mezcla</v>
+      </c>
+      <c r="D306" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B306,$B$2,D$2)</f>
+        <v>Votre Mix</v>
+      </c>
+    </row>
+    <row r="307" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
         <v>599</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B307" t="s">
         <v>600</v>
       </c>
-      <c r="C305" t="str">
-        <f>_xlfn.TRANSLATE($B305,$B$2,C$2)</f>
+      <c r="C307" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B307,$B$2,C$2)</f>
         <v>Vídeos de YouTube</v>
       </c>
-      <c r="D305" t="str">
-        <f>_xlfn.TRANSLATE($B305,$B$2,D$2)</f>
+      <c r="D307" t="str">
+        <f ca="1">_xlfn.TRANSLATE($B307,$B$2,D$2)</f>
         <v>Vidéos YouTube</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance media upload functionality with image support for songs and videos
- Updated upload endpoints to accept image files for songs and videos.
- Modified data models to include artist names, disc numbers, and track numbers.
- Implemented streaming responses for audio and video files with range support.
- Added new utility functions for extracting media duration using ffprobe.
- Refactored frontend upload components to handle image file selection and submission.
- Introduced new vocabulary strings for upload actions and hints.
- Improved error handling and response parsing in HTTP methods.
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D310" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D329" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D307"/>
   <sortState ref="A3:D307">
     <sortCondition ref="A2:A307"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D310"/>
+  <dimension ref="A1:D329"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6655,6 +6655,386 @@
         <v/>
       </c>
     </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>UPLOAD_ACTION</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Upload</t>
+        </is>
+      </c>
+      <c r="C311">
+        <f>_xlfn.TRANSLATE($B311,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D311">
+        <f>_xlfn.TRANSLATE($B311,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>UPLOAD_ADD_MORE</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Add More</t>
+        </is>
+      </c>
+      <c r="C312">
+        <f>_xlfn.TRANSLATE($B312,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D312">
+        <f>_xlfn.TRANSLATE($B312,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>UPLOAD_ALBUM</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Album</t>
+        </is>
+      </c>
+      <c r="C313">
+        <f>_xlfn.TRANSLATE($B313,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D313">
+        <f>_xlfn.TRANSLATE($B313,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>UPLOAD_ALBUM_TITLE</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Album title</t>
+        </is>
+      </c>
+      <c r="C314">
+        <f>_xlfn.TRANSLATE($B314,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D314">
+        <f>_xlfn.TRANSLATE($B314,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>UPLOAD_ARTIST_FIELD</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+      <c r="C315">
+        <f>_xlfn.TRANSLATE($B315,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D315">
+        <f>_xlfn.TRANSLATE($B315,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>UPLOAD_BROWSE</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>or browse files</t>
+        </is>
+      </c>
+      <c r="C316">
+        <f>_xlfn.TRANSLATE($B316,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D316">
+        <f>_xlfn.TRANSLATE($B316,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>UPLOAD_COVER_HINT</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Add cover image</t>
+        </is>
+      </c>
+      <c r="C317">
+        <f>_xlfn.TRANSLATE($B317,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D317">
+        <f>_xlfn.TRANSLATE($B317,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>UPLOAD_DROP_ZONE</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Drop your files here</t>
+        </is>
+      </c>
+      <c r="C318">
+        <f>_xlfn.TRANSLATE($B318,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D318">
+        <f>_xlfn.TRANSLATE($B318,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>UPLOAD_ERROR</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Upload error</t>
+        </is>
+      </c>
+      <c r="C319">
+        <f>_xlfn.TRANSLATE($B319,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D319">
+        <f>_xlfn.TRANSLATE($B319,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>UPLOAD_FILES_READY</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>files ready</t>
+        </is>
+      </c>
+      <c r="C320">
+        <f>_xlfn.TRANSLATE($B320,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D320">
+        <f>_xlfn.TRANSLATE($B320,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>UPLOAD_HINT</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Upload your music files</t>
+        </is>
+      </c>
+      <c r="C321">
+        <f>_xlfn.TRANSLATE($B321,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D321">
+        <f>_xlfn.TRANSLATE($B321,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>UPLOAD_IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Uploading…</t>
+        </is>
+      </c>
+      <c r="C322">
+        <f>_xlfn.TRANSLATE($B322,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D322">
+        <f>_xlfn.TRANSLATE($B322,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>UPLOAD_NO_FILES</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>No files</t>
+        </is>
+      </c>
+      <c r="C323">
+        <f>_xlfn.TRANSLATE($B323,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D323">
+        <f>_xlfn.TRANSLATE($B323,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>UPLOAD_SONGS</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Songs</t>
+        </is>
+      </c>
+      <c r="C324">
+        <f>_xlfn.TRANSLATE($B324,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D324">
+        <f>_xlfn.TRANSLATE($B324,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>UPLOAD_TITLE</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Upload</t>
+        </is>
+      </c>
+      <c r="C325">
+        <f>_xlfn.TRANSLATE($B325,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D325">
+        <f>_xlfn.TRANSLATE($B325,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>UPLOAD_TITLE_FIELD</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C326">
+        <f>_xlfn.TRANSLATE($B326,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D326">
+        <f>_xlfn.TRANSLATE($B326,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>UPLOAD_TRACK_FIELD</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="C327">
+        <f>_xlfn.TRANSLATE($B327,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D327">
+        <f>_xlfn.TRANSLATE($B327,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>UPLOAD_VIDEO</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C328">
+        <f>_xlfn.TRANSLATE($B328,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D328">
+        <f>_xlfn.TRANSLATE($B328,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>UPLOAD_VIDEO_TITLE</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Video title</t>
+        </is>
+      </c>
+      <c r="C329">
+        <f>_xlfn.TRANSLATE($B329,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D329">
+        <f>_xlfn.TRANSLATE($B329,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Implement delete media functionality with UI integration and vocabulary updates
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D329" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D332" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D307"/>
   <sortState ref="A3:D307">
     <sortCondition ref="A2:A307"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D329"/>
+  <dimension ref="A1:D332"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7035,6 +7035,66 @@
         <v/>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>DELETE_ERROR</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Delete error</t>
+        </is>
+      </c>
+      <c r="C330">
+        <f>_xlfn.TRANSLATE($B330,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D330">
+        <f>_xlfn.TRANSLATE($B330,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Delete</t>
+        </is>
+      </c>
+      <c r="C331">
+        <f>_xlfn.TRANSLATE($B331,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D331">
+        <f>_xlfn.TRANSLATE($B331,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>DELETE_SUCCESS</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Delete success</t>
+        </is>
+      </c>
+      <c r="C332">
+        <f>_xlfn.TRANSLATE($B332,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D332">
+        <f>_xlfn.TRANSLATE($B332,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: add Listen Together and Sharing functionality
- Implement ListenTogetherManager for managing listen-together sessions, including fetching sessions, inviting users, joining/leaving sessions, and syncing media.
- Create SharingManager for handling shared media items, including fetching inbox and sent items, sharing media, and marking items as seen.
- Enhance WebSocketManager to register handlers for friend activity and listen-together sync messages.
- Introduce new DTOs for friend activities, sharing media, listen-together sessions, and related requests/responses.
- Extend BaseHttp with new API methods for friend management, listen-together sessions, and media sharing.
- Update webSocketMessages to include new message types for friend activity and listen-together sync.
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="225" yWindow="3840" windowWidth="22650" windowHeight="14325" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D333"/>
+  <dimension ref="A1:D359"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7115,6 +7115,526 @@
         <v/>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C334">
+        <f>_xlfn.TRANSLATE($B$334,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D334">
+        <f>_xlfn.TRANSLATE($B$334,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>FRIENDS_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C335">
+        <f>_xlfn.TRANSLATE($B$335,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D335">
+        <f>_xlfn.TRANSLATE($B$335,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="C336">
+        <f>_xlfn.TRANSLATE($B$336,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D336">
+        <f>_xlfn.TRANSLATE($B$336,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>FRIENDS_PARTY</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C337">
+        <f>_xlfn.TRANSLATE($B$337,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D337">
+        <f>_xlfn.TRANSLATE($B$337,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>FRIENDS_RANKS</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Ranks</t>
+        </is>
+      </c>
+      <c r="C338">
+        <f>_xlfn.TRANSLATE($B$338,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D338">
+        <f>_xlfn.TRANSLATE($B$338,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>FRIENDS_SEARCH_PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Search users...</t>
+        </is>
+      </c>
+      <c r="C339">
+        <f>_xlfn.TRANSLATE($B$339,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D339">
+        <f>_xlfn.TRANSLATE($B$339,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>No friends yet</t>
+        </is>
+      </c>
+      <c r="C340">
+        <f>_xlfn.TRANSLATE($B$340,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D340">
+        <f>_xlfn.TRANSLATE($B$340,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>FRIENDS_PENDING</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C341">
+        <f>_xlfn.TRANSLATE($B$341,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D341">
+        <f>_xlfn.TRANSLATE($B$341,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>FRIENDS_ADD</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C342">
+        <f>_xlfn.TRANSLATE($B$342,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D342">
+        <f>_xlfn.TRANSLATE($B$342,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>FRIENDS_ALREADY_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Already friends</t>
+        </is>
+      </c>
+      <c r="C343">
+        <f>_xlfn.TRANSLATE($B$343,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D343">
+        <f>_xlfn.TRANSLATE($B$343,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>FRIENDS_FRIEND_REQUESTS</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Friend Requests</t>
+        </is>
+      </c>
+      <c r="C344">
+        <f>_xlfn.TRANSLATE($B$344,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D344">
+        <f>_xlfn.TRANSLATE($B$344,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>No activity yet</t>
+        </is>
+      </c>
+      <c r="C345">
+        <f>_xlfn.TRANSLATE($B$345,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D345">
+        <f>_xlfn.TRANSLATE($B$345,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>FRIENDS_ONLINE</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="C346">
+        <f>_xlfn.TRANSLATE($B$346,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D346">
+        <f>_xlfn.TRANSLATE($B$346,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>FRIENDS_OFFLINE</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C347">
+        <f>_xlfn.TRANSLATE($B$347,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D347">
+        <f>_xlfn.TRANSLATE($B$347,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>FRIENDS_REMOVE</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="C348">
+        <f>_xlfn.TRANSLATE($B$348,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D348">
+        <f>_xlfn.TRANSLATE($B$348,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>FRIENDS_INVITE</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Invite</t>
+        </is>
+      </c>
+      <c r="C349">
+        <f>_xlfn.TRANSLATE($B$349,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D349">
+        <f>_xlfn.TRANSLATE($B$349,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>FRIENDS_LEAVE</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Leave Session</t>
+        </is>
+      </c>
+      <c r="C350">
+        <f>_xlfn.TRANSLATE($B$350,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D350">
+        <f>_xlfn.TRANSLATE($B$350,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_SESSIONS</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>No active sessions</t>
+        </is>
+      </c>
+      <c r="C351">
+        <f>_xlfn.TRANSLATE($B$351,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D351">
+        <f>_xlfn.TRANSLATE($B$351,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACTIVE</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C352">
+        <f>_xlfn.TRANSLATE($B$352,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D352">
+        <f>_xlfn.TRANSLATE($B$352,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>FRIENDS_JOIN</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="C353">
+        <f>_xlfn.TRANSLATE($B$353,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D353">
+        <f>_xlfn.TRANSLATE($B$353,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>FRIENDS_LEADERBOARD</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Leaderboard</t>
+        </is>
+      </c>
+      <c r="C354">
+        <f>_xlfn.TRANSLATE($B$354,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D354">
+        <f>_xlfn.TRANSLATE($B$354,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="C355">
+        <f>_xlfn.TRANSLATE($B$355,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D355">
+        <f>_xlfn.TRANSLATE($B$355,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE_SENT</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="C356">
+        <f>_xlfn.TRANSLATE($B$356,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D356">
+        <f>_xlfn.TRANSLATE($B$356,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_SHARED</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>No shared media yet</t>
+        </is>
+      </c>
+      <c r="C357">
+        <f>_xlfn.TRANSLATE($B$357,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D357">
+        <f>_xlfn.TRANSLATE($B$357,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>FRIENDS_LIVE</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C358">
+        <f>_xlfn.TRANSLATE($B$358,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D358">
+        <f>_xlfn.TRANSLATE($B$358,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>FRIENDS_MY_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>My Friends</t>
+        </is>
+      </c>
+      <c r="C359">
+        <f>_xlfn.TRANSLATE($B$359,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D359">
+        <f>_xlfn.TRANSLATE($B$359,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: add vocabulary keys for friends feature, fix AResult patterns, clean up imports and webSocket handlers
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="225" yWindow="3840" windowWidth="22650" windowHeight="14325" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3465" yWindow="3465" windowWidth="38700" windowHeight="15285" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
@@ -124,8 +124,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D333" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A2:D307"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D403" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A2:D333"/>
   <sortState ref="A3:D307">
     <sortCondition ref="A2:A307"/>
   </sortState>
@@ -432,8 +432,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D359"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:D403"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="42.7109375" customWidth="1" min="2" max="2"/>
@@ -7118,520 +7118,1400 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>FRIENDS_ACTIVITY</t>
+          <t>JUST_NOW</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Just now</t>
         </is>
       </c>
       <c r="C334">
-        <f>_xlfn.TRANSLATE($B$334,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B334,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D334">
-        <f>_xlfn.TRANSLATE($B$334,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B334,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>FRIENDS_FRIENDS</t>
+          <t>NOTHING_PLAYING_YET</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Friends</t>
+          <t>Nothing playing yet</t>
         </is>
       </c>
       <c r="C335">
-        <f>_xlfn.TRANSLATE($B$335,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B335,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D335">
-        <f>_xlfn.TRANSLATE($B$335,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B335,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>FRIENDS_SHARE</t>
+          <t>FRIENDS_ACTIVITY_WILL_APPEAR</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Share</t>
+          <t>Your friends' activity will appear here</t>
         </is>
       </c>
       <c r="C336">
-        <f>_xlfn.TRANSLATE($B$336,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B336,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D336">
-        <f>_xlfn.TRANSLATE($B$336,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B336,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>FRIENDS_PARTY</t>
+          <t>NOW_PLAYING</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Party</t>
+          <t>Now Playing</t>
         </is>
       </c>
       <c r="C337">
-        <f>_xlfn.TRANSLATE($B$337,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B337,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D337">
-        <f>_xlfn.TRANSLATE($B$337,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B337,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>FRIENDS_RANKS</t>
+          <t>RECENT</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Ranks</t>
+          <t>Recent</t>
         </is>
       </c>
       <c r="C338">
-        <f>_xlfn.TRANSLATE($B$338,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B338,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D338">
-        <f>_xlfn.TRANSLATE($B$338,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B338,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>FRIENDS_SEARCH_PLACEHOLDER</t>
+          <t>FRIENDS_LISTENING_NOW</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Search users...</t>
+          <t>{count} friends listening now</t>
         </is>
       </c>
       <c r="C339">
-        <f>_xlfn.TRANSLATE($B$339,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B339,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D339">
-        <f>_xlfn.TRANSLATE($B$339,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B339,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>FRIENDS_NO_FRIENDS</t>
+          <t>SEE_WHAT_WORLD_LISTENING</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>No friends yet</t>
+          <t>See what the world is listening to</t>
         </is>
       </c>
       <c r="C340">
-        <f>_xlfn.TRANSLATE($B$340,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B340,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D340">
-        <f>_xlfn.TRANSLATE($B$340,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B340,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>FRIENDS_PENDING</t>
+          <t>FRIEND_REQUEST</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Friend Request</t>
         </is>
       </c>
       <c r="C341">
-        <f>_xlfn.TRANSLATE($B$341,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B341,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D341">
-        <f>_xlfn.TRANSLATE($B$341,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B341,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>FRIENDS_ADD</t>
+          <t>FRIEND_REQUESTS</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>Friend Requests</t>
         </is>
       </c>
       <c r="C342">
-        <f>_xlfn.TRANSLATE($B$342,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B342,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D342">
-        <f>_xlfn.TRANSLATE($B$342,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B342,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>FRIENDS_ALREADY_FRIENDS</t>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Already friends</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C343">
-        <f>_xlfn.TRANSLATE($B$343,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B343,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D343">
-        <f>_xlfn.TRANSLATE($B$343,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B343,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>FRIENDS_FRIEND_REQUESTS</t>
+          <t>LISTENING_WITH</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Friend Requests</t>
+          <t>Listening with</t>
         </is>
       </c>
       <c r="C344">
-        <f>_xlfn.TRANSLATE($B$344,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B344,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D344">
-        <f>_xlfn.TRANSLATE($B$344,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B344,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>FRIENDS_NO_ACTIVITY</t>
+          <t>LEAVE_SESSION</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>No activity yet</t>
+          <t>Leave Session</t>
         </is>
       </c>
       <c r="C345">
-        <f>_xlfn.TRANSLATE($B$345,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B345,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D345">
-        <f>_xlfn.TRANSLATE($B$345,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B345,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>FRIENDS_ONLINE</t>
+          <t>ACTIVE_SESSIONS</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Active Sessions</t>
         </is>
       </c>
       <c r="C346">
-        <f>_xlfn.TRANSLATE($B$346,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B346,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D346">
-        <f>_xlfn.TRANSLATE($B$346,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B346,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>FRIENDS_OFFLINE</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="C347">
-        <f>_xlfn.TRANSLATE($B$347,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B347,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D347">
-        <f>_xlfn.TRANSLATE($B$347,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B347,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>FRIENDS_REMOVE</t>
+          <t>ENDED</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Remove</t>
+          <t>Ended</t>
         </is>
       </c>
       <c r="C348">
-        <f>_xlfn.TRANSLATE($B$348,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B348,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D348">
-        <f>_xlfn.TRANSLATE($B$348,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B348,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>FRIENDS_INVITE</t>
+          <t>JOIN</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Invite</t>
+          <t>Join</t>
         </is>
       </c>
       <c r="C349">
-        <f>_xlfn.TRANSLATE($B$349,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B349,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D349">
-        <f>_xlfn.TRANSLATE($B$349,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B349,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>FRIENDS_LEAVE</t>
+          <t>NO_ACTIVE_SESSIONS</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Leave Session</t>
+          <t>No active sessions</t>
         </is>
       </c>
       <c r="C350">
-        <f>_xlfn.TRANSLATE($B$350,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B350,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D350">
-        <f>_xlfn.TRANSLATE($B$350,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B350,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>FRIENDS_NO_SESSIONS</t>
+          <t>INVITE_FRIEND_LISTEN</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>No active sessions</t>
+          <t>Invite a friend to listen together in real time</t>
         </is>
       </c>
       <c r="C351">
-        <f>_xlfn.TRANSLATE($B$351,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B351,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D351">
-        <f>_xlfn.TRANSLATE($B$351,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B351,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>FRIENDS_ACTIVE</t>
+          <t>INVITE_A_FRIEND</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Invite a friend</t>
         </is>
       </c>
       <c r="C352">
-        <f>_xlfn.TRANSLATE($B$352,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B352,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D352">
-        <f>_xlfn.TRANSLATE($B$352,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B352,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>FRIENDS_JOIN</t>
+          <t>RECEIVED</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Join</t>
+          <t>Received</t>
         </is>
       </c>
       <c r="C353">
-        <f>_xlfn.TRANSLATE($B$353,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B353,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D353">
-        <f>_xlfn.TRANSLATE($B$353,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B353,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>FRIENDS_LEADERBOARD</t>
+          <t>SENT</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Leaderboard</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="C354">
-        <f>_xlfn.TRANSLATE($B$354,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B354,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D354">
-        <f>_xlfn.TRANSLATE($B$354,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B354,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>FRIENDS_SHARE_RECEIVED</t>
+          <t>NO_SHARED_MEDIA_YET</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>No shared media yet</t>
         </is>
       </c>
       <c r="C355">
-        <f>_xlfn.TRANSLATE($B$355,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B355,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D355">
-        <f>_xlfn.TRANSLATE($B$355,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B355,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>FRIENDS_SHARE_SENT</t>
+          <t>NOTHING_SHARED_YET</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Nothing shared yet</t>
         </is>
       </c>
       <c r="C356">
-        <f>_xlfn.TRANSLATE($B$356,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B356,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D356">
-        <f>_xlfn.TRANSLATE($B$356,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B356,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>FRIENDS_NO_SHARED</t>
+          <t>FROM_USER</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>No shared media yet</t>
+          <t>from {username}</t>
         </is>
       </c>
       <c r="C357">
-        <f>_xlfn.TRANSLATE($B$357,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B357,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D357">
-        <f>_xlfn.TRANSLATE($B$357,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B357,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>FRIENDS_LIVE</t>
+          <t>TO_USER</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>to {username}</t>
         </is>
       </c>
       <c r="C358">
-        <f>_xlfn.TRANSLATE($B$358,$B$2,C$2)</f>
+        <f>_xlfn.TRANSLATE($B358,$B$2,C$2)</f>
         <v/>
       </c>
       <c r="D358">
-        <f>_xlfn.TRANSLATE($B$358,$B$2,D$2)</f>
+        <f>_xlfn.TRANSLATE($B358,$B$2,D$2)</f>
         <v/>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
+          <t>LEVEL</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C359">
+        <f>_xlfn.TRANSLATE($B359,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D359">
+        <f>_xlfn.TRANSLATE($B359,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="C360">
+        <f>_xlfn.TRANSLATE($B360,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D360">
+        <f>_xlfn.TRANSLATE($B360,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>LEADERBOARD</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Leaderboard</t>
+        </is>
+      </c>
+      <c r="C361">
+        <f>_xlfn.TRANSLATE($B361,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D361">
+        <f>_xlfn.TRANSLATE($B361,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>RESULTS</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="C362">
+        <f>_xlfn.TRANSLATE($B363,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D362">
+        <f>_xlfn.TRANSLATE($B363,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>NO_USERS_FOUND</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>No users found</t>
+        </is>
+      </c>
+      <c r="C363">
+        <f>_xlfn.TRANSLATE($B364,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D363">
+        <f>_xlfn.TRANSLATE($B364,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>ALREADY_FRIENDS_LABEL</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C364">
+        <f>_xlfn.TRANSLATE($B365,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D364">
+        <f>_xlfn.TRANSLATE($B365,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>REQUEST_SENT_LABEL</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Request sent</t>
+        </is>
+      </c>
+      <c r="C365">
+        <f>_xlfn.TRANSLATE($B366,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D365">
+        <f>_xlfn.TRANSLATE($B366,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>ADD_FRIEND</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C366">
+        <f>_xlfn.TRANSLATE($B367,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D366">
+        <f>_xlfn.TRANSLATE($B367,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>MY_FRIENDS_TITLE</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>My Friends</t>
+        </is>
+      </c>
+      <c r="C367">
+        <f>_xlfn.TRANSLATE($B368,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D367">
+        <f>_xlfn.TRANSLATE($B368,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>NO_FRIENDS_YET</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>No friends yet</t>
+        </is>
+      </c>
+      <c r="C368">
+        <f>_xlfn.TRANSLATE($B369,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D368">
+        <f>_xlfn.TRANSLATE($B369,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>SEARCH_ABOVE_FIND</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Search above to find people</t>
+        </is>
+      </c>
+      <c r="C369">
+        <f>_xlfn.TRANSLATE($B370,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D369">
+        <f>_xlfn.TRANSLATE($B370,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>ONLINE_LABEL</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="C370">
+        <f>_xlfn.TRANSLATE($B371,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D370">
+        <f>_xlfn.TRANSLATE($B371,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>OFFLINE_LABEL</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C371">
+        <f>_xlfn.TRANSLATE($B372,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D371">
+        <f>_xlfn.TRANSLATE($B372,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>REMOVE_FRIEND</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Remove friend</t>
+        </is>
+      </c>
+      <c r="C372">
+        <f>_xlfn.TRANSLATE($B373,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D372">
+        <f>_xlfn.TRANSLATE($B373,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>SHARE</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="C373">
+        <f>_xlfn.TRANSLATE($B376,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D373">
+        <f>_xlfn.TRANSLATE($B376,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>TIME_MINUTES</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>{n}m</t>
+        </is>
+      </c>
+      <c r="C374">
+        <f>_xlfn.TRANSLATE($B377,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D374">
+        <f>_xlfn.TRANSLATE($B377,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>TIME_HOURS</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>{n}h</t>
+        </is>
+      </c>
+      <c r="C375">
+        <f>_xlfn.TRANSLATE($B378,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D375">
+        <f>_xlfn.TRANSLATE($B378,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>TIME_DAYS</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>{n}d</t>
+        </is>
+      </c>
+      <c r="C376">
+        <f>_xlfn.TRANSLATE($B379,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D376">
+        <f>_xlfn.TRANSLATE($B379,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>LISTENING_LIVE</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C377">
+        <f>_xlfn.TRANSLATE($B380,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D377">
+        <f>_xlfn.TRANSLATE($B380,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C378">
+        <f>_xlfn.TRANSLATE($B381,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D378">
+        <f>_xlfn.TRANSLATE($B381,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>FRIENDS_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C379">
+        <f>_xlfn.TRANSLATE($B382,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D379">
+        <f>_xlfn.TRANSLATE($B382,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="C380">
+        <f>_xlfn.TRANSLATE($B383,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D380">
+        <f>_xlfn.TRANSLATE($B383,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>FRIENDS_PARTY</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C381">
+        <f>_xlfn.TRANSLATE($B384,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D381">
+        <f>_xlfn.TRANSLATE($B384,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>FRIENDS_RANKS</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Ranks</t>
+        </is>
+      </c>
+      <c r="C382">
+        <f>_xlfn.TRANSLATE($B385,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D382">
+        <f>_xlfn.TRANSLATE($B385,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>FRIENDS_SEARCH_PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Search users...</t>
+        </is>
+      </c>
+      <c r="C383">
+        <f>_xlfn.TRANSLATE($B386,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D383">
+        <f>_xlfn.TRANSLATE($B386,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>No friends yet</t>
+        </is>
+      </c>
+      <c r="C384">
+        <f>_xlfn.TRANSLATE($B387,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D384">
+        <f>_xlfn.TRANSLATE($B387,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>FRIENDS_PENDING</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C385">
+        <f>_xlfn.TRANSLATE($B388,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D385">
+        <f>_xlfn.TRANSLATE($B388,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>FRIENDS_ADD</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="C386">
+        <f>_xlfn.TRANSLATE($B389,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D386">
+        <f>_xlfn.TRANSLATE($B389,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>FRIENDS_ALREADY_FRIENDS</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Already friends</t>
+        </is>
+      </c>
+      <c r="C387">
+        <f>_xlfn.TRANSLATE($B390,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D387">
+        <f>_xlfn.TRANSLATE($B390,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>FRIENDS_FRIEND_REQUESTS</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Friend Requests</t>
+        </is>
+      </c>
+      <c r="C388">
+        <f>_xlfn.TRANSLATE($B391,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D388">
+        <f>_xlfn.TRANSLATE($B391,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_ACTIVITY</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>No activity</t>
+        </is>
+      </c>
+      <c r="C389">
+        <f>_xlfn.TRANSLATE($B392,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D389">
+        <f>_xlfn.TRANSLATE($B392,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>FRIENDS_ONLINE</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="C390">
+        <f>_xlfn.TRANSLATE($B393,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D390">
+        <f>_xlfn.TRANSLATE($B393,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>FRIENDS_OFFLINE</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C391">
+        <f>_xlfn.TRANSLATE($B394,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D391">
+        <f>_xlfn.TRANSLATE($B394,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>FRIENDS_REMOVE</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="C392">
+        <f>_xlfn.TRANSLATE($B395,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D392">
+        <f>_xlfn.TRANSLATE($B395,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>FRIENDS_INVITE</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Invite</t>
+        </is>
+      </c>
+      <c r="C393">
+        <f>_xlfn.TRANSLATE($B396,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D393">
+        <f>_xlfn.TRANSLATE($B396,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>FRIENDS_LEAVE</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Leave</t>
+        </is>
+      </c>
+      <c r="C394">
+        <f>_xlfn.TRANSLATE($B397,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D394">
+        <f>_xlfn.TRANSLATE($B397,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_SESSIONS</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>No sessions</t>
+        </is>
+      </c>
+      <c r="C395">
+        <f>_xlfn.TRANSLATE($B398,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D395">
+        <f>_xlfn.TRANSLATE($B398,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>FRIENDS_ACTIVE</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C396">
+        <f>_xlfn.TRANSLATE($B399,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D396">
+        <f>_xlfn.TRANSLATE($B399,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>FRIENDS_JOIN</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="C397">
+        <f>_xlfn.TRANSLATE($B400,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D397">
+        <f>_xlfn.TRANSLATE($B400,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>FRIENDS_LEADERBOARD</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Leaderboard</t>
+        </is>
+      </c>
+      <c r="C398">
+        <f>_xlfn.TRANSLATE($B401,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D398">
+        <f>_xlfn.TRANSLATE($B401,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="C399">
+        <f>_xlfn.TRANSLATE($B402,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D399">
+        <f>_xlfn.TRANSLATE($B402,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>FRIENDS_SHARE_SENT</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="C400">
+        <f>_xlfn.TRANSLATE($B403,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D400">
+        <f>_xlfn.TRANSLATE($B403,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>FRIENDS_NO_SHARED</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>No shared media yet</t>
+        </is>
+      </c>
+      <c r="C401">
+        <f>_xlfn.TRANSLATE($B404,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D401">
+        <f>_xlfn.TRANSLATE($B404,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>FRIENDS_LIVE</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="C402">
+        <f>_xlfn.TRANSLATE($B405,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D402">
+        <f>_xlfn.TRANSLATE($B405,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
           <t>FRIENDS_MY_FRIENDS</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B403" t="inlineStr">
         <is>
           <t>My Friends</t>
         </is>
       </c>
-      <c r="C359">
-        <f>_xlfn.TRANSLATE($B$359,$B$2,C$2)</f>
-        <v/>
-      </c>
-      <c r="D359">
-        <f>_xlfn.TRANSLATE($B$359,$B$2,D$2)</f>
+      <c r="C403">
+        <f>_xlfn.TRANSLATE($B406,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D403">
+        <f>_xlfn.TRANSLATE($B406,$B$2,D$2)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixes in adding spotify url
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D354" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D355" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D351"/>
   <sortState ref="A3:D351">
     <sortCondition ref="A2:A351"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D354"/>
+  <dimension ref="A1:D355"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7536,6 +7536,26 @@
         <v/>
       </c>
     </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>NO_MEDIA_FOUND</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>No media found</t>
+        </is>
+      </c>
+      <c r="C355">
+        <f>_xlfn.TRANSLATE($B355,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D355">
+        <f>_xlfn.TRANSLATE($B355,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Fixed spotify scrapper access layer
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D355" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D357" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D351"/>
   <sortState ref="A3:D351">
     <sortCondition ref="A2:A351"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D355"/>
+  <dimension ref="A1:D357"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7556,6 +7556,46 @@
         <v/>
       </c>
     </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>ADDED_TO_LIBRARY</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Added to library</t>
+        </is>
+      </c>
+      <c r="C356">
+        <f>_xlfn.TRANSLATE($B356,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D356">
+        <f>_xlfn.TRANSLATE($B356,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>ADDING_MEDIA_TO_LIBRARY</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Adding media to library</t>
+        </is>
+      </c>
+      <c r="C357">
+        <f>_xlfn.TRANSLATE($B357,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D357">
+        <f>_xlfn.TRANSLATE($B357,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add download actions for search results and update vocabulary
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4335" yWindow="2475" windowWidth="38700" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D368" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D370" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D361"/>
   <sortState ref="A3:D361">
     <sortCondition ref="A2:A361"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D368"/>
+  <dimension ref="A1:D370"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7816,6 +7816,46 @@
         <v/>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>DOWNLOAD_TO_SERVER</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Download to Server</t>
+        </is>
+      </c>
+      <c r="C369">
+        <f>_xlfn.TRANSLATE($B369,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D369">
+        <f>_xlfn.TRANSLATE($B369,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>DOWNLOAD_AND_ADD_TO_LIBRARY</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Download and Add to Library</t>
+        </is>
+      </c>
+      <c r="C370">
+        <f>_xlfn.TRANSLATE($B370,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D370">
+        <f>_xlfn.TRANSLATE($B370,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Removed media type repeated lists
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D394" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D400" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D389"/>
   <sortState ref="A3:D386">
     <sortCondition ref="A2:A386"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D393"/>
+  <dimension ref="A1:D400"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8314,6 +8314,126 @@
         <v/>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_TITLE</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Admin search</t>
+        </is>
+      </c>
+      <c r="C395">
+        <f>_xlfn.TRANSLATE($B395,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D395">
+        <f>_xlfn.TRANSLATE($B395,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_SUBTITLE</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Search all media in database</t>
+        </is>
+      </c>
+      <c r="C396">
+        <f>_xlfn.TRANSLATE($B396,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D396">
+        <f>_xlfn.TRANSLATE($B396,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Type anything...</t>
+        </is>
+      </c>
+      <c r="C397">
+        <f>_xlfn.TRANSLATE($B397,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D397">
+        <f>_xlfn.TRANSLATE($B397,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_RESULTS</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="C398">
+        <f>_xlfn.TRANSLATE($B398,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D398">
+        <f>_xlfn.TRANSLATE($B398,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_NO_RESULTS</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>No results</t>
+        </is>
+      </c>
+      <c r="C399">
+        <f>_xlfn.TRANSLATE($B399,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D399">
+        <f>_xlfn.TRANSLATE($B399,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>ADMIN_SEARCH_PROMPT</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Type anything to start searching</t>
+        </is>
+      </c>
+      <c r="C400">
+        <f>_xlfn.TRANSLATE($B400,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D400">
+        <f>_xlfn.TRANSLATE($B400,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add ADMIN_TAB_SEARCH to vocabulary interface
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D400" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table2" displayName="Table2" ref="A2:D401" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A2:D389"/>
   <sortState ref="A3:D386">
     <sortCondition ref="A2:A386"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D400"/>
+  <dimension ref="A1:D401"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8434,6 +8434,26 @@
         <v/>
       </c>
     </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>ADMIN_TAB_SEARCH</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="C401">
+        <f>_xlfn.TRANSLATE($B401,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D401">
+        <f>_xlfn.TRANSLATE($B401,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Implement recommendation system with Last.fm integration
- Added RecommendationAccess for fetching similar songs based on co-occurrence and user listening history.
- Created recommendationController to handle API requests for personalized song recommendations.
- Developed LastfmClient to interact with Last.fm API for discovering similar tracks.
- Introduced recommendation framework to manage user-specific song recommendations and playlist suggestions.
- Added SongListResponse model for structured response of song recommendations.
- Enhanced mobile and web components to display related songs and handle user interactions for downloading and queuing songs.
- Implemented SimilarSongsAction for creating playlists of similar songs based on user selection.
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D410"/>
+  <dimension ref="A1:D413"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8634,6 +8634,66 @@
         <v/>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>PLAYER_RELATED_TITLE</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Related songs</t>
+        </is>
+      </c>
+      <c r="C411">
+        <f>_xlfn.TRANSLATE($B411,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D411">
+        <f>_xlfn.TRANSLATE($B411,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>PLAYER_RELATED_EMPTY</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>No related songs yet</t>
+        </is>
+      </c>
+      <c r="C412">
+        <f>_xlfn.TRANSLATE($B412,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D412">
+        <f>_xlfn.TRANSLATE($B412,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>PLAYER_DISCOVER_TITLE</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Discover</t>
+        </is>
+      </c>
+      <c r="C413">
+        <f>_xlfn.TRANSLATE($B413,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D413">
+        <f>_xlfn.TRANSLATE($B413,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add recommendations feature with personalized and playlist-based suggestions
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D413"/>
+  <dimension ref="A1:D415"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8694,6 +8694,46 @@
         <v/>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>FOR_YOU</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>For you</t>
+        </is>
+      </c>
+      <c r="C414">
+        <f>_xlfn.TRANSLATE($B414,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D414">
+        <f>_xlfn.TRANSLATE($B414,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>RECOMMENDED_FOR_THIS_PLAYLIST</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Recommended for this playlist</t>
+        </is>
+      </c>
+      <c r="C415">
+        <f>_xlfn.TRANSLATE($B415,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D415">
+        <f>_xlfn.TRANSLATE($B415,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add new vocabulary entries for recommendations feature
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D415"/>
+  <dimension ref="A1:D419"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8734,6 +8734,86 @@
         <v/>
       </c>
     </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>NO_SIMILAR_SONGS_FOUND</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>No similar songs found</t>
+        </is>
+      </c>
+      <c r="C416">
+        <f>_xlfn.TRANSLATE($B416,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D416">
+        <f>_xlfn.TRANSLATE($B416,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>SIMILAR_TO_SONG_PLAYLIST_PREFIX</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Similar to</t>
+        </is>
+      </c>
+      <c r="C417">
+        <f>_xlfn.TRANSLATE($B417,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D417">
+        <f>_xlfn.TRANSLATE($B417,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>SIMILAR_SONGS_PLAYLIST_CREATED</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Playlist created</t>
+        </is>
+      </c>
+      <c r="C418">
+        <f>_xlfn.TRANSLATE($B418,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D418">
+        <f>_xlfn.TRANSLATE($B418,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>SIMILAR_TO_SONG</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Similar to this song</t>
+        </is>
+      </c>
+      <c r="C419">
+        <f>_xlfn.TRANSLATE($B419,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D419">
+        <f>_xlfn.TRANSLATE($B419,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Implement autoplay feature with recommendations for queue end
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D419"/>
+  <dimension ref="A1:D420"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8814,6 +8814,26 @@
         <v/>
       </c>
     </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>AUTOPLAY_ON</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Autoplay on</t>
+        </is>
+      </c>
+      <c r="C420">
+        <f>_xlfn.TRANSLATE($B420,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D420">
+        <f>_xlfn.TRANSLATE($B420,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add recommendations feature with song-seeded suggestions and personalized picks
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D420"/>
+  <dimension ref="A1:D421"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8834,6 +8834,26 @@
         <v/>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>RECOMMENDED_SONGS</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Recommended songs</t>
+        </is>
+      </c>
+      <c r="C421">
+        <f>_xlfn.TRANSLATE($B421,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D421">
+        <f>_xlfn.TRANSLATE($B421,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix: optimize offline song download process with bounded concurrency and caching for albums/playlists
</commit_message>
<xml_diff>
--- a/Vocabulary.xlsx
+++ b/Vocabulary.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D410"/>
+  <dimension ref="A1:D415"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="42.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8454,6 +8454,7 @@
         <v/>
       </c>
     </row>
+    <row r="401"/>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
@@ -8631,6 +8632,106 @@
       </c>
       <c r="D410">
         <f>_xlfn.TRANSLATE($B410,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>OFFLINE</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="C411">
+        <f>_xlfn.TRANSLATE(B411,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D411">
+        <f>_xlfn.TRANSLATE(B411,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>NO_OFFLINE_MEDIA</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>No offline media</t>
+        </is>
+      </c>
+      <c r="C412">
+        <f>_xlfn.TRANSLATE(B412,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D412">
+        <f>_xlfn.TRANSLATE(B412,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>OFFLINE_DOWNLOAD_SUMMARY</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>saved offline</t>
+        </is>
+      </c>
+      <c r="C413">
+        <f>_xlfn.TRANSLATE(B413,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D413">
+        <f>_xlfn.TRANSLATE(B413,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>OFFLINE_DOWNLOAD_FAILED_SUMMARY</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>failed to save offline</t>
+        </is>
+      </c>
+      <c r="C414">
+        <f>_xlfn.TRANSLATE(B414,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D414">
+        <f>_xlfn.TRANSLATE(B414,$B$2,D$2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>OFFLINE_REMOVE_SUMMARY</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>removed from offline</t>
+        </is>
+      </c>
+      <c r="C415">
+        <f>_xlfn.TRANSLATE(B415,$B$2,C$2)</f>
+        <v/>
+      </c>
+      <c r="D415">
+        <f>_xlfn.TRANSLATE(B415,$B$2,D$2)</f>
         <v/>
       </c>
     </row>

</xml_diff>